<commit_message>
Actualizo tableros (2026-09-13 07:44) - 133 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="90">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="98">
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>1494</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>382</v>
+        <v>404</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>382</v>
+        <v>404</v>
       </c>
     </row>
     <row r="121">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="123">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="125">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="128">
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="133">
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="134">
@@ -5297,12 +5297,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="136">
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5389,7 +5389,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137">
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="138">
@@ -5441,12 +5441,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139">
@@ -5585,12 +5585,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5605,7 +5605,7 @@
         </is>
       </c>
       <c r="H142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143">
@@ -5621,12 +5621,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5657,12 +5657,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5729,12 +5729,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5801,12 +5801,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -5821,7 +5821,7 @@
         </is>
       </c>
       <c r="H148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -5837,12 +5837,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -5873,12 +5873,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
@@ -5909,12 +5909,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
@@ -5945,12 +5945,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
@@ -5981,12 +5981,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E153" t="inlineStr"/>
@@ -6017,12 +6017,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
@@ -6053,12 +6053,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -6089,12 +6089,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -6125,12 +6125,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -6161,12 +6161,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -6197,12 +6197,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -6233,12 +6233,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -11660,7 +11660,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="109">
@@ -11748,7 +11748,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="110">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="124">
@@ -12484,7 +12484,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="126">
@@ -12836,7 +12836,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="134">
@@ -13764,7 +13764,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>63</v>
+        <v>85</v>
       </c>
     </row>
     <row r="151">
@@ -13896,7 +13896,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="154">
@@ -13940,7 +13940,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="155">
@@ -15044,7 +15044,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>1494</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="176">
@@ -15176,7 +15176,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="179">
@@ -15396,7 +15396,7 @@
         </is>
       </c>
       <c r="L183" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="184">
@@ -15828,7 +15828,7 @@
         </is>
       </c>
       <c r="L192" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="193">
@@ -17508,7 +17508,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223">
@@ -17684,7 +17684,7 @@
         </is>
       </c>
       <c r="L226" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="227">
@@ -17728,7 +17728,7 @@
         </is>
       </c>
       <c r="L227" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="228">
@@ -17816,7 +17816,7 @@
         </is>
       </c>
       <c r="L229" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-14 07:44) - 133 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="92">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="98">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>1506</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="119">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>356</v>
+        <v>352</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="123">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>271</v>
+        <v>260</v>
       </c>
     </row>
     <row r="124">
@@ -6732,7 +6732,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
@@ -7084,7 +7084,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -8420,7 +8420,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
@@ -11484,7 +11484,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
@@ -11572,7 +11572,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="106">
@@ -12836,7 +12836,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="134">
@@ -12980,7 +12980,7 @@
         </is>
       </c>
       <c r="L136" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="137">
@@ -13596,7 +13596,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>292</v>
+        <v>276</v>
       </c>
     </row>
     <row r="148">
@@ -13940,7 +13940,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="155">
@@ -14028,7 +14028,7 @@
         </is>
       </c>
       <c r="L156" t="n">
-        <v>271</v>
+        <v>260</v>
       </c>
     </row>
     <row r="157">
@@ -14172,7 +14172,7 @@
         </is>
       </c>
       <c r="L159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -14732,7 +14732,7 @@
         </is>
       </c>
       <c r="L169" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="170">
@@ -14788,7 +14788,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="171">
@@ -15044,7 +15044,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>1506</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="176">
@@ -15132,7 +15132,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>356</v>
+        <v>352</v>
       </c>
     </row>
     <row r="178">
@@ -15176,7 +15176,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="179">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-16 07:37) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31">
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="47">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50">
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2473,12 +2473,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2617,12 +2617,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2725,12 +2725,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2797,12 +2797,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2833,12 +2833,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2869,12 +2869,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -2905,12 +2905,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -2941,12 +2941,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="82">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="87">
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="88">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89">
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="92">
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="95">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="99">
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=09e9193a-f463-498d-9e90-493d77f30de4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4325,12 +4325,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=09e9193a-f463-498d-9e90-493d77f30de4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>416</v>
+        <v>429</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>416</v>
+        <v>429</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="119">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="123">
@@ -4901,12 +4901,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="124">
@@ -4937,12 +4937,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125">
@@ -4973,12 +4973,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="128">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="129">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134">
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
@@ -6300,7 +6300,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10">
@@ -6476,7 +6476,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14">
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16">
@@ -6652,7 +6652,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18">
@@ -6696,7 +6696,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
@@ -9104,7 +9104,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
@@ -9284,7 +9284,7 @@
         </is>
       </c>
       <c r="L68" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="69">
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="93">
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="100">
@@ -11008,7 +11008,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="103">
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="105">
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="106">
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="107">
@@ -11228,7 +11228,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108">
@@ -11316,7 +11316,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -11656,7 +11656,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="117">
@@ -11876,7 +11876,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="122">
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="124">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="129">
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="133">
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>260</v>
+        <v>248</v>
       </c>
     </row>
     <row r="146">
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>97</v>
+        <v>110</v>
       </c>
     </row>
     <row r="149">
@@ -13332,7 +13332,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="151">
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="152">
@@ -13464,7 +13464,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="154">
@@ -14392,7 +14392,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171">
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="176">
@@ -14956,7 +14956,7 @@
         </is>
       </c>
       <c r="L182" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="183">
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="215">
@@ -16768,7 +16768,7 @@
         </is>
       </c>
       <c r="L215" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="216">
@@ -16856,7 +16856,7 @@
         </is>
       </c>
       <c r="L217" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="218">
@@ -16900,7 +16900,7 @@
         </is>
       </c>
       <c r="L218" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-17 07:37) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30">
@@ -1537,12 +1537,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CONTROL DE COSTOS</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>CONTROL DE COSTOS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="47">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="50">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="51">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="82">
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="88">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="89">
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="96">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="98">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="100">
@@ -4073,12 +4073,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101">
@@ -4109,12 +4109,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="103">
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4309,7 +4309,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>429</v>
+        <v>437</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>429</v>
+        <v>437</v>
       </c>
     </row>
     <row r="117">
@@ -4829,12 +4829,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4865,12 +4865,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="123">
@@ -4901,12 +4901,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="124">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="125">
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="126">
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="129">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="130">
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="131">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="134">
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -6476,7 +6476,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14">
@@ -6652,7 +6652,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
@@ -6740,7 +6740,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20">
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44">
@@ -8804,7 +8804,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59">
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93">
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="100">
@@ -11008,7 +11008,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="103">
@@ -11052,7 +11052,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="105">
@@ -11316,7 +11316,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="110">
@@ -11656,7 +11656,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="117">
@@ -11832,7 +11832,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="121">
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="124">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="132">
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="133">
@@ -12852,7 +12852,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="142">
@@ -12964,7 +12964,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="144">
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>248</v>
+        <v>220</v>
       </c>
     </row>
     <row r="146">
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="149">
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="152">
@@ -14392,7 +14392,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171">
@@ -14656,7 +14656,7 @@
         </is>
       </c>
       <c r="L176" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="177">
@@ -14956,7 +14956,7 @@
         </is>
       </c>
       <c r="L182" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="183">
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215">
@@ -16768,7 +16768,7 @@
         </is>
       </c>
       <c r="L215" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="216">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-18 07:37) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CONTROL DE COSTOS</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CONTROL DE COSTOS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41">
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47">
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56">
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57">
@@ -2725,12 +2725,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="89">
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="97">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="110">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>437</v>
+        <v>453</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>437</v>
+        <v>453</v>
       </c>
     </row>
     <row r="117">
@@ -4685,12 +4685,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6afd1ddb-25f2-4631-bf59-fbaceff88e1b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="118">
@@ -4721,12 +4721,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6afd1ddb-25f2-4631-bf59-fbaceff88e1b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>246</v>
+        <v>252</v>
       </c>
     </row>
     <row r="119">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="122">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="130">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="131">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134">
@@ -5992,7 +5992,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
@@ -6300,7 +6300,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10">
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38">
@@ -7856,7 +7856,7 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
@@ -8972,7 +8972,7 @@
         </is>
       </c>
       <c r="L61" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62">
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="93">
@@ -10604,7 +10604,7 @@
         </is>
       </c>
       <c r="L93" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="94">
@@ -11008,7 +11008,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="103">
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="107">
@@ -11228,7 +11228,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="108">
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="124">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="129">
@@ -12272,7 +12272,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="131">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="132">
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="149">
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="152">
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="176">
@@ -14956,7 +14956,7 @@
         </is>
       </c>
       <c r="L182" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="183">
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="215">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-19 07:38) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1537,12 +1537,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34">
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40">
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -2617,12 +2617,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -2725,12 +2725,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="87">
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92">
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="93">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>142</v>
+        <v>149</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="99">
@@ -4109,12 +4109,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="110">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="111">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="118">
@@ -4793,12 +4793,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=bdfe582a-c303-4732-b9b7-2390e04aa58e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4829,12 +4829,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=bdfe582a-c303-4732-b9b7-2390e04aa58e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="122">
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="129">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="130">
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="131">
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="132">
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -6300,7 +6300,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10">
@@ -6344,7 +6344,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -6696,7 +6696,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
@@ -7900,7 +7900,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="106">
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="107">
@@ -11228,7 +11228,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="108">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -11656,7 +11656,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="117">
@@ -11876,7 +11876,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="122">
@@ -11920,7 +11920,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="123">
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>142</v>
+        <v>149</v>
       </c>
     </row>
     <row r="124">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="129">
@@ -12272,7 +12272,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="131">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="132">
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="149">
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="152">
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="176">
@@ -14656,7 +14656,7 @@
         </is>
       </c>
       <c r="L176" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="177">
@@ -14956,7 +14956,7 @@
         </is>
       </c>
       <c r="L182" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="183">
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="215">
@@ -16768,7 +16768,7 @@
         </is>
       </c>
       <c r="L215" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="216">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-20 07:38) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2725,12 +2725,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83">
@@ -3605,12 +3605,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88">
@@ -3641,12 +3641,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="89">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="99">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>456</v>
+        <v>475</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>456</v>
+        <v>475</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="122">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="124">
@@ -4937,12 +4937,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="125">
@@ -4973,12 +4973,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="127">
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="129">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="130">
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="132">
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="135">
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5389,7 +5389,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="137">
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
@@ -5441,12 +5441,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5477,12 +5477,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5513,12 +5513,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5657,12 +5657,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5729,12 +5729,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5801,12 +5801,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -6652,7 +6652,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44">
@@ -8076,7 +8076,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -8804,7 +8804,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59">
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68">
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="105">
@@ -11656,7 +11656,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="117">
@@ -11876,7 +11876,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="122">
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="124">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="129">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="132">
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="133">
@@ -12404,7 +12404,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134">
@@ -12628,7 +12628,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="138">
@@ -12964,7 +12964,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="144">
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>220</v>
+        <v>202</v>
       </c>
     </row>
     <row r="146">
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>137</v>
+        <v>156</v>
       </c>
     </row>
     <row r="149">
@@ -13332,7 +13332,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="151">
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="152">
@@ -13464,7 +13464,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="154">
@@ -13552,7 +13552,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="156">
@@ -14224,7 +14224,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="168">
@@ -14480,7 +14480,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="173">
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="176">
@@ -14956,7 +14956,7 @@
         </is>
       </c>
       <c r="L182" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="183">
@@ -15964,7 +15964,7 @@
         </is>
       </c>
       <c r="L200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -16356,7 +16356,7 @@
         </is>
       </c>
       <c r="L207" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208">
@@ -16468,7 +16468,7 @@
         </is>
       </c>
       <c r="L209" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="210">
@@ -16680,7 +16680,7 @@
         </is>
       </c>
       <c r="L213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="215">
@@ -16768,7 +16768,7 @@
         </is>
       </c>
       <c r="L215" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="216">
@@ -16900,7 +16900,7 @@
         </is>
       </c>
       <c r="L218" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-21 07:38) - 121 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41">
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -3605,12 +3605,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88">
@@ -3641,12 +3641,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
     </row>
     <row r="89">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="90">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="96">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>262</v>
+        <v>250</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="119">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="122">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128">
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -6652,7 +6652,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -6828,7 +6828,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44">
@@ -8804,7 +8804,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="101">
@@ -11008,7 +11008,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="103">
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="105">
@@ -11272,7 +11272,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="109">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="132">
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>202</v>
+        <v>180</v>
       </c>
     </row>
     <row r="146">
@@ -13464,7 +13464,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="154">
@@ -13508,7 +13508,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="155">
@@ -14224,7 +14224,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="168">
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>262</v>
+        <v>250</v>
       </c>
     </row>
     <row r="176">
@@ -16900,7 +16900,7 @@
         </is>
       </c>
       <c r="L218" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-21 12:17) - 116 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$145</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5621,12 +5621,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a9871445-40ed-48b8-b22f-f36ed0a3e5fa&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5652,17 +5652,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5680,44 +5680,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>MENOR COSTE</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>INFORME</t>
-        </is>
-      </c>
-      <c r="H145" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H145"/>
+  <autoFilter ref="A1:H144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5728,7 +5692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L214"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16337,7 +16301,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16345,7 +16309,7 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Stock unificado</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
@@ -16356,7 +16320,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>a9871445-40ed-48b8-b22f-f36ed0a3e5fa</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L209" t="n">
@@ -16381,7 +16345,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16389,7 +16353,7 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I210" t="inlineStr"/>
@@ -16400,11 +16364,11 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L210" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="211">
@@ -16425,7 +16389,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16433,7 +16397,7 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I211" t="inlineStr"/>
@@ -16444,11 +16408,11 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
         </is>
       </c>
       <c r="L211" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="212">
@@ -16469,7 +16433,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16477,7 +16441,7 @@
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -16488,11 +16452,11 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L212" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213">
@@ -16513,7 +16477,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16521,7 +16485,7 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I213" t="inlineStr"/>
@@ -16532,61 +16496,17 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
       <c r="L213" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>HERGO - DISTRIBUCION</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>VENTA MAYORISTA DETALLE</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>Venta Mayorista Detalle</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>Grupo Hergo - Jefes</t>
-        </is>
-      </c>
-      <c r="K214" t="inlineStr">
-        <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
-        </is>
-      </c>
-      <c r="L214" t="n">
         <v>47</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L214"/>
+  <autoFilter ref="A1:L213"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Login por usuario: cada area ve solo sus tableros
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableros" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$144</definedName>
@@ -64,12 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -16512,4 +16514,336 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Areas</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Iteraciones</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Hash</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0cILV2uqKc4jGDDC8yo2mg==</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>vbJeYyfcKNb3vhfVu5K9UyOFzwtoRb/C/UwBE/4vJ1s=</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>administracion01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Administracion 01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>e0WoCrEGvyAfFalzjsE1jQ==</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>B8J7dPPj2ucAJz3JVvpXRR9C2Yxvx96GEBhkXOwRll8=</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>administracion02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Administracion 02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>yg4EVntqLYjtRhcwffhUMw==</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NECqDF21ZyEY9liEeD4MeN27klbg6zPxq62uICf3wi8=</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>administracion03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Administracion 03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GfdoK30pfRpewh5deP9PEg==</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+4QI2rQrZ/j2WxEWFFz1L6PyAuL3yOGFaXf7yOG/G2Q=</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>administracion04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Administracion 04</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GERENCIA;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>o5ohDweOUWAjvW0dIx9wLA==</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>eldif//zVkfe/hO9E4w/1M8PeJRUqqM2DRcZpTe17QY=</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>administracion05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Administracion 05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Yfy9hfbf1dhF5x2aZt+cOg==</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EV361FYqYY+TgFy3raDW9spHlqAVG5Zg3tYdddzA+Hs=</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>administracion06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Administracion 06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>COMPRAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3RN5vSMCWjqcEM2fir8ziw==</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>QKbSnd5GGzwbd+QUzp0dkIEN4IvWn+3Fs6WPhpsj76A=</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>administracion07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Administracion 07</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1pAuM0slao+4wutINTIwEw==</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>kl8MNOyJe8W93IjmQwwR2MfFn6SuomY7kbyJVwzZM/I=</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>directorio</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Directorio</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DIRECTORIO;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>w/MGkOPlIv1UJSL/5/VHsg==</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OMJWemvKk/SwHagRSknprfTmoHepitNNQVPExf8Rpe8=</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizo tableros (2026-09-21 16:30) - 116 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -16834,12 +16834,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>w/MGkOPlIv1UJSL/5/VHsg==</t>
+          <t>w/MGkOPlIv1UJSL/5/VHsg==;/NTh0t7FDmU+L9z1ek5Muw==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>OMJWemvKk/SwHagRSknprfTmoHepitNNQVPExf8Rpe8=</t>
+          <t>OMJWemvKk/SwHagRSknprfTmoHepitNNQVPExf8Rpe8=;B8gFjXcpc6KehUgpVmBq44MNYXJ3i6Xr33KrNU5LcFQ=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-22 07:38) - 116 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6339ca7-bf01-48b1-a5ce-930d679671a2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6339ca7-bf01-48b1-a5ce-930d679671a2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="51">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -2655,12 +2655,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="85">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="89">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="90">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="92">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6f91c54d-24ae-4d7a-a580-596cc52ec510&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="97">
@@ -3967,12 +3967,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6f91c54d-24ae-4d7a-a580-596cc52ec510&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="98">
@@ -4003,12 +4003,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="99">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4075,12 +4075,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4131,7 +4131,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="102">
@@ -4147,12 +4147,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="107">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>475</v>
+        <v>490</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>475</v>
+        <v>490</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="115">
@@ -4615,12 +4615,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="116">
@@ -4651,12 +4651,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="117">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="121">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="122">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="124">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="125">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="127">
@@ -5858,7 +5858,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -6078,7 +6078,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -6122,7 +6122,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10">
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16">
@@ -6518,7 +6518,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19">
@@ -6606,7 +6606,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -7334,7 +7334,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
@@ -7446,7 +7446,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36">
@@ -7502,7 +7502,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37">
@@ -7546,7 +7546,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -7590,7 +7590,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -7678,7 +7678,7 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
@@ -8582,7 +8582,7 @@
         </is>
       </c>
       <c r="L57" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -9018,7 +9018,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67">
@@ -9062,7 +9062,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="68">
@@ -10830,7 +10830,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="103">
@@ -10874,7 +10874,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="104">
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="105">
@@ -10962,7 +10962,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="106">
@@ -11214,7 +11214,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="111">
@@ -11346,7 +11346,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="114">
@@ -11478,7 +11478,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
@@ -11566,7 +11566,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="119">
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="120">
@@ -11654,7 +11654,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="121">
@@ -12722,7 +12722,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>180</v>
+        <v>164</v>
       </c>
     </row>
     <row r="142">
@@ -12890,7 +12890,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>156</v>
+        <v>171</v>
       </c>
     </row>
     <row r="145">
@@ -12978,7 +12978,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="147">
@@ -13022,7 +13022,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
     </row>
     <row r="148">
@@ -13110,7 +13110,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="150">
@@ -13870,7 +13870,7 @@
         </is>
       </c>
       <c r="L163" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="164">
@@ -13982,7 +13982,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="166">
@@ -14038,7 +14038,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167">
@@ -14258,7 +14258,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="172">
@@ -14302,7 +14302,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="173">
@@ -14602,7 +14602,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="179">
@@ -16370,7 +16370,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="211">
@@ -16414,7 +16414,7 @@
         </is>
       </c>
       <c r="L211" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="212">

</xml_diff>

<commit_message>
Las claves se aplican solas al publicar, desde CLAVES TABLERO.xlsx
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -16588,12 +16588,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0cILV2uqKc4jGDDC8yo2mg==</t>
+          <t>LDQeRxVsYl0vE4EW/sT5nw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>vbJeYyfcKNb3vhfVu5K9UyOFzwtoRb/C/UwBE/4vJ1s=</t>
+          <t>0mPkAA+WnC/1dzrh0MqwqiTnvO+xVxZ6IVNb89XlX7g=</t>
         </is>
       </c>
     </row>
@@ -16620,12 +16620,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>e0WoCrEGvyAfFalzjsE1jQ==</t>
+          <t>1ae5oLox/0gVa+gneZ5f+A==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>B8J7dPPj2ucAJz3JVvpXRR9C2Yxvx96GEBhkXOwRll8=</t>
+          <t>AZEqnVybPLDxGkLjzMs5GhtiHIhnoQ34TgrcNmazGsI=</t>
         </is>
       </c>
     </row>
@@ -16652,12 +16652,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>yg4EVntqLYjtRhcwffhUMw==</t>
+          <t>TPgVRSq3iz/qF1Z7UXENzw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NECqDF21ZyEY9liEeD4MeN27klbg6zPxq62uICf3wi8=</t>
+          <t>qVBjKLjlGlSb2Kg1ozReKULE3BTwUevqFjp688DP/D8=</t>
         </is>
       </c>
     </row>
@@ -16679,12 +16679,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GfdoK30pfRpewh5deP9PEg==</t>
+          <t>Ei498/IfpwOW4yqaLd2C+A==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>+4QI2rQrZ/j2WxEWFFz1L6PyAuL3yOGFaXf7yOG/G2Q=</t>
+          <t>6BxZdp2Dzkpx+9SurGOE0EHkzhBjvE/zDbSvFJNvARo=</t>
         </is>
       </c>
     </row>
@@ -16711,12 +16711,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>o5ohDweOUWAjvW0dIx9wLA==</t>
+          <t>yPdXLgLYPbsvo4Z6leTYOA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>eldif//zVkfe/hO9E4w/1M8PeJRUqqM2DRcZpTe17QY=</t>
+          <t>Lfx8cSIVbMQqji5Ay6zypiwVzMZrySiYtX6z7z4E1xQ=</t>
         </is>
       </c>
     </row>
@@ -16743,12 +16743,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Yfy9hfbf1dhF5x2aZt+cOg==</t>
+          <t>EUeoD3PZD4T4hwqlqRzcIA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>EV361FYqYY+TgFy3raDW9spHlqAVG5Zg3tYdddzA+Hs=</t>
+          <t>+xPXF+x7zVVBIyk88gRygrEUlxZHe1zZr9j9YBZm54s=</t>
         </is>
       </c>
     </row>
@@ -16775,12 +16775,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3RN5vSMCWjqcEM2fir8ziw==</t>
+          <t>/3Yt4pa8aIgU1Tz/x+YHRQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>QKbSnd5GGzwbd+QUzp0dkIEN4IvWn+3Fs6WPhpsj76A=</t>
+          <t>qsDERwI4ITIgan8YQmt3wLMU1KwhHTRVoFyfxLU322M=</t>
         </is>
       </c>
     </row>
@@ -16802,12 +16802,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1pAuM0slao+4wutINTIwEw==</t>
+          <t>TWYAUvIDsBZnBi2CbqBqow==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>kl8MNOyJe8W93IjmQwwR2MfFn6SuomY7kbyJVwzZM/I=</t>
+          <t>L0dgwp1IRzAZyEM+yWI/8NCeKe3jATy1799TNNb8bU4=</t>
         </is>
       </c>
     </row>
@@ -16834,12 +16834,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>w/MGkOPlIv1UJSL/5/VHsg==;/NTh0t7FDmU+L9z1ek5Muw==</t>
+          <t>R+veWS9paL753q8ESrixYQ==;B+zDfbZqeuwJYMekGKo6xQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>OMJWemvKk/SwHagRSknprfTmoHepitNNQVPExf8Rpe8=;B8gFjXcpc6KehUgpVmBq44MNYXJ3i6Xr33KrNU5LcFQ=</t>
+          <t>pgGqyRZay+k/st6WmDaxEEhbq477gPvYeD4PRRHGvus=;alSoy/Sayf1tP4gtBtnieTKKb4ohyCZDP1IiWJgHUZc=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Usuarios personales que heredan areas de su cuenta de Power BI
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$144</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4579,12 +4579,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>236</v>
+        <v>71</v>
       </c>
     </row>
     <row r="115">
@@ -4615,12 +4615,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="116">
@@ -4651,12 +4651,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="117">
@@ -4687,12 +4687,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="120">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="123">
@@ -4903,12 +4903,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="124">
@@ -4939,12 +4939,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="125">
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="126">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129">
@@ -5119,12 +5119,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="130">
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132">
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5247,7 +5247,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5618,17 +5618,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5646,44 +5646,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>MENOR COSTE</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>INFORME</t>
-        </is>
-      </c>
-      <c r="H144" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H144"/>
+  <autoFilter ref="A1:H143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5694,7 +5658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L213"/>
+  <dimension ref="A1:L212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13087,7 +13051,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -13095,7 +13059,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -13106,11 +13070,11 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>849ac12f-c28b-4306-a0fe-6a00c6c9c8e8</t>
+          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
         </is>
       </c>
       <c r="L149" t="n">
-        <v>236</v>
+        <v>30</v>
       </c>
     </row>
     <row r="150">
@@ -13131,7 +13095,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
@@ -13139,7 +13103,7 @@
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>Grupo Clientes BLACK 2026</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -13150,11 +13114,11 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
+          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
         </is>
       </c>
       <c r="L150" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151">
@@ -13175,18 +13139,30 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>HECTOLITROS 07-2025</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>HECTOLITROS</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Grupo Clientes BLACK 2026</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr"/>
+          <t>Informe Hctos - Julio 25</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J151" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -13194,11 +13170,11 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
+          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
         </is>
       </c>
       <c r="L151" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -13219,7 +13195,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2025</t>
+          <t>HECTOLITROS 08-2025</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
@@ -13230,17 +13206,17 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 25</t>
+          <t>Informe Hctos - Agosto 25</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -13250,7 +13226,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
+          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -13275,7 +13251,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2025</t>
+          <t>HECTOLITROS 09-2025</t>
         </is>
       </c>
       <c r="E153" t="inlineStr"/>
@@ -13286,17 +13262,17 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 25</t>
+          <t>Informe Hctos - Septiembre 25</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -13306,7 +13282,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
+          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -13331,7 +13307,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2025</t>
+          <t>HECTOLITROS 10-2025</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
@@ -13342,17 +13318,17 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 25</t>
+          <t>Informe Hctos - Octubre 25</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -13362,7 +13338,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
+          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -13387,7 +13363,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2025</t>
+          <t>HECTOLITROS 11-2025</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -13398,17 +13374,17 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 25</t>
+          <t>Informe Hctos - Noviembre 25</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -13418,7 +13394,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
+          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -13443,7 +13419,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>HECTOLITROS 11-2025</t>
+          <t>HECTOLITROS 12-2025</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -13454,17 +13430,17 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Informe Hctos - Noviembre 25</t>
+          <t>Informe Hctos - Diciembre 25</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -13474,7 +13450,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
+          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -13499,7 +13475,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>HECTOLITROS 12-2025</t>
+          <t>HECTOLITROS 01-2026</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -13510,17 +13486,17 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Informe Hctos - Diciembre 25</t>
+          <t>Informe Hctos - Enero 26</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -13530,7 +13506,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
+          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -13555,7 +13531,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>HECTOLITROS 01-2026</t>
+          <t>HECTOLITROS 02-2026</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -13566,17 +13542,17 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Informe Hctos - Enero 26</t>
+          <t>Informe Hctos - Febrero 26</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -13586,7 +13562,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
+          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -13611,7 +13587,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>HECTOLITROS 02-2026</t>
+          <t>HECTOLITROS 03-2026</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -13622,17 +13598,17 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Informe Hctos - Febrero 26</t>
+          <t>Informe Hctos - Marzo 26</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -13642,7 +13618,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
+          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -13667,7 +13643,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HECTOLITROS 03-2026</t>
+          <t>HECTOLITROS 04-2026</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -13678,17 +13654,17 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Informe Hctos - Marzo 26</t>
+          <t>Informe Hctos - Abril 26</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -13698,11 +13674,11 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
+          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
         </is>
       </c>
       <c r="L160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -13723,7 +13699,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>HECTOLITROS 04-2026</t>
+          <t>HECTOLITROS 05-2026</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -13734,17 +13710,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Informe Hctos - Abril 26</t>
+          <t>Informe Hctos - Mayo 26</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -13754,11 +13730,11 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
+          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
         </is>
       </c>
       <c r="L161" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="162">
@@ -13779,7 +13755,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>HECTOLITROS 05-2026</t>
+          <t>HECTOLITROS 06-2026</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -13790,17 +13766,17 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Informe Hctos - Mayo 26</t>
+          <t>Informe Hctos - Junio 26</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -13810,11 +13786,11 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
+          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
         </is>
       </c>
       <c r="L162" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="163">
@@ -13835,7 +13811,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -13846,17 +13822,17 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 26</t>
+          <t>Informe Hctos - Julio 26</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -13866,11 +13842,11 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
+          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
         </is>
       </c>
       <c r="L163" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="164">
@@ -13891,7 +13867,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -13902,17 +13878,17 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 26</t>
+          <t>Informe Hctos - Agosto 26</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -13922,11 +13898,11 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
+          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
         </is>
       </c>
       <c r="L164" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="165">
@@ -13947,7 +13923,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -13958,17 +13934,17 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 26</t>
+          <t>Informe Hctos - Septiembre 26</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -13978,11 +13954,11 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
+          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
         </is>
       </c>
       <c r="L165" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
     </row>
     <row r="166">
@@ -14003,30 +13979,18 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>HECTOLITROS</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>09-2026</t>
-        </is>
-      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 26</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>Septiembre - 26</t>
-        </is>
-      </c>
+          <t>INFO MARCA CORE CCU</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14034,11 +13998,11 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
+          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
         </is>
       </c>
       <c r="L166" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
@@ -14059,7 +14023,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -14067,7 +14031,7 @@
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -14078,11 +14042,11 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
+          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
         </is>
       </c>
       <c r="L167" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="168">
@@ -14103,7 +14067,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
@@ -14111,7 +14075,7 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -14122,11 +14086,11 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
+          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
         </is>
       </c>
       <c r="L168" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -14147,7 +14111,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
@@ -14155,7 +14119,7 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -14166,11 +14130,11 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
+          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
         </is>
       </c>
       <c r="L169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170">
@@ -14191,7 +14155,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
@@ -14199,7 +14163,7 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -14210,11 +14174,11 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
+          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
         </is>
       </c>
       <c r="L170" t="n">
-        <v>0</v>
+        <v>244</v>
       </c>
     </row>
     <row r="171">
@@ -14235,7 +14199,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -14243,7 +14207,7 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
@@ -14254,11 +14218,11 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L171" t="n">
-        <v>244</v>
+        <v>18</v>
       </c>
     </row>
     <row r="172">
@@ -14279,18 +14243,30 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>PARTICIPACION VENTAS CCU</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr"/>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14298,11 +14274,11 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
+          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
       </c>
       <c r="L172" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173">
@@ -14323,28 +14299,28 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -14354,11 +14330,11 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
+          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
       </c>
       <c r="L173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -14379,13 +14355,13 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -14395,7 +14371,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
+          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -14410,11 +14386,11 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
+          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
       </c>
       <c r="L174" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -14435,30 +14411,18 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP COSTA</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>Agosto - 25</t>
-        </is>
-      </c>
+          <t>PLAN TRADI</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14466,11 +14430,11 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
+          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
         </is>
       </c>
       <c r="L175" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176">
@@ -14486,12 +14450,12 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
@@ -14499,7 +14463,7 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -14510,11 +14474,11 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
+          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
@@ -14530,12 +14494,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
@@ -14543,7 +14507,7 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>RECHAZOS ago 26</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -14554,11 +14518,11 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
+          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="178">
@@ -14579,18 +14543,30 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO DE MARCAS</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>RECHAZOS ago 26</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr"/>
+          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14598,11 +14574,11 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
+          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
       <c r="L178" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179">
@@ -14623,7 +14599,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -14634,17 +14610,17 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -14654,7 +14630,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
+          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -14679,7 +14655,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -14690,17 +14666,17 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -14710,7 +14686,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
+          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -14735,7 +14711,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -14746,17 +14722,17 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -14766,7 +14742,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
+          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -14791,7 +14767,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
@@ -14802,17 +14778,17 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -14822,7 +14798,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
+          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -14847,7 +14823,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
@@ -14858,17 +14834,17 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -14878,7 +14854,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
+          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
       <c r="L183" t="n">
@@ -14903,7 +14879,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
@@ -14914,17 +14890,17 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -14934,7 +14910,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
+          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
       <c r="L184" t="n">
@@ -14959,7 +14935,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -14970,17 +14946,17 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -14990,7 +14966,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
+          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
       <c r="L185" t="n">
@@ -15015,7 +14991,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -15026,17 +15002,17 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -15046,7 +15022,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
+          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
       <c r="L186" t="n">
@@ -15071,7 +15047,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
@@ -15082,17 +15058,17 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -15102,7 +15078,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
+          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
       <c r="L187" t="n">
@@ -15127,7 +15103,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -15138,17 +15114,17 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -15158,7 +15134,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
+          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
       <c r="L188" t="n">
@@ -15183,7 +15159,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
@@ -15194,17 +15170,17 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -15214,7 +15190,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
+          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
       <c r="L189" t="n">
@@ -15239,7 +15215,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -15250,17 +15226,17 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -15270,7 +15246,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
+          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
       <c r="L190" t="n">
@@ -15295,7 +15271,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -15306,17 +15282,17 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -15326,11 +15302,11 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
+          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
       <c r="L191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -15351,7 +15327,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
@@ -15362,17 +15338,17 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -15382,11 +15358,11 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
+          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
         </is>
       </c>
       <c r="L192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -15407,28 +15383,28 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -15438,11 +15414,11 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L193" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194">
@@ -15463,7 +15439,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -15474,17 +15450,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15494,11 +15470,11 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195">
@@ -15519,7 +15495,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -15530,17 +15506,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15550,11 +15526,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -15575,7 +15551,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -15586,17 +15562,17 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -15606,7 +15582,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L196" t="n">
@@ -15631,7 +15607,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -15642,17 +15618,17 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -15662,11 +15638,11 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L197" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -15687,7 +15663,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -15698,17 +15674,17 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -15718,7 +15694,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L198" t="n">
@@ -15743,7 +15719,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -15754,17 +15730,17 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -15774,7 +15750,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L199" t="n">
@@ -15799,7 +15775,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -15810,17 +15786,17 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15830,7 +15806,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L200" t="n">
@@ -15855,7 +15831,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -15866,17 +15842,17 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15886,7 +15862,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L201" t="n">
@@ -15911,7 +15887,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
@@ -15922,17 +15898,17 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -15942,11 +15918,11 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L202" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203">
@@ -15967,7 +15943,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
@@ -15978,17 +15954,17 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -15998,11 +15974,11 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204">
@@ -16023,7 +15999,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16034,17 +16010,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16054,11 +16030,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="205">
@@ -16079,7 +16055,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16090,17 +16066,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16110,11 +16086,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="206">
@@ -16135,7 +16111,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16146,17 +16122,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16166,11 +16142,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="207">
@@ -16191,7 +16167,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
@@ -16202,17 +16178,17 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16222,11 +16198,11 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L207" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208">
@@ -16247,30 +16223,18 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
-        </is>
-      </c>
-      <c r="G208" t="inlineStr">
-        <is>
-          <t>09-2026</t>
-        </is>
-      </c>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>Septiembre - 26</t>
-        </is>
-      </c>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr"/>
       <c r="J208" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16278,11 +16242,11 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L208" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209">
@@ -16303,7 +16267,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16311,7 +16275,7 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
@@ -16322,11 +16286,11 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L209" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="210">
@@ -16347,7 +16311,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16355,7 +16319,7 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I210" t="inlineStr"/>
@@ -16366,11 +16330,11 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
         </is>
       </c>
       <c r="L210" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="211">
@@ -16391,7 +16355,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16399,7 +16363,7 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I211" t="inlineStr"/>
@@ -16410,11 +16374,11 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L211" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="212">
@@ -16435,7 +16399,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16443,7 +16407,7 @@
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -16454,61 +16418,17 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
       <c r="L212" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>HERGO - DISTRIBUCION</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>VENTA MAYORISTA DETALLE</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>Venta Mayorista Detalle</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>Grupo Hergo - Jefes</t>
-        </is>
-      </c>
-      <c r="K213" t="inlineStr">
-        <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
-        </is>
-      </c>
-      <c r="L213" t="n">
         <v>47</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L213"/>
+  <autoFilter ref="A1:L212"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16522,7 +16442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16588,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LDQeRxVsYl0vE4EW/sT5nw==</t>
+          <t>XpCbS/tg7dxs/1szzYzxvw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0mPkAA+WnC/1dzrh0MqwqiTnvO+xVxZ6IVNb89XlX7g=</t>
+          <t>/Fh85PA1Z3uHyQisEfpGIq9MX72F0+4Y/b3+IpqNGks=</t>
         </is>
       </c>
     </row>
@@ -16620,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1ae5oLox/0gVa+gneZ5f+A==</t>
+          <t>6M7iAkgj6krKFUlKTU91sg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AZEqnVybPLDxGkLjzMs5GhtiHIhnoQ34TgrcNmazGsI=</t>
+          <t>S+pFMl4Ahfr0PVVGtDuh1Ia5HtoN0VChr6pSZFtaa5M=</t>
         </is>
       </c>
     </row>
@@ -16652,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TPgVRSq3iz/qF1Z7UXENzw==</t>
+          <t>G3iBHpD3j2xsUj73n/skgQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>qVBjKLjlGlSb2Kg1ozReKULE3BTwUevqFjp688DP/D8=</t>
+          <t>WbsKVx6sKlKCHirpru9Lev5B3nE3lgZZUx5oHDMvOBc=</t>
         </is>
       </c>
     </row>
@@ -16679,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ei498/IfpwOW4yqaLd2C+A==</t>
+          <t>cwqDzA6bW5uiNCzRAWbllg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6BxZdp2Dzkpx+9SurGOE0EHkzhBjvE/zDbSvFJNvARo=</t>
+          <t>LA5iWd7J8fbZNmZ+9Eqqq3oAA+TuypVrdH0SbtWasmU=</t>
         </is>
       </c>
     </row>
@@ -16711,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>yPdXLgLYPbsvo4Z6leTYOA==</t>
+          <t>XH7w5xcMAV2EBoeuKjQ+lQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Lfx8cSIVbMQqji5Ay6zypiwVzMZrySiYtX6z7z4E1xQ=</t>
+          <t>gzjF6mQdRApOMh0gtbMgrywvW64H8He2/7wJ7xV6p04=</t>
         </is>
       </c>
     </row>
@@ -16743,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EUeoD3PZD4T4hwqlqRzcIA==</t>
+          <t>HV1PLTVoG2eUEgF9hyIM2A==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>+xPXF+x7zVVBIyk88gRygrEUlxZHe1zZr9j9YBZm54s=</t>
+          <t>ihPMoROlU3qnrMtUuCWcTwqt7dshRGSzHabFWZuksTw=</t>
         </is>
       </c>
     </row>
@@ -16775,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>/3Yt4pa8aIgU1Tz/x+YHRQ==</t>
+          <t>Lib8E+JsNNIZvUS25LDeJA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>qsDERwI4ITIgan8YQmt3wLMU1KwhHTRVoFyfxLU322M=</t>
+          <t>+Jek0A/gvm683MygVNp2alEhZLM3Yk+ZKngfuEpDFDk=</t>
         </is>
       </c>
     </row>
@@ -16802,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TWYAUvIDsBZnBi2CbqBqow==</t>
+          <t>qUrMvEsMG8n/kiCbWKwVzQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>L0dgwp1IRzAZyEM+yWI/8NCeKe3jATy1799TNNb8bU4=</t>
+          <t>GQMiQGxszfF06F1fgOGx+4e+E4dVK5S0y8vVROL06NA=</t>
         </is>
       </c>
     </row>
@@ -16834,12 +16754,908 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>R+veWS9paL753q8ESrixYQ==;B+zDfbZqeuwJYMekGKo6xQ==</t>
+          <t>ZL+8vcVZPTpTgdW+GIIdWQ==;SI+6ijjftqTMpyTq+OyqKA==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>pgGqyRZay+k/st6WmDaxEEhbq477gPvYeD4PRRHGvus=;alSoy/Sayf1tP4gtBtnieTKKb4ohyCZDP1IiWJgHUZc=</t>
+          <t>jZcl/UNs27gQMZnComyi0XOIzLuL5aY/dlfzCI/WYSQ=;5TAZgIDnCJQiV4tloliU7qyjNgy3wucPrxXS/CY70GA=</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rtm</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rtm</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>aJWXAa1QY0MtxQGMAICunA==</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>vh0MneFTX0rTVuFnynm6oJhN6LXEOdJo/IXRuZPg8eI=</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>gabriel.mariani</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Gabriel Mariani</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>6vBDROa2S3UHknFkAazX8w==</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EwnO+gut7aHt2GzZXOOdv0ArIMu365tHlTxHOiY7WDc=</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>juanpablo.diserio</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Juanpablo Diserio</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>NSlOJrHOTaArGIB4hqeOhA==</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SenMcCRbw4BkE2+hm90PrhntwIqKe6JsNXvRGnlxs6Q=</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>matias.dasilva</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Matias Dasilva</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>56CBXWoc3AK5myBap7DE4g==</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>MMyN5pJp+flL6xOSolYLI7jIjtU2GHuSvwltBll8654=</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>andrea.juarez</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Andrea Juarez</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>uKGYpKgEeznWzME0+7ZP9g==</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>p+FZoQ7uwDWjYGDv1Qn483lTkQRs/5VYx1bc2i0p2Ac=</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lucas.ceballos</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lucas Ceballos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>aHYBLD0J+jhazGeUenybMw==</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>c4jIn9yCljd7DArboV0P4IfGd9UMr2v1WNczFo0cQL8=</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>david.leon</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>David Leon</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WIKlLO62LbTs9+60pNKM1w==</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>/qC22nVvni2gd0UWYeiqQmd/FK/6QBbkjSqpbzgcAyw=</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>matias.abelando</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Matias Abelando</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3QEVCHK8xtdSULh9RVQYLA==</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>eHIYVo2+XojOFbupRAjoHh3Va3/yCJudwuNlUJ/hU3E=</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gaston.daoud</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gaston Daoud</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>mZdnWX+w5gweUN9ABeRkeg==</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>YAoeNh0otP+wy3D2V3J7TyYOA5CQ/zMkpjwZhmgdV8Q=</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cristian.mena</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cristian Mena</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>9qcjnJ0hjrs2NyhaCSQ3pg==</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>bH9A8CHC/Zxufp41CK2ZNzslt7KSOmSKC+8k7MXLXWk=</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>hernan.bertola</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hernan Bertola</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0w7PypKLpTnO/aN+1n4iTA==</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>IAbtnZO/2PEnNB64eZVjPSXleYHZSvhJJYFuiiZIdxI=</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>diego.lopez</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Diego Lopez</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TwsHKhFfAoMynIE3pb79LA==</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>WEYJjkLLJNfrA6k9UvX+WOE7PR4JNGObhiebSZnQ8fk=</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>directorio.directorio</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Directorio Directorio</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>DIRECTORIO;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>o5/WGTouNBCZj75g7mQRyg==</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>A0kNeygEacKxZTHy7nSfwvrObksibNCxsVsvPkey82U=</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>felicitas.scianna</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Felicitas Scianna</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>T4hGTcwpwujxyu3L5WR3Uw==</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>q4IGTgJxfy9Sq0vvOe8UVCSt+ChuKQr4fWzKBACZG1Q=</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>florencia.guerendiain</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Florencia Guerendiain</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>9+N1nrG8rW3qI217hBPjAQ==</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>8Fi/mmWt1i2F6NTQwOlPbBb2NY22/HsCUf7cfDS/1ww=</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>florencia.lopez</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Florencia Lopez</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>kWLaFcAGPB6SVatPiHVWmw==</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>dBfMn83s2kapYH5OMXYhm58pOoFEZrsL/JfA+icxB2g=</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ivana.paladini</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ivana Paladini</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>NcU1VwY3ca4MmXZ3tmuYvQ==</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>lojps2yS+f99ID+2uF4sJcc58xhxggs7yJP5MM1BwV0=</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>juanignacio.garberi</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Juanignacio Garberi</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GERENCIA;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>rRgvhQSDO2HxufdB29fz3A==</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>cTgTPia3ftoHu7gmEk7Qd94iCtiCYpcPm4aPDlHI59k=</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>paula.pezzelato</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Paula Pezzelato</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>mbNyxgseRIj96L174sDUAQ==</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>k/dVTQsyFut4RDhP57VT59zmuXEE1kn81Wl4mjwRBig=</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sebastian.dopazo</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sebastian Dopazo</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GERENCIA;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>8XQiOg+9kX9LzSRp3h3cWw==</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>J39z2ZctkFSgXLXsCGrtCbNrMhnwAtWIfppxymizn5M=</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mariaemilia.bibbo</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Mariaemilia Bibbo</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>cEHY/+AobwP5FYwdJQeifw==</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>kQK+4/i3wnydd5mxHGwXwOK8TWl4lQPlzCwtQzZvB4I=</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>agustin.sarraute</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Agustin Sarraute</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>aeY1bbqPvFOemC7t22LKbA==</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>4N5zneogX8+L6ZkqKt5fmGXislUsXYs2bwLnyN/RTwo=</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>inaki.turza</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Inaki Turza</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>t5xyJfT/FZePF+OUZRAZYQ==</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>FiWqD9wN1N+oM45taLbyCvPi/GIG45UhXfWol1D3UJg=</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>nadia.kozlovski</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Nadia Kozlovski</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>VqjJNV5lyihFKQRGQC8j4A==</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d6/YGhZOHnTSqMdrP+X/BZ/oceOCdBLhoHUCh/dJ1Sw=</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>pablo.ferre</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Pablo Ferre</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GERENCIA;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>U1RviQDU0b1afhg+KS/i7g==</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>t1Y51WW36YFgolLObttxfV5bqMokTmrlsMnzYR9Eang=</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ramiro.bibiloni</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ramiro Bibiloni</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GYvW+mYTFPxD+PW7eaZ5Gg==</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>diGemc30ZS6QZ80vi3wm+93TacYgmalwDEZi+d1/89M=</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mkt</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mkt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>JEFES;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>AxshHGoNylblE9oKqyCAqQ==</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>9Yhw2QQRrTXn4h3RiQDQ3//II3Cw1dTUpec5iCEj0fY=</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>soledad.martin</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Soledad Martin</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>FINANZAS;AREAS COMUNES</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>jKJqzQbrpbptmVPTVBbf0Q==</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0anSemi4IkkeFXU7+E91EsEUIw7NehcDMHlsZGt/P24=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-23 07:38) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43">
@@ -2007,12 +2007,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="85">
@@ -3535,12 +3535,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="86">
@@ -3571,12 +3571,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="97">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="106">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="107">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=243f52b1-78cb-4c1a-9689-e0f18217f77a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=551a92c1-4681-4327-9d2a-c0e1263fe997&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4399,12 +4399,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=551a92c1-4681-4327-9d2a-c0e1263fe997&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=243f52b1-78cb-4c1a-9689-e0f18217f77a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>490</v>
+        <v>510</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>490</v>
+        <v>510</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="117">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="124">
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14">
@@ -6306,7 +6306,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16">
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18">
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43">
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="92">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="103">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="105">
@@ -11178,7 +11178,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="111">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="114">
@@ -11354,7 +11354,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="119">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="120">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="126">
@@ -11926,7 +11926,7 @@
         </is>
       </c>
       <c r="L127" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="128">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="142">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>171</v>
+        <v>191</v>
       </c>
     </row>
     <row r="145">
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="148">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="163">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="171">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="178">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="211">
@@ -16422,7 +16422,7 @@
         </is>
       </c>
       <c r="L212" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>XpCbS/tg7dxs/1szzYzxvw==</t>
+          <t>jtIlnyjY2tCd7GPhxcwKuQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>/Fh85PA1Z3uHyQisEfpGIq9MX72F0+4Y/b3+IpqNGks=</t>
+          <t>dY3WMlVSPF6xaG8e8y0Xm6o3EsHgAkHvdnH68LfUyIk=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6M7iAkgj6krKFUlKTU91sg==</t>
+          <t>UVyEGPpGyQG2FRZJVqnedg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>S+pFMl4Ahfr0PVVGtDuh1Ia5HtoN0VChr6pSZFtaa5M=</t>
+          <t>Znlx5urY9ntzJeCVPAcj3QQEQTFulS1ut2eZ7sVPIfA=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>G3iBHpD3j2xsUj73n/skgQ==</t>
+          <t>dGUZuqYoWbGUt9X5CV8UNA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>WbsKVx6sKlKCHirpru9Lev5B3nE3lgZZUx5oHDMvOBc=</t>
+          <t>vgNPgSSzC5uoOB/JyUpBbB2mwPM8vAvyPAe2O2+b7sI=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>cwqDzA6bW5uiNCzRAWbllg==</t>
+          <t>8NrU5C8LSkHxLeWDp7sahg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LA5iWd7J8fbZNmZ+9Eqqq3oAA+TuypVrdH0SbtWasmU=</t>
+          <t>ageX7ebH0/3FXga8HAXefDwUcRagd60sXmY5ZAB2i5Q=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>XH7w5xcMAV2EBoeuKjQ+lQ==</t>
+          <t>+aAp2+D0bbspmFlyXH0gKw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>gzjF6mQdRApOMh0gtbMgrywvW64H8He2/7wJ7xV6p04=</t>
+          <t>Mx8+ga6JOoNqm9uY1SYGDCyAN+RW9K06BBgIKpvNfVQ=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HV1PLTVoG2eUEgF9hyIM2A==</t>
+          <t>/YzK2FEpupKKd7UAIucYmQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ihPMoROlU3qnrMtUuCWcTwqt7dshRGSzHabFWZuksTw=</t>
+          <t>CJ0lHO3FwGMtH0DKDvF1hlFOBFkBBVmKX6iuIbcUBt8=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Lib8E+JsNNIZvUS25LDeJA==</t>
+          <t>sy2caYGmJaiKMxgjI7fJbA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>+Jek0A/gvm683MygVNp2alEhZLM3Yk+ZKngfuEpDFDk=</t>
+          <t>Pjdm/GWV3bXcdIQp9jNTuHdih/4+QAnCmFmBXZ3OAjQ=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>qUrMvEsMG8n/kiCbWKwVzQ==</t>
+          <t>5ZeXEYBNk32TMHg+IUZWJQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>GQMiQGxszfF06F1fgOGx+4e+E4dVK5S0y8vVROL06NA=</t>
+          <t>NE/IgnBygZCvODvy5EOI9RQMbmKgdrWyfl+Yz3blnUQ=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ZL+8vcVZPTpTgdW+GIIdWQ==;SI+6ijjftqTMpyTq+OyqKA==</t>
+          <t>P6PC/6fHMef8Gp/SFQuDew==;sbrAJFGeTAr0oDeefJAZVg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>jZcl/UNs27gQMZnComyi0XOIzLuL5aY/dlfzCI/WYSQ=;5TAZgIDnCJQiV4tloliU7qyjNgy3wucPrxXS/CY70GA=</t>
+          <t>EXPamnsvVpNAqT9TW8DPVH+qm7uqErQo1ZhoX1Waef8=;iVHZgkgBEWL7qYhubek0RQS5cel0QW9G1mcOzf3OE2g=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>aJWXAa1QY0MtxQGMAICunA==</t>
+          <t>919fjD8yJfOB4FYoRXzPtA==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>vh0MneFTX0rTVuFnynm6oJhN6LXEOdJo/IXRuZPg8eI=</t>
+          <t>zk0gEc1ZzT2TySzWnc+ckmRaD46WNoHARz+3a5ZZTCo=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>6vBDROa2S3UHknFkAazX8w==</t>
+          <t>LKu3WqfFSAEbhHOwSoFYjg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>EwnO+gut7aHt2GzZXOOdv0ArIMu365tHlTxHOiY7WDc=</t>
+          <t>JG8ajM1JiiW4ESXRTu00xOoGRq9XmZxdRDoYYmHWllU=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NSlOJrHOTaArGIB4hqeOhA==</t>
+          <t>sHYO9g1SZYyn5C4oTfFZ3Q==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SenMcCRbw4BkE2+hm90PrhntwIqKe6JsNXvRGnlxs6Q=</t>
+          <t>x+OWDuiQK+6BvND9/8/sWpavXUsvGm07L061IKqquhg=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>56CBXWoc3AK5myBap7DE4g==</t>
+          <t>ZtGk7tWL9nZiZj6Ynt8xXw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MMyN5pJp+flL6xOSolYLI7jIjtU2GHuSvwltBll8654=</t>
+          <t>qq2CnePJe9p1GUoJIuiT6/fG6m5Ih6Zrx4tuYhBIpgc=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>uKGYpKgEeznWzME0+7ZP9g==</t>
+          <t>wq0t7ldKRiHfABFIVdnIWA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>p+FZoQ7uwDWjYGDv1Qn483lTkQRs/5VYx1bc2i0p2Ac=</t>
+          <t>eQPJneHS7zicSkqFQkrdcaro1W0W7WHuKWJE7aM/jFo=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>aHYBLD0J+jhazGeUenybMw==</t>
+          <t>3zL/XwSf5HxUm6iKrvzTKQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>c4jIn9yCljd7DArboV0P4IfGd9UMr2v1WNczFo0cQL8=</t>
+          <t>0/5Y89Qbcnv5PsS0gqtPdX/vxofbDVEdHVAcJnmN5vI=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>WIKlLO62LbTs9+60pNKM1w==</t>
+          <t>V/yJaBzVThQjFuqrksw+Ug==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>/qC22nVvni2gd0UWYeiqQmd/FK/6QBbkjSqpbzgcAyw=</t>
+          <t>YAAO5m/K8E61CWV/4sqzEMCD0LUdqcGeIc3XX9F89M4=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3QEVCHK8xtdSULh9RVQYLA==</t>
+          <t>ov6kDx8BR7TkQkjuIP7FLg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>eHIYVo2+XojOFbupRAjoHh3Va3/yCJudwuNlUJ/hU3E=</t>
+          <t>kRA8PWF1lElHeZxLWMtpC/pzHaWY9U+FVqU9r0sNk7Q=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>mZdnWX+w5gweUN9ABeRkeg==</t>
+          <t>YLwqD05N8cul3emVU7gd2Q==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>YAoeNh0otP+wy3D2V3J7TyYOA5CQ/zMkpjwZhmgdV8Q=</t>
+          <t>bNODLTKV0MeMA3aylLo2F4spoWafhB5JP9v7wo6Y30M=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>9qcjnJ0hjrs2NyhaCSQ3pg==</t>
+          <t>60FKggSpp4MHXHAnMSYrdA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>bH9A8CHC/Zxufp41CK2ZNzslt7KSOmSKC+8k7MXLXWk=</t>
+          <t>aobIJn60UIKA46VDvF/Cu7g16YdTVKFzuTgXHuLAReg=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0w7PypKLpTnO/aN+1n4iTA==</t>
+          <t>0eptERUqpDDdQMt63QuMrg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>IAbtnZO/2PEnNB64eZVjPSXleYHZSvhJJYFuiiZIdxI=</t>
+          <t>BhqBMNI3OQ9EW42Rkmh4hd2TNOW9SzcLAF+psc4NK4E=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TwsHKhFfAoMynIE3pb79LA==</t>
+          <t>55e64YcvNOAMDcjaDo8Rbw==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>WEYJjkLLJNfrA6k9UvX+WOE7PR4JNGObhiebSZnQ8fk=</t>
+          <t>Nllekt+qnX3cohFTu4ts1pWs6DWwEvw7JKWmTwFyCws=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>o5/WGTouNBCZj75g7mQRyg==</t>
+          <t>vZA63aoeo383oKRQIheYYQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>A0kNeygEacKxZTHy7nSfwvrObksibNCxsVsvPkey82U=</t>
+          <t>K0OSrASBHr5rNk34eI00xbf6OKEMrZoSdmruEnMeB4s=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>T4hGTcwpwujxyu3L5WR3Uw==</t>
+          <t>kRn9yyaJ7hcHHvgaci5wdw==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>q4IGTgJxfy9Sq0vvOe8UVCSt+ChuKQr4fWzKBACZG1Q=</t>
+          <t>lsFRXaAWovbUVuzbm0qCNjieNeygHpnS8eQBPMD1p/I=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>9+N1nrG8rW3qI217hBPjAQ==</t>
+          <t>jkXCSWV6mgKnfUs8XNmCDg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>8Fi/mmWt1i2F6NTQwOlPbBb2NY22/HsCUf7cfDS/1ww=</t>
+          <t>aRn/RCnYu+ZLxy3KTRiyzGFLBma47IInbH0If7Cs/m4=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>kWLaFcAGPB6SVatPiHVWmw==</t>
+          <t>XpGOY/4uF1DHVk/zi/2umQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dBfMn83s2kapYH5OMXYhm58pOoFEZrsL/JfA+icxB2g=</t>
+          <t>G/UC2v4vFz9Z9eFuIZ7lp326UilgrbQ+px/NcSDnQBc=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NcU1VwY3ca4MmXZ3tmuYvQ==</t>
+          <t>QJdZDVvjEzTywl7YH/7mvg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>lojps2yS+f99ID+2uF4sJcc58xhxggs7yJP5MM1BwV0=</t>
+          <t>jFyRbyV8ORcSr/i4GfDS09DYWgW9NNqdHmGrVqrdFVA=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>rRgvhQSDO2HxufdB29fz3A==</t>
+          <t>kX61QNvMXsyojKQoPFC+DQ==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>cTgTPia3ftoHu7gmEk7Qd94iCtiCYpcPm4aPDlHI59k=</t>
+          <t>wJsJMXT/hzyoFchp+wmI6zJEwCnyYbmNdHjD1FXy9SU=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mbNyxgseRIj96L174sDUAQ==</t>
+          <t>Rc1AMI/QiyTdBPhiCOLDlA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>k/dVTQsyFut4RDhP57VT59zmuXEE1kn81Wl4mjwRBig=</t>
+          <t>9Sqe/gQuRCvYc4ziJ25RUGj5Jip/fJruZIKjJaHzNUQ=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>8XQiOg+9kX9LzSRp3h3cWw==</t>
+          <t>4I1kGTld2/kQnKk3aRsXDQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>J39z2ZctkFSgXLXsCGrtCbNrMhnwAtWIfppxymizn5M=</t>
+          <t>dwGWXB8ZGmagrAjyp29FvsFxQNhRwze+FdmXYiq/7oY=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>cEHY/+AobwP5FYwdJQeifw==</t>
+          <t>ad5V5WrcCdGsvycx0bdZqA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>kQK+4/i3wnydd5mxHGwXwOK8TWl4lQPlzCwtQzZvB4I=</t>
+          <t>gXhwyVUHs9AzRUlf3CComug11fexHUs9WczS1LcbwBM=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>aeY1bbqPvFOemC7t22LKbA==</t>
+          <t>P3WGy2F7XceTnFKmrEmCKA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>4N5zneogX8+L6ZkqKt5fmGXislUsXYs2bwLnyN/RTwo=</t>
+          <t>M3IAoUFbg9m+uANoZwL6wiPhevwlqrd/VZZFULJfzRE=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>t5xyJfT/FZePF+OUZRAZYQ==</t>
+          <t>F07lPY+yBEKZk4MIECJ1UQ==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>FiWqD9wN1N+oM45taLbyCvPi/GIG45UhXfWol1D3UJg=</t>
+          <t>AbdxSK7LuQHhFX8s9YVwjKdnBKoWr9bWF1p9Y9a9geU=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VqjJNV5lyihFKQRGQC8j4A==</t>
+          <t>8cHIaBWC02vIXiXxbpwWTg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d6/YGhZOHnTSqMdrP+X/BZ/oceOCdBLhoHUCh/dJ1Sw=</t>
+          <t>v7ArCYx+1lXz3tRROPr30aaVzpBqudCPiH/D0nKp62o=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>U1RviQDU0b1afhg+KS/i7g==</t>
+          <t>gLgX+orkR1iTZIj45q4uYA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>t1Y51WW36YFgolLObttxfV5bqMokTmrlsMnzYR9Eang=</t>
+          <t>AcuRsG1v37tc75/uMGqPnEWMHHi+YoP5PWCYDNiCsrg=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>GYvW+mYTFPxD+PW7eaZ5Gg==</t>
+          <t>DaNjOIE9LclwWoeTvkQqeA==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>diGemc30ZS6QZ80vi3wm+93TacYgmalwDEZi+d1/89M=</t>
+          <t>sZ9Zk+NiMvnSpu4UO2pPDzSHfMJyXxaphXGDtd1u0Jw=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AxshHGoNylblE9oKqyCAqQ==</t>
+          <t>1QzhDNvXioa6v6RXcP/PRQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>9Yhw2QQRrTXn4h3RiQDQ3//II3Cw1dTUpec5iCEj0fY=</t>
+          <t>tTNg3WBoyiqyDPQ61FMrJDQUytvkElqY0m23xYpZN08=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>jKJqzQbrpbptmVPTVBbf0Q==</t>
+          <t>mwHSckrhr1ux2t/XJBbIhA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>0anSemi4IkkeFXU7+E91EsEUIw7NehcDMHlsZGt/P24=</t>
+          <t>RG/70c5ILYb7WgqfR5XMnr7ze1CZClUm6VSCXpByjl4=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-24 07:38) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46">
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>182</v>
+        <v>196</v>
       </c>
     </row>
     <row r="85">
@@ -3535,12 +3535,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="86">
@@ -3571,12 +3571,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="89">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="107">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>510</v>
+        <v>523</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>510</v>
+        <v>523</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="117">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="121">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="122">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124">
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
@@ -6306,7 +6306,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16">
@@ -7298,7 +7298,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -8982,7 +8982,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="67">
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="92">
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="100">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="101">
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="102">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="103">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="104">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>182</v>
+        <v>196</v>
       </c>
     </row>
     <row r="105">
@@ -10970,7 +10970,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="107">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="114">
@@ -11354,7 +11354,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="120">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="126">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="142">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="145">
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="148">
@@ -13678,7 +13678,7 @@
         </is>
       </c>
       <c r="L160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -13958,7 +13958,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="171">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="178">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="211">
@@ -16422,7 +16422,7 @@
         </is>
       </c>
       <c r="L212" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>jtIlnyjY2tCd7GPhxcwKuQ==</t>
+          <t>V9odpBAPvIDU22nEUk6aag==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dY3WMlVSPF6xaG8e8y0Xm6o3EsHgAkHvdnH68LfUyIk=</t>
+          <t>TZlgmTktUAAJUbh+qsrJ/sqcmtzLZ/j0vE2GtySWJBU=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>UVyEGPpGyQG2FRZJVqnedg==</t>
+          <t>/jdNM7OoEC31TPmO+0tkTg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Znlx5urY9ntzJeCVPAcj3QQEQTFulS1ut2eZ7sVPIfA=</t>
+          <t>wXviW1u46LjTaWneD3m/lRYQTqzXYULn9geDAIwQ5Vw=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>dGUZuqYoWbGUt9X5CV8UNA==</t>
+          <t>qGSc6fkgVor0XP0imKbTVw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>vgNPgSSzC5uoOB/JyUpBbB2mwPM8vAvyPAe2O2+b7sI=</t>
+          <t>Fq/hM2SuGTU8RpWeU3ky7rbf1S57evepdRYbCO5PePQ=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8NrU5C8LSkHxLeWDp7sahg==</t>
+          <t>F0SMyBx7VXE+SDqk1u1KVg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ageX7ebH0/3FXga8HAXefDwUcRagd60sXmY5ZAB2i5Q=</t>
+          <t>TmaK4wOUREY8cOUfB2siQNMMBGMQsMFrM6+moAmzxEc=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+aAp2+D0bbspmFlyXH0gKw==</t>
+          <t>KNgXdcoP0feN/iXzNzhxew==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mx8+ga6JOoNqm9uY1SYGDCyAN+RW9K06BBgIKpvNfVQ=</t>
+          <t>k7n+lU7DfwXGFcKRTpkZkJ8rdvVmC9THtD0ZsGGBPts=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>/YzK2FEpupKKd7UAIucYmQ==</t>
+          <t>vjnlBaYiKywJWL0+AfH7QA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CJ0lHO3FwGMtH0DKDvF1hlFOBFkBBVmKX6iuIbcUBt8=</t>
+          <t>zEgUxrafAnEMyhWbYKFaaVfHh9DpI584qY5UIsO2bJ8=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>sy2caYGmJaiKMxgjI7fJbA==</t>
+          <t>GMLgqukXnx0KD+tMAN99wQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Pjdm/GWV3bXcdIQp9jNTuHdih/4+QAnCmFmBXZ3OAjQ=</t>
+          <t>9C1IUxUxiIaDKOcAU3Y8nr4ikg4a1yg5Nj8YFYmNRQs=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5ZeXEYBNk32TMHg+IUZWJQ==</t>
+          <t>YC6WM2LrUCmN5k39Zi6MbQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>NE/IgnBygZCvODvy5EOI9RQMbmKgdrWyfl+Yz3blnUQ=</t>
+          <t>uc9H0R0xssU4aZmHvGjWAJvmYQUSS7wgjvSGS0vkoCk=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>P6PC/6fHMef8Gp/SFQuDew==;sbrAJFGeTAr0oDeefJAZVg==</t>
+          <t>dy7wWmx0y3C+F5DvfPuEig==;9qq84tvZtJ8mZArUyY3KgQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>EXPamnsvVpNAqT9TW8DPVH+qm7uqErQo1ZhoX1Waef8=;iVHZgkgBEWL7qYhubek0RQS5cel0QW9G1mcOzf3OE2g=</t>
+          <t>hN+tZYMegV7TcQfBN/EuNkXSLLT2+I02gnX55z2nQEQ=;NX4/EMg4cnpwOsHWWkPnhH5Moear0pbbpiELKHAgkaY=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>919fjD8yJfOB4FYoRXzPtA==</t>
+          <t>S7eguCFUj9Pt42gQiqe7HA==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>zk0gEc1ZzT2TySzWnc+ckmRaD46WNoHARz+3a5ZZTCo=</t>
+          <t>7I7ip8Or+NWOJWCq2VhYMYb2+1zNV+vfzbsLnqJqgEY=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LKu3WqfFSAEbhHOwSoFYjg==</t>
+          <t>Gh83VbAlvwoGelHu8LBFJg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>JG8ajM1JiiW4ESXRTu00xOoGRq9XmZxdRDoYYmHWllU=</t>
+          <t>RaYDbePG0rtdgcpXbzeO+BEwqpluCahJ95O7QVPGt3E=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sHYO9g1SZYyn5C4oTfFZ3Q==</t>
+          <t>hBkwmfnDOyG4FU15l8T6sA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>x+OWDuiQK+6BvND9/8/sWpavXUsvGm07L061IKqquhg=</t>
+          <t>f99mMSRr8cbEdVqPfhR1QA1hf/RDdSdq5lQgOrrz5tY=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ZtGk7tWL9nZiZj6Ynt8xXw==</t>
+          <t>TYnFcjdKAzxST9+hClJoMQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>qq2CnePJe9p1GUoJIuiT6/fG6m5Ih6Zrx4tuYhBIpgc=</t>
+          <t>yUYBhTVvW34/XCBQPMdb6mUWF5AV1jq8qdUWDuKXjnA=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>wq0t7ldKRiHfABFIVdnIWA==</t>
+          <t>huiZxQj2uan64znDH5GlAg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>eQPJneHS7zicSkqFQkrdcaro1W0W7WHuKWJE7aM/jFo=</t>
+          <t>wCBjrdBFxneZEqOaWdTKEn3LX5VIv6w14uMYk/oJMvA=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3zL/XwSf5HxUm6iKrvzTKQ==</t>
+          <t>ggIWrqjUn64iWTpLGFOgew==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0/5Y89Qbcnv5PsS0gqtPdX/vxofbDVEdHVAcJnmN5vI=</t>
+          <t>uOkNIjTOJMpzmzUj76wGG2MXk4F7bcuZKno6skch3Wg=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>V/yJaBzVThQjFuqrksw+Ug==</t>
+          <t>4451ILlC8Ka70h/lYAop9A==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>YAAO5m/K8E61CWV/4sqzEMCD0LUdqcGeIc3XX9F89M4=</t>
+          <t>ttki3NUMvkb8SA7nkK9zdrSJtAPX1Ae7/SasKtSMnpQ=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ov6kDx8BR7TkQkjuIP7FLg==</t>
+          <t>FbNPs8DGEN6GJqsOZfRBaQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>kRA8PWF1lElHeZxLWMtpC/pzHaWY9U+FVqU9r0sNk7Q=</t>
+          <t>VK94Eq1Er3FJ1ejVgJGmGotRqZnrk30RcNLDnDKbfLw=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YLwqD05N8cul3emVU7gd2Q==</t>
+          <t>vMmIgkR9XRa4S6B1gs7gPA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>bNODLTKV0MeMA3aylLo2F4spoWafhB5JP9v7wo6Y30M=</t>
+          <t>UdpBnHOdshh0aln7pl8cb6koa4G0TSV6EzW/rzbfWFc=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>60FKggSpp4MHXHAnMSYrdA==</t>
+          <t>ogwxi6yKVtT+zqqs+eLBew==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>aobIJn60UIKA46VDvF/Cu7g16YdTVKFzuTgXHuLAReg=</t>
+          <t>0WlhNIna5UVCEbItUahqUMyKotGdlFz1HUQ5nMW4vgQ=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0eptERUqpDDdQMt63QuMrg==</t>
+          <t>e8tmUiySaOGyl75LnfC0yg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BhqBMNI3OQ9EW42Rkmh4hd2TNOW9SzcLAF+psc4NK4E=</t>
+          <t>PwfCt4nGCstw5J9iykXnXp6Wts6EkhMqzYUjJe5KuoU=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>55e64YcvNOAMDcjaDo8Rbw==</t>
+          <t>eB64b0tlmMG8GYU6ln4BpQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Nllekt+qnX3cohFTu4ts1pWs6DWwEvw7JKWmTwFyCws=</t>
+          <t>4piv63szNXFjjWWTHw2X5pZEFnjBrD46YjWkF0745EY=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vZA63aoeo383oKRQIheYYQ==</t>
+          <t>mpzZlqixjMpP2LyYyIbicA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>K0OSrASBHr5rNk34eI00xbf6OKEMrZoSdmruEnMeB4s=</t>
+          <t>uCZEq8ZUXWgqBBNmKhULXPMCvtFhOaN5dWlOuqmfkiM=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>kRn9yyaJ7hcHHvgaci5wdw==</t>
+          <t>LadiN4IDv0a+g4m3Vt6DsQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>lsFRXaAWovbUVuzbm0qCNjieNeygHpnS8eQBPMD1p/I=</t>
+          <t>pTppiSJPBWal28LFT6nLdg2wDQkJkvFIFbR15BwwxKE=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>jkXCSWV6mgKnfUs8XNmCDg==</t>
+          <t>8g/v3KbtYHhyqLYz8KI/Ow==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>aRn/RCnYu+ZLxy3KTRiyzGFLBma47IInbH0If7Cs/m4=</t>
+          <t>pGafT5o/k3X8wDbbZinmDKz4N8CosgHWvVH7ORD/iAM=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>XpGOY/4uF1DHVk/zi/2umQ==</t>
+          <t>US0wOi4U9gk39xWEsb3sEQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>G/UC2v4vFz9Z9eFuIZ7lp326UilgrbQ+px/NcSDnQBc=</t>
+          <t>2hMUArJ2xmDXa03v86sGIIcH3/dC11iSz/4eJvRmd6w=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>QJdZDVvjEzTywl7YH/7mvg==</t>
+          <t>zFQ+WY4MooBN3Xf9BsbKMA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>jFyRbyV8ORcSr/i4GfDS09DYWgW9NNqdHmGrVqrdFVA=</t>
+          <t>XqkB5XYYC9Q+C4oOLlWkzNlpCi9RK1jJvypC+l6fOsI=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>kX61QNvMXsyojKQoPFC+DQ==</t>
+          <t>mpBB5JpOJ9chI/ztjNN8tg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>wJsJMXT/hzyoFchp+wmI6zJEwCnyYbmNdHjD1FXy9SU=</t>
+          <t>Mu/AU7XUSFAIE8Q9G4L2cVigJlQ9OgDv6GxG7p9as7Q=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Rc1AMI/QiyTdBPhiCOLDlA==</t>
+          <t>paOVaLY2QDZgkeBi+Ppclw==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>9Sqe/gQuRCvYc4ziJ25RUGj5Jip/fJruZIKjJaHzNUQ=</t>
+          <t>4O/w3QJxf5UROgd7mdx2ECElhDX44g95WACYozE1V1Y=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>4I1kGTld2/kQnKk3aRsXDQ==</t>
+          <t>5YKNcVFDGK8+tnDJFzei9Q==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dwGWXB8ZGmagrAjyp29FvsFxQNhRwze+FdmXYiq/7oY=</t>
+          <t>VgCF0MhldioinBzrVTEE+q3b81g9IJxb9fPdWAj1z5U=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ad5V5WrcCdGsvycx0bdZqA==</t>
+          <t>p5UrLDVFKsFWVMgJoZor2g==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>gXhwyVUHs9AzRUlf3CComug11fexHUs9WczS1LcbwBM=</t>
+          <t>OL6r2LPHAYfplOI1tK20Ed6W1UloLB9f4IQ+vtDuiF0=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>P3WGy2F7XceTnFKmrEmCKA==</t>
+          <t>WJCqo9vuZjwkrx4wjciOBA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>M3IAoUFbg9m+uANoZwL6wiPhevwlqrd/VZZFULJfzRE=</t>
+          <t>Hc2IodZwV5kFdYVbeqKGHa6+foHFnDWnD3RsRl11h2c=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>F07lPY+yBEKZk4MIECJ1UQ==</t>
+          <t>r5B6R0ieWSmLEOfMli7dFA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AbdxSK7LuQHhFX8s9YVwjKdnBKoWr9bWF1p9Y9a9geU=</t>
+          <t>qKFdHh0Y98HqEqchpi23bQvGz+YHQ8KJ5m6SjfB0iOE=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>8cHIaBWC02vIXiXxbpwWTg==</t>
+          <t>GESt9oQoabDlDXGtOccnXg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>v7ArCYx+1lXz3tRROPr30aaVzpBqudCPiH/D0nKp62o=</t>
+          <t>4Gi3a5uAxa1tZ+9Eh5NpugY4WzvVQvZiOc4UsFdjatc=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>gLgX+orkR1iTZIj45q4uYA==</t>
+          <t>OmrCnxW5ASS/s2+VNh7P7A==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AcuRsG1v37tc75/uMGqPnEWMHHi+YoP5PWCYDNiCsrg=</t>
+          <t>itMpUVz6O6kIX8tsQvZyUeiTwkM5Tr9lDNodriweR7A=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DaNjOIE9LclwWoeTvkQqeA==</t>
+          <t>sUtWxF+d8duibC4CIwMmrQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>sZ9Zk+NiMvnSpu4UO2pPDzSHfMJyXxaphXGDtd1u0Jw=</t>
+          <t>Sqbs2ShIB/7syUoTwHWMfByWfhGUIFV9YuM7HhU3ehg=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1QzhDNvXioa6v6RXcP/PRQ==</t>
+          <t>LCToVY3DG+kn6FDIs86rDQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tTNg3WBoyiqyDPQ61FMrJDQUytvkElqY0m23xYpZN08=</t>
+          <t>4FLgp7l6JklUyZA6UUXfd0ICSDr75ARBIgbXvw3BB8g=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mwHSckrhr1ux2t/XJBbIhA==</t>
+          <t>EvaNVGcYHz7eWTzEaC6Fgg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>RG/70c5ILYb7WgqfR5XMnr7ze1CZClUm6VSCXpByjl4=</t>
+          <t>f5LYA14s2U2hnXBVydlphhDjBx0SZ4McwMSNRbTlBWU=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-25 07:38) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50">
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="53">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="80">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>196</v>
+        <v>203</v>
       </c>
     </row>
     <row r="85">
@@ -3535,12 +3535,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="86">
@@ -3571,12 +3571,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="90">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="95">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4075,12 +4075,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4147,12 +4147,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="103">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="107">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>523</v>
+        <v>540</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>523</v>
+        <v>540</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="115">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123">
@@ -4903,12 +4903,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5355,7 +5355,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10">
@@ -6306,7 +6306,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16">
@@ -6482,7 +6482,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
@@ -7466,7 +7466,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
@@ -9026,7 +9026,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68">
@@ -10618,7 +10618,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="99">
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="100">
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="102">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="103">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>196</v>
+        <v>203</v>
       </c>
     </row>
     <row r="105">
@@ -10926,7 +10926,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="106">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="114">
@@ -11398,7 +11398,7 @@
         </is>
       </c>
       <c r="L115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="116">
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="119">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="120">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="126">
@@ -12574,7 +12574,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="140">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="142">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>204</v>
+        <v>221</v>
       </c>
     </row>
     <row r="145">
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="148">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="163">
@@ -14090,7 +14090,7 @@
         </is>
       </c>
       <c r="L168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="171">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="178">
@@ -16034,7 +16034,7 @@
         </is>
       </c>
       <c r="L204" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="205">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="211">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>V9odpBAPvIDU22nEUk6aag==</t>
+          <t>i2DLKTG0H/F12ftJrGX8IA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TZlgmTktUAAJUbh+qsrJ/sqcmtzLZ/j0vE2GtySWJBU=</t>
+          <t>VnSwyLDypMhQuGsyK2IHbT5QCISs4jB7QHqG8/EWfkc=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/jdNM7OoEC31TPmO+0tkTg==</t>
+          <t>y/IIOVa4Prkr63YubcRs3w==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>wXviW1u46LjTaWneD3m/lRYQTqzXYULn9geDAIwQ5Vw=</t>
+          <t>MReR+WjkSm2FBb3PxrKe0iTW80Nr2VVXA5zs3bXULIs=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>qGSc6fkgVor0XP0imKbTVw==</t>
+          <t>Lt0jZtri6kEn5EFs4fvZLw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Fq/hM2SuGTU8RpWeU3ky7rbf1S57evepdRYbCO5PePQ=</t>
+          <t>utK/OGENHYo9Z/QoIhFIyHbpWuHrx9Ccb7wbSLMb0us=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>F0SMyBx7VXE+SDqk1u1KVg==</t>
+          <t>Gq/pgd9HMtX2UFFiZlW6iQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TmaK4wOUREY8cOUfB2siQNMMBGMQsMFrM6+moAmzxEc=</t>
+          <t>nBBSZf/3ez24a3oVFgx62GAgWRU/LEyNwQSX1lqnJDA=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>KNgXdcoP0feN/iXzNzhxew==</t>
+          <t>pDw0yzE9tbM6MNpjPNR0GA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>k7n+lU7DfwXGFcKRTpkZkJ8rdvVmC9THtD0ZsGGBPts=</t>
+          <t>lGGC0xcOhFBuVbMGCwtBsHeACY8AvvDb6vjK0Qi0+U4=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>vjnlBaYiKywJWL0+AfH7QA==</t>
+          <t>cNSDLXjiqw70coBafvWrbw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>zEgUxrafAnEMyhWbYKFaaVfHh9DpI584qY5UIsO2bJ8=</t>
+          <t>wfOwTvo6FfO5mFrzGLh6V3+3qe7ex+4tLU4xe1LSJMA=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GMLgqukXnx0KD+tMAN99wQ==</t>
+          <t>Dmfnb7v+pzmwlVL1QwQE2w==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9C1IUxUxiIaDKOcAU3Y8nr4ikg4a1yg5Nj8YFYmNRQs=</t>
+          <t>Mh3RhCZMFmgo2gX0EDFWJtMmJTY3rAjHuln+8rFStrY=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>YC6WM2LrUCmN5k39Zi6MbQ==</t>
+          <t>FXaHc3gW3PDMkatzF+RiTA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>uc9H0R0xssU4aZmHvGjWAJvmYQUSS7wgjvSGS0vkoCk=</t>
+          <t>zrXAg3DQGRP70WLUGhUImSaRRFMLYlbrW6WzFdRICtU=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>dy7wWmx0y3C+F5DvfPuEig==;9qq84tvZtJ8mZArUyY3KgQ==</t>
+          <t>GkSKkqMMe0STEY9qQ6sTNQ==;gkhuP8iqdqhKbY7GJy/GkA==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>hN+tZYMegV7TcQfBN/EuNkXSLLT2+I02gnX55z2nQEQ=;NX4/EMg4cnpwOsHWWkPnhH5Moear0pbbpiELKHAgkaY=</t>
+          <t>PWmOsmxzZOuk0Cl0jJl5QmG2RzF1Rau3T/920ACkSHU=;ptJXEM02i3QfBdhNDrd8kodkTHTJreBHS2P9JXbttys=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>S7eguCFUj9Pt42gQiqe7HA==</t>
+          <t>zPjOmHj37hIQbJCNU3thiQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>7I7ip8Or+NWOJWCq2VhYMYb2+1zNV+vfzbsLnqJqgEY=</t>
+          <t>DSbCkMPOaD8MUnKvqgO7FkGoPBDnyUP06hdrUZ9AgC0=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Gh83VbAlvwoGelHu8LBFJg==</t>
+          <t>/xU9c+HWE5vKrspiWvYT5g==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RaYDbePG0rtdgcpXbzeO+BEwqpluCahJ95O7QVPGt3E=</t>
+          <t>HHpCRR9fg2OThV3IK8Vl9bBfx5SvULNtNo8uaJ41ggo=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>hBkwmfnDOyG4FU15l8T6sA==</t>
+          <t>d8ZoBf2RoUPe+eWjyG4fww==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>f99mMSRr8cbEdVqPfhR1QA1hf/RDdSdq5lQgOrrz5tY=</t>
+          <t>lfDDog3R4XZHnTdfP7+TuNJbK/yAvkda4PVcSWk/omI=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TYnFcjdKAzxST9+hClJoMQ==</t>
+          <t>76J+mVGW5LySnh3IHQWHLg==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>yUYBhTVvW34/XCBQPMdb6mUWF5AV1jq8qdUWDuKXjnA=</t>
+          <t>9cckea8Una4EZKYVJ9Svmv+W75s2n1c2JdUd7hlLaOw=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>huiZxQj2uan64znDH5GlAg==</t>
+          <t>X+FzSAc171E/1Kr8h1hGcg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>wCBjrdBFxneZEqOaWdTKEn3LX5VIv6w14uMYk/oJMvA=</t>
+          <t>ZCsaoxDe15Pd/QLOImJztoU8sRGMInBaf7JZqJTmTDU=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ggIWrqjUn64iWTpLGFOgew==</t>
+          <t>tUmO7C6RLLum1C6dlzucIA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>uOkNIjTOJMpzmzUj76wGG2MXk4F7bcuZKno6skch3Wg=</t>
+          <t>GtjEdXVTdGsAW2ly0MB6oZ0Gi1LJm+5eTipOhYmgZpI=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4451ILlC8Ka70h/lYAop9A==</t>
+          <t>73l+tGsKAyOHHfwGQUFG4w==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ttki3NUMvkb8SA7nkK9zdrSJtAPX1Ae7/SasKtSMnpQ=</t>
+          <t>ITylB7Cn1QMQj192ACZ01kEfoylqeM1qHuE9vL1YmIo=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FbNPs8DGEN6GJqsOZfRBaQ==</t>
+          <t>aeenqQMJJirzyYn9YDmUcw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>VK94Eq1Er3FJ1ejVgJGmGotRqZnrk30RcNLDnDKbfLw=</t>
+          <t>/RcwZTqxf8Xm3QnyRQFGfVoz9pbDjLGvCUMWzZMO1VE=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>vMmIgkR9XRa4S6B1gs7gPA==</t>
+          <t>zwJixJeUtWkGhwazcfVXWA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>UdpBnHOdshh0aln7pl8cb6koa4G0TSV6EzW/rzbfWFc=</t>
+          <t>l2pbRpW22oApjKMtvAt0IlNHb/bAT8qZK6RI6YZgynw=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ogwxi6yKVtT+zqqs+eLBew==</t>
+          <t>lMsxDZJI/13C5WOXsJMQQg==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0WlhNIna5UVCEbItUahqUMyKotGdlFz1HUQ5nMW4vgQ=</t>
+          <t>n15hJsdVxVp6rghkb/K2kxslQdH2jSH80BIb7z1VTt4=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>e8tmUiySaOGyl75LnfC0yg==</t>
+          <t>mUQdWgZUpkmy0cpvBo6a3g==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PwfCt4nGCstw5J9iykXnXp6Wts6EkhMqzYUjJe5KuoU=</t>
+          <t>UVh1PODIpksTAfCh0R2yOVctYM/qHmaDHd6CteeD5V8=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>eB64b0tlmMG8GYU6ln4BpQ==</t>
+          <t>SxnAgJAQcwms3ZNVi1bn3g==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>4piv63szNXFjjWWTHw2X5pZEFnjBrD46YjWkF0745EY=</t>
+          <t>J/Eufub00ToEjqlsYbWmzLG/SRTDAHehCTgs+J6/jB0=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mpzZlqixjMpP2LyYyIbicA==</t>
+          <t>4wfhU3BhNisLsna/SP5t3w==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>uCZEq8ZUXWgqBBNmKhULXPMCvtFhOaN5dWlOuqmfkiM=</t>
+          <t>Y/s8xC7Q5tYz90v4BmJn8EkHPHf01al5qh58cwbGcxg=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LadiN4IDv0a+g4m3Vt6DsQ==</t>
+          <t>w95DRpnaezHiDRSxSwhlZw==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>pTppiSJPBWal28LFT6nLdg2wDQkJkvFIFbR15BwwxKE=</t>
+          <t>jYYac01xXuuF2n4S0ZMSZ4bV9nECWcWCcw2k2jhe/9I=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>8g/v3KbtYHhyqLYz8KI/Ow==</t>
+          <t>ZpXJPoc91fZ7eeQhDgavKA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>pGafT5o/k3X8wDbbZinmDKz4N8CosgHWvVH7ORD/iAM=</t>
+          <t>cZ0MFIznpVf66HSyU+lpROpKPPhAgXlRjeZm0CN790w=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>US0wOi4U9gk39xWEsb3sEQ==</t>
+          <t>jjZ9x8DKiyB5s6Ufk0QYrw==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2hMUArJ2xmDXa03v86sGIIcH3/dC11iSz/4eJvRmd6w=</t>
+          <t>+Oza1DXBmshBWKlYI76HaT1/e+TuAIZoEhq2aw+Xuhw=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>zFQ+WY4MooBN3Xf9BsbKMA==</t>
+          <t>XZvtP2Ut7btYW+2FZyQQzg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>XqkB5XYYC9Q+C4oOLlWkzNlpCi9RK1jJvypC+l6fOsI=</t>
+          <t>v2f1zwWzt9WmEceUUJf+vC1P4IMVKsTZTYN5HZUIw0s=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mpBB5JpOJ9chI/ztjNN8tg==</t>
+          <t>3rY8Fwgn8OX5t7CFD2Ultw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Mu/AU7XUSFAIE8Q9G4L2cVigJlQ9OgDv6GxG7p9as7Q=</t>
+          <t>t4bbHVM6vdg2cz04/aTszjSDVy906hKe34AJomgD4iU=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>paOVaLY2QDZgkeBi+Ppclw==</t>
+          <t>uTA2jKXlP24Bo0Mx9PSKbg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>4O/w3QJxf5UROgd7mdx2ECElhDX44g95WACYozE1V1Y=</t>
+          <t>FRB7zBXmKVYN3eMuBx2fm4QTMYzDIzSsrgicuQmrpNw=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5YKNcVFDGK8+tnDJFzei9Q==</t>
+          <t>9gZUKnZWuo0SKl+ri35gXA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>VgCF0MhldioinBzrVTEE+q3b81g9IJxb9fPdWAj1z5U=</t>
+          <t>XuMN0svBfxX2ySqkiFUHowmIwpcbvEYvYuTYey3ZF/8=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>p5UrLDVFKsFWVMgJoZor2g==</t>
+          <t>YQH0H8xJAPkd9YZFieTNSg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>OL6r2LPHAYfplOI1tK20Ed6W1UloLB9f4IQ+vtDuiF0=</t>
+          <t>8mZRzRezBIFlAelimmOK1pOWLLxWzPOnrcQtETUB9iw=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WJCqo9vuZjwkrx4wjciOBA==</t>
+          <t>cBJyJ4GY/py2H6j5q7QCzw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Hc2IodZwV5kFdYVbeqKGHa6+foHFnDWnD3RsRl11h2c=</t>
+          <t>s9Tu+ouR7wFykkUyvvO26wfyA9Xfb9IKC7V6zdNhWJo=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>r5B6R0ieWSmLEOfMli7dFA==</t>
+          <t>OSmPkUKiwx/4y20WpFbZRg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>qKFdHh0Y98HqEqchpi23bQvGz+YHQ8KJ5m6SjfB0iOE=</t>
+          <t>YG+B3eRDTTOJgtN4mX88++FkoPxvce0NkmyFmcxIEZg=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>GESt9oQoabDlDXGtOccnXg==</t>
+          <t>1bqTh+rSmQ3b+DanS4YAPg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>4Gi3a5uAxa1tZ+9Eh5NpugY4WzvVQvZiOc4UsFdjatc=</t>
+          <t>UWto3obkWWHigShbPDpi4m377a9pz7zv0MwQ0G9YMGA=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OmrCnxW5ASS/s2+VNh7P7A==</t>
+          <t>HfaV75wDnutGmtlBeOwgqw==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>itMpUVz6O6kIX8tsQvZyUeiTwkM5Tr9lDNodriweR7A=</t>
+          <t>1QW3nlY6oc1ExQFVqi/vN9YzG3JoOpME8IiGrqghaws=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>sUtWxF+d8duibC4CIwMmrQ==</t>
+          <t>XqyMHP1qEaqpWvdymYML2g==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sqbs2ShIB/7syUoTwHWMfByWfhGUIFV9YuM7HhU3ehg=</t>
+          <t>skHv356LxkT9zwZ88U3jxIacKGeHqCC9bmWhQnSBrV4=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>LCToVY3DG+kn6FDIs86rDQ==</t>
+          <t>1Rlm69EIcJ8nxaKX2sV4Ww==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4FLgp7l6JklUyZA6UUXfd0ICSDr75ARBIgbXvw3BB8g=</t>
+          <t>KmEglVqQd32LNYMJJdtlmkiCVa6MDYj2MSkAPqtzvgc=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>EvaNVGcYHz7eWTzEaC6Fgg==</t>
+          <t>2t01syym1CMJL4Tgy/zbJQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>f5LYA14s2U2hnXBVydlphhDjBx0SZ4McwMSNRbTlBWU=</t>
+          <t>eC8jYzKNgHUsU4MRPwrkkUb+tBDG5G5ujQ67zwpgowk=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-26 07:39) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="52">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="54">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55">
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="85">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="95">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="106">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>540</v>
+        <v>549</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>540</v>
+        <v>549</v>
       </c>
     </row>
     <row r="113">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="115">
@@ -4651,12 +4651,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="117">
@@ -4687,12 +4687,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="119">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="122">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="123">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="126">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130">
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
@@ -6306,7 +6306,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16">
@@ -7466,7 +7466,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37">
@@ -8714,7 +8714,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="61">
@@ -9026,7 +9026,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68">
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="93">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="101">
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="102">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="105">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="114">
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="119">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="126">
@@ -11926,7 +11926,7 @@
         </is>
       </c>
       <c r="L127" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="128">
@@ -11970,7 +11970,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="129">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>221</v>
+        <v>230</v>
       </c>
     </row>
     <row r="145">
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="148">
@@ -13118,7 +13118,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="178">
@@ -16290,7 +16290,7 @@
         </is>
       </c>
       <c r="L209" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="210">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="211">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>i2DLKTG0H/F12ftJrGX8IA==</t>
+          <t>tUBi0IjaXdP2RcNkz9aBGg==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>VnSwyLDypMhQuGsyK2IHbT5QCISs4jB7QHqG8/EWfkc=</t>
+          <t>CZhz+Wby/02b9Krcu5TCjZT7ooUm4pSeAccyp4itnFc=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>y/IIOVa4Prkr63YubcRs3w==</t>
+          <t>s8DUZNjJ+EWId+PSbFlvxQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MReR+WjkSm2FBb3PxrKe0iTW80Nr2VVXA5zs3bXULIs=</t>
+          <t>SVbwRwriUGD66kN5BMaDuHLLG6biYImwqC45JbKYmnc=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lt0jZtri6kEn5EFs4fvZLw==</t>
+          <t>lpWoPWUbkpRlEo6DTELPeQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>utK/OGENHYo9Z/QoIhFIyHbpWuHrx9Ccb7wbSLMb0us=</t>
+          <t>jsldnw4SzH95nQIb3s5ZOV9GoIUGjmjyAGLlrCYYUPs=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Gq/pgd9HMtX2UFFiZlW6iQ==</t>
+          <t>p5I3y8qUKXn9fLKCkXE8ug==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>nBBSZf/3ez24a3oVFgx62GAgWRU/LEyNwQSX1lqnJDA=</t>
+          <t>IB99yTCutDVx8PTM+QlDSHazME6UTFE3Po6hE3MNy2U=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>pDw0yzE9tbM6MNpjPNR0GA==</t>
+          <t>1TD2fSsscLO8BkT4tShYrA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>lGGC0xcOhFBuVbMGCwtBsHeACY8AvvDb6vjK0Qi0+U4=</t>
+          <t>PULcxLk35SvaH0dl3sl5LJKGowt1t7VG1whpV5lBshs=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>cNSDLXjiqw70coBafvWrbw==</t>
+          <t>UfpRRewYUkyWAbIpi+RiOA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>wfOwTvo6FfO5mFrzGLh6V3+3qe7ex+4tLU4xe1LSJMA=</t>
+          <t>QT5xxv2OGde6tfiWxFkZ7+FE5BG9G6Yq4nHsy6Ej53g=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dmfnb7v+pzmwlVL1QwQE2w==</t>
+          <t>F99kekQ4V4xTyNlogZKqJw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mh3RhCZMFmgo2gX0EDFWJtMmJTY3rAjHuln+8rFStrY=</t>
+          <t>BBfXOGlcprsiAQFHXOBwJAdJSdVdkjTiiaGD8l0K4Rc=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FXaHc3gW3PDMkatzF+RiTA==</t>
+          <t>GUMaAxe68fkBuJNpDqx5NQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>zrXAg3DQGRP70WLUGhUImSaRRFMLYlbrW6WzFdRICtU=</t>
+          <t>TTrtZx9rAcjsGZkEbTyctqli0zrzQ/qQBYP9mgnGF2M=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GkSKkqMMe0STEY9qQ6sTNQ==;gkhuP8iqdqhKbY7GJy/GkA==</t>
+          <t>h9zcDcqLjNM9HOdlrwxNZA==;I+UXEOIFurtoVh/Y7lPM+A==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PWmOsmxzZOuk0Cl0jJl5QmG2RzF1Rau3T/920ACkSHU=;ptJXEM02i3QfBdhNDrd8kodkTHTJreBHS2P9JXbttys=</t>
+          <t>btvMpPrup9CT7d3fFZQmb4opl8/AtV0YDi8iPKUjJUs=;LTM8aDgZQSIE80mUGVqhai3iAuIl9fefW49O5LCyEvI=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>zPjOmHj37hIQbJCNU3thiQ==</t>
+          <t>2W6jr9iB7VXO3R2nLIG9PQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DSbCkMPOaD8MUnKvqgO7FkGoPBDnyUP06hdrUZ9AgC0=</t>
+          <t>kvMDQfQrEhRoTp3g6uyO1XSeNBFzlajHM2l/9VsLD6A=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/xU9c+HWE5vKrspiWvYT5g==</t>
+          <t>xgfVXMvNii26dLmMp+IR4A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HHpCRR9fg2OThV3IK8Vl9bBfx5SvULNtNo8uaJ41ggo=</t>
+          <t>GRaVmJ+Fy+wEZr9Iwu+xE6rqqm/5wzFysCYeJc20ciM=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>d8ZoBf2RoUPe+eWjyG4fww==</t>
+          <t>KKWnodhbV7VuKCuTPY1ZmA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>lfDDog3R4XZHnTdfP7+TuNJbK/yAvkda4PVcSWk/omI=</t>
+          <t>o0iRo9RW9NFB9SoWL/lKItKKeIHR/7l8yWvrPIXiYKo=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>76J+mVGW5LySnh3IHQWHLg==</t>
+          <t>xNkxNssGot2tT2J+xzo/8g==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>9cckea8Una4EZKYVJ9Svmv+W75s2n1c2JdUd7hlLaOw=</t>
+          <t>Pzst3SrOcQ73kWwWX1ZBAxgTNcUHtUn7jxWmT8BnmHU=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>X+FzSAc171E/1Kr8h1hGcg==</t>
+          <t>PFAkZKRJPlTPEnyD9LGtDw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ZCsaoxDe15Pd/QLOImJztoU8sRGMInBaf7JZqJTmTDU=</t>
+          <t>ZUxWdoTShk+P2rjNdX56OtECYlyE4I7I45lOd5j1m9A=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>tUmO7C6RLLum1C6dlzucIA==</t>
+          <t>ZjuktToBHb/vx+65Jlcgpw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>GtjEdXVTdGsAW2ly0MB6oZ0Gi1LJm+5eTipOhYmgZpI=</t>
+          <t>euw+I3z6MN6BJX8dzC+2exlO3NPr5DUTlwxVrzQFdko=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>73l+tGsKAyOHHfwGQUFG4w==</t>
+          <t>Mp2dw2JGgBOSmEZjgPcnKQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ITylB7Cn1QMQj192ACZ01kEfoylqeM1qHuE9vL1YmIo=</t>
+          <t>dLkwo4HTI2HhQNmqkQkDqvkFuMulHCgCeRox6blWp/Q=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>aeenqQMJJirzyYn9YDmUcw==</t>
+          <t>Vj5fwO9tnroIhzDdhBGqUw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>/RcwZTqxf8Xm3QnyRQFGfVoz9pbDjLGvCUMWzZMO1VE=</t>
+          <t>p1k7dHp41c2yWCY3VAY/4zFicb/UeeoFUQl+qR1/MSc=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>zwJixJeUtWkGhwazcfVXWA==</t>
+          <t>Gs5ja5IU6so8EYcGveC/xA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>l2pbRpW22oApjKMtvAt0IlNHb/bAT8qZK6RI6YZgynw=</t>
+          <t>BbOoU4gr86QfIvAgNQq2SQCXHwTOmidCnZSLtAqgtKA=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>lMsxDZJI/13C5WOXsJMQQg==</t>
+          <t>B4BGYRBIsbHmSNdcV/06zw==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>n15hJsdVxVp6rghkb/K2kxslQdH2jSH80BIb7z1VTt4=</t>
+          <t>hZ4z7MzZPeJ/ifCANXgV0k2BWUzDgwvpOwS4H6hAp/E=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>mUQdWgZUpkmy0cpvBo6a3g==</t>
+          <t>/OBnij4tFRWlRCnuNFh3SA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>UVh1PODIpksTAfCh0R2yOVctYM/qHmaDHd6CteeD5V8=</t>
+          <t>EMO14aWx7BvQioM7H5dI8McHQSf5JyCKLI4XCiAmuEw=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SxnAgJAQcwms3ZNVi1bn3g==</t>
+          <t>W4g+xyTgbY9nrMZm4p1S+A==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>J/Eufub00ToEjqlsYbWmzLG/SRTDAHehCTgs+J6/jB0=</t>
+          <t>qH7FtR1Ju4YOFuhbwToR2NAX95d7GUb5/YU0EvSocVw=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4wfhU3BhNisLsna/SP5t3w==</t>
+          <t>UfGZMDPoZzeuJ6svBmuhyA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Y/s8xC7Q5tYz90v4BmJn8EkHPHf01al5qh58cwbGcxg=</t>
+          <t>JGA9foTR+FzjXqY01Ow8dHvGmB52lFmMDl2ti5fnVuQ=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>w95DRpnaezHiDRSxSwhlZw==</t>
+          <t>5XOFan8KXdrVTWzambjejQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>jYYac01xXuuF2n4S0ZMSZ4bV9nECWcWCcw2k2jhe/9I=</t>
+          <t>NMOhfbS//vHWccpt2MMx1HBKQaRzeCf4h+yymznx8lo=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ZpXJPoc91fZ7eeQhDgavKA==</t>
+          <t>xVXdhLF084DFRZE4OF0mZw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>cZ0MFIznpVf66HSyU+lpROpKPPhAgXlRjeZm0CN790w=</t>
+          <t>4NwxQ2V6kWIwdEXmqL6k2hV9IfPappvEP5GOc5nWsY4=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>jjZ9x8DKiyB5s6Ufk0QYrw==</t>
+          <t>0Nyll2R5Tec12En6d1nIjg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>+Oza1DXBmshBWKlYI76HaT1/e+TuAIZoEhq2aw+Xuhw=</t>
+          <t>tKrzzva196gnHo/4zbVjl3PNzKPMVEUtgAsdtfKORtI=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>XZvtP2Ut7btYW+2FZyQQzg==</t>
+          <t>Rkq72IaTjlerjCxNUHNgaQ==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>v2f1zwWzt9WmEceUUJf+vC1P4IMVKsTZTYN5HZUIw0s=</t>
+          <t>CDoeGufDAQ+ExPtOMCs199K7Nv6mik+oHnskllAnXaw=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3rY8Fwgn8OX5t7CFD2Ultw==</t>
+          <t>LhCX3wby1wf5qdJVJVmBiw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>t4bbHVM6vdg2cz04/aTszjSDVy906hKe34AJomgD4iU=</t>
+          <t>uPiDKHX8hlHj+46PUHzoidg6iYFFNfVwHH7EKb+23yQ=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>uTA2jKXlP24Bo0Mx9PSKbg==</t>
+          <t>t9qykw+YJ6U/Im1Hxriudw==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>FRB7zBXmKVYN3eMuBx2fm4QTMYzDIzSsrgicuQmrpNw=</t>
+          <t>pdMWG3a5VAuJlAftd4eQMumC8xtqKgR06ixFb9nLkvs=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>9gZUKnZWuo0SKl+ri35gXA==</t>
+          <t>DCcj1cvbaTrRqGC7BS/r8Q==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>XuMN0svBfxX2ySqkiFUHowmIwpcbvEYvYuTYey3ZF/8=</t>
+          <t>DuPOxQ9uY7owQ41HuKTm/fb5gIRe10Gf4ytyR1z00Rs=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>YQH0H8xJAPkd9YZFieTNSg==</t>
+          <t>r9jjn5SyiJnIoJ6Rlgc1FA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>8mZRzRezBIFlAelimmOK1pOWLLxWzPOnrcQtETUB9iw=</t>
+          <t>Z68BVlmIegaBLyO6i17fwHfzVsUeePylT0ygcSG//Lk=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>cBJyJ4GY/py2H6j5q7QCzw==</t>
+          <t>yJgZote83P8q/F74xiKW4w==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>s9Tu+ouR7wFykkUyvvO26wfyA9Xfb9IKC7V6zdNhWJo=</t>
+          <t>ocjdYaFhylHZPZk/ijF7y3kPnpp3LZYTD7L9okafxTE=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OSmPkUKiwx/4y20WpFbZRg==</t>
+          <t>SJuLEIMHpSQArrCKsy3igQ==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>YG+B3eRDTTOJgtN4mX88++FkoPxvce0NkmyFmcxIEZg=</t>
+          <t>NDlrEp8hox1S6d+BCMMVeHbzMrfQqTxNla40RsaNnjo=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1bqTh+rSmQ3b+DanS4YAPg==</t>
+          <t>KXl3sz5EypHJBo0/sj6uZw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>UWto3obkWWHigShbPDpi4m377a9pz7zv0MwQ0G9YMGA=</t>
+          <t>nfnQcbHIlUl30StkHsG86uit/+SJXzfW5OHK+Oe12v4=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>HfaV75wDnutGmtlBeOwgqw==</t>
+          <t>sJHdXFlC1sXC22F6CvPRCQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1QW3nlY6oc1ExQFVqi/vN9YzG3JoOpME8IiGrqghaws=</t>
+          <t>t4De+mlbaXMybJTAZxPd6xJchxQnsNsyAtRJ/ddg+co=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>XqyMHP1qEaqpWvdymYML2g==</t>
+          <t>5p+kVvNPJwQPIVHxyj4Y0Q==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>skHv356LxkT9zwZ88U3jxIacKGeHqCC9bmWhQnSBrV4=</t>
+          <t>1MI27bnBfYgpIilRvVEETYK/pSgYpnD9xFKjj2j6X18=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1Rlm69EIcJ8nxaKX2sV4Ww==</t>
+          <t>tA9rRtkhVNhU7eet8N8jkA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>KmEglVqQd32LNYMJJdtlmkiCVa6MDYj2MSkAPqtzvgc=</t>
+          <t>LC/dk5IMz4+l/ejNZKA7hmZ4ct/h3uWQugeFltbr8l4=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2t01syym1CMJL4Tgy/zbJQ==</t>
+          <t>RvOlvGzS+fs+95TyT7e6rA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>eC8jYzKNgHUsU4MRPwrkkUb+tBDG5G5ujQ67zwpgowk=</t>
+          <t>UyZHBTeZE4UYGS77ig8dSkoGBoCJDwcUu9UB2qJDIS4=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-27 07:39) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="85">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="87">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="91">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="98">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -4075,12 +4075,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>549</v>
+        <v>559</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>549</v>
+        <v>559</v>
       </c>
     </row>
     <row r="113">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="122">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="123">
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9">
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
     </row>
     <row r="92">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93">
@@ -10618,7 +10618,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="99">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="101">
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="102">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="103">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="105">
@@ -11442,7 +11442,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117">
@@ -11486,7 +11486,7 @@
         </is>
       </c>
       <c r="L117" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="118">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="126">
@@ -12574,7 +12574,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="140">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>131</v>
+        <v>118</v>
       </c>
     </row>
     <row r="142">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="145">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="178">
@@ -16034,7 +16034,7 @@
         </is>
       </c>
       <c r="L204" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="211">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tUBi0IjaXdP2RcNkz9aBGg==</t>
+          <t>ILaIxfZoWEm6+ZNO9g+BLA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CZhz+Wby/02b9Krcu5TCjZT7ooUm4pSeAccyp4itnFc=</t>
+          <t>SbUDxG5VyMf1oFf6AgPJJ3CPLV9SxZ5lBctVrgx4BpE=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>s8DUZNjJ+EWId+PSbFlvxQ==</t>
+          <t>XAZO8Tgy9tc75v+8kg050Q==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SVbwRwriUGD66kN5BMaDuHLLG6biYImwqC45JbKYmnc=</t>
+          <t>F/q/l9AQEiCcHpP6+Z27ik06aWG92GWqnlG15//WQfY=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>lpWoPWUbkpRlEo6DTELPeQ==</t>
+          <t>i0aWEkkf3aQnWao/dshWxg==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>jsldnw4SzH95nQIb3s5ZOV9GoIUGjmjyAGLlrCYYUPs=</t>
+          <t>GLnqBK5dsZyXO5vJr0qFlMSVy0+bqbDQx58wlvI34Cw=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>p5I3y8qUKXn9fLKCkXE8ug==</t>
+          <t>ddb0xltRWWHdJdytezPixw==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IB99yTCutDVx8PTM+QlDSHazME6UTFE3Po6hE3MNy2U=</t>
+          <t>d2NCyAh8/n29DO69p0uNjh42Zw08e4azSXbeLVejFV0=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1TD2fSsscLO8BkT4tShYrA==</t>
+          <t>1zIEJbN8/AmsELFo0NH9qQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PULcxLk35SvaH0dl3sl5LJKGowt1t7VG1whpV5lBshs=</t>
+          <t>WHNINvLrbKLxN9aClOXc+jTf+x+H748XJx7Woko3u2o=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>UfpRRewYUkyWAbIpi+RiOA==</t>
+          <t>tt/tLhMU4O/9E+/m3dbR1w==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>QT5xxv2OGde6tfiWxFkZ7+FE5BG9G6Yq4nHsy6Ej53g=</t>
+          <t>Y7QZYEymlftgo2hQ9MIfuUzvGp9WmHXP5T/9jWWlo/0=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>F99kekQ4V4xTyNlogZKqJw==</t>
+          <t>LrLji6yKUwmvYEPZxgIaZA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>BBfXOGlcprsiAQFHXOBwJAdJSdVdkjTiiaGD8l0K4Rc=</t>
+          <t>TDppOSConwyQWBmbWC7xeg124Cq3quphNuF3ACxulGA=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GUMaAxe68fkBuJNpDqx5NQ==</t>
+          <t>1pBFbc7ne8JUWQGqc0t2mg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TTrtZx9rAcjsGZkEbTyctqli0zrzQ/qQBYP9mgnGF2M=</t>
+          <t>kvJh4DmU4OeqWcTyYGWO7RkTyc2ZRquaHWTzVZ3vHXo=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>h9zcDcqLjNM9HOdlrwxNZA==;I+UXEOIFurtoVh/Y7lPM+A==</t>
+          <t>4XIvywS1qYBJo1hDSP47OA==;ijvzXweh8W9JRuMXwmcNPw==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>btvMpPrup9CT7d3fFZQmb4opl8/AtV0YDi8iPKUjJUs=;LTM8aDgZQSIE80mUGVqhai3iAuIl9fefW49O5LCyEvI=</t>
+          <t>lIfqqQ41ggR1yey839FX3zb59FRyFYeDFehbKJsVxcw=;2FCU1n2g5cf191WnvsLZSab9Xew8rrz2/NCgoV1sXMk=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2W6jr9iB7VXO3R2nLIG9PQ==</t>
+          <t>s9baOaDLaxGEfK1gK3d3Gw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>kvMDQfQrEhRoTp3g6uyO1XSeNBFzlajHM2l/9VsLD6A=</t>
+          <t>IltOXGZsvfQUrQ8prZNh9CSPYLOrXc531mxKuHddO4A=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>xgfVXMvNii26dLmMp+IR4A==</t>
+          <t>v8FyuYdX7tB0E/maTRwVuA==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>GRaVmJ+Fy+wEZr9Iwu+xE6rqqm/5wzFysCYeJc20ciM=</t>
+          <t>myOX90Y+XCIVszTjRwTdGp3An/LUJRorJAobSdabQx0=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>KKWnodhbV7VuKCuTPY1ZmA==</t>
+          <t>mg9w8y61/FhFhN2zX29LMw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>o0iRo9RW9NFB9SoWL/lKItKKeIHR/7l8yWvrPIXiYKo=</t>
+          <t>hZUUCJqKKu7eD6NXEX4qkM+JT/IZ2BsnNuD3otOyZSA=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xNkxNssGot2tT2J+xzo/8g==</t>
+          <t>PTuG+zD69M88ZoeqSR35MA==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Pzst3SrOcQ73kWwWX1ZBAxgTNcUHtUn7jxWmT8BnmHU=</t>
+          <t>FOhRt5SsEbgF57lsnaCr8DzfcOng6uw++6NM0jWwjvg=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PFAkZKRJPlTPEnyD9LGtDw==</t>
+          <t>FhHllmJ2fVQJNHvpQKggDQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ZUxWdoTShk+P2rjNdX56OtECYlyE4I7I45lOd5j1m9A=</t>
+          <t>m66t93G8yW2G/5Z1RJryo4dNTl+RnturB/f/YwtBfp0=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ZjuktToBHb/vx+65Jlcgpw==</t>
+          <t>LML57cFPH0hknrE0/YYpMw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>euw+I3z6MN6BJX8dzC+2exlO3NPr5DUTlwxVrzQFdko=</t>
+          <t>25+e4/+FiKLlh57FKi9bR3xRRpsjoVK1LC5sR8OdOk4=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mp2dw2JGgBOSmEZjgPcnKQ==</t>
+          <t>auLScaIecu2iQhbKVTSBJw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>dLkwo4HTI2HhQNmqkQkDqvkFuMulHCgCeRox6blWp/Q=</t>
+          <t>DKa05WD6VOz4vqb/Bbm59bFWU86IUOmGfr9fW4e02ic=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Vj5fwO9tnroIhzDdhBGqUw==</t>
+          <t>ZHbFGEkfzQFNrb48rnQRCA==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>p1k7dHp41c2yWCY3VAY/4zFicb/UeeoFUQl+qR1/MSc=</t>
+          <t>Dmo6XtS4QP3fAVnUU6Tijz1J9YXLnd24vf/Lq8OYvHI=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Gs5ja5IU6so8EYcGveC/xA==</t>
+          <t>hhpNkrbG1+fXPKYzPPZupg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>BbOoU4gr86QfIvAgNQq2SQCXHwTOmidCnZSLtAqgtKA=</t>
+          <t>rs0jb6Fk0t0Tip6a03N0pS5MjJjreH/8ARF1DfZaeds=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>B4BGYRBIsbHmSNdcV/06zw==</t>
+          <t>WeFgHq+PkHPj0axBg1QS2Q==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>hZ4z7MzZPeJ/ifCANXgV0k2BWUzDgwvpOwS4H6hAp/E=</t>
+          <t>dMotWP9X50GZsOWfbAYevIoHRqKasDoZgF1eHxMNNBs=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>/OBnij4tFRWlRCnuNFh3SA==</t>
+          <t>HnIrDHdP1H8td2jyKsTKjQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>EMO14aWx7BvQioM7H5dI8McHQSf5JyCKLI4XCiAmuEw=</t>
+          <t>ksdb09/WlbIbfDAUuo2ljMgvR46W6qMg8hkr8Y3AQU0=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>W4g+xyTgbY9nrMZm4p1S+A==</t>
+          <t>kX+1I3PlGsvqxUMetHwHAg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>qH7FtR1Ju4YOFuhbwToR2NAX95d7GUb5/YU0EvSocVw=</t>
+          <t>zydsZdWe5VrFL9hfUXYjKgavwkb2+zef0dVb/YBmxbE=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>UfGZMDPoZzeuJ6svBmuhyA==</t>
+          <t>GYxo3Mg7XnpPmRICk9wTYQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>JGA9foTR+FzjXqY01Ow8dHvGmB52lFmMDl2ti5fnVuQ=</t>
+          <t>t9aef8ffNuMfy/LCXmfzsFoKjW9e7xMNmBfVtnz/g0g=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>5XOFan8KXdrVTWzambjejQ==</t>
+          <t>f67asZ1+wRgmdAb08iM93Q==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>NMOhfbS//vHWccpt2MMx1HBKQaRzeCf4h+yymznx8lo=</t>
+          <t>HACYHC2trk5a30IiPNbYeZ5WtQg+q3FuE4PD9rjIyZQ=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>xVXdhLF084DFRZE4OF0mZw==</t>
+          <t>i4NVbEktaFe7FX6WnrPiWA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>4NwxQ2V6kWIwdEXmqL6k2hV9IfPappvEP5GOc5nWsY4=</t>
+          <t>le2BUWTWwkWhWJ4wI/eBVXKVAXa3WkfIpoGYAhO0qPo=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0Nyll2R5Tec12En6d1nIjg==</t>
+          <t>HHcyVRI6dbBoUQDItgB/8A==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>tKrzzva196gnHo/4zbVjl3PNzKPMVEUtgAsdtfKORtI=</t>
+          <t>J2OQnluAKFLU1Y8eWT91vSHDuMgKs3h8is98H8LBMng=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Rkq72IaTjlerjCxNUHNgaQ==</t>
+          <t>hFrXE9cMo5VERpX1TjwS6A==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CDoeGufDAQ+ExPtOMCs199K7Nv6mik+oHnskllAnXaw=</t>
+          <t>piCx6quZYbsEeeeaf4P4vCGnqU9T+9r2zz+BbfQUP9Q=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>LhCX3wby1wf5qdJVJVmBiw==</t>
+          <t>LlY25v4z9Fe/ut1H0r/aAA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>uPiDKHX8hlHj+46PUHzoidg6iYFFNfVwHH7EKb+23yQ=</t>
+          <t>2FskVnKPmKkGUhxbtB4/UkljRUmJZzPGVqIW5dSpnJE=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>t9qykw+YJ6U/Im1Hxriudw==</t>
+          <t>VUoFtq28PfNIE8pvDRUEgA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>pdMWG3a5VAuJlAftd4eQMumC8xtqKgR06ixFb9nLkvs=</t>
+          <t>1QuRnf7sUdjlnm5unZAG8n/9Nh5dS7ToMQM+ukvZEMA=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>DCcj1cvbaTrRqGC7BS/r8Q==</t>
+          <t>/Nar7ehtFDunOFthA8o/BA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>DuPOxQ9uY7owQ41HuKTm/fb5gIRe10Gf4ytyR1z00Rs=</t>
+          <t>fhFakufDU6BWHLjs1SYvVhMP4snc/fj8EL+zf0UTh6s=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>r9jjn5SyiJnIoJ6Rlgc1FA==</t>
+          <t>zmAPNyyN9b7w5A6j8lYwKA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Z68BVlmIegaBLyO6i17fwHfzVsUeePylT0ygcSG//Lk=</t>
+          <t>ECUapJs6mT6UBWa0xocbmSqgOvKZXQQMIevf8KNivTw=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>yJgZote83P8q/F74xiKW4w==</t>
+          <t>1ap3xqeEj7O4AqCTzltJgQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ocjdYaFhylHZPZk/ijF7y3kPnpp3LZYTD7L9okafxTE=</t>
+          <t>nbejQd3P9ZfgE1NH0cvQJ5tXDbQu0S9HMBwsh7RbWrI=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SJuLEIMHpSQArrCKsy3igQ==</t>
+          <t>uhSema47uVuBp5NAXXD22A==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>NDlrEp8hox1S6d+BCMMVeHbzMrfQqTxNla40RsaNnjo=</t>
+          <t>BRnImmCy2xJZU8XyHo25Rc3WuwEv2ZsiqHMwMDauVjI=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KXl3sz5EypHJBo0/sj6uZw==</t>
+          <t>xQCsU09z2zcu1oCTo+kgtw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nfnQcbHIlUl30StkHsG86uit/+SJXzfW5OHK+Oe12v4=</t>
+          <t>PGKCRjHsdn+ntBd8rAJ7RqQQkDcO973tb2LEQI0F9eE=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sJHdXFlC1sXC22F6CvPRCQ==</t>
+          <t>7JnfD/nhMZC32O+00ID+HQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>t4De+mlbaXMybJTAZxPd6xJchxQnsNsyAtRJ/ddg+co=</t>
+          <t>A6g5+6qSNRZwMpzTMBroDu2xczEZqsLUmtM5ou0F8tk=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>5p+kVvNPJwQPIVHxyj4Y0Q==</t>
+          <t>tV8VNsbvldYb+oou3THcbA==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1MI27bnBfYgpIilRvVEETYK/pSgYpnD9xFKjj2j6X18=</t>
+          <t>gLJox07igNB+VvQBxOIQ7AZX6Ee24QS24wXQ1YpFCpg=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>tA9rRtkhVNhU7eet8N8jkA==</t>
+          <t>WI62B5iAdsom9zbcUTw0sQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>LC/dk5IMz4+l/ejNZKA7hmZ4ct/h3uWQugeFltbr8l4=</t>
+          <t>HPfzM+yqxs++4TycSPYQO/GhSFlB/z0i1dAULBmAW9U=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RvOlvGzS+fs+95TyT7e6rA==</t>
+          <t>o7MaRtRyhjJXYZ3UwLMgAg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>UyZHBTeZE4UYGS77ig8dSkoGBoCJDwcUu9UB2qJDIS4=</t>
+          <t>QYCpvPjmnSQxUgqXRdbQMzhdE02vQlkxvvj1xvRjQ+Y=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-28 07:39) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="87">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="107">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="114">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10">
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="101">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="103">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="114">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="120">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -12574,7 +12574,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="140">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="142">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="163">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="171">
@@ -16034,7 +16034,7 @@
         </is>
       </c>
       <c r="L204" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="205">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ILaIxfZoWEm6+ZNO9g+BLA==</t>
+          <t>BiHVnMOornczgvTol6VeGw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SbUDxG5VyMf1oFf6AgPJJ3CPLV9SxZ5lBctVrgx4BpE=</t>
+          <t>V728sNz82IGhcFZUqO57fXCWmuWuSLAJ1iZLummZtW8=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XAZO8Tgy9tc75v+8kg050Q==</t>
+          <t>iNfDRN81OxamnKjx0ueoMg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>F/q/l9AQEiCcHpP6+Z27ik06aWG92GWqnlG15//WQfY=</t>
+          <t>f2hg3CPQzGC+GaVynq0ku5cEWm/GcgQww593UaZBFuU=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>i0aWEkkf3aQnWao/dshWxg==</t>
+          <t>pUUmWw+ln83IdabNbboNRA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GLnqBK5dsZyXO5vJr0qFlMSVy0+bqbDQx58wlvI34Cw=</t>
+          <t>2PUy8+qXbpcOYSWTIuDSmMltC/LEJDUItKUvBQ3WaQM=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ddb0xltRWWHdJdytezPixw==</t>
+          <t>LQdPjCSSRni6WFa1TlHrOg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>d2NCyAh8/n29DO69p0uNjh42Zw08e4azSXbeLVejFV0=</t>
+          <t>kSXxUYVweb/Isc06iaQY8zOvE0BSo0oTRVanzDHoXy0=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1zIEJbN8/AmsELFo0NH9qQ==</t>
+          <t>+vXhffkYj8tNLAD7m2SDOw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WHNINvLrbKLxN9aClOXc+jTf+x+H748XJx7Woko3u2o=</t>
+          <t>54/6Sqqvn/J7OoBo1H4l7pFIacOZe1x5oYPwscjeXUg=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>tt/tLhMU4O/9E+/m3dbR1w==</t>
+          <t>a+9ijCfL0regtOMOiLqO1A==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Y7QZYEymlftgo2hQ9MIfuUzvGp9WmHXP5T/9jWWlo/0=</t>
+          <t>7TCXCsa/msYO+96Y912+3O6cCiZqDzROGWdrizvzl8U=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LrLji6yKUwmvYEPZxgIaZA==</t>
+          <t>2EEsJRXaFERrpULxJrlk4Q==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TDppOSConwyQWBmbWC7xeg124Cq3quphNuF3ACxulGA=</t>
+          <t>WW3YhByc0GH+DDyX0iQWlm9CIhAHne0RVJNsqocXqkg=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1pBFbc7ne8JUWQGqc0t2mg==</t>
+          <t>4Vv4ycbkadMQG7/R4PLnRA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>kvJh4DmU4OeqWcTyYGWO7RkTyc2ZRquaHWTzVZ3vHXo=</t>
+          <t>YyXeHOdBByidk95L5XilpTQRP9zjEkXicH6Gtm7Jr5k=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4XIvywS1qYBJo1hDSP47OA==;ijvzXweh8W9JRuMXwmcNPw==</t>
+          <t>4FK+9ZB7l1H6/JMAQrtKFg==;Frr5AAWSEQSX1u57Fhcv8w==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>lIfqqQ41ggR1yey839FX3zb59FRyFYeDFehbKJsVxcw=;2FCU1n2g5cf191WnvsLZSab9Xew8rrz2/NCgoV1sXMk=</t>
+          <t>rlcorKNhtrUP/jEVSeVugTdLKgO2NNkht0Ov1fZkEDQ=;lSO47vTkhSw9DH9KwB3lji4KMX6IzwsYXF+iZQFbYeY=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>s9baOaDLaxGEfK1gK3d3Gw==</t>
+          <t>V366IeDqIyfQ1UA3T3BU7g==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>IltOXGZsvfQUrQ8prZNh9CSPYLOrXc531mxKuHddO4A=</t>
+          <t>rBfptDKX+WW9RnF8zsg72sQomRmwO7a9en/jMBE0q50=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>v8FyuYdX7tB0E/maTRwVuA==</t>
+          <t>Z8WY092WF0lIBQeDOjAz0A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>myOX90Y+XCIVszTjRwTdGp3An/LUJRorJAobSdabQx0=</t>
+          <t>A8+jNLIEomL4E/DbaZ4W9tkO0eHGAxKyyIaTuSVc448=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>mg9w8y61/FhFhN2zX29LMw==</t>
+          <t>2m3EfASoXmSoQfh8kZS+3w==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>hZUUCJqKKu7eD6NXEX4qkM+JT/IZ2BsnNuD3otOyZSA=</t>
+          <t>xdeiBucuxPMeCpC2idyM3EIPIDCW7NhS1ejsC7X7PkU=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PTuG+zD69M88ZoeqSR35MA==</t>
+          <t>tCyl1OR3rb/fM7gtsek6ZA==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FOhRt5SsEbgF57lsnaCr8DzfcOng6uw++6NM0jWwjvg=</t>
+          <t>vwASiQDzdB07Krmtb9gNbJsLiyHXVq/ayyluyUsjXTE=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FhHllmJ2fVQJNHvpQKggDQ==</t>
+          <t>RV8Gwz3l5Tt+E60uFXXgEQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>m66t93G8yW2G/5Z1RJryo4dNTl+RnturB/f/YwtBfp0=</t>
+          <t>osmCNq8azbd0tBU1t0DL9dUDDj/s2axzq+OhaMRElnI=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LML57cFPH0hknrE0/YYpMw==</t>
+          <t>0gMvwSeJeMrHba6SM5GB2g==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>25+e4/+FiKLlh57FKi9bR3xRRpsjoVK1LC5sR8OdOk4=</t>
+          <t>YHiYFAbHSJpwASEK8mACgEzvLZivWlqZ0l1m1CDUa9A=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>auLScaIecu2iQhbKVTSBJw==</t>
+          <t>H3xeY7MD/wiA4fAXoBMUZw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>DKa05WD6VOz4vqb/Bbm59bFWU86IUOmGfr9fW4e02ic=</t>
+          <t>4Lklue3zH0LV51Ipv64GovWpW2K76Vo1M8pH+4KO1ns=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ZHbFGEkfzQFNrb48rnQRCA==</t>
+          <t>Rql9QzuTsUSGE58FrCUgZQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Dmo6XtS4QP3fAVnUU6Tijz1J9YXLnd24vf/Lq8OYvHI=</t>
+          <t>FDm1Ysod2AhpvIliIaMmuH5ZhlFLYYNgK3s8fgd642c=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>hhpNkrbG1+fXPKYzPPZupg==</t>
+          <t>7gOsLpROdBHdWDmVSLQj6g==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>rs0jb6Fk0t0Tip6a03N0pS5MjJjreH/8ARF1DfZaeds=</t>
+          <t>UhEtTnZA5kVPSh6bepTPcrDlrHcvzxJfGjyLyhMVVRk=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WeFgHq+PkHPj0axBg1QS2Q==</t>
+          <t>aye5JmUgFzI2cdalIRz1MQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dMotWP9X50GZsOWfbAYevIoHRqKasDoZgF1eHxMNNBs=</t>
+          <t>Dde+h04gVU96W99cs4U/IHrpKEgz6VinwJlwzVnNA24=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>HnIrDHdP1H8td2jyKsTKjQ==</t>
+          <t>iW3JYZTVMQyeZEC/gp3cog==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ksdb09/WlbIbfDAUuo2ljMgvR46W6qMg8hkr8Y3AQU0=</t>
+          <t>pQsu5F0GJKmj8bo+szG+8V9Rj5H0uVZ/hAilIwEGT9M=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>kX+1I3PlGsvqxUMetHwHAg==</t>
+          <t>T2Io01SkMslCdFN6Urd/GQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>zydsZdWe5VrFL9hfUXYjKgavwkb2+zef0dVb/YBmxbE=</t>
+          <t>KcpOLjWenbj4M/nVCRsGa5K5rmau6bFLvbOs/NKuvkI=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GYxo3Mg7XnpPmRICk9wTYQ==</t>
+          <t>7w8bQthjJhB4GZlgAkStaQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>t9aef8ffNuMfy/LCXmfzsFoKjW9e7xMNmBfVtnz/g0g=</t>
+          <t>csnDhZuhewK4wG6+G/5FGoGXUKb1XHdsY9VokUjPocg=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>f67asZ1+wRgmdAb08iM93Q==</t>
+          <t>0HSulEBeU0D7QGOTDodIfg==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>HACYHC2trk5a30IiPNbYeZ5WtQg+q3FuE4PD9rjIyZQ=</t>
+          <t>8sCN3h2tHLcGbk5jjQctAxzCsds+3hV6kL9P9GFxE6k=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>i4NVbEktaFe7FX6WnrPiWA==</t>
+          <t>wAz4j6n7eRAR64tfd4a+1g==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>le2BUWTWwkWhWJ4wI/eBVXKVAXa3WkfIpoGYAhO0qPo=</t>
+          <t>5sqhIxiWqFOvjSA9GbokmFbJX/9P+taOwiwsNnFGzzY=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HHcyVRI6dbBoUQDItgB/8A==</t>
+          <t>U6g/gP2wH2ORktEgolNIqA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>J2OQnluAKFLU1Y8eWT91vSHDuMgKs3h8is98H8LBMng=</t>
+          <t>4nYGYAAHXZZHJ78SVZTdgpHJth5dfnE+/ufz2zTFAv4=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>hFrXE9cMo5VERpX1TjwS6A==</t>
+          <t>I6c5bdQhBQFWpg6lg+5f/A==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>piCx6quZYbsEeeeaf4P4vCGnqU9T+9r2zz+BbfQUP9Q=</t>
+          <t>nyGERz36mOXZBH8SEjiw5XWyn/8FTejMNlpOYdjQNAk=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>LlY25v4z9Fe/ut1H0r/aAA==</t>
+          <t>34OOdqWW8cGX9WXbxU2fKg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2FskVnKPmKkGUhxbtB4/UkljRUmJZzPGVqIW5dSpnJE=</t>
+          <t>T8vhZbl/alaTKukTeD+WgpUUsoyHUs3m+ea/r3SrnsA=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>VUoFtq28PfNIE8pvDRUEgA==</t>
+          <t>XSZKEelZCDfkGgQsAlVmKA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1QuRnf7sUdjlnm5unZAG8n/9Nh5dS7ToMQM+ukvZEMA=</t>
+          <t>GemnbLbxHtVwVybpgpLvc0uzoBs3/rxZVPzcVnHXON4=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>/Nar7ehtFDunOFthA8o/BA==</t>
+          <t>g7B7XHd2RcxbhQSOzmZtqw==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>fhFakufDU6BWHLjs1SYvVhMP4snc/fj8EL+zf0UTh6s=</t>
+          <t>MglpQAIUaRaK3AtZaZykpmJ7PGenirJwgEl5QXFGt58=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>zmAPNyyN9b7w5A6j8lYwKA==</t>
+          <t>TCFNPVI4h57/ADNb9OxpwQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ECUapJs6mT6UBWa0xocbmSqgOvKZXQQMIevf8KNivTw=</t>
+          <t>R5c3TW96DXGtaxD0NEPwROFl6W3zCdmHiAIENgVC8Ws=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1ap3xqeEj7O4AqCTzltJgQ==</t>
+          <t>JmkH///NmYQU08AtA+Da3w==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>nbejQd3P9ZfgE1NH0cvQJ5tXDbQu0S9HMBwsh7RbWrI=</t>
+          <t>CfRmtOjQGILSDtv+wTkoSa7+vDHkPV5/23PLI6HnjkI=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>uhSema47uVuBp5NAXXD22A==</t>
+          <t>COU+2JOHpTcvu1WMrWwOOA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BRnImmCy2xJZU8XyHo25Rc3WuwEv2ZsiqHMwMDauVjI=</t>
+          <t>B1wJf/CHh9N/R3M+FyG38PHt6Z0ttV/YOPD5IG0vgeo=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>xQCsU09z2zcu1oCTo+kgtw==</t>
+          <t>nrQRmJIXhTmmSu0cQtRJFw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PGKCRjHsdn+ntBd8rAJ7RqQQkDcO973tb2LEQI0F9eE=</t>
+          <t>H7+h+ArM4UgMu22xXxhBLOdZYGwuazp8hIzC0bfyjjs=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>7JnfD/nhMZC32O+00ID+HQ==</t>
+          <t>5+iAcvcs4jHMod4RlZk5FA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A6g5+6qSNRZwMpzTMBroDu2xczEZqsLUmtM5ou0F8tk=</t>
+          <t>hbh93j+jmKXRijHy9aCJ+lr2Yo6QeJHBx8hMOf2hgnE=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>tV8VNsbvldYb+oou3THcbA==</t>
+          <t>FIkYkqMjkgS9XlxYW4F1Nw==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>gLJox07igNB+VvQBxOIQ7AZX6Ee24QS24wXQ1YpFCpg=</t>
+          <t>UdProHbVWpkB6ErKJvQWQxf0Sk9Kj+C2q9O0zz9R7Fc=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WI62B5iAdsom9zbcUTw0sQ==</t>
+          <t>bKjvQhNqBbnCSPzrnpx8ww==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>HPfzM+yqxs++4TycSPYQO/GhSFlB/z0i1dAULBmAW9U=</t>
+          <t>IoewI2Kd5Tr5b8FOC4CVApdXdQk2ItLrygcYVEIDJ7s=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>o7MaRtRyhjJXYZ3UwLMgAg==</t>
+          <t>FsE1cgoV/gD4t3te2Tyvtg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>QYCpvPjmnSQxUgqXRdbQMzhdE02vQlkxvvj1xvRjQ+Y=</t>
+          <t>I3AXuolyP/JVE+bPfw5MudQEJdHfYwMu3Mne5U/PV0M=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-29 07:39) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="87">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="114">
@@ -6086,7 +6086,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10">
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="103">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="120">
@@ -12574,7 +12574,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="140">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
     </row>
     <row r="142">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="163">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="171">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BiHVnMOornczgvTol6VeGw==</t>
+          <t>TGye8oS9xOO2zCkYdFPtiA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>V728sNz82IGhcFZUqO57fXCWmuWuSLAJ1iZLummZtW8=</t>
+          <t>Ny3kYbHPjzNXfrWf5WDJ70awLpzUeQbrWxsZINHqcxo=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>iNfDRN81OxamnKjx0ueoMg==</t>
+          <t>2Vwe3otRzL4YgCuZb05RyA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>f2hg3CPQzGC+GaVynq0ku5cEWm/GcgQww593UaZBFuU=</t>
+          <t>z3+4Xr3DMEk2fdAJpfzJvhUlxnH8j/R5jV6D1goXd+4=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pUUmWw+ln83IdabNbboNRA==</t>
+          <t>DUQeOLTQMVP8OE+6unMGGA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2PUy8+qXbpcOYSWTIuDSmMltC/LEJDUItKUvBQ3WaQM=</t>
+          <t>zKXlbTd8b/sn9W6LrTjEgKqeCxzNUOD+v1otuZoANwE=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LQdPjCSSRni6WFa1TlHrOg==</t>
+          <t>YECCQJXGmkYXsm8cbM2lXQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>kSXxUYVweb/Isc06iaQY8zOvE0BSo0oTRVanzDHoXy0=</t>
+          <t>qoVsihzO2Q7ltpdGW1Z4h0y3cS9UatyC/sUfHYtkBfg=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+vXhffkYj8tNLAD7m2SDOw==</t>
+          <t>pb5Rv3PSQAdSHdMuKT/bsQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>54/6Sqqvn/J7OoBo1H4l7pFIacOZe1x5oYPwscjeXUg=</t>
+          <t>mBkqDxWbjAtQm2K0A0xZN6q1EtM7iPQXwTehCcCkC50=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>a+9ijCfL0regtOMOiLqO1A==</t>
+          <t>Hx0H+NSrYQlbveg/BlFQ6g==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7TCXCsa/msYO+96Y912+3O6cCiZqDzROGWdrizvzl8U=</t>
+          <t>sRckP+opjMMrnfdv/UXiyN9W7owQPeVjFeSDknKvS40=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2EEsJRXaFERrpULxJrlk4Q==</t>
+          <t>iI0jRh5k0/emfmPD9qQhoA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>WW3YhByc0GH+DDyX0iQWlm9CIhAHne0RVJNsqocXqkg=</t>
+          <t>8UYFtR+6FzRxJtUeAl9+406XkoiQtSdRfHucr8UNSaI=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4Vv4ycbkadMQG7/R4PLnRA==</t>
+          <t>3SNynI6r4rFG1jq+GrnUOw==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>YyXeHOdBByidk95L5XilpTQRP9zjEkXicH6Gtm7Jr5k=</t>
+          <t>maayaN1H4V8QoOekzG1/F8vIhvFUl18ljs4n6Yt1oKE=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4FK+9ZB7l1H6/JMAQrtKFg==;Frr5AAWSEQSX1u57Fhcv8w==</t>
+          <t>HLC4DEAdCau6mgmNEbKDZQ==;Angkb4ybiTcw16Xvrv1+fQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>rlcorKNhtrUP/jEVSeVugTdLKgO2NNkht0Ov1fZkEDQ=;lSO47vTkhSw9DH9KwB3lji4KMX6IzwsYXF+iZQFbYeY=</t>
+          <t>1ggpHN2SSnQqdNCG4G4kLVdOyp0bRtNRp9SBgEuZ1EY=;xl8V+OV55jJnylbgHwUogyYAWptrJLOCYqwMt9PvCmw=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>V366IeDqIyfQ1UA3T3BU7g==</t>
+          <t>IMnENL5PePsFEEa38miPAQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>rBfptDKX+WW9RnF8zsg72sQomRmwO7a9en/jMBE0q50=</t>
+          <t>SQPbfwkCKU5eXbkmFcDIi7TjB5knRDgvYbucwC1AcvM=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Z8WY092WF0lIBQeDOjAz0A==</t>
+          <t>s9DsWJcD8abbLangEbm/eA==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A8+jNLIEomL4E/DbaZ4W9tkO0eHGAxKyyIaTuSVc448=</t>
+          <t>jXMqYfQD4ULC6LEThq4G47TFtzylb4NSaslggRCxwl4=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2m3EfASoXmSoQfh8kZS+3w==</t>
+          <t>QbJ6mMDZFMqYHEsdtWM14Q==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>xdeiBucuxPMeCpC2idyM3EIPIDCW7NhS1ejsC7X7PkU=</t>
+          <t>WZy3n4kUJaw1Kw8mTZ87YZ0q5dzDBb4w9eP4b7fM560=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>tCyl1OR3rb/fM7gtsek6ZA==</t>
+          <t>sKP7cMLC2g74n4c1OEWV3g==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>vwASiQDzdB07Krmtb9gNbJsLiyHXVq/ayyluyUsjXTE=</t>
+          <t>/89gchQ8TDUfmwAERHzP92e7Zj0apSrHdyA5qOKTS+4=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RV8Gwz3l5Tt+E60uFXXgEQ==</t>
+          <t>dIt+GbNBIOzWinN5U6ellg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>osmCNq8azbd0tBU1t0DL9dUDDj/s2axzq+OhaMRElnI=</t>
+          <t>cHJa1iT+B2r4+LykNebG2j7xYPXbsXFi+J9ryXLb2FU=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0gMvwSeJeMrHba6SM5GB2g==</t>
+          <t>iEYVOWGajUGBU3RmBbCsMw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>YHiYFAbHSJpwASEK8mACgEzvLZivWlqZ0l1m1CDUa9A=</t>
+          <t>VAviw/5MzGbkQwLOD7fKogQVvP1sRKydAikizksfxCE=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>H3xeY7MD/wiA4fAXoBMUZw==</t>
+          <t>wZ2H0KJ/TNcca6Alm15wxQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4Lklue3zH0LV51Ipv64GovWpW2K76Vo1M8pH+4KO1ns=</t>
+          <t>PIsRN+1ktT3r9zfV3GpagNrT9zoe55okIse/rcPncA0=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Rql9QzuTsUSGE58FrCUgZQ==</t>
+          <t>GbXe8n3YnTYf2OpM8P5JPg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>FDm1Ysod2AhpvIliIaMmuH5ZhlFLYYNgK3s8fgd642c=</t>
+          <t>xQyhMJVLbB+05Ph7rNW5yDngZOIy7w4TOqaaJiHdiLs=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>7gOsLpROdBHdWDmVSLQj6g==</t>
+          <t>AWmrTbLKFZTxw4QsDiYa7A==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>UhEtTnZA5kVPSh6bepTPcrDlrHcvzxJfGjyLyhMVVRk=</t>
+          <t>ac84uGq+PxusQj02sRieHYqaktRNviELmsOnF+wcj28=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>aye5JmUgFzI2cdalIRz1MQ==</t>
+          <t>plUmwYL5A0LN/qjMP2vupg==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Dde+h04gVU96W99cs4U/IHrpKEgz6VinwJlwzVnNA24=</t>
+          <t>BLu7mtnVp1X97JZAlJveK9Psb9Pws6ep8bHU/mcMMj8=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>iW3JYZTVMQyeZEC/gp3cog==</t>
+          <t>W5cRWkcbx3nVmblzLxbOSg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>pQsu5F0GJKmj8bo+szG+8V9Rj5H0uVZ/hAilIwEGT9M=</t>
+          <t>B12/4rnrlfYBPbTkhWp5VWPyH25fk9Ah2Fa5ltiNeoA=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>T2Io01SkMslCdFN6Urd/GQ==</t>
+          <t>TabeuDxNq0dxO8kXtfWG4w==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>KcpOLjWenbj4M/nVCRsGa5K5rmau6bFLvbOs/NKuvkI=</t>
+          <t>T5ugo17PP3xaoIUtiha1o+o9bFl5fK5ioXpJ74g+Wjs=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7w8bQthjJhB4GZlgAkStaQ==</t>
+          <t>koV75PgRyY5AGLFgQ/sfmA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>csnDhZuhewK4wG6+G/5FGoGXUKb1XHdsY9VokUjPocg=</t>
+          <t>1cC5UhLuFh3AJt04xhSjmTri0N0XYtqw6KRZmTrPvG0=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0HSulEBeU0D7QGOTDodIfg==</t>
+          <t>YhN+Fp5avgB6WppuM+UW0Q==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>8sCN3h2tHLcGbk5jjQctAxzCsds+3hV6kL9P9GFxE6k=</t>
+          <t>vH1IiK1Q5kbepEVVo0Dx7vjDA4tOg7fUEehfxhIpc/g=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>wAz4j6n7eRAR64tfd4a+1g==</t>
+          <t>7kLrDV/jpuBVhrzq/worAQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>5sqhIxiWqFOvjSA9GbokmFbJX/9P+taOwiwsNnFGzzY=</t>
+          <t>p19NWDIjRQc6Pbxq94rstYJm1a7bDtig7KsOM7/eN+I=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>U6g/gP2wH2ORktEgolNIqA==</t>
+          <t>GqbQ4I2gfzsrMNXgTEyWWA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4nYGYAAHXZZHJ78SVZTdgpHJth5dfnE+/ufz2zTFAv4=</t>
+          <t>5fVHHKphHqJXaxPEi4ztcCArjdX+W16qcumwvx1+orY=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>I6c5bdQhBQFWpg6lg+5f/A==</t>
+          <t>BRClmasgllE1LQzbsDasMA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>nyGERz36mOXZBH8SEjiw5XWyn/8FTejMNlpOYdjQNAk=</t>
+          <t>zeLUURuzYjXFxITn81aAWOFXZeoZJ6vS1pRc+TOFQb8=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>34OOdqWW8cGX9WXbxU2fKg==</t>
+          <t>GO9BTBOd9abiS8UktMdkWg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>T8vhZbl/alaTKukTeD+WgpUUsoyHUs3m+ea/r3SrnsA=</t>
+          <t>zvpQs44mTbv3uWXLd6CZzk3DAERoas+5/PzfcKWtiBo=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>XSZKEelZCDfkGgQsAlVmKA==</t>
+          <t>GavPgKTPGqsUSSld9YFvYg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>GemnbLbxHtVwVybpgpLvc0uzoBs3/rxZVPzcVnHXON4=</t>
+          <t>rIY2pFFB9nZKF6T/KbHcavV0Aumn04whPqji9JYhr2E=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>g7B7XHd2RcxbhQSOzmZtqw==</t>
+          <t>xcCpkyP8VsDwjwQ5ZlA++w==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>MglpQAIUaRaK3AtZaZykpmJ7PGenirJwgEl5QXFGt58=</t>
+          <t>CZ/dvKalLiY+zQB8xHte5PkgOXK5LqDVrnODSkrTqgA=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TCFNPVI4h57/ADNb9OxpwQ==</t>
+          <t>xHS3APpypT9CN7VpDSTrxw==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>R5c3TW96DXGtaxD0NEPwROFl6W3zCdmHiAIENgVC8Ws=</t>
+          <t>7ywuKRXgJEfUoBQNG/xNuX14gm74lUOEprb1YDUVyTk=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>JmkH///NmYQU08AtA+Da3w==</t>
+          <t>aogvr08jnqYewdvD9Lq8sw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CfRmtOjQGILSDtv+wTkoSa7+vDHkPV5/23PLI6HnjkI=</t>
+          <t>1HRzg9WDEQwZWax+xbSPayXA4tbiZGZF5KxlhaqQYYk=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>COU+2JOHpTcvu1WMrWwOOA==</t>
+          <t>egD9IcbNihseWeScd5t2iA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>B1wJf/CHh9N/R3M+FyG38PHt6Z0ttV/YOPD5IG0vgeo=</t>
+          <t>jDjguY/efOcM60BkFucG+RDlupjZrx+POgh5QypllQQ=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>nrQRmJIXhTmmSu0cQtRJFw==</t>
+          <t>cyojw7Ci/Ga31cO9xdx7Pw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>H7+h+ArM4UgMu22xXxhBLOdZYGwuazp8hIzC0bfyjjs=</t>
+          <t>Oc5xFwn+qlLSP1Imfx12p0N8osJUYe7rgpcF5/iqV7w=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>5+iAcvcs4jHMod4RlZk5FA==</t>
+          <t>uAG7TUgN9UHakIIB3df+qw==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>hbh93j+jmKXRijHy9aCJ+lr2Yo6QeJHBx8hMOf2hgnE=</t>
+          <t>zn7FsCXMMEGMyxN4BgOtpCb7yhttqMAUX7jlUaZstEw=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FIkYkqMjkgS9XlxYW4F1Nw==</t>
+          <t>cU44LM7wIzxBe5o+unVotQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>UdProHbVWpkB6ErKJvQWQxf0Sk9Kj+C2q9O0zz9R7Fc=</t>
+          <t>Qy83EFderZnNu1gWHJVoBWthcxdWMPmeHJeKdd1LWBY=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>bKjvQhNqBbnCSPzrnpx8ww==</t>
+          <t>blQZ1ezudMsNdZE3JTBZyg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>IoewI2Kd5Tr5b8FOC4CVApdXdQk2ItLrygcYVEIDJ7s=</t>
+          <t>pv/uzeobtl0K18rNY9+WBoagpB4HnzdKYuB66C1urlo=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FsE1cgoV/gD4t3te2Tyvtg==</t>
+          <t>QMDZQysbSKKOMWdwWTtrDQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>I3AXuolyP/JVE+bPfw5MudQEJdHfYwMu3Mne5U/PV0M=</t>
+          <t>N0aUMSX9/VRduDVQw5rGyYSmKQS7WWga3vFJtCbiPdQ=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-30 07:39) - 115 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="46">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="54">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2799,12 +2799,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2871,12 +2871,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a22fe5fb-0b92-436c-b710-db69d8ea7c47&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -2943,12 +2943,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 06-2025</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a22fe5fb-0b92-436c-b710-db69d8ea7c47&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -2979,12 +2979,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PARTICIPACION VENTAS CCU 06-2025</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ed3b5a8c-8ac6-4d65-8961-df938488eb29&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS DISTR</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=74da6bde-8f40-4f5a-881e-c79da99f35a1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ed3b5a8c-8ac6-4d65-8961-df938488eb29&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -3051,12 +3051,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PRESUPUESTO MARKETING</t>
+          <t>PRECIOS Y OFERTAS DISTR</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cf5e22c9-8925-4779-8f00-d8de2fa957eb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=74da6bde-8f40-4f5a-881e-c79da99f35a1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -3087,12 +3087,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE OFERTAS</t>
+          <t>PRESUPUESTO MARKETING</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=467411be-b152-4571-aab6-634eb4bf23fc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cf5e22c9-8925-4779-8f00-d8de2fa957eb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -3123,12 +3123,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO DE OFERTAS</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2271183e-fad9-4f2f-94a4-656ddc3e2327&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=467411be-b152-4571-aab6-634eb4bf23fc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -3159,12 +3159,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0f0d31e7-0dbf-4e4b-b4bf-79b7b6781d35&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2271183e-fad9-4f2f-94a4-656ddc3e2327&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -3195,12 +3195,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>TRAFICO</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ffd69225-dff5-4250-8c81-775a75de3777&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0f0d31e7-0dbf-4e4b-b4bf-79b7b6781d35&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -3231,12 +3231,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a09b2740-4617-4450-a263-e63c7ab47158&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ffd69225-dff5-4250-8c81-775a75de3777&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -3267,12 +3267,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4bdda3e7-2a7d-4b74-a484-4551b4873c03&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a09b2740-4617-4450-a263-e63c7ab47158&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>212</v>
+        <v>225</v>
       </c>
     </row>
     <row r="85">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="87">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="90">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="93">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="95">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="107">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="115">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="121">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="122">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="123">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="126">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -6467,7 +6467,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -6478,11 +6478,11 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>18fd2917-e128-47d7-b930-81698225d577</t>
+          <t>c81e4915-018b-44c6-a93d-efe70059b2ac</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -6498,12 +6498,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FINANZAS</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -6511,7 +6511,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -6522,11 +6522,11 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>ef4634d6-33e3-4dc4-a17c-6bd0b81ec138</t>
+          <t>18fd2917-e128-47d7-b930-81698225d577</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -6555,7 +6555,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -6566,7 +6566,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>e6339ca7-bf01-48b1-a5ce-930d679671a2</t>
+          <t>ef4634d6-33e3-4dc4-a17c-6bd0b81ec138</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -6586,35 +6586,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>FINANZAS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COMPARATIVO 06-2025</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>COMPARATIVO</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>06-2025</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>COMPARATIVO JUNIO 2025</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Junio - 25</t>
-        </is>
-      </c>
+          <t>CASH FLOW</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -6622,11 +6610,11 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>e9341165-ec5f-48f9-abfd-d7fe80c14842</t>
+          <t>e6339ca7-bf01-48b1-a5ce-930d679671a2</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -6647,7 +6635,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2025</t>
+          <t>COMPARATIVO 06-2025</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -6658,17 +6646,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>06-2025</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>COMPARATIVO JULIO 2025</t>
+          <t>COMPARATIVO JUNIO 2025</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Junio - 25</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6678,7 +6666,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>0a2ec774-224d-49f8-be1c-a0bf9568e471</t>
+          <t>e9341165-ec5f-48f9-abfd-d7fe80c14842</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -6703,7 +6691,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2025</t>
+          <t>COMPARATIVO 07-2025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -6714,17 +6702,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>COMPARATIVO AGOSTO 2025</t>
+          <t>COMPARATIVO JULIO 2025</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -6734,7 +6722,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>e15c4cf7-8e43-4586-b5d6-3f23aa9e5738</t>
+          <t>0a2ec774-224d-49f8-be1c-a0bf9568e471</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -6759,7 +6747,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2025</t>
+          <t>COMPARATIVO 08-2025</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -6770,17 +6758,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>COMPARATIVO SEPTIEMBRE 2025</t>
+          <t>COMPARATIVO AGOSTO 2025</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -6790,7 +6778,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>9c210891-9419-44fd-8ba4-e3857e7d805b</t>
+          <t>e15c4cf7-8e43-4586-b5d6-3f23aa9e5738</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -6815,7 +6803,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>COMPARATIVO 10-2025</t>
+          <t>COMPARATIVO 09-2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -6826,17 +6814,17 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>COMPARATIVO OCTUBRE 2025</t>
+          <t>COMPARATIVO SEPTIEMBRE 2025</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -6846,7 +6834,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>0fe483f9-028b-417e-8ef5-8f93156abcbe</t>
+          <t>9c210891-9419-44fd-8ba4-e3857e7d805b</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -6871,7 +6859,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>COMPARATIVO 11-2025</t>
+          <t>COMPARATIVO 10-2025</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -6882,17 +6870,17 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>COMPARATIVO NOVIEMBRE 2025</t>
+          <t>COMPARATIVO OCTUBRE 2025</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -6902,7 +6890,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>07f8cb25-b8f7-48a3-af1e-b5c1fd3e109f</t>
+          <t>0fe483f9-028b-417e-8ef5-8f93156abcbe</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -6927,7 +6915,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>COMPARATIVO 12-2025</t>
+          <t>COMPARATIVO 11-2025</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -6938,17 +6926,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>COMPARATIVO DICIEMBRE 2025</t>
+          <t>COMPARATIVO NOVIEMBRE 2025</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -6958,7 +6946,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>9ece0bac-ba3c-4063-a0eb-03b231f021d5</t>
+          <t>07f8cb25-b8f7-48a3-af1e-b5c1fd3e109f</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -6983,7 +6971,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>COMPARATIVO 01-2026</t>
+          <t>COMPARATIVO 12-2025</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -6994,17 +6982,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>COMPARATIVO ENERO 2026</t>
+          <t>COMPARATIVO DICIEMBRE 2025</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -7014,7 +7002,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>d94dbbd9-6cd5-4c9a-94a4-4e5a8bc7c8a1</t>
+          <t>9ece0bac-ba3c-4063-a0eb-03b231f021d5</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -7039,7 +7027,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>COMPARATIVO 02-2026</t>
+          <t>COMPARATIVO 01-2026</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -7050,17 +7038,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>COMPARATIVO FEBRERO 2026</t>
+          <t>COMPARATIVO ENERO 2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -7070,7 +7058,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>3832edd0-03c0-4ff1-8a1f-abf56dd93932</t>
+          <t>d94dbbd9-6cd5-4c9a-94a4-4e5a8bc7c8a1</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -7095,7 +7083,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>COMPARATIVO 03-2026</t>
+          <t>COMPARATIVO 02-2026</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -7106,17 +7094,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>COMPARATIVO MARZO 2026</t>
+          <t>COMPARATIVO FEBRERO 2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -7126,7 +7114,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>20d7c15a-131e-4488-831e-d1fe0804779c</t>
+          <t>3832edd0-03c0-4ff1-8a1f-abf56dd93932</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -7151,7 +7139,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>COMPARATIVO 04-2026</t>
+          <t>COMPARATIVO 03-2026</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -7162,17 +7150,17 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>COMPARATIVO ABRIL 2026</t>
+          <t>COMPARATIVO MARZO 2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -7182,7 +7170,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>ddc96523-0162-4bc1-8a67-c5b00e1a7b5c</t>
+          <t>20d7c15a-131e-4488-831e-d1fe0804779c</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -7207,7 +7195,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>COMPARATIVO 05-2026</t>
+          <t>COMPARATIVO 04-2026</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -7218,17 +7206,17 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>COMPARATIVO MAYO 2026</t>
+          <t>COMPARATIVO ABRIL 2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -7238,7 +7226,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>7d56118f-e9a2-4439-af4e-3f6d4eb77929</t>
+          <t>ddc96523-0162-4bc1-8a67-c5b00e1a7b5c</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -7263,7 +7251,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>COMPARATIVO 06-2026</t>
+          <t>COMPARATIVO 05-2026</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -7274,17 +7262,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>COMPARATIVO JUNIO 2026</t>
+          <t>COMPARATIVO MAYO 2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -7294,11 +7282,11 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>e87b9f6f-d894-4e54-9353-f17aa155e82b</t>
+          <t>7d56118f-e9a2-4439-af4e-3f6d4eb77929</t>
         </is>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -7319,7 +7307,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2026</t>
+          <t>COMPARATIVO 06-2026</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -7330,17 +7318,17 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>COMPARATIVO JULIO 2026</t>
+          <t>COMPARATIVO JUNIO 2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -7350,11 +7338,11 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>402b5c26-c94e-44f2-958b-e71cb071ff31</t>
+          <t>e87b9f6f-d894-4e54-9353-f17aa155e82b</t>
         </is>
       </c>
       <c r="L34" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -7375,7 +7363,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>COMPARATIVO 07-2026</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -7386,17 +7374,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>COMPARATIVO AGOSTO 2026</t>
+          <t>COMPARATIVO JULIO 2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -7406,11 +7394,11 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>4e0903c4-5dde-45ce-ad9f-6aed6e2a4136</t>
+          <t>402b5c26-c94e-44f2-958b-e71cb071ff31</t>
         </is>
       </c>
       <c r="L35" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
@@ -7431,7 +7419,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -7442,17 +7430,17 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>COMPARATIVO SEPTIEMBRE 2026</t>
+          <t>COMPARATIVO AGOSTO 2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -7462,11 +7450,11 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>9387acc1-2f91-4921-9891-fb194c770f25</t>
+          <t>4e0903c4-5dde-45ce-ad9f-6aed6e2a4136</t>
         </is>
       </c>
       <c r="L36" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37">
@@ -7487,18 +7475,30 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>COMPARATIVO</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Comparativo Cervezas</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>COMPARATIVO SEPTIEMBRE 2026</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -7506,11 +7506,11 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>b427136c-6785-4e5f-8e88-026b03a2bbe1</t>
+          <t>9387acc1-2f91-4921-9891-fb194c770f25</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -7539,7 +7539,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Comportamiento Clientes</t>
+          <t>Comparativo Cervezas</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -7550,11 +7550,11 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>45ca0371-6f94-430e-be96-2ec8fc691b21</t>
+          <t>b427136c-6785-4e5f-8e88-026b03a2bbe1</t>
         </is>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -7583,7 +7583,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Consumos por cliente</t>
+          <t>Comportamiento Clientes</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>27dfaf71-9641-46a8-a9d2-21a7299ca705</t>
+          <t>45ca0371-6f94-430e-be96-2ec8fc691b21</t>
         </is>
       </c>
       <c r="L39" t="n">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -7627,7 +7627,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>Consumos por cliente</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -7638,11 +7638,11 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>ab000668-c7ee-4c12-8689-e4afdbe23b96</t>
+          <t>27dfaf71-9641-46a8-a9d2-21a7299ca705</t>
         </is>
       </c>
       <c r="L40" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -7671,7 +7671,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -7682,11 +7682,11 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>899444c9-cd01-4bcf-b726-d4ae8d7fa432</t>
+          <t>ab000668-c7ee-4c12-8689-e4afdbe23b96</t>
         </is>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -7715,7 +7715,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -7726,11 +7726,11 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>595175a9-fe3a-49ce-abde-bd1b578273ff</t>
+          <t>899444c9-cd01-4bcf-b726-d4ae8d7fa432</t>
         </is>
       </c>
       <c r="L42" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -7759,7 +7759,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -7770,11 +7770,11 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>883ebe8e-09ee-4631-b55b-337f9560d8ac</t>
+          <t>595175a9-fe3a-49ce-abde-bd1b578273ff</t>
         </is>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -7803,7 +7803,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>363d9b37-f245-4192-9224-0b00b4fd1ea5</t>
+          <t>883ebe8e-09ee-4631-b55b-337f9560d8ac</t>
         </is>
       </c>
       <c r="L44" t="n">
@@ -7839,30 +7839,18 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2025</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>HECTOLITROS</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>06-2025</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 25</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Junio - 25</t>
-        </is>
-      </c>
+          <t>FRATELLI REPRESENTADAS 2026</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -7870,7 +7858,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>e03d8d14-befe-40b7-b6ab-4472bef23ff7</t>
+          <t>363d9b37-f245-4192-9224-0b00b4fd1ea5</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -7895,7 +7883,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2025</t>
+          <t>HECTOLITROS 06-2025</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -7906,17 +7894,17 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>06-2025</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 25</t>
+          <t>Informe Hctos - Junio 25</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Junio - 25</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -7926,7 +7914,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>9e7a5358-3efa-4301-ad21-e924721689b5</t>
+          <t>e03d8d14-befe-40b7-b6ab-4472bef23ff7</t>
         </is>
       </c>
       <c r="L46" t="n">
@@ -7951,7 +7939,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2025</t>
+          <t>HECTOLITROS 07-2025</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -7962,17 +7950,17 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 25</t>
+          <t>Informe Hctos - Julio 25</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -7982,7 +7970,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>9e294012-4f82-47df-9c9f-5375df0a5e69</t>
+          <t>9e7a5358-3efa-4301-ad21-e924721689b5</t>
         </is>
       </c>
       <c r="L47" t="n">
@@ -8007,7 +7995,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2025</t>
+          <t>HECTOLITROS 08-2025</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -8018,17 +8006,17 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 25</t>
+          <t>Informe Hctos - Agosto 25</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -8038,7 +8026,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>43799b86-b983-4162-8c36-dd40b7aac74b</t>
+          <t>9e294012-4f82-47df-9c9f-5375df0a5e69</t>
         </is>
       </c>
       <c r="L48" t="n">
@@ -8063,7 +8051,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2025</t>
+          <t>HECTOLITROS 09-2025</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -8074,17 +8062,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 25</t>
+          <t>Informe Hctos - Septiembre 25</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -8094,7 +8082,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>1c86f6da-ba1b-4e21-b7b1-e91107da1bee</t>
+          <t>43799b86-b983-4162-8c36-dd40b7aac74b</t>
         </is>
       </c>
       <c r="L49" t="n">
@@ -8119,7 +8107,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>HECTOLITROS 11-2025</t>
+          <t>HECTOLITROS 10-2025</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -8130,17 +8118,17 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Informe Hctos - Noviembre 25</t>
+          <t>Informe Hctos - Octubre 25</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -8150,7 +8138,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>d1aed816-e28a-4ffb-a158-06ef60b75add</t>
+          <t>1c86f6da-ba1b-4e21-b7b1-e91107da1bee</t>
         </is>
       </c>
       <c r="L50" t="n">
@@ -8175,7 +8163,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>HECTOLITROS 12-2025</t>
+          <t>HECTOLITROS 11-2025</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -8186,17 +8174,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Informe Hctos - Diciembre 25</t>
+          <t>Informe Hctos - Noviembre 25</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -8206,7 +8194,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>11c20815-6856-4b18-8729-d9a7e64c6496</t>
+          <t>d1aed816-e28a-4ffb-a158-06ef60b75add</t>
         </is>
       </c>
       <c r="L51" t="n">
@@ -8231,7 +8219,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>HECTOLITROS 01-2026</t>
+          <t>HECTOLITROS 12-2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -8242,17 +8230,17 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Informe Hctos - Enero 26</t>
+          <t>Informe Hctos - Diciembre 25</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -8262,7 +8250,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>044d5eda-11e1-4f03-8af6-58eea7a265e5</t>
+          <t>11c20815-6856-4b18-8729-d9a7e64c6496</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -8287,7 +8275,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>HECTOLITROS 02-2026</t>
+          <t>HECTOLITROS 01-2026</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -8298,17 +8286,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Informe Hctos - Febrero 26</t>
+          <t>Informe Hctos - Enero 26</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -8318,7 +8306,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>f160738c-ce43-45ce-87a3-3da53b3cb493</t>
+          <t>044d5eda-11e1-4f03-8af6-58eea7a265e5</t>
         </is>
       </c>
       <c r="L53" t="n">
@@ -8343,7 +8331,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>HECTOLITROS 03-2026</t>
+          <t>HECTOLITROS 02-2026</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -8354,17 +8342,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Informe Hctos - Marzo 26</t>
+          <t>Informe Hctos - Febrero 26</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -8374,7 +8362,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>f5923390-9c4e-43ab-9848-de3e4e5e09f0</t>
+          <t>f160738c-ce43-45ce-87a3-3da53b3cb493</t>
         </is>
       </c>
       <c r="L54" t="n">
@@ -8399,7 +8387,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>HECTOLITROS 04-2026</t>
+          <t>HECTOLITROS 03-2026</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -8410,17 +8398,17 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Informe Hctos - Abril 26</t>
+          <t>Informe Hctos - Marzo 26</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -8430,7 +8418,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>bb82063a-b49c-48c3-b898-66f8d7550169</t>
+          <t>f5923390-9c4e-43ab-9848-de3e4e5e09f0</t>
         </is>
       </c>
       <c r="L55" t="n">
@@ -8455,7 +8443,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>HECTOLITROS 05-2026</t>
+          <t>HECTOLITROS 04-2026</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -8466,17 +8454,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Informe Hctos - Mayo 26</t>
+          <t>Informe Hctos - Abril 26</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -8486,11 +8474,11 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>3e50d2a1-e143-431c-9480-dd556374f28a</t>
+          <t>bb82063a-b49c-48c3-b898-66f8d7550169</t>
         </is>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -8511,7 +8499,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2026</t>
+          <t>HECTOLITROS 05-2026</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -8522,17 +8510,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 26</t>
+          <t>Informe Hctos - Mayo 26</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -8542,11 +8530,11 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>32fc6955-cc43-4154-9769-e57335f68ef1</t>
+          <t>3e50d2a1-e143-431c-9480-dd556374f28a</t>
         </is>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -8567,7 +8555,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 06-2026</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -8578,17 +8566,17 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 26</t>
+          <t>Informe Hctos - Junio 26</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -8598,11 +8586,11 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8</t>
+          <t>32fc6955-cc43-4154-9769-e57335f68ef1</t>
         </is>
       </c>
       <c r="L58" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -8623,7 +8611,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -8634,17 +8622,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 26</t>
+          <t>Informe Hctos - Julio 26</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -8654,11 +8642,11 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>db3b1962-96b8-49b8-ab8b-c7c13fd197df</t>
+          <t>d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8</t>
         </is>
       </c>
       <c r="L59" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="60">
@@ -8679,7 +8667,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -8690,17 +8678,17 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 26</t>
+          <t>Informe Hctos - Agosto 26</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -8710,11 +8698,11 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>8e7f08c1-fd17-4367-85f0-9af0618ec50f</t>
+          <t>db3b1962-96b8-49b8-ab8b-c7c13fd197df</t>
         </is>
       </c>
       <c r="L60" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61">
@@ -8735,18 +8723,30 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>HECTOLITROS</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr"/>
+          <t>Informe Hctos - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -8754,11 +8754,11 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>8a7194e4-c02a-4fb6-a108-b214302c8a96</t>
+          <t>8e7f08c1-fd17-4367-85f0-9af0618ec50f</t>
         </is>
       </c>
       <c r="L61" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -8787,7 +8787,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -8798,7 +8798,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>34982d0f-52be-4a8b-935f-9aa3ee3915bb</t>
+          <t>8a7194e4-c02a-4fb6-a108-b214302c8a96</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -8831,7 +8831,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -8842,11 +8842,11 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>220bac31-1b58-44ff-8b44-2e0dffd8fc5a</t>
+          <t>34982d0f-52be-4a8b-935f-9aa3ee3915bb</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS DISTR</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -8875,7 +8875,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -8886,11 +8886,11 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>74da6bde-8f40-4f5a-881e-c79da99f35a1</t>
+          <t>220bac31-1b58-44ff-8b44-2e0dffd8fc5a</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>PRECIOS Y OFERTAS DISTR</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -8919,7 +8919,7 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -8930,11 +8930,11 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>3bc172f4-88c0-403c-9c60-483089c17d75</t>
+          <t>74da6bde-8f40-4f5a-881e-c79da99f35a1</t>
         </is>
       </c>
       <c r="L65" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -8950,24 +8950,20 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MARGENES MC</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Analiza la rentabilidad de las ventas: margen $ y % por sucursal, sección, rubro, línea, proveedor y artículo. Cruza facturación, importe s/IVA, costo, descuentos y mermas para mostrar dónde se gana y dónde se pierde rentabilidad.</t>
-        </is>
-      </c>
+          <t>MARGENES MAYORISTA</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>MARGENES MC</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -8978,11 +8974,11 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>c189c73d-9a18-477b-8c39-c855849020d0</t>
+          <t>3bc172f4-88c0-403c-9c60-483089c17d75</t>
         </is>
       </c>
       <c r="L66" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
@@ -8998,20 +8994,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
+          <t>MARGENES MC</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Analiza la rentabilidad de las ventas: margen $ y % por sucursal, sección, rubro, línea, proveedor y artículo. Cruza facturación, importe s/IVA, costo, descuentos y mermas para mostrar dónde se gana y dónde se pierde rentabilidad.</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>MARGENES MC</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9022,11 +9022,11 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>e00515fb-8071-400a-bf39-fa070c0f663c</t>
+          <t>c189c73d-9a18-477b-8c39-c855849020d0</t>
         </is>
       </c>
       <c r="L67" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68">
@@ -9042,24 +9042,20 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Controla las pérdidas de mercadería (roturas, vencimientos) en unidades y valorizadas, por sucursal, sección y artículo.</t>
-        </is>
-      </c>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Mermas MC</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9070,11 +9066,11 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b</t>
+          <t>e00515fb-8071-400a-bf39-fa070c0f663c</t>
         </is>
       </c>
       <c r="L68" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="69">
@@ -9090,20 +9086,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
+          <t>MERMAS MC</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Controla las pérdidas de mercadería (roturas, vencimientos) en unidades y valorizadas, por sucursal, sección y artículo.</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Ofertas desempeño</t>
+          <t>Mermas MC</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>a22fe5fb-0b92-436c-b710-db69d8ea7c47</t>
+          <t>dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b</t>
         </is>
       </c>
       <c r="L69" t="n">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE OFERTAS</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -9153,12 +9153,12 @@
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Grupo Hergo - Jefes</t>
+          <t>Directorio</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>467411be-b152-4571-aab6-634eb4bf23fc</t>
+          <t>a22fe5fb-0b92-436c-b710-db69d8ea7c47</t>
         </is>
       </c>
       <c r="L70" t="n">
@@ -9183,38 +9183,26 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 06-2025</t>
+          <t>SEGUIMIENTO DE OFERTAS</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>PARTICIPACION VENTAS CCU</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>06-2025</t>
-        </is>
-      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Junio 25</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Junio - 25</t>
-        </is>
-      </c>
+          <t>Ofertas desempeño</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Directorio</t>
+          <t>Grupo Hergo - Jefes</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3</t>
+          <t>467411be-b152-4571-aab6-634eb4bf23fc</t>
         </is>
       </c>
       <c r="L71" t="n">
@@ -9239,7 +9227,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PARTICIPACION VENTAS CCU 06-2025</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -9250,17 +9238,17 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>06-2025</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+          <t>PARTICIPACION VENTAS CCU - Junio 25</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Junio - 25</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -9270,7 +9258,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>ed3b5a8c-8ac6-4d65-8961-df938488eb29</t>
+          <t>a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3</t>
         </is>
       </c>
       <c r="L72" t="n">
@@ -9290,23 +9278,35 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>PARTICIPACION VENTAS CCU</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J73" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -9314,7 +9314,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>48b6a50f-e36a-4be6-9fe5-ba74ff2c0afc</t>
+          <t>ed3b5a8c-8ac6-4d65-8961-df938488eb29</t>
         </is>
       </c>
       <c r="L73" t="n">
@@ -9334,12 +9334,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PRESUPUESTO MARKETING</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -9347,7 +9347,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>PRESUPUESTO MARKETING</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>cf5e22c9-8925-4779-8f00-d8de2fa957eb</t>
+          <t>48b6a50f-e36a-4be6-9fe5-ba74ff2c0afc</t>
         </is>
       </c>
       <c r="L74" t="n">
@@ -9383,30 +9383,18 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2025</t>
+          <t>PRESUPUESTO MARKETING</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>06-2025</t>
-        </is>
-      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 25</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>Junio - 25</t>
-        </is>
-      </c>
+          <t>PRESUPUESTO MARKETING</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -9414,7 +9402,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>b2a5fae9-92c4-46d3-b364-372aea858f72</t>
+          <t>cf5e22c9-8925-4779-8f00-d8de2fa957eb</t>
         </is>
       </c>
       <c r="L75" t="n">
@@ -9439,7 +9427,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2025</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -9450,17 +9438,17 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>06-2025</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 25</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Junio - 25</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -9470,7 +9458,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>0a3ae277-8590-4478-b8d5-804f67d03891</t>
+          <t>b2a5fae9-92c4-46d3-b364-372aea858f72</t>
         </is>
       </c>
       <c r="L76" t="n">
@@ -9495,7 +9483,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -9506,17 +9494,17 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -9526,7 +9514,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>abf8c306-8989-4b41-b690-61b081be32e6</t>
+          <t>0a3ae277-8590-4478-b8d5-804f67d03891</t>
         </is>
       </c>
       <c r="L77" t="n">
@@ -9551,7 +9539,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -9562,17 +9550,17 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -9582,7 +9570,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>f0d47671-2942-4899-ba80-022688764653</t>
+          <t>abf8c306-8989-4b41-b690-61b081be32e6</t>
         </is>
       </c>
       <c r="L78" t="n">
@@ -9607,7 +9595,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -9618,17 +9606,17 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -9638,7 +9626,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>ecc0aee3-c751-4e88-b738-4d0611d42f0a</t>
+          <t>f0d47671-2942-4899-ba80-022688764653</t>
         </is>
       </c>
       <c r="L79" t="n">
@@ -9663,7 +9651,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -9674,17 +9662,17 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -9694,7 +9682,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>8be45a46-a4fe-47f7-8e14-0d8b88c8bc08</t>
+          <t>ecc0aee3-c751-4e88-b738-4d0611d42f0a</t>
         </is>
       </c>
       <c r="L80" t="n">
@@ -9719,7 +9707,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -9730,17 +9718,17 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9750,7 +9738,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>0ed4d6a9-e127-48da-bb35-b80be311a816</t>
+          <t>8be45a46-a4fe-47f7-8e14-0d8b88c8bc08</t>
         </is>
       </c>
       <c r="L81" t="n">
@@ -9775,7 +9763,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -9786,17 +9774,17 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9806,7 +9794,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>9bb19246-4084-4e1b-98b3-751e272d0cd9</t>
+          <t>0ed4d6a9-e127-48da-bb35-b80be311a816</t>
         </is>
       </c>
       <c r="L82" t="n">
@@ -9831,7 +9819,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -9842,17 +9830,17 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9862,7 +9850,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>33609288-f489-4d89-84b7-70823a5a276d</t>
+          <t>9bb19246-4084-4e1b-98b3-751e272d0cd9</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -9887,7 +9875,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -9898,17 +9886,17 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -9918,7 +9906,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>3c08fbd5-25e3-47fb-9f66-a076efa2ab2e</t>
+          <t>33609288-f489-4d89-84b7-70823a5a276d</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -9943,7 +9931,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -9954,17 +9942,17 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -9974,7 +9962,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>3f0a1b1b-e90e-4324-8479-bdf6259f6040</t>
+          <t>3c08fbd5-25e3-47fb-9f66-a076efa2ab2e</t>
         </is>
       </c>
       <c r="L85" t="n">
@@ -9999,7 +9987,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -10010,17 +9998,17 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -10030,7 +10018,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>c7ec947a-c40b-4710-a08f-0a436442ba97</t>
+          <t>3f0a1b1b-e90e-4324-8479-bdf6259f6040</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -10055,7 +10043,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -10066,17 +10054,17 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -10086,7 +10074,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>1a7a09ca-f8b7-4f55-8441-ffb04e0d63f6</t>
+          <t>c7ec947a-c40b-4710-a08f-0a436442ba97</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -10111,7 +10099,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -10122,17 +10110,17 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10142,7 +10130,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>8cc08bae-0659-4b71-af6a-b3f830c2d9c8</t>
+          <t>1a7a09ca-f8b7-4f55-8441-ffb04e0d63f6</t>
         </is>
       </c>
       <c r="L88" t="n">
@@ -10167,7 +10155,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -10178,17 +10166,17 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10198,7 +10186,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>2271183e-fad9-4f2f-94a4-656ddc3e2327</t>
+          <t>8cc08bae-0659-4b71-af6a-b3f830c2d9c8</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -10223,7 +10211,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -10234,17 +10222,17 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -10254,7 +10242,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>0f0d31e7-0dbf-4e4b-b4bf-79b7b6781d35</t>
+          <t>2271183e-fad9-4f2f-94a4-656ddc3e2327</t>
         </is>
       </c>
       <c r="L90" t="n">
@@ -10274,23 +10262,35 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FINANZAS</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>SITUACION FINANCIERA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>SITUACION FINANCIERA</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J91" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -10298,11 +10298,11 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>7ed33ee7-275e-4af5-8ddc-3e67ce01ce50</t>
+          <t>0f0d31e7-0dbf-4e4b-b4bf-79b7b6781d35</t>
         </is>
       </c>
       <c r="L91" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -10318,12 +10318,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>FINANZAS</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>SITUACION FINANCIERA</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -10331,7 +10331,7 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Stock unificado</t>
+          <t>SITUACION FINANCIERA</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -10342,11 +10342,11 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>589dc885-5ca9-4b06-9776-ebb80e7ea81d</t>
+          <t>7ed33ee7-275e-4af5-8ddc-3e67ce01ce50</t>
         </is>
       </c>
       <c r="L92" t="n">
-        <v>23</v>
+        <v>119</v>
       </c>
     </row>
     <row r="93">
@@ -10362,24 +10362,20 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MENOR COSTE</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Dashboard con el stock valorizado de las sucursales de menor coste y los dias de stock por seccion/linea/producto</t>
-        </is>
-      </c>
+          <t>STOCK UNIFICADO</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Stock valorizado MC</t>
+          <t>Stock unificado</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -10390,11 +10386,11 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>4900a270-06ee-458b-9793-2f98b3644748</t>
+          <t>589dc885-5ca9-4b06-9776-ebb80e7ea81d</t>
         </is>
       </c>
       <c r="L93" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
     </row>
     <row r="94">
@@ -10410,20 +10406,24 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>TRAFICO</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr"/>
+          <t>STOCK VALORIZADO MENOR COSTE</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Dashboard con el stock valorizado de las sucursales de menor coste y los dias de stock por seccion/linea/producto</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TRAFICO</t>
+          <t>Stock valorizado MC</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -10434,11 +10434,11 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>ffd69225-dff5-4250-8c81-775a75de3777</t>
+          <t>4900a270-06ee-458b-9793-2f98b3644748</t>
         </is>
       </c>
       <c r="L94" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -10467,7 +10467,7 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>a09b2740-4617-4450-a263-e63c7ab47158</t>
+          <t>ffd69225-dff5-4250-8c81-775a75de3777</t>
         </is>
       </c>
       <c r="L95" t="n">
@@ -10503,7 +10503,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -10511,7 +10511,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -10522,11 +10522,11 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>3d9a0917-34b5-4ac6-8b6a-f2244892db15</t>
+          <t>a09b2740-4617-4450-a263-e63c7ab47158</t>
         </is>
       </c>
       <c r="L96" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -10555,7 +10555,7 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -10566,11 +10566,11 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>4bdda3e7-2a7d-4b74-a484-4551b4873c03</t>
+          <t>3d9a0917-34b5-4ac6-8b6a-f2244892db15</t>
         </is>
       </c>
       <c r="L97" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="98">
@@ -10706,7 +10706,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101">
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="102">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="103">
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>212</v>
+        <v>225</v>
       </c>
     </row>
     <row r="105">
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="119">
@@ -11574,7 +11574,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="120">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="126">
@@ -12686,7 +12686,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
     <row r="142">
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="145">
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="148">
@@ -13790,7 +13790,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="163">
@@ -13958,7 +13958,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166">
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="171">
@@ -14522,7 +14522,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="178">
@@ -16290,7 +16290,7 @@
         </is>
       </c>
       <c r="L209" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="210">
@@ -16334,7 +16334,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="211">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TGye8oS9xOO2zCkYdFPtiA==</t>
+          <t>aksT43m+wZJrIuqyuLgkjg==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ny3kYbHPjzNXfrWf5WDJ70awLpzUeQbrWxsZINHqcxo=</t>
+          <t>cil515MLzL6S+Zhxqcup04G/lXLC+j0NbQ1MixJinpc=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16540,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2Vwe3otRzL4YgCuZb05RyA==</t>
+          <t>XZ93E8AeedazPIe7prWUzw==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>z3+4Xr3DMEk2fdAJpfzJvhUlxnH8j/R5jV6D1goXd+4=</t>
+          <t>WV3PrRPx1iutu7Ei88mMaScKjMb1AWVIScojTuon4xY=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16572,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DUQeOLTQMVP8OE+6unMGGA==</t>
+          <t>aVuxeogh+cPUjhCv5w66mg==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>zKXlbTd8b/sn9W6LrTjEgKqeCxzNUOD+v1otuZoANwE=</t>
+          <t>sV24ZMAfz57Nd1q9cZJWP+1wDLWTn9QcytCW86kTfIk=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>YECCQJXGmkYXsm8cbM2lXQ==</t>
+          <t>ydUszkNT91jNX+zrBRypqA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>qoVsihzO2Q7ltpdGW1Z4h0y3cS9UatyC/sUfHYtkBfg=</t>
+          <t>cBCCY4+ZXTuOOK4mVSmdtD14AEI8fIhjU9m/mRK/BEM=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16631,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>pb5Rv3PSQAdSHdMuKT/bsQ==</t>
+          <t>JZh21kizkDatq202imOWIg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>mBkqDxWbjAtQm2K0A0xZN6q1EtM7iPQXwTehCcCkC50=</t>
+          <t>yr5+CVG4UQ1xT/kHiZUq1iXAg6NUMyY12uj8Vgx+1wk=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16663,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hx0H+NSrYQlbveg/BlFQ6g==</t>
+          <t>jJ6QByQ4RPjksI+6HuxaWQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>sRckP+opjMMrnfdv/UXiyN9W7owQPeVjFeSDknKvS40=</t>
+          <t>1x9voCl1nPIWAjL0SSDwEj56KG8yYuKZQuB/JgzS1DM=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>iI0jRh5k0/emfmPD9qQhoA==</t>
+          <t>y6tzFgNGeZvqATziyT2Q5Q==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8UYFtR+6FzRxJtUeAl9+406XkoiQtSdRfHucr8UNSaI=</t>
+          <t>4Q6y/hhq3+b9q884IUEJp9tGKrbngwO/I+5EvBgGXJQ=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3SNynI6r4rFG1jq+GrnUOw==</t>
+          <t>0liUSt9wiDH9/wAYl/qmeg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>maayaN1H4V8QoOekzG1/F8vIhvFUl18ljs4n6Yt1oKE=</t>
+          <t>ASSAg4A3l1Ch+PQ5eJfVVUV+JeUGK/9dkjDAGoKyfBM=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HLC4DEAdCau6mgmNEbKDZQ==;Angkb4ybiTcw16Xvrv1+fQ==</t>
+          <t>kNs9XPQX+60ypyuS+fVxeA==;1/QCM9ycjx8OqS4dvOOC5A==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1ggpHN2SSnQqdNCG4G4kLVdOyp0bRtNRp9SBgEuZ1EY=;xl8V+OV55jJnylbgHwUogyYAWptrJLOCYqwMt9PvCmw=</t>
+          <t>Uh8sLoscXPW+CukThJZQWMYFWGoHLvn1BsOkFzElq6w=;aeE7M4Znp2ASmYm4JnQVNiOMpc1BT/yueC8WUr8bS+0=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>IMnENL5PePsFEEa38miPAQ==</t>
+          <t>OQNwaGtOOSrTKunZI6WJ7w==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SQPbfwkCKU5eXbkmFcDIi7TjB5knRDgvYbucwC1AcvM=</t>
+          <t>mxgItOGznrC8n1IsKk/NhtK6qkZ9lWekbGeXc9jYr7w=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16818,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>s9DsWJcD8abbLangEbm/eA==</t>
+          <t>5Ly+VoxLGHs2mdKVFE0xMg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>jXMqYfQD4ULC6LEThq4G47TFtzylb4NSaslggRCxwl4=</t>
+          <t>ZB7+jkv12nPll15C8NmXOPKdF3f+kAmPbm5QemsKd3U=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16850,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>QbJ6mMDZFMqYHEsdtWM14Q==</t>
+          <t>8h+X/TfXoCzjUy4RQluDMw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WZy3n4kUJaw1Kw8mTZ87YZ0q5dzDBb4w9eP4b7fM560=</t>
+          <t>doUiPMH+UKR1iU7CCvrar2+YTn+PkvIXp7U3m33w4y0=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16882,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>sKP7cMLC2g74n4c1OEWV3g==</t>
+          <t>c2SqqwKA7jw7rXMX1qvD9A==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>/89gchQ8TDUfmwAERHzP92e7Zj0apSrHdyA5qOKTS+4=</t>
+          <t>5Q8HIubxJTmcAQZY33792U8/Yxa/E4/nO/qgVdCme5s=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16914,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>dIt+GbNBIOzWinN5U6ellg==</t>
+          <t>TEzQNUzCS82O8o6VZQW/fw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cHJa1iT+B2r4+LykNebG2j7xYPXbsXFi+J9ryXLb2FU=</t>
+          <t>whnbegwuAo3Ru2eQ8gt8Fg5+lIVex9I3++X9uYs0RYE=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +16946,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>iEYVOWGajUGBU3RmBbCsMw==</t>
+          <t>UBM4KuR45VS9zEFDeQCmfQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>VAviw/5MzGbkQwLOD7fKogQVvP1sRKydAikizksfxCE=</t>
+          <t>WuQrY9Dv0PAJyD7uyhJApm5StmaRy5GfMX5ImFLHf2Y=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +16978,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>wZ2H0KJ/TNcca6Alm15wxQ==</t>
+          <t>68M92ZCgT35mIQGtNQxoCg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PIsRN+1ktT3r9zfV3GpagNrT9zoe55okIse/rcPncA0=</t>
+          <t>9BdppOaph386HZEzrQP/VF0MJxQGFaOXfCKqvhtheJ8=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GbXe8n3YnTYf2OpM8P5JPg==</t>
+          <t>FjBmFNAW4z4tTOvd5U0Hlw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>xQyhMJVLbB+05Ph7rNW5yDngZOIy7w4TOqaaJiHdiLs=</t>
+          <t>OoX47VmUPMaMF7ZJwsw3XHb4SL1Gjwq408/xx9P/zBo=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17042,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AWmrTbLKFZTxw4QsDiYa7A==</t>
+          <t>q5tcDYQV10TcfsElVUB0Hw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ac84uGq+PxusQj02sRieHYqaktRNviELmsOnF+wcj28=</t>
+          <t>bkQqy6PWsnFEbFKIa71ZKlDfiaue0ti0gEl61AARnAY=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17074,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>plUmwYL5A0LN/qjMP2vupg==</t>
+          <t>S2OrrKSAPS2SCPD5KXl00A==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>BLu7mtnVp1X97JZAlJveK9Psb9Pws6ep8bHU/mcMMj8=</t>
+          <t>o4fNKYY2BwRcUmfwpNq8GhLvQmyQT/gj22ERIP0PO7Y=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17106,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>W5cRWkcbx3nVmblzLxbOSg==</t>
+          <t>1yms592TPgpSGTVknO2HLA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>B12/4rnrlfYBPbTkhWp5VWPyH25fk9Ah2Fa5ltiNeoA=</t>
+          <t>//xriyP0N3wUQziu1345Q4M6D+/OhWBSky1xXX39TA8=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TabeuDxNq0dxO8kXtfWG4w==</t>
+          <t>ddi/s7f7ww1hNsQ/oA4R6w==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>T5ugo17PP3xaoIUtiha1o+o9bFl5fK5ioXpJ74g+Wjs=</t>
+          <t>HgtbuqfHebbAwyQVPIsACdnWAEo0RhXsmPLxnZhXOWs=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17170,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>koV75PgRyY5AGLFgQ/sfmA==</t>
+          <t>ToFm4v/E5ACmN7U9G8rmjw==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1cC5UhLuFh3AJt04xhSjmTri0N0XYtqw6KRZmTrPvG0=</t>
+          <t>glYLxBmbX3bKvbVFATK1lic9Ly+X4ePN+ed7Mypo0Y0=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17202,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YhN+Fp5avgB6WppuM+UW0Q==</t>
+          <t>bcuYnRZiNbPmlxP9ZJa7Hg==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>vH1IiK1Q5kbepEVVo0Dx7vjDA4tOg7fUEehfxhIpc/g=</t>
+          <t>IycDcbMmSMvWRscC+411AImnpTrK2TxjvS13c2ABVAw=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17234,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7kLrDV/jpuBVhrzq/worAQ==</t>
+          <t>TYNV0zR/MbeMQ2qClApIXQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>p19NWDIjRQc6Pbxq94rstYJm1a7bDtig7KsOM7/eN+I=</t>
+          <t>f3FUg/syfF28TCnZYPONZFRN+liF7TYFJ/NgNBSAEeI=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17266,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>GqbQ4I2gfzsrMNXgTEyWWA==</t>
+          <t>yBVguuNxwzZUGM4fpaIqIA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5fVHHKphHqJXaxPEi4ztcCArjdX+W16qcumwvx1+orY=</t>
+          <t>lN9r7/HA5IhJFXtmp60vRphy2L2gUFePncJBCe/YNOo=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17298,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BRClmasgllE1LQzbsDasMA==</t>
+          <t>CF9m5xKjxwr8ZUeCCgDjbA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>zeLUURuzYjXFxITn81aAWOFXZeoZJ6vS1pRc+TOFQb8=</t>
+          <t>JxZAO8O0Oa6S/zDVYXkGxP60rGJyGDJSWgeaLp/wuhQ=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17330,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>GO9BTBOd9abiS8UktMdkWg==</t>
+          <t>Ry/5a7LzdRisM2BpJQWgAA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>zvpQs44mTbv3uWXLd6CZzk3DAERoas+5/PzfcKWtiBo=</t>
+          <t>KMDJMf3JE6EuCs/DWyBH+3ldXTrYvChQoJpjsi7jP1M=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17362,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>GavPgKTPGqsUSSld9YFvYg==</t>
+          <t>DSBED+8DVUwvsjbr68nwVA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>rIY2pFFB9nZKF6T/KbHcavV0Aumn04whPqji9JYhr2E=</t>
+          <t>ocRPt0YCByF0JHnmU9DJ1FHLvVVLipAM8ffSWNcjoPA=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17394,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>xcCpkyP8VsDwjwQ5ZlA++w==</t>
+          <t>UjRXt56YXo29ijVrrxCIdg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CZ/dvKalLiY+zQB8xHte5PkgOXK5LqDVrnODSkrTqgA=</t>
+          <t>UCgsSy969GkjY24totBFvT8aWMN2SUx4jbqfVvLUDxo=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>xHS3APpypT9CN7VpDSTrxw==</t>
+          <t>CFxWhV6tZ5ILDzhhFZzDpQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>7ywuKRXgJEfUoBQNG/xNuX14gm74lUOEprb1YDUVyTk=</t>
+          <t>bvAcJQM6u9kuksQQ4cLQQqJv0ggieLdRQMMI9kwLABk=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17458,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>aogvr08jnqYewdvD9Lq8sw==</t>
+          <t>NVuqgbtGTRNXl7Ss9QrMtQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1HRzg9WDEQwZWax+xbSPayXA4tbiZGZF5KxlhaqQYYk=</t>
+          <t>P2SE7J5DM+2TUiwCkh74voQaUHBR2IiHe3exudQFEaE=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17490,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>egD9IcbNihseWeScd5t2iA==</t>
+          <t>CmAqbtFbAfF8hc11SRqWgw==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>jDjguY/efOcM60BkFucG+RDlupjZrx+POgh5QypllQQ=</t>
+          <t>OMYC2IEb9X/2qII8panwNXGBe5uZyFiSMEHIkYGJIUs=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17522,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>cyojw7Ci/Ga31cO9xdx7Pw==</t>
+          <t>NPdlgAT4sOtDglHrVlYQsg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Oc5xFwn+qlLSP1Imfx12p0N8osJUYe7rgpcF5/iqV7w=</t>
+          <t>qwC4mId56sB+AT6emuYqcadg28eHjkFvx7f/RfvcNyQ=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17554,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>uAG7TUgN9UHakIIB3df+qw==</t>
+          <t>wbxYGfvz1xl9iBCbI5TkpQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>zn7FsCXMMEGMyxN4BgOtpCb7yhttqMAUX7jlUaZstEw=</t>
+          <t>5jC9SCLyZMIXRMi/swQlChzn2bA42WKJLS4WARNHP8I=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>cU44LM7wIzxBe5o+unVotQ==</t>
+          <t>XQFqtNg39SSZ2sKjovhwFg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Qy83EFderZnNu1gWHJVoBWthcxdWMPmeHJeKdd1LWBY=</t>
+          <t>Aq0MMGnLsWGRvUgEyQA8bnzQsFQ5spbb5KdbsSx5mQE=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>blQZ1ezudMsNdZE3JTBZyg==</t>
+          <t>pyr1SQNQpisme6HPcomm+w==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>pv/uzeobtl0K18rNY9+WBoagpB4HnzdKYuB66C1urlo=</t>
+          <t>e9aro7yOdzryN71aOSfxfZYMBTzP1H9cS0yJdae4roE=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17650,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>QMDZQysbSKKOMWdwWTtrDQ==</t>
+          <t>PbphOL/ffXDnx1gK9JwLVQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>N0aUMSX9/VRduDVQw5rGyYSmKQS7WWga3vFJtCbiPdQ=</t>
+          <t>TQmwtGG6Ewd6Pqvmosxs6Hm8txd+XQUV8NgNrCrSo78=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-01 07:38) - 116 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$143</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="80">
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="85">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="90">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="95">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="106">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="107">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>562</v>
+        <v>571</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>562</v>
+        <v>571</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="115">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="121">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="122">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5618,17 +5618,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5646,8 +5646,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>MENOR COSTE</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>INFORME</t>
+        </is>
+      </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H143"/>
+  <autoFilter ref="A1:H144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5658,7 +5694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L212"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5822,7 +5858,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -6042,7 +6078,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
@@ -6086,7 +6122,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10">
@@ -6350,7 +6386,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16">
@@ -7686,7 +7722,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
@@ -7774,7 +7810,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44">
@@ -8646,7 +8682,7 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="60">
@@ -9026,7 +9062,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68">
@@ -9070,7 +9106,7 @@
         </is>
       </c>
       <c r="L68" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69">
@@ -10346,7 +10382,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="93">
@@ -10390,7 +10426,7 @@
         </is>
       </c>
       <c r="L93" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94">
@@ -10618,7 +10654,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99">
@@ -10662,7 +10698,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="100">
@@ -10706,7 +10742,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="101">
@@ -10750,7 +10786,7 @@
         </is>
       </c>
       <c r="L101" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="102">
@@ -10794,7 +10830,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="103">
@@ -10838,7 +10874,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="104">
@@ -10882,7 +10918,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="105">
@@ -11310,7 +11346,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="114">
@@ -11530,7 +11566,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="119">
@@ -11574,7 +11610,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="120">
@@ -11618,7 +11654,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="121">
@@ -11838,7 +11874,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="126">
@@ -11926,7 +11962,7 @@
         </is>
       </c>
       <c r="L127" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="128">
@@ -11947,7 +11983,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -11955,7 +11991,7 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -11966,11 +12002,11 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>5d2131f2-f6b5-41f6-b864-e0534c499950</t>
+          <t>f81dd4b4-8d4e-4a57-a673-eff19a270837</t>
         </is>
       </c>
       <c r="L128" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -11991,7 +12027,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -11999,7 +12035,7 @@
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
-          <t>AnalisisOfertas</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -12010,11 +12046,11 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>034fc54a-d18c-44b2-9915-aa86bd8b02f1</t>
+          <t>5d2131f2-f6b5-41f6-b864-e0534c499950</t>
         </is>
       </c>
       <c r="L129" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
     </row>
     <row r="130">
@@ -12035,30 +12071,18 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2025</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>COMPARATIVO</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>COMPARATIVO JULIO 2025</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>AnalisisOfertas</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -12066,11 +12090,11 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>3d26ba08-de7b-4635-b801-959f2751c0ea</t>
+          <t>034fc54a-d18c-44b2-9915-aa86bd8b02f1</t>
         </is>
       </c>
       <c r="L130" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="131">
@@ -12091,7 +12115,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2025</t>
+          <t>COMPARATIVO 07-2025</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -12102,17 +12126,17 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>COMPARATIVO AGOSTO 2025</t>
+          <t>COMPARATIVO JULIO 2025</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -12122,11 +12146,11 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>2ebaf008-5151-4818-941c-1fb09e7ece5d</t>
+          <t>3d26ba08-de7b-4635-b801-959f2751c0ea</t>
         </is>
       </c>
       <c r="L131" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -12147,7 +12171,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2025</t>
+          <t>COMPARATIVO 08-2025</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -12158,17 +12182,17 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>COMPARATIVO SEPTIEMBRE 2025</t>
+          <t>COMPARATIVO AGOSTO 2025</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -12178,11 +12202,11 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>5b114d82-e229-482c-9756-a9461a47fa76</t>
+          <t>2ebaf008-5151-4818-941c-1fb09e7ece5d</t>
         </is>
       </c>
       <c r="L132" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
     </row>
     <row r="133">
@@ -12203,7 +12227,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>COMPARATIVO 10-2025</t>
+          <t>COMPARATIVO 09-2025</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -12214,17 +12238,17 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>COMPARATIVO OCTUBRE 2025</t>
+          <t>COMPARATIVO SEPTIEMBRE 2025</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -12234,11 +12258,11 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>79627458-97b4-408e-b057-93369d32e0fc</t>
+          <t>5b114d82-e229-482c-9756-a9461a47fa76</t>
         </is>
       </c>
       <c r="L133" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="134">
@@ -12259,7 +12283,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>COMPARATIVO 11-2025</t>
+          <t>COMPARATIVO 10-2025</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -12270,17 +12294,17 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>COMPARATIVO NOVIEMBRE 2025</t>
+          <t>COMPARATIVO OCTUBRE 2025</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -12290,11 +12314,11 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>4c69e9ea-c9fe-4853-8b65-0944c71c846f</t>
+          <t>79627458-97b4-408e-b057-93369d32e0fc</t>
         </is>
       </c>
       <c r="L134" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="135">
@@ -12315,7 +12339,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>COMPARATIVO 12-2025</t>
+          <t>COMPARATIVO 11-2025</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -12326,17 +12350,17 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>COMPARATIVO DICIEMBRE 2025</t>
+          <t>COMPARATIVO NOVIEMBRE 2025</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -12346,7 +12370,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>bb053133-fab4-44ba-beef-b3cc5a883d8b</t>
+          <t>4c69e9ea-c9fe-4853-8b65-0944c71c846f</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -12371,7 +12395,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>COMPARATIVO 01-2026</t>
+          <t>COMPARATIVO 12-2025</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -12382,17 +12406,17 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>COMPARATIVO ENERO 2026</t>
+          <t>COMPARATIVO DICIEMBRE 2025</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -12402,7 +12426,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>be821246-ab66-4f6d-8723-345a31c51584</t>
+          <t>bb053133-fab4-44ba-beef-b3cc5a883d8b</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -12427,7 +12451,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>COMPARATIVO 02-2026</t>
+          <t>COMPARATIVO 01-2026</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -12438,17 +12462,17 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>COMPARATIVO FEBRERO 2026</t>
+          <t>COMPARATIVO ENERO 2026</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -12458,11 +12482,11 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>864f9511-ae08-4152-be61-da8b02e0d10d</t>
+          <t>be821246-ab66-4f6d-8723-345a31c51584</t>
         </is>
       </c>
       <c r="L137" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -12483,7 +12507,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>COMPARATIVO 03-2026</t>
+          <t>COMPARATIVO 02-2026</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -12494,17 +12518,17 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>COMPARATIVO MARZO 2026</t>
+          <t>COMPARATIVO FEBRERO 2026</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -12514,11 +12538,11 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>62dad30f-7d22-4048-80a6-dda3df482533</t>
+          <t>864f9511-ae08-4152-be61-da8b02e0d10d</t>
         </is>
       </c>
       <c r="L138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="139">
@@ -12539,7 +12563,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>COMPARATIVO 04-2026</t>
+          <t>COMPARATIVO 03-2026</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -12550,17 +12574,17 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>COMPARATIVO ABRIL 2026</t>
+          <t>COMPARATIVO MARZO 2026</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -12570,11 +12594,11 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>7a756d76-6d55-4541-ac3c-9c9f20aa3bb6</t>
+          <t>62dad30f-7d22-4048-80a6-dda3df482533</t>
         </is>
       </c>
       <c r="L139" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140">
@@ -12595,7 +12619,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>COMPARATIVO 05-2026</t>
+          <t>COMPARATIVO 04-2026</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -12606,17 +12630,17 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>COMPARATIVO MAYO 2026</t>
+          <t>COMPARATIVO ABRIL 2026</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -12626,11 +12650,11 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>a34b1e3d-829e-467c-81fb-9e7e446afeee</t>
+          <t>7a756d76-6d55-4541-ac3c-9c9f20aa3bb6</t>
         </is>
       </c>
       <c r="L140" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141">
@@ -12651,7 +12675,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>COMPARATIVO 06-2026</t>
+          <t>COMPARATIVO 05-2026</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -12662,17 +12686,17 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>COMPARATIVO JUNIO 2026</t>
+          <t>COMPARATIVO MAYO 2026</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -12682,11 +12706,11 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>8e1fe016-e2ae-4085-8c03-6ba689cd0be0</t>
+          <t>a34b1e3d-829e-467c-81fb-9e7e446afeee</t>
         </is>
       </c>
       <c r="L141" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
@@ -12707,7 +12731,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2026</t>
+          <t>COMPARATIVO 06-2026</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -12718,17 +12742,17 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>COMPARATIVO JULIO 2026</t>
+          <t>COMPARATIVO JUNIO 2026</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -12738,11 +12762,11 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>ef671aec-c05d-4a42-b941-bc2f967d6226</t>
+          <t>8e1fe016-e2ae-4085-8c03-6ba689cd0be0</t>
         </is>
       </c>
       <c r="L142" t="n">
-        <v>360</v>
+        <v>58</v>
       </c>
     </row>
     <row r="143">
@@ -12763,7 +12787,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>COMPARATIVO 07-2026</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -12774,17 +12798,17 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>COMPARATIVO AGOSTO 2026</t>
+          <t>COMPARATIVO JULIO 2026</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -12794,11 +12818,11 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>c6e72043-9449-4d47-992c-d5e6075ec51d</t>
+          <t>ef671aec-c05d-4a42-b941-bc2f967d6226</t>
         </is>
       </c>
       <c r="L143" t="n">
-        <v>319</v>
+        <v>353</v>
       </c>
     </row>
     <row r="144">
@@ -12819,7 +12843,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -12830,17 +12854,17 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>COMPARATIVO SEPTIEMBRE 2026</t>
+          <t>COMPARATIVO AGOSTO 2026</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -12850,11 +12874,11 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>6968ebe5-cca7-4c17-8bb2-31e518e0171e</t>
+          <t>c6e72043-9449-4d47-992c-d5e6075ec51d</t>
         </is>
       </c>
       <c r="L144" t="n">
-        <v>243</v>
+        <v>319</v>
       </c>
     </row>
     <row r="145">
@@ -12875,18 +12899,30 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>COMPARATIVO</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Comparativo Cervezas</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr"/>
+          <t>COMPARATIVO SEPTIEMBRE 2026</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J145" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -12894,11 +12930,11 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>30580dcd-18a8-4764-b965-e447e8860cf4</t>
+          <t>6968ebe5-cca7-4c17-8bb2-31e518e0171e</t>
         </is>
       </c>
       <c r="L145" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
     </row>
     <row r="146">
@@ -12919,7 +12955,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -12927,7 +12963,7 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Comportamiento Clientes</t>
+          <t>Comparativo Cervezas</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -12938,11 +12974,11 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>7de99d39-41a8-4578-994d-377c9a1c334e</t>
+          <t>30580dcd-18a8-4764-b965-e447e8860cf4</t>
         </is>
       </c>
       <c r="L146" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -12963,7 +12999,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -12971,7 +13007,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Consumos por cliente</t>
+          <t>Comportamiento Clientes</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -12982,11 +13018,11 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>e6b113ec-729a-4d3c-934c-f54c1f9689d9</t>
+          <t>7de99d39-41a8-4578-994d-377c9a1c334e</t>
         </is>
       </c>
       <c r="L147" t="n">
-        <v>96</v>
+        <v>44</v>
       </c>
     </row>
     <row r="148">
@@ -13007,7 +13043,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -13015,7 +13051,7 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>Consumos por cliente</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -13026,11 +13062,11 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>1632e5a1-1d96-42be-b9c6-a2d58321335e</t>
+          <t>e6b113ec-729a-4d3c-934c-f54c1f9689d9</t>
         </is>
       </c>
       <c r="L148" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
     </row>
     <row r="149">
@@ -13051,7 +13087,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -13059,7 +13095,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -13070,11 +13106,11 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
+          <t>1632e5a1-1d96-42be-b9c6-a2d58321335e</t>
         </is>
       </c>
       <c r="L149" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -13095,7 +13131,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
@@ -13103,7 +13139,7 @@
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Grupo Clientes BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -13114,11 +13150,11 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
+          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
         </is>
       </c>
       <c r="L150" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="151">
@@ -13139,30 +13175,18 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2025</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>HECTOLITROS</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 25</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>Grupo Clientes BLACK 2026</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -13170,11 +13194,11 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
+          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
         </is>
       </c>
       <c r="L151" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="152">
@@ -13195,7 +13219,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2025</t>
+          <t>HECTOLITROS 07-2025</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
@@ -13206,17 +13230,17 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 25</t>
+          <t>Informe Hctos - Julio 25</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -13226,7 +13250,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
+          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -13251,7 +13275,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2025</t>
+          <t>HECTOLITROS 08-2025</t>
         </is>
       </c>
       <c r="E153" t="inlineStr"/>
@@ -13262,17 +13286,17 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 25</t>
+          <t>Informe Hctos - Agosto 25</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -13282,7 +13306,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
+          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -13307,7 +13331,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2025</t>
+          <t>HECTOLITROS 09-2025</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
@@ -13318,17 +13342,17 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 25</t>
+          <t>Informe Hctos - Septiembre 25</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -13338,7 +13362,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
+          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -13363,7 +13387,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>HECTOLITROS 11-2025</t>
+          <t>HECTOLITROS 10-2025</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -13374,17 +13398,17 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Informe Hctos - Noviembre 25</t>
+          <t>Informe Hctos - Octubre 25</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -13394,7 +13418,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
+          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -13419,7 +13443,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>HECTOLITROS 12-2025</t>
+          <t>HECTOLITROS 11-2025</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -13430,17 +13454,17 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Informe Hctos - Diciembre 25</t>
+          <t>Informe Hctos - Noviembre 25</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -13450,7 +13474,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
+          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -13475,7 +13499,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>HECTOLITROS 01-2026</t>
+          <t>HECTOLITROS 12-2025</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -13486,17 +13510,17 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Informe Hctos - Enero 26</t>
+          <t>Informe Hctos - Diciembre 25</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -13506,7 +13530,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
+          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -13531,7 +13555,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>HECTOLITROS 02-2026</t>
+          <t>HECTOLITROS 01-2026</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -13542,17 +13566,17 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Informe Hctos - Febrero 26</t>
+          <t>Informe Hctos - Enero 26</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -13562,7 +13586,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
+          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -13587,7 +13611,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>HECTOLITROS 03-2026</t>
+          <t>HECTOLITROS 02-2026</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -13598,17 +13622,17 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Informe Hctos - Marzo 26</t>
+          <t>Informe Hctos - Febrero 26</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -13618,7 +13642,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
+          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -13643,7 +13667,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HECTOLITROS 04-2026</t>
+          <t>HECTOLITROS 03-2026</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -13654,17 +13678,17 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Informe Hctos - Abril 26</t>
+          <t>Informe Hctos - Marzo 26</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -13674,7 +13698,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
+          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -13699,7 +13723,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>HECTOLITROS 05-2026</t>
+          <t>HECTOLITROS 04-2026</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -13710,17 +13734,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Informe Hctos - Mayo 26</t>
+          <t>Informe Hctos - Abril 26</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -13730,11 +13754,11 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
+          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
         </is>
       </c>
       <c r="L161" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -13755,7 +13779,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2026</t>
+          <t>HECTOLITROS 05-2026</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -13766,17 +13790,17 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 26</t>
+          <t>Informe Hctos - Mayo 26</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -13786,7 +13810,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
+          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -13811,7 +13835,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 06-2026</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -13822,17 +13846,17 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 26</t>
+          <t>Informe Hctos - Junio 26</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -13842,11 +13866,11 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
+          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
         </is>
       </c>
       <c r="L163" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
     </row>
     <row r="164">
@@ -13867,7 +13891,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -13878,17 +13902,17 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 26</t>
+          <t>Informe Hctos - Julio 26</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -13898,11 +13922,11 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
+          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
         </is>
       </c>
       <c r="L164" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="165">
@@ -13923,7 +13947,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -13934,17 +13958,17 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 26</t>
+          <t>Informe Hctos - Agosto 26</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -13954,11 +13978,11 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
+          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
         </is>
       </c>
       <c r="L165" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="166">
@@ -13979,18 +14003,30 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>HECTOLITROS</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr"/>
+          <t>Informe Hctos - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J166" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -13998,11 +14034,11 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
+          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
         </is>
       </c>
       <c r="L166" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="167">
@@ -14023,7 +14059,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -14031,7 +14067,7 @@
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -14042,11 +14078,11 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
+          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
         </is>
       </c>
       <c r="L167" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -14067,7 +14103,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
@@ -14075,7 +14111,7 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -14086,11 +14122,11 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
+          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
         </is>
       </c>
       <c r="L168" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="169">
@@ -14111,7 +14147,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
@@ -14119,7 +14155,7 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -14130,7 +14166,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
+          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -14155,7 +14191,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
@@ -14163,7 +14199,7 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -14174,11 +14210,11 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
+          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
         </is>
       </c>
       <c r="L170" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171">
@@ -14199,7 +14235,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -14207,7 +14243,7 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
@@ -14218,11 +14254,11 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
+          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
         </is>
       </c>
       <c r="L171" t="n">
-        <v>18</v>
+        <v>224</v>
       </c>
     </row>
     <row r="172">
@@ -14243,30 +14279,18 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>PARTICIPACION VENTAS CCU</t>
-        </is>
-      </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14274,11 +14298,11 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L172" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="173">
@@ -14299,28 +14323,28 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PARTICIPACION VENTAS CCU</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -14330,11 +14354,11 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
+          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
       </c>
       <c r="L173" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174">
@@ -14355,13 +14379,13 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -14371,7 +14395,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
+          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -14386,11 +14410,11 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
+          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
       </c>
       <c r="L174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -14411,18 +14435,30 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>PLAN ESPACIO APP COSTA</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>08-2025</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr"/>
+          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Agosto - 25</t>
+        </is>
+      </c>
       <c r="J175" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14430,11 +14466,11 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
+          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
       </c>
       <c r="L175" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">
@@ -14450,12 +14486,12 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
@@ -14463,7 +14499,7 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -14474,11 +14510,11 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
+          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177">
@@ -14494,12 +14530,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
@@ -14507,7 +14543,7 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>RECHAZOS ago 26</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -14518,11 +14554,11 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
+          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -14543,30 +14579,18 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO DE MARCAS</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>RECHAZOS ago 26</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14574,11 +14598,11 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
+          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
         </is>
       </c>
       <c r="L178" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="179">
@@ -14599,7 +14623,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -14610,17 +14634,17 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -14630,7 +14654,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
+          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -14655,7 +14679,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -14666,17 +14690,17 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -14686,7 +14710,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
+          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -14711,7 +14735,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -14722,17 +14746,17 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -14742,7 +14766,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
+          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -14767,7 +14791,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
@@ -14778,17 +14802,17 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -14798,7 +14822,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
+          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -14823,7 +14847,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
@@ -14834,17 +14858,17 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -14854,7 +14878,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
+          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
       <c r="L183" t="n">
@@ -14879,7 +14903,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
@@ -14890,17 +14914,17 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -14910,7 +14934,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
+          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
       <c r="L184" t="n">
@@ -14935,7 +14959,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -14946,17 +14970,17 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -14966,7 +14990,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
+          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
       <c r="L185" t="n">
@@ -14991,7 +15015,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -15002,17 +15026,17 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -15022,7 +15046,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
+          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
       <c r="L186" t="n">
@@ -15047,7 +15071,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
@@ -15058,17 +15082,17 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -15078,7 +15102,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
+          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
       <c r="L187" t="n">
@@ -15103,7 +15127,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -15114,17 +15138,17 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -15134,7 +15158,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
+          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
       <c r="L188" t="n">
@@ -15159,7 +15183,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
@@ -15170,17 +15194,17 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -15190,7 +15214,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
+          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
       <c r="L189" t="n">
@@ -15215,7 +15239,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -15226,17 +15250,17 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -15246,7 +15270,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
+          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
       <c r="L190" t="n">
@@ -15271,7 +15295,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -15282,17 +15306,17 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -15302,11 +15326,11 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
+          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
       <c r="L191" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192">
@@ -15327,7 +15351,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
@@ -15338,17 +15362,17 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -15358,11 +15382,11 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
+          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
       <c r="L192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -15383,28 +15407,28 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
+          <t>SEGUIMIENTO DE MARCAS</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -15414,11 +15438,11 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
         </is>
       </c>
       <c r="L193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194">
@@ -15439,7 +15463,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -15450,17 +15474,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15470,11 +15494,11 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L194" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195">
@@ -15495,7 +15519,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -15506,17 +15530,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15526,11 +15550,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196">
@@ -15551,7 +15575,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -15562,17 +15586,17 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -15582,7 +15606,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L196" t="n">
@@ -15607,7 +15631,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -15618,17 +15642,17 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -15638,7 +15662,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L197" t="n">
@@ -15663,7 +15687,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -15674,17 +15698,17 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -15694,7 +15718,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L198" t="n">
@@ -15719,7 +15743,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -15730,17 +15754,17 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -15750,7 +15774,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L199" t="n">
@@ -15775,7 +15799,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -15786,17 +15810,17 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15806,7 +15830,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L200" t="n">
@@ -15831,7 +15855,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -15842,17 +15866,17 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15862,7 +15886,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L201" t="n">
@@ -15887,7 +15911,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
@@ -15898,17 +15922,17 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -15918,11 +15942,11 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L202" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203">
@@ -15943,7 +15967,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
@@ -15954,17 +15978,17 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -15974,11 +15998,11 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204">
@@ -15999,7 +16023,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16010,17 +16034,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16030,11 +16054,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205">
@@ -16055,7 +16079,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16066,17 +16090,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16086,11 +16110,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="206">
@@ -16111,7 +16135,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16122,17 +16146,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16142,11 +16166,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="207">
@@ -16167,7 +16191,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
@@ -16178,17 +16202,17 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16198,11 +16222,11 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L207" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="208">
@@ -16223,18 +16247,30 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J208" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16242,11 +16278,11 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L208" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="209">
@@ -16267,7 +16303,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16275,7 +16311,7 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
@@ -16286,11 +16322,11 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L209" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="210">
@@ -16311,7 +16347,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16319,7 +16355,7 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I210" t="inlineStr"/>
@@ -16330,11 +16366,11 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L210" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="211">
@@ -16355,7 +16391,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16363,7 +16399,7 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I211" t="inlineStr"/>
@@ -16374,11 +16410,11 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
         </is>
       </c>
       <c r="L211" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="212">
@@ -16399,7 +16435,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16407,7 +16443,7 @@
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -16418,17 +16454,61 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+        </is>
+      </c>
+      <c r="L212" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>HERGO - DISTRIBUCION</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>VENTA MAYORISTA DETALLE</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Venta Mayorista Detalle</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Grupo Hergo - Jefes</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
           <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
-      <c r="L212" t="n">
+      <c r="L213" t="n">
         <v>52</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L212"/>
+  <autoFilter ref="A1:L213"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16508,12 +16588,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>aksT43m+wZJrIuqyuLgkjg==</t>
+          <t>BVwfrxO2eC+aN2Ayeu29dQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>cil515MLzL6S+Zhxqcup04G/lXLC+j0NbQ1MixJinpc=</t>
+          <t>tD3LBlf1cjPCSw5pQeK0SnbGpXF2P6lY45rznqIiv9w=</t>
         </is>
       </c>
     </row>
@@ -16540,12 +16620,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XZ93E8AeedazPIe7prWUzw==</t>
+          <t>3UtaRRWFgUaTN2yoEeZjfw==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>WV3PrRPx1iutu7Ei88mMaScKjMb1AWVIScojTuon4xY=</t>
+          <t>CNkrAJnpGjo1lWmUQ1D8w/wHTit/owWJwQWvaIifnQM=</t>
         </is>
       </c>
     </row>
@@ -16572,12 +16652,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>aVuxeogh+cPUjhCv5w66mg==</t>
+          <t>8AiJvf0io7Tgod5n/uWC1Q==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>sV24ZMAfz57Nd1q9cZJWP+1wDLWTn9QcytCW86kTfIk=</t>
+          <t>y1ZQCcZ3MiCAO1cK4jORv60I7QPMtuCfN78KZ/JKfaU=</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16679,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ydUszkNT91jNX+zrBRypqA==</t>
+          <t>LM3xkqQ2MFuKBwRIEeoedA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>cBCCY4+ZXTuOOK4mVSmdtD14AEI8fIhjU9m/mRK/BEM=</t>
+          <t>KAqjCIqarQcTVjzilV7gAStBIiS18nb0ghXfxykcxtg=</t>
         </is>
       </c>
     </row>
@@ -16631,12 +16711,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JZh21kizkDatq202imOWIg==</t>
+          <t>I8vyP2rjFoPha7PzjK/IYg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>yr5+CVG4UQ1xT/kHiZUq1iXAg6NUMyY12uj8Vgx+1wk=</t>
+          <t>AF//C2wjyadEigvr6qcrFQfvb2Av7YvQOZ7OgQEuKy4=</t>
         </is>
       </c>
     </row>
@@ -16663,12 +16743,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>jJ6QByQ4RPjksI+6HuxaWQ==</t>
+          <t>RA5Uy4SYjTpkw6mM13kSeQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1x9voCl1nPIWAjL0SSDwEj56KG8yYuKZQuB/JgzS1DM=</t>
+          <t>UE8uBZHamzhgAhP2DWIC1eO0YrsYWgn6uNuxxXhVnfY=</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16775,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>y6tzFgNGeZvqATziyT2Q5Q==</t>
+          <t>mxUUl3x72fMgjkuFvHojBg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>4Q6y/hhq3+b9q884IUEJp9tGKrbngwO/I+5EvBgGXJQ=</t>
+          <t>fGDuULEhQg15ogG6djUocpgYDiGkt6SEGvHYboqbg6Y=</t>
         </is>
       </c>
     </row>
@@ -16722,12 +16802,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0liUSt9wiDH9/wAYl/qmeg==</t>
+          <t>pQixDZpX7pDHLOW6kWCYbQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ASSAg4A3l1Ch+PQ5eJfVVUV+JeUGK/9dkjDAGoKyfBM=</t>
+          <t>04/A5Ls9w5b3ff4HS8W1QOjMMUacgHQviqB5GeQmoPg=</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16834,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>kNs9XPQX+60ypyuS+fVxeA==;1/QCM9ycjx8OqS4dvOOC5A==</t>
+          <t>Zjyjah4fw+sqLJa9WZjD4g==;QUyKep+s2T6AhLDgcVBJ9w==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Uh8sLoscXPW+CukThJZQWMYFWGoHLvn1BsOkFzElq6w=;aeE7M4Znp2ASmYm4JnQVNiOMpc1BT/yueC8WUr8bS+0=</t>
+          <t>tdZJLRc1THdjG6sVCETdhc6EApWHC2FB7w4dgygpr6o=;1MxImoLyGNVrSoNlEGAFNAOLREhwgFiFQOOgrvi9fOE=</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16866,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OQNwaGtOOSrTKunZI6WJ7w==</t>
+          <t>QUAyb1OZ2+8gu1VEljd/2A==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>mxgItOGznrC8n1IsKk/NhtK6qkZ9lWekbGeXc9jYr7w=</t>
+          <t>wZi4Hoika3ouvx2ePZ13sZq06O2qRaOLs47QN9zrXOw=</t>
         </is>
       </c>
     </row>
@@ -16818,12 +16898,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>5Ly+VoxLGHs2mdKVFE0xMg==</t>
+          <t>EJyTkp/HX/YrflIzFRinog==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ZB7+jkv12nPll15C8NmXOPKdF3f+kAmPbm5QemsKd3U=</t>
+          <t>vTiPZWcu57vMN7EGGrAizjVDmZCPeHqqKqDemRDdCnw=</t>
         </is>
       </c>
     </row>
@@ -16850,12 +16930,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8h+X/TfXoCzjUy4RQluDMw==</t>
+          <t>ulnOSIDXIk2LgqMRgh0xJQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>doUiPMH+UKR1iU7CCvrar2+YTn+PkvIXp7U3m33w4y0=</t>
+          <t>L/9S6s42KCCJ3NO8tXWEUM8zV28U4maNMMYQQW4t9p8=</t>
         </is>
       </c>
     </row>
@@ -16882,12 +16962,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>c2SqqwKA7jw7rXMX1qvD9A==</t>
+          <t>lD7gQRejhELTMFY8Fm1bug==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>5Q8HIubxJTmcAQZY33792U8/Yxa/E4/nO/qgVdCme5s=</t>
+          <t>eQGaw/5T2bzKlKuPnqsD0uMj4WDZWXPe8qGjxv0Le5I=</t>
         </is>
       </c>
     </row>
@@ -16914,12 +16994,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TEzQNUzCS82O8o6VZQW/fw==</t>
+          <t>yjO2rodil2WpRqgWeMW8Og==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>whnbegwuAo3Ru2eQ8gt8Fg5+lIVex9I3++X9uYs0RYE=</t>
+          <t>iF6GAzanAa8X8K7KBQAkwzgSuXa30D/K+Huqwcfq+cs=</t>
         </is>
       </c>
     </row>
@@ -16946,12 +17026,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UBM4KuR45VS9zEFDeQCmfQ==</t>
+          <t>49NKPq6X9rFVqniXusqTOQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>WuQrY9Dv0PAJyD7uyhJApm5StmaRy5GfMX5ImFLHf2Y=</t>
+          <t>6VyRbvcs5OlVIeoqEZusxgiKA1p2Qx/ODqpkgwCWvro=</t>
         </is>
       </c>
     </row>
@@ -16978,12 +17058,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>68M92ZCgT35mIQGtNQxoCg==</t>
+          <t>DxhW24skhlbLkh+IzC593A==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>9BdppOaph386HZEzrQP/VF0MJxQGFaOXfCKqvhtheJ8=</t>
+          <t>J3/nzdNL/MJf1Ql2d1M8TDI6l1t7s7KmnZiqN87hhdA=</t>
         </is>
       </c>
     </row>
@@ -17010,12 +17090,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FjBmFNAW4z4tTOvd5U0Hlw==</t>
+          <t>9Jfg/sMA8CD/aoaPTKCNyg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>OoX47VmUPMaMF7ZJwsw3XHb4SL1Gjwq408/xx9P/zBo=</t>
+          <t>6wp+YuatoLQbZcVJKpFks8CHSboETc9Kh0pZj5i9gmA=</t>
         </is>
       </c>
     </row>
@@ -17042,12 +17122,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>q5tcDYQV10TcfsElVUB0Hw==</t>
+          <t>5cgokStsNTga4elvcbFlrA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>bkQqy6PWsnFEbFKIa71ZKlDfiaue0ti0gEl61AARnAY=</t>
+          <t>xT7EXzNmUr7BYDTgaCd6yDe77wPFpA2RbJ2edKXYGv8=</t>
         </is>
       </c>
     </row>
@@ -17074,12 +17154,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>S2OrrKSAPS2SCPD5KXl00A==</t>
+          <t>Kgdh/9gOuF9tG1ipuI+/Yg==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>o4fNKYY2BwRcUmfwpNq8GhLvQmyQT/gj22ERIP0PO7Y=</t>
+          <t>ZK8aNs3Xc/CF3hUMbWxcEcss3FReARAl7KKwo2qKKy4=</t>
         </is>
       </c>
     </row>
@@ -17106,12 +17186,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1yms592TPgpSGTVknO2HLA==</t>
+          <t>ZPyFCvlzfrk1rusAm6e34Q==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>//xriyP0N3wUQziu1345Q4M6D+/OhWBSky1xXX39TA8=</t>
+          <t>1Ly8YiJQ3P4Hrm8Iv0iU6dy8ShPoQOBh5On1F7wiYAw=</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17218,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ddi/s7f7ww1hNsQ/oA4R6w==</t>
+          <t>za0qyIZmA5iCMQtIpY/CtA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>HgtbuqfHebbAwyQVPIsACdnWAEo0RhXsmPLxnZhXOWs=</t>
+          <t>6XYO2RA3yHFu+/+B6KFzlVAII9d5D7ekL6CFg3oOVLo=</t>
         </is>
       </c>
     </row>
@@ -17170,12 +17250,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ToFm4v/E5ACmN7U9G8rmjw==</t>
+          <t>ApWjemCRqWe+iT9WcCpESw==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>glYLxBmbX3bKvbVFATK1lic9Ly+X4ePN+ed7Mypo0Y0=</t>
+          <t>0DE+M93Atqd9/YQGjpYCkMd/CgZxx5ogr5e35PR1qQ4=</t>
         </is>
       </c>
     </row>
@@ -17202,12 +17282,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>bcuYnRZiNbPmlxP9ZJa7Hg==</t>
+          <t>nud6ru//wcsrd1c1AUP8rg==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>IycDcbMmSMvWRscC+411AImnpTrK2TxjvS13c2ABVAw=</t>
+          <t>iICulYlNLS+rpcp3O2YsZiV6vS8jJDQh4+cATlSa0mQ=</t>
         </is>
       </c>
     </row>
@@ -17234,12 +17314,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TYNV0zR/MbeMQ2qClApIXQ==</t>
+          <t>3rmd7Nb9vzsFRAVBQP8qkw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>f3FUg/syfF28TCnZYPONZFRN+liF7TYFJ/NgNBSAEeI=</t>
+          <t>H07QqNBxd9lVwpCzkThSNa61myl1zL9yd7jl4qkHh6c=</t>
         </is>
       </c>
     </row>
@@ -17266,12 +17346,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>yBVguuNxwzZUGM4fpaIqIA==</t>
+          <t>TxnB6HMytm81FyVvekFjDQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>lN9r7/HA5IhJFXtmp60vRphy2L2gUFePncJBCe/YNOo=</t>
+          <t>kXC9OwEnrTT7b/fo4lR74CINhWlyqkGuFf618Vx5/Ac=</t>
         </is>
       </c>
     </row>
@@ -17298,12 +17378,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CF9m5xKjxwr8ZUeCCgDjbA==</t>
+          <t>/d/dt88CXc/22OrOeILWfA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>JxZAO8O0Oa6S/zDVYXkGxP60rGJyGDJSWgeaLp/wuhQ=</t>
+          <t>MAwjDIH9mT7W4wkuZiYGobclxF81LnLLaiSOE1hQ7Bo=</t>
         </is>
       </c>
     </row>
@@ -17330,12 +17410,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ry/5a7LzdRisM2BpJQWgAA==</t>
+          <t>WOzd1Tni9aR22YRy/TZ45Q==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>KMDJMf3JE6EuCs/DWyBH+3ldXTrYvChQoJpjsi7jP1M=</t>
+          <t>Yblq3zq1L4dyWSmTFuHp27lQd8qnED4oyr5fCPLjNCM=</t>
         </is>
       </c>
     </row>
@@ -17362,12 +17442,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DSBED+8DVUwvsjbr68nwVA==</t>
+          <t>fjqaUcsa3k9ww2285uMnNA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ocRPt0YCByF0JHnmU9DJ1FHLvVVLipAM8ffSWNcjoPA=</t>
+          <t>+s8EunVlEQjdPPPUMp926UfxSAZvJ4BkEyctzGdfbwU=</t>
         </is>
       </c>
     </row>
@@ -17394,12 +17474,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>UjRXt56YXo29ijVrrxCIdg==</t>
+          <t>r7E6Uexybc0Hu6KRHS3V1A==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UCgsSy969GkjY24totBFvT8aWMN2SUx4jbqfVvLUDxo=</t>
+          <t>YC1YysTTI5aN1WNuUuQ5Txsc2HexXPwgtKtYG7jhfSM=</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17506,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CFxWhV6tZ5ILDzhhFZzDpQ==</t>
+          <t>STCmQcVnfO+XjGdN7WDgaw==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>bvAcJQM6u9kuksQQ4cLQQqJv0ggieLdRQMMI9kwLABk=</t>
+          <t>TvnhwLRevgtXZ21TFViRjeTl1GY/K4k4JQfgPfcM+xU=</t>
         </is>
       </c>
     </row>
@@ -17458,12 +17538,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NVuqgbtGTRNXl7Ss9QrMtQ==</t>
+          <t>FCEKO5OxzVSUNa8uHkHMcA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>P2SE7J5DM+2TUiwCkh74voQaUHBR2IiHe3exudQFEaE=</t>
+          <t>UdC2NdKbnlp2zlRNslLfgXYn6HUt9gZZ2ta12930+dc=</t>
         </is>
       </c>
     </row>
@@ -17490,12 +17570,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CmAqbtFbAfF8hc11SRqWgw==</t>
+          <t>KxpD5HXAzSB0QLoVBFqUvA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>OMYC2IEb9X/2qII8panwNXGBe5uZyFiSMEHIkYGJIUs=</t>
+          <t>ifhJL3/ZgcQFaZ+RJALn2NV3OTcsaEDxc5ha4Kir7zU=</t>
         </is>
       </c>
     </row>
@@ -17522,12 +17602,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>NPdlgAT4sOtDglHrVlYQsg==</t>
+          <t>w59YhScrhcyNSZnfCa0t+Q==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>qwC4mId56sB+AT6emuYqcadg28eHjkFvx7f/RfvcNyQ=</t>
+          <t>3TGL/eEgjt8pJIOkYkFFXLyRpX+e+p87II4cTwSd2mM=</t>
         </is>
       </c>
     </row>
@@ -17554,12 +17634,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>wbxYGfvz1xl9iBCbI5TkpQ==</t>
+          <t>XZMSDNGblQWBOHBcoq/pxw==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>5jC9SCLyZMIXRMi/swQlChzn2bA42WKJLS4WARNHP8I=</t>
+          <t>+yOJVi2rwrb6uV1F/8KrW+GLuGynQYmKsyt0x4+3WMw=</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17666,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>XQFqtNg39SSZ2sKjovhwFg==</t>
+          <t>afkSIQGjrExRRpUL5NVf9Q==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Aq0MMGnLsWGRvUgEyQA8bnzQsFQ5spbb5KdbsSx5mQE=</t>
+          <t>6NvYfVxipZ+s40lE3nulf5tUBvG5AnfIyPrEU4frd7I=</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17698,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>pyr1SQNQpisme6HPcomm+w==</t>
+          <t>T21RvgiBMT6uFKjGJAWrGQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e9aro7yOdzryN71aOSfxfZYMBTzP1H9cS0yJdae4roE=</t>
+          <t>iuKljfHsKE8ziQIsRNDRbP81bah5aqDUvw5QI4caB7Q=</t>
         </is>
       </c>
     </row>
@@ -17650,12 +17730,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PbphOL/ffXDnx1gK9JwLVQ==</t>
+          <t>QjCaC7u7uYafQDmWbfTM0w==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TQmwtGG6Ewd6Pqvmosxs6Hm8txd+XQUV8NgNrCrSo78=</t>
+          <t>iabwZQGNhLmL0sQMmMsetzCPBJwD09V5JIB37ug9gmY=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-04 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="82">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="88">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3967,12 +3967,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6f91c54d-24ae-4d7a-a580-596cc52ec510&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="98">
@@ -4003,12 +4003,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 10-2026</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0731c094-27aa-438c-a4f0-d5d3c0e5e8a7&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="99">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COMPARATIVO 10-2026</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0731c094-27aa-438c-a4f0-d5d3c0e5e8a7&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6f91c54d-24ae-4d7a-a580-596cc52ec510&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="100">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="117">
@@ -4687,12 +4687,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="119">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="121">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="123">
@@ -4903,12 +4903,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="124">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="125">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="127">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16">
@@ -7542,7 +7542,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="L69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="103">
@@ -10994,7 +10994,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104">
@@ -11038,7 +11038,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="105">
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="108">
@@ -11466,7 +11466,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="114">
@@ -11870,7 +11870,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="123">
@@ -11958,7 +11958,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="125">
@@ -12178,7 +12178,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="130">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="147">
@@ -13126,7 +13126,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="148">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="150">
@@ -13294,7 +13294,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="151">
@@ -13382,7 +13382,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="153">
@@ -13426,7 +13426,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="154">
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="173">
@@ -14530,7 +14530,7 @@
         </is>
       </c>
       <c r="L174" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="175">
@@ -14662,7 +14662,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="178">
@@ -15006,7 +15006,7 @@
         </is>
       </c>
       <c r="L184" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="185">
@@ -16774,7 +16774,7 @@
         </is>
       </c>
       <c r="L216" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="217">
@@ -16818,7 +16818,7 @@
         </is>
       </c>
       <c r="L217" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="218">
@@ -16906,7 +16906,7 @@
         </is>
       </c>
       <c r="L219" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -16992,12 +16992,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>lslLZG3fBMWwl1RMdxxlPA==</t>
+          <t>9ZvV8XpDAFAqf37NfQa4WQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>+RBaLC9PLaJE+xN4rp6qD4xFPPHI209GT27l/DK5MyY=</t>
+          <t>V4ei42vlMC+t76RQjQKoEtX8qwbWe3aPMTLm+KAQczw=</t>
         </is>
       </c>
     </row>
@@ -17024,12 +17024,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5HdeZfHkb5FanSRghsHSBg==</t>
+          <t>cWjolxSuDEn8HgnNPwUhCA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ZhixLBz/Esp06yKOTYgRRg0h+h//lR2YJ7EqIIFkPqk=</t>
+          <t>VNR9rhR1TV40h6n2HCc29VwOAXo1+JLJ3CT/BQugH0Q=</t>
         </is>
       </c>
     </row>
@@ -17056,12 +17056,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+rc6ZqHTyT4H4ChUBMLxNA==</t>
+          <t>pRjqMHUTFZFy+K69iJdRaw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4m/HF5vLJ6mdUuEKD7x6TAFPPGJ/qqLEDbVyggtuQuY=</t>
+          <t>HF3uhBo+s/JB5ZPFMLOpXNk73iF5JGyuP3I5dJqNjVs=</t>
         </is>
       </c>
     </row>
@@ -17083,12 +17083,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Uj2fN06gf63r3tS21K4bBA==</t>
+          <t>D1VAont9/1Z0dGSfUIU+5Q==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dc6TYh6nIaVvp1cG5HACN79dXT/WJL9sQ8n6t7ZWvf4=</t>
+          <t>U21VpZR350phVtKsFqF1PlpJvWnXntzX6Ls0x6y+ysU=</t>
         </is>
       </c>
     </row>
@@ -17115,12 +17115,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>suKzdO19h8aolL+kYbDIuQ==</t>
+          <t>Fsg33gxVmRIODIslYTuoOQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>eXVF0y+tfcVHqpDx8dOdzF9p8GyFrCBOWhE1dV9tvrM=</t>
+          <t>RJ6O5nGoxHC0zv2GO85CSkYaJGNA0VMDZKhlGApuqh8=</t>
         </is>
       </c>
     </row>
@@ -17147,12 +17147,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1mB40CE/Qe53hNiQOcX4eg==</t>
+          <t>lsRTgq5CpX/y6E7CdFS4oQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>/RLw7v9qQcXJ4QD6cK0J+k+BjrrhldPBybwgldxMpv0=</t>
+          <t>lHdysB8FPdXCvycye63hZIKYvOnc9PDQg19Fsdv2On8=</t>
         </is>
       </c>
     </row>
@@ -17179,12 +17179,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ro42vtws41cxoqcWS4qG2w==</t>
+          <t>iPdUGC4pn83kXZkKG4Ce3w==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>+tbfiJUwMo0KltUwrUwdr+ggpPSFFM5ueGGm0513xio=</t>
+          <t>19GIT+Z1NQaZc3TD1ojC84HPJDSCVPijnZMSwt0y+/Y=</t>
         </is>
       </c>
     </row>
@@ -17206,12 +17206,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8h6hmMYZaQ8KvaI57iL3tw==</t>
+          <t>vVOB/cA4VLy1qGjrleE+WA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1F7RWVHcAhXpk6ciPZkRHznO61Wcj731P60D4BHoHnY=</t>
+          <t>leLo90fQqgNE5wbDyOXsTfTqB34fMxT+yZlEuQVfteI=</t>
         </is>
       </c>
     </row>
@@ -17238,12 +17238,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>jAhqlAyhotQ2dp6RznU5Rg==;BzmyyiYU9GJXoH9DQVMhzQ==</t>
+          <t>kX/VOZd9Xx+/u1nGBzTihw==;mp8WhVokE9TD1KoMtXCp4Q==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>twRpwUuCpToNZFxFkL9zGLw3HrdzKmWS0rXvAxQUwNw=;rNpDqUHPs2Fn3vBHMkrGdxo6dunacNlFw79UVW8OTXE=</t>
+          <t>CgGEOma37YULFjE0zCyfrDSKQ+S8uE0PRWtnGQ4jGRc=;EFGaecEIer4FHMvRpSalDJWh41eBv8UkxpxfzvK8lwA=</t>
         </is>
       </c>
     </row>
@@ -17270,12 +17270,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>XaCgt03ZQFfqfDWox4vOjQ==</t>
+          <t>AdGObZMuBGf/R6P3aD8a6Q==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>fMYllWe8VuVWl77kgDhRsgn9gBVBqK010NBD2tHRAV8=</t>
+          <t>ROORYGTSSOxwM6oG/3imxCRE4cCjkhUEtfTU38n0/cY=</t>
         </is>
       </c>
     </row>
@@ -17302,12 +17302,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>XPQ2QooKVYyCmKtny0dKVQ==</t>
+          <t>7wuEX6N4XWeQ30ArSTyGrw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>yGUMjnYbiuV9ApUYxueT3OWhto0aLukAxX1SGkiXhDU=</t>
+          <t>nndZgALVjzmO2GbtZEHD9ayHAnDHP7wlPt/KJmxvAAM=</t>
         </is>
       </c>
     </row>
@@ -17334,12 +17334,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2KAtb0GL7B2Xeg0HiHBXaA==</t>
+          <t>OT36okELDpCFxSS1Hf6TSA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>xY6+kJSTT8krdk1bCQimC9EceB81+p2dID75tKZHx8Y=</t>
+          <t>wY28Oz9+f5YVBjHkxzNMiUZn2LwkjzvGyod9RX+tWGg=</t>
         </is>
       </c>
     </row>
@@ -17366,12 +17366,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>lduP5mTmJeiqRD6KN8chGg==</t>
+          <t>Eu+PDh3joXAqwLR4jbT3vw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>6LUOLDSgKxZsjKkUql0CdnpIicsIpRqyov+e4UKbl1s=</t>
+          <t>cmx/JO0Ffs2LFpZiKAajQyy/GtEmstfy3WhNLFtu9VA=</t>
         </is>
       </c>
     </row>
@@ -17398,12 +17398,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tjs+AFlEa4GISaBXJ1nRDA==</t>
+          <t>B03GR+QtctU08n3TKmi0Ug==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ZdBgSyWIniJjG95gXHCHzja7dQcCO1IgfpjtHw9/QZY=</t>
+          <t>HCfnTs4cpOl0cPR6iwbi/mQb56mzu2CASTHUY6VxvDM=</t>
         </is>
       </c>
     </row>
@@ -17430,12 +17430,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>jklph6WdrOImpYBEWK294g==</t>
+          <t>PPMUjn/2edPGz+mZI2EjRg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>wEMrZ8xO1kPO27vvJuQPTfhfZVXAWApyHf5t2wKXAlg=</t>
+          <t>WiCOLbsxy2MF1AvOixMV5MM23e2ZzyVUpR3m+pIxuMk=</t>
         </is>
       </c>
     </row>
@@ -17462,12 +17462,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>h/XBZ2n9YQYKPajQC/axtA==</t>
+          <t>pXJayUOGHRoadywDocdtXQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2qo1OXgL105kVXqZWLVlrbvZMfydes20SQfj8gGkfWA=</t>
+          <t>a6fcUeAmdxyxvoQlxQQ7OFcPC6HTR2IxSHj6COLXL2Y=</t>
         </is>
       </c>
     </row>
@@ -17494,12 +17494,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PNr39zaTOdn741o3ewTZPA==</t>
+          <t>5k0qrtDRzI7DPLb6DKZ1yw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SuXlw+eXEI592ABtIhqXNSN8VJ5ALczWHddtIqFkGA4=</t>
+          <t>mPoxU9azNaBEuaoiicD1YVNzK9Xo0tjI62KUzmUCzOI=</t>
         </is>
       </c>
     </row>
@@ -17526,12 +17526,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>avsC7CvLPqBVjWTMycoe+g==</t>
+          <t>rZzhJDbKTwjazB/0+70zBg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>VAdaF6iBMGo5FZ1KoIVOPy9f9KEBXnlDzSve/xoXF2A=</t>
+          <t>SclGTd2+WfKN7CwDudSWU29jg2KfHCCjXZi/NVWcZ48=</t>
         </is>
       </c>
     </row>
@@ -17558,12 +17558,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RhvDUFrXaOO0SIEdlgZ0OQ==</t>
+          <t>m9CQbBD5QnuUdSfZpbU1Gg==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>JXxgmEQdtvrDo36VpHDOQa0AR2mf+os8YxM++59Rdbs=</t>
+          <t>Cnu9qmqXS8Tfm1Ut0906nl9u20P2gGpMKgc24s5zIu4=</t>
         </is>
       </c>
     </row>
@@ -17590,12 +17590,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>hP+G056neRViRPFXeV87lQ==</t>
+          <t>k4quVCfwOEdIrWhm9+azWA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0gqvNMPVELfO+Xjmn83QH3GiGNSv35BbnqDy/S3q8sA=</t>
+          <t>fNyM546Gat8JAZxoy/5bXzo33y8F51kEjdJSR+AWnSI=</t>
         </is>
       </c>
     </row>
@@ -17622,12 +17622,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>sroVXuW4JYcTdSwdH6bo6g==</t>
+          <t>kS6IKoJ/9+5xT2yxJoJFpg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>+2oJR0B4sTaS4GOD6wY2clULlCALHOKXkVp3Cc8aprM=</t>
+          <t>aIJK0CQ8jDyRt+Zr1iXq8pFrcjuyxpiNpZvAb/OmPUs=</t>
         </is>
       </c>
     </row>
@@ -17654,12 +17654,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>kOrzvNyx0thLAXP7UsyTmQ==</t>
+          <t>d4am9ONAAqqDCu5cV7dPrg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>REh9rqDvJd+3ziCzAJoh5HxF9O1v4yMNZRfHT/n1FR0=</t>
+          <t>VNTfPt/LqXFoOJzeae8Y6PsowwqucNr7s8GSN7gAIsk=</t>
         </is>
       </c>
     </row>
@@ -17686,12 +17686,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>D91lHeWDvULEHYpnlY7SOA==</t>
+          <t>MPYsLFSRswKdfnvMoFzH1Q==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4HbrxyF9YvcQiu9I0xEsr7mYp5+mjP+vvknaTTREDeg=</t>
+          <t>qSw5rTzMD7tYIvc1jTkwRtKRZOKEtTPf6AokJJmtQyA=</t>
         </is>
       </c>
     </row>
@@ -17718,12 +17718,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>zvSMZVu12JrRdAHdEYgFLA==</t>
+          <t>xMB6K8F3fQEIXY1OKbJjnw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>VrVuEsEIZLGQK2vlnDFesXFNqwIrD0iW7+bjlno29mg=</t>
+          <t>elCqVG7nNqBX8hiJwdsN6W+4bZK+Vr8isaFn46lhBm4=</t>
         </is>
       </c>
     </row>
@@ -17750,12 +17750,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>biHDTAjT7oGYB3PLculokA==</t>
+          <t>0VpT2YhDnrxFY2lrwhpg+w==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>aWXQhX3MmojiDnQlNY4VTCyQQiA+SQt27GDehXBUOds=</t>
+          <t>5NmAVtUZMXPTnTEZl23XRhbuHlB7MS/qDedqsfJ25wE=</t>
         </is>
       </c>
     </row>
@@ -17782,12 +17782,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>27yya1PxyL+aVZRGs61Z6Q==</t>
+          <t>5DCGOGhvIbrwPiMvZyx8cg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dEH2nr0qtozl01/REqbVXpBvw58lIHLc6WeBY9KpKlM=</t>
+          <t>LfBzmbF8ibQeCj3PlnG6X5/1aMF5o2/e8xDCXltjnTU=</t>
         </is>
       </c>
     </row>
@@ -17814,12 +17814,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>YeJbEAEHFZZlJdkc3P77fg==</t>
+          <t>I0QKsCWq+HC0C6k31SRSLg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>p3FMffLTxu/RxB0631n0rmb0HN/YaKoh+b4czss+ItY=</t>
+          <t>5df+pPweNa9626Tr/D+PovjhsHQjekxyDygc5YmXZCg=</t>
         </is>
       </c>
     </row>
@@ -17846,12 +17846,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>6hBO6TAA0yCUddxeIOMCEw==</t>
+          <t>v1cw2kfAcEhboNrpJdG7gQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>uBKC+nabPJxe7tX3G69Vi0Fy77gV88S19tzL81BlnXQ=</t>
+          <t>qiDjYyrvnj4JqzFHn6FHVBffDr0nVVG7JeMvwMm+lVk=</t>
         </is>
       </c>
     </row>
@@ -17878,12 +17878,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>qn6Cqy8PeMh4xO7Gx/Wyrg==</t>
+          <t>KQJtkpmQt4DWCcfPK/drqg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UEsssMZnKwynSzoidlesyZAc9ga0KUKvIHNDEVQyJrc=</t>
+          <t>XjTH3Wjsw/BDECHEX8zN2uj0C7gdr+HWfiJBHlqLqfo=</t>
         </is>
       </c>
     </row>
@@ -17910,12 +17910,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>bCr7ZzdsjXfRnE2U3rrkVA==</t>
+          <t>FWTgA4UQacasDhPE19qVsQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>gaHMUbjZ9ri5iLqe607eSJw3bTuEPzN5V12jelGtSiA=</t>
+          <t>8WVgRXrBKg6D1YhkwxyLfBpWWuMJbZfzLrhtXpGg20o=</t>
         </is>
       </c>
     </row>
@@ -17942,12 +17942,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0TO1UIxdMUKrUnrRoxXFww==</t>
+          <t>5yNMOvoELVeVolSjuOvoNQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dKdonvg6MeI8kT03Wgu7/7ar+eqsbhtTLuKyMa34faQ=</t>
+          <t>3Rv/6aq6G6dO0wOXxhGf8DilKjeJPVR8Ad88s5jDsJc=</t>
         </is>
       </c>
     </row>
@@ -17974,12 +17974,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PGuLAMAMJhhLIxb9i85Zlg==</t>
+          <t>d211OZD4CH4nv5n7GZ6djg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>vxHlNCWXqKMZuB6dXd8WXtdgr8XucbSWaIyf3uwQnfk=</t>
+          <t>oWGrcppQoZ4H89Zm2kc6dNaEwXHwn2mdi5iubGQVfZs=</t>
         </is>
       </c>
     </row>
@@ -18006,12 +18006,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ghKOKPwBPy36lYpx92242w==</t>
+          <t>J5Py3VjsQGhr2L84USVYMA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>iDgDyo3yKlcs0l8vaCEd/06T39lZAzVq6R/Hadk3ukY=</t>
+          <t>GmpkxrYxPIiMfBnpInozHR+5Nx4BcUMclBHERsG+3E8=</t>
         </is>
       </c>
     </row>
@@ -18038,12 +18038,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>rqtW1OTfKeJvr0/AJ7Fsyw==</t>
+          <t>WwOr9I5EQFtblWoFkcBcBA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>5F1H0hK4khzg9M/3Dp8t+8i8jnfJJ9rjarDAwY0IQow=</t>
+          <t>YM6AuE1uCT+5bdDR9R5vp72zIFMjK0vLqK0DLHOkkTE=</t>
         </is>
       </c>
     </row>
@@ -18070,12 +18070,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>vXw/qzTynzEW4j5srdGrEA==</t>
+          <t>JEgKqeiD6g0TuJlUwrsnBw==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>6NcArBwDiBGqBKrVwz6gQa5l/E4IDUolFfkjkkF7pGM=</t>
+          <t>i/DbYgufQueNwjyaktWAV5dPhDqN7GzdgfB6Y0Z9uB8=</t>
         </is>
       </c>
     </row>
@@ -18102,12 +18102,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>8c75hOgaqKFDnmT2eOCpgQ==</t>
+          <t>PGKxYKK2spHwHV8uCPTpgA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>crB4Sz2XoHf34pPbFcxu1TCJrgJUpXvB1NPQQgKfUfk=</t>
+          <t>kWAs9PxneBtoswZjtB0RWC32x8a3NfEjGutaHfoGbR8=</t>
         </is>
       </c>
     </row>
@@ -18134,12 +18134,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>lmPUUEk+waVc3MtXMKPWuQ==</t>
+          <t>1diAcdDF2xYHQDt0SEehvg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>3zRGyXaYcYwBSJ4p619sLVk56SC2kNWHP/2ZM8DwZyU=</t>
+          <t>GGMsMfSB/ZPGknoDtNq72VfHov7CL51re4/RVUI3MTI=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-05 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="88">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="116">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="120">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="121">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18">
@@ -7542,7 +7542,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="L69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -11038,7 +11038,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="105">
@@ -11650,7 +11650,7 @@
         </is>
       </c>
       <c r="L117" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="118">
@@ -12398,7 +12398,7 @@
         </is>
       </c>
       <c r="L134" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="135">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="147">
@@ -13126,7 +13126,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>347</v>
+        <v>340</v>
       </c>
     </row>
     <row r="148">
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="173">
@@ -14530,7 +14530,7 @@
         </is>
       </c>
       <c r="L174" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="175">
@@ -14662,7 +14662,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="178">
@@ -16992,12 +16992,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9ZvV8XpDAFAqf37NfQa4WQ==</t>
+          <t>oWdcbiHY5Vrd3qF7KFpNFQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>V4ei42vlMC+t76RQjQKoEtX8qwbWe3aPMTLm+KAQczw=</t>
+          <t>r7WtEkUJLp0kFrZU55A2sX9Uy4Q7RkKn/7YjOfNb4LE=</t>
         </is>
       </c>
     </row>
@@ -17024,12 +17024,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>cWjolxSuDEn8HgnNPwUhCA==</t>
+          <t>0JhwPesSCI3DtrnEiorbzg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>VNR9rhR1TV40h6n2HCc29VwOAXo1+JLJ3CT/BQugH0Q=</t>
+          <t>go6ntu5aLZ9YrwhapZQ3oz6+OlR64xXriRYZBAuxv3c=</t>
         </is>
       </c>
     </row>
@@ -17056,12 +17056,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pRjqMHUTFZFy+K69iJdRaw==</t>
+          <t>I0JfF1W9YB3jPKS62is9Jw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>HF3uhBo+s/JB5ZPFMLOpXNk73iF5JGyuP3I5dJqNjVs=</t>
+          <t>7l8XHehCjpUuxH2VpNMhnXOhbZUIqUnxM6+CLEEf8gQ=</t>
         </is>
       </c>
     </row>
@@ -17083,12 +17083,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D1VAont9/1Z0dGSfUIU+5Q==</t>
+          <t>XZ+qGsy5g7Yuu2mIBHerOw==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>U21VpZR350phVtKsFqF1PlpJvWnXntzX6Ls0x6y+ysU=</t>
+          <t>yYzvOHL3iQhwY0CMklxXcD3iUBob5a3Yw+wuAt/KqJ0=</t>
         </is>
       </c>
     </row>
@@ -17115,12 +17115,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fsg33gxVmRIODIslYTuoOQ==</t>
+          <t>J01Tu10SCS9SHzrk8MCXoA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>RJ6O5nGoxHC0zv2GO85CSkYaJGNA0VMDZKhlGApuqh8=</t>
+          <t>E+KLeN6y8ks5DaTDGtlcTP1EzIsSA9abSDO+T32fXC0=</t>
         </is>
       </c>
     </row>
@@ -17147,12 +17147,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>lsRTgq5CpX/y6E7CdFS4oQ==</t>
+          <t>SKEvrgN1tdeITmeYbkv9gw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>lHdysB8FPdXCvycye63hZIKYvOnc9PDQg19Fsdv2On8=</t>
+          <t>Qj/kbCyNOGjCMS3vgc8yIZUs3H3c35dTfau69Zw9bUM=</t>
         </is>
       </c>
     </row>
@@ -17179,12 +17179,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>iPdUGC4pn83kXZkKG4Ce3w==</t>
+          <t>0KKQdt8PS2iu4piyy1VGfQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>19GIT+Z1NQaZc3TD1ojC84HPJDSCVPijnZMSwt0y+/Y=</t>
+          <t>wJpKyxRKBSc6C6ypUZISJ2LKFihHRKtiJ9cKVshvzZA=</t>
         </is>
       </c>
     </row>
@@ -17206,12 +17206,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>vVOB/cA4VLy1qGjrleE+WA==</t>
+          <t>mjd8JASSvRFAGP6/6lsQIg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>leLo90fQqgNE5wbDyOXsTfTqB34fMxT+yZlEuQVfteI=</t>
+          <t>lN/Mx1uJx1Naqlb1kntTdDyXRuGSXItU7n09AjPisZI=</t>
         </is>
       </c>
     </row>
@@ -17238,12 +17238,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>kX/VOZd9Xx+/u1nGBzTihw==;mp8WhVokE9TD1KoMtXCp4Q==</t>
+          <t>nYdhFONYWw0JYj6NXIv09A==;+21RtNdbM+tdHJ+lHIn6sg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CgGEOma37YULFjE0zCyfrDSKQ+S8uE0PRWtnGQ4jGRc=;EFGaecEIer4FHMvRpSalDJWh41eBv8UkxpxfzvK8lwA=</t>
+          <t>9Za1RNk9nC45Oh3kjTy3N52sGaBC8FKZGhfjRIAgQvs=;ljAqdvxPbjcoD1T3s+9nGa09b/1vF7KQHeOJlt2shls=</t>
         </is>
       </c>
     </row>
@@ -17270,12 +17270,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AdGObZMuBGf/R6P3aD8a6Q==</t>
+          <t>uC7d7w8g2lkVLbVPvki8Sw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ROORYGTSSOxwM6oG/3imxCRE4cCjkhUEtfTU38n0/cY=</t>
+          <t>+J17OJGXUDaKJhP0ua8fh8dgQYCir3ZJ6BmFb31SCAY=</t>
         </is>
       </c>
     </row>
@@ -17302,12 +17302,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>7wuEX6N4XWeQ30ArSTyGrw==</t>
+          <t>gmp2wygPLtySL+EqqLmgTQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>nndZgALVjzmO2GbtZEHD9ayHAnDHP7wlPt/KJmxvAAM=</t>
+          <t>Hee2qCGfvRKEplHoqn/J64nJA2/k4Dioe+yQBmEGWEo=</t>
         </is>
       </c>
     </row>
@@ -17334,12 +17334,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OT36okELDpCFxSS1Hf6TSA==</t>
+          <t>RJC6NIHS4QvWZo6ztxhdTw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>wY28Oz9+f5YVBjHkxzNMiUZn2LwkjzvGyod9RX+tWGg=</t>
+          <t>ARhZZZKuYmBHToCxnN9jsriu5XP8BvMkyzu0B33qAt8=</t>
         </is>
       </c>
     </row>
@@ -17366,12 +17366,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Eu+PDh3joXAqwLR4jbT3vw==</t>
+          <t>qIJsE8tOimluIKV4+9NHZQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>cmx/JO0Ffs2LFpZiKAajQyy/GtEmstfy3WhNLFtu9VA=</t>
+          <t>81iu5BPOkR+AXGBUKGKiOsgmXOP1WwZQRzGtD5AyEDM=</t>
         </is>
       </c>
     </row>
@@ -17398,12 +17398,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B03GR+QtctU08n3TKmi0Ug==</t>
+          <t>OAdElTsDRxFGSt7v8UP4lg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HCfnTs4cpOl0cPR6iwbi/mQb56mzu2CASTHUY6VxvDM=</t>
+          <t>aYUEVH8gxXIMuw0CMjFHb0c4L9LKyrzaxYdQPdQHJS0=</t>
         </is>
       </c>
     </row>
@@ -17430,12 +17430,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PPMUjn/2edPGz+mZI2EjRg==</t>
+          <t>5ggJLdkXZfnyvc481aKCZQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>WiCOLbsxy2MF1AvOixMV5MM23e2ZzyVUpR3m+pIxuMk=</t>
+          <t>PQT3DtzRxDgvFoKJxEkccqi5AMb42Sl2pfkIvrKNetM=</t>
         </is>
       </c>
     </row>
@@ -17462,12 +17462,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>pXJayUOGHRoadywDocdtXQ==</t>
+          <t>GfYRjzADYDOhfWuGBVrqag==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>a6fcUeAmdxyxvoQlxQQ7OFcPC6HTR2IxSHj6COLXL2Y=</t>
+          <t>TXCY/akXwqb8XxEEKmOM8bUnn/ud30/1iWvTSffbcvI=</t>
         </is>
       </c>
     </row>
@@ -17494,12 +17494,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5k0qrtDRzI7DPLb6DKZ1yw==</t>
+          <t>UjzzX2ygLOPl1uM8nlymNw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>mPoxU9azNaBEuaoiicD1YVNzK9Xo0tjI62KUzmUCzOI=</t>
+          <t>5Xg7PtX6eC9mJFGOA5SQqxjWDUAekj8lY9gXOsm1hx8=</t>
         </is>
       </c>
     </row>
@@ -17526,12 +17526,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>rZzhJDbKTwjazB/0+70zBg==</t>
+          <t>mL0ifiTnrpoPYMh4cketyw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SclGTd2+WfKN7CwDudSWU29jg2KfHCCjXZi/NVWcZ48=</t>
+          <t>0HfvakCUn4ul3sQIuIzRO8HFkmi46UPkRod4sCKMa8g=</t>
         </is>
       </c>
     </row>
@@ -17558,12 +17558,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>m9CQbBD5QnuUdSfZpbU1Gg==</t>
+          <t>57i1R6sgn86tah35RTtwHA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cnu9qmqXS8Tfm1Ut0906nl9u20P2gGpMKgc24s5zIu4=</t>
+          <t>Djb8Y1vEfxWXMLjuwngF0afUnx61Q0MtfjlXJdzwPkw=</t>
         </is>
       </c>
     </row>
@@ -17590,12 +17590,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>k4quVCfwOEdIrWhm9+azWA==</t>
+          <t>rgmfpp4CB8OFKFlnYKX6Tg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>fNyM546Gat8JAZxoy/5bXzo33y8F51kEjdJSR+AWnSI=</t>
+          <t>RM9QcAOAN1h6sVRVMrzD9y0AFd7YqNFmtZRMg/AqwPE=</t>
         </is>
       </c>
     </row>
@@ -17622,12 +17622,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>kS6IKoJ/9+5xT2yxJoJFpg==</t>
+          <t>yB7/SuL53jcZ4mSp4cFt5w==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>aIJK0CQ8jDyRt+Zr1iXq8pFrcjuyxpiNpZvAb/OmPUs=</t>
+          <t>xT/EFLflEhuXUngYDHlkKdy1xctnX51ki6UiLPiH5lc=</t>
         </is>
       </c>
     </row>
@@ -17654,12 +17654,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>d4am9ONAAqqDCu5cV7dPrg==</t>
+          <t>8wFfhiolZ4/hrP0gXUsOcQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>VNTfPt/LqXFoOJzeae8Y6PsowwqucNr7s8GSN7gAIsk=</t>
+          <t>kwcOXb3oGybfLhuAn90g7Qt84xtV4wUiG2BmJaaGTxE=</t>
         </is>
       </c>
     </row>
@@ -17686,12 +17686,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MPYsLFSRswKdfnvMoFzH1Q==</t>
+          <t>C4vGq5EEGGcB8Ou2xVZP6A==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>qSw5rTzMD7tYIvc1jTkwRtKRZOKEtTPf6AokJJmtQyA=</t>
+          <t>gfAIBMOWVCS/x3EsCEh9VBMmi5D/RSLI8oVN02K6SeM=</t>
         </is>
       </c>
     </row>
@@ -17718,12 +17718,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>xMB6K8F3fQEIXY1OKbJjnw==</t>
+          <t>M2uMyehhy5tZ+m91ZhCcFg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>elCqVG7nNqBX8hiJwdsN6W+4bZK+Vr8isaFn46lhBm4=</t>
+          <t>G0LuliCfmb+1jbfqgZM7fHktzJkI2OpjlqnHPM7WxZ0=</t>
         </is>
       </c>
     </row>
@@ -17750,12 +17750,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0VpT2YhDnrxFY2lrwhpg+w==</t>
+          <t>4td9mgmbc033il/vgljW9w==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5NmAVtUZMXPTnTEZl23XRhbuHlB7MS/qDedqsfJ25wE=</t>
+          <t>n0vBTD9UxLZMTiR+WOtZFJYT9x6a90+a80YDKJ45gKY=</t>
         </is>
       </c>
     </row>
@@ -17782,12 +17782,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>5DCGOGhvIbrwPiMvZyx8cg==</t>
+          <t>gv3jHZuyjn+ZR3oMd/J1FQ==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>LfBzmbF8ibQeCj3PlnG6X5/1aMF5o2/e8xDCXltjnTU=</t>
+          <t>YGhG++ZINuSNMTZcXmzQp1LwYANMTV+rQgBL2S9xFns=</t>
         </is>
       </c>
     </row>
@@ -17814,12 +17814,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>I0QKsCWq+HC0C6k31SRSLg==</t>
+          <t>7kDPuBKkzNwilKZgsO96IQ==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>5df+pPweNa9626Tr/D+PovjhsHQjekxyDygc5YmXZCg=</t>
+          <t>diZDuZm18cxuPbR7UpsnYIKVHLEsW6GKaZvPkXP1yrk=</t>
         </is>
       </c>
     </row>
@@ -17846,12 +17846,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>v1cw2kfAcEhboNrpJdG7gQ==</t>
+          <t>l35N7evdG40Yy7glbv14MA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>qiDjYyrvnj4JqzFHn6FHVBffDr0nVVG7JeMvwMm+lVk=</t>
+          <t>Rnv7gXWfl1fY60mLRFXFBVIlfBI2of57NedGDGx6KhM=</t>
         </is>
       </c>
     </row>
@@ -17878,12 +17878,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KQJtkpmQt4DWCcfPK/drqg==</t>
+          <t>fiKWaZz21mEj0y5QneUgBA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>XjTH3Wjsw/BDECHEX8zN2uj0C7gdr+HWfiJBHlqLqfo=</t>
+          <t>pS2MTYRrJmRCayXF6Ol44NGKXOrvufUIMjIB90s/BE8=</t>
         </is>
       </c>
     </row>
@@ -17910,12 +17910,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FWTgA4UQacasDhPE19qVsQ==</t>
+          <t>SteENJ5NFjLysIPBwM5rPw==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>8WVgRXrBKg6D1YhkwxyLfBpWWuMJbZfzLrhtXpGg20o=</t>
+          <t>cVI//0CUWvFrX5Jms44CnOMXquYyBKLIozAUoaf+iOg=</t>
         </is>
       </c>
     </row>
@@ -17942,12 +17942,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5yNMOvoELVeVolSjuOvoNQ==</t>
+          <t>hgqUtCX5eWkvXJ75k8x4wA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3Rv/6aq6G6dO0wOXxhGf8DilKjeJPVR8Ad88s5jDsJc=</t>
+          <t>NhYYMfQ5WAbpS/6+y90cjPueXS+sIRJ6jyodnf1qyOY=</t>
         </is>
       </c>
     </row>
@@ -17974,12 +17974,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>d211OZD4CH4nv5n7GZ6djg==</t>
+          <t>XUuNXVByDcEmjeYo0D67tA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>oWGrcppQoZ4H89Zm2kc6dNaEwXHwn2mdi5iubGQVfZs=</t>
+          <t>WOOvDDF8yCZdY1b+xd/B0mZb5iWwFotFOHntroPDoL0=</t>
         </is>
       </c>
     </row>
@@ -18006,12 +18006,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>J5Py3VjsQGhr2L84USVYMA==</t>
+          <t>ujk+IfwEOUudER8XfpSumA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>GmpkxrYxPIiMfBnpInozHR+5Nx4BcUMclBHERsG+3E8=</t>
+          <t>p1wumjFaRddtiY8LwAvVN0zU23GSzUWl1aD8weBvCao=</t>
         </is>
       </c>
     </row>
@@ -18038,12 +18038,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WwOr9I5EQFtblWoFkcBcBA==</t>
+          <t>vaIWncyBIQUV1JhWUq6O/A==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>YM6AuE1uCT+5bdDR9R5vp72zIFMjK0vLqK0DLHOkkTE=</t>
+          <t>QgEID7ESBLrw5Xe28gBuFxhBAh/kWgNTuQ9FV5Fty74=</t>
         </is>
       </c>
     </row>
@@ -18070,12 +18070,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JEgKqeiD6g0TuJlUwrsnBw==</t>
+          <t>CYNvACTwZ+7VhdHBdcFyug==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>i/DbYgufQueNwjyaktWAV5dPhDqN7GzdgfB6Y0Z9uB8=</t>
+          <t>+AYLTzH+geb4ZoUj6hghCPCQ4f4SAExkHgsj4iIC+rQ=</t>
         </is>
       </c>
     </row>
@@ -18102,12 +18102,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PGKxYKK2spHwHV8uCPTpgA==</t>
+          <t>jCHUqHwFHQhm1BblLpUUiA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>kWAs9PxneBtoswZjtB0RWC32x8a3NfEjGutaHfoGbR8=</t>
+          <t>YjIbSh58Wm8kix0vuInZ8MUTUpG40Q7abWZuo8/oIqQ=</t>
         </is>
       </c>
     </row>
@@ -18134,12 +18134,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1diAcdDF2xYHQDt0SEehvg==</t>
+          <t>M4WPkEjjpcI4sMFzO854yg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>GGMsMfSB/ZPGknoDtNq72VfHov7CL51re4/RVUI3MTI=</t>
+          <t>sFr8en6jOkO8Dj1YXBxK54DwceZYP+UR5IKiGP7EbNU=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-06 09:40) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0ujDLb+Tb/S2eHowQDV0iw==</t>
+          <t>1rao27DsCJcz84rq34WbmQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>mSz5NH4ChFiJK1vBleXFkfjv9BT9hAmhaA9rW7kQ1y0=</t>
+          <t>67zVwlAHih3dvANwuYR+INzB0dYO3KTgT8Qo/rxzSAo=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JXqkgF7czOeQk9tHbGhHvg==</t>
+          <t>qBoJiubApTv/l3DnhrI7Ow==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>27OXdxqMXi9pZgmMlvkVBgtP4EU/1bhF6HZeLUgt5zE=</t>
+          <t>1gO7AUSN3XSwfCbeBBhu0gTPuAL78qKV6Lrhu4WXkhE=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>cEbwIyI0kE+MrUuGkCjl4A==</t>
+          <t>9NGOYWzjWbvapzWOkeq+Qw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>uSJ14kWtI0SKgaY5+fAHFZ1ryZ0TNVkktZP0u+aKctI=</t>
+          <t>FizPmwbuVXcOaUngZHCt8zxGp0qHWbBoEOrw/nDAL6s=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>oYMZMAE82tWZrPwXSgBegQ==</t>
+          <t>P/TUjpq8tpeTT53FCTfQtQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Vv87UcHrHkgVgUwN8Z9I44YT0VR6ICZZ7Mwa9NSFXgY=</t>
+          <t>755Zt1wKCBzAOGj/jh6MdUEr0Vr8bsMD+VM73elpltk=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JWD6B6BF0ustazXkoEENFQ==</t>
+          <t>dmAlD0zJHDnNICd5QNZomQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>mB3VwKeZK2K5WnfkPZwXzTiSq8j8NcCFw6fMt2YqNlU=</t>
+          <t>fyH/8jvwsYYJj5H7z4m/ZskCXN/zG/jCUDS0OcIW7ME=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>seqNQyr1cJBsqnL10refJg==</t>
+          <t>ptsGBLjLM9DLJi3rhpgxPg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ZdIJfNc9FQpgDN7iD5/UtcnJVj1KeX5+hfcjE1WSSQA=</t>
+          <t>6BpAeBaCDScr5RRpnN1mzfh0+QrakwQe3aXKHIQpbeo=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>uGmkKHYus6BWWY1sNVVBWA==</t>
+          <t>8Gd5swA0qV1OH1ZKyOHMaQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>aq3HHXhDoX/iOVWAeEvyvl0dqp7c7DyuRm+UVCXMKFM=</t>
+          <t>FXlqAYZwhKEHCaG1AOwvgtV/MReX/DcUwp2i09gEX0Q=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SdPYPlhHp5jWTGb6/PZ35Q==</t>
+          <t>ZvJ2NRL36pQpDzGvDBIyIw==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>msG2aqKQ4PGJgh9ylJoWUI0H26Nc9bXHOsSzTZi8G2Y=</t>
+          <t>KayMe7cFOB61FxsNxraQzDepKa0Dhts6+d4wUZd1/hE=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EogdhBrQEQ62Sndr7VAf1A==;8mMSPCciZgud1If6erqnEA==</t>
+          <t>OksomJqgkLuP/soxUjWr5Q==;566POo2ZZMEvPnuUhJGA1w==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>i2qJgqsx1/rpak38SpjtMxYjQkRjkAa3Qw0GZj2ETOQ=;R7yJTLlNXweBF64Z0rCdcb6+G9XyWL4OmwFMAfWGkAA=</t>
+          <t>pJyw4IOgQAf8WlboXNral4FGT53Q2C2s8RPhr1Q2Jgs=;XQDTV30zQCpTVNiKzpLgoyOaHwXM5/4zt5nVP5x2Ce0=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>927t9UdyBt3JVdjjcvf2ag==</t>
+          <t>Tahyxi2ALInOUMZGqwShlw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ckFnY3tSLL3esQWlMudVwXrCkwwDAW9i5B32zbe/vpU=</t>
+          <t>SkPZj2+HtZCgm534eKxg5CJDsxuRWXqU5rQaGvBdjBM=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>vyTLEOJf5c8ZV4YjCj+Ggw==</t>
+          <t>b1ETZ8agKjepLgwXIzrRBw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>7UVNOYAqu3xh6ilbOnDnh/St0fS0TsBizmq4O6ZAgZ8=</t>
+          <t>C8d696vHiKKfETniM1PdaNAotvwTuHzgiK+w0f15Lgw=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>nTKgjFj/1TUzdIlzHaQKJA==</t>
+          <t>eBO1UsOAru6UB4hq8THkew==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>7DB/GaP4mpYReQdYpvlzOBjtWkCPdm4fgneeOM3ptts=</t>
+          <t>+WG57WE3dEYhRFI0D6Kg8RD9KxaVNMXzBZcQiWdcPkY=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>JKZd7YsDL7CM/iMV4mpK0A==</t>
+          <t>XqgBoCUdnBhZh6pmy4+l0Q==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>lTXi4nlf/OQzfBEO4xPPhTSmCPVXwO0ItRuagzYBq44=</t>
+          <t>9mr6hd7lCcdIVbDxOMeYJNQrF73ZluLO2fK/kxSog/0=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EhdkwA6R+rJeU8tvcMrvLg==</t>
+          <t>wMP/1k31SgchhGfS+lAb0w==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Pm6604Jw2bZLt3lHhXAWAZzhSYAaAq7G7IqxzEcEt84=</t>
+          <t>3M1+U9YSP4MRDQTNfkSkXeLkLPK80m+e2cg9Rbj9BLs=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>6o13kZrM4UrB99o8XRV+AA==</t>
+          <t>++TzdZg5iLdiMFDQ/9aajA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>xbNwzqKTY2DLsvbD1D26VmNl+IWGZVOMK/zTDP0TKCY=</t>
+          <t>NRbvkOnV6hab7+IKP/rCAeEhuTD0jufJsFh/26kpY1U=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>iJOMsTrEFt1WE72W7r47Ow==</t>
+          <t>bUaNcuJPqK/ZrmRk5n7xSQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>6+eN7OjX5WggH/D4QiwyhYgzE+cqt3+jkIycUnBQYKI=</t>
+          <t>ASUy8kCg5MCAmucFI3LvZG3oi5N8DxMTDXS9Vwg62cY=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>jdTUq5N3sJXMxz6w4dXaDQ==</t>
+          <t>Nmv5yacL70zVJ1xcBJ2zeQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>NIkobmimV0heweysX0KGRBaBZToNT4o9PXLMtZCu2io=</t>
+          <t>b/X1gVEHxtAco3DlJz1g2vaTvyGcRhGvdYJEw9jC+rQ=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ROAEop1ZOsRXkKF9vZvfgg==</t>
+          <t>xfVmy/iUWxmoild3iQRI2A==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>wLu9t3Ua+ODcDdPvIXvQ2Rd0eq5iocSeMWn0ypUEtBo=</t>
+          <t>Rb0hFlH3gsoBaJtiLPsaVOUDMYuvQcTs3yJtmcJ/A98=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>dyyI9tdSXOpM/MG0dilJIw==</t>
+          <t>SsTBFAZxnLas/mUezaqvmw==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ar9bdQWuhb3cdacl7TW7rKvWuhIxi0/15cHMESciCAE=</t>
+          <t>DZuXgagcNzfZ4pSupiTGKE6G3H/VGC2HCa3H4US16R8=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7si6+qS3eZQRdUpfi7JOew==</t>
+          <t>zPP/yA+pal1hSxZFMVof1w==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ypQIxOe3u4X2Fpd1844fT/uNW+b8u0j0Hm77SjIpB1A=</t>
+          <t>4DxJ73X4M5qXSWZt6C88P11xTdkc2VAjaWYnAI9us1s=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>dKtf7XN8yOcWT3vq6uGyEw==</t>
+          <t>N6Zk0ujRSLdnxk21u1jKlg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>6yCJoHZvMIKjXe6Q8d6SEWtBn63pgchwzmCchTRG1u4=</t>
+          <t>K3wR/AcFJDiHN8Gk4rOnhfArjT/LqotQ7iRNaOJXUno=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>HerJ4KTdr8OUAl6pxIufjw==</t>
+          <t>3HT2OGil7P/j5CS/VPW8NA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>YqZ4RfZD3xb4qoHqwDOaVsJQLOO9FdQ4ywhZ/dO43mI=</t>
+          <t>9DaLYgXrUgARnB+PddQTMizgti/TSCg/SAaDTkZGXmw=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AAR4CmxoxZ1TqoET+ZOJwA==</t>
+          <t>BIbjE3ZuTn6rIYfffE9dbA==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>G76Z8sTlOVpN8TLzmKNlrZh0jnSSCRctpVmbcQqGj54=</t>
+          <t>KAfE3p5EV5A/D5GixMgPuT/p9AKwmv7/XpBgLmRMzqk=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>04g0Pk7gD35WGMRupSwkLA==</t>
+          <t>sQPPwYXIYoLXRPJ2K/HewA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>mPZCRpYfNX5a5wIKbrSZz2JS5BGcr/TuxKfEx7hbpqU=</t>
+          <t>/ObHEhDtyiObkKLBN3xpjGH2b2z0MgaXCBwskplD1G0=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>jF+0/Id/lIMJ1sxG4QsmfA==</t>
+          <t>F1w45Om7UlzL5FSwFv4YFw==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>iv0uP2rzoDIRY7zmNTjWFy63rF4RZ/ugBdGgU1F6r1E=</t>
+          <t>8DCuzogtwfn+14d0YJeTGDjwmxGQaJHydfJZUSllyGA=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>+Wt18QcpZyFRbxRP4THBjw==</t>
+          <t>3rkTel7fhJmXP++FfYYH1g==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>kfronSnkCgMiJtmMMszKUvhAqh4hFpwjnkGs4SDNnjA=</t>
+          <t>5Va5k2kFlwaMIu4R2BvWryQ95GbWF8+7vS9YN+goKU0=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>VHsWakngVCL3I2S7Itfuaw==</t>
+          <t>YZWCrZtFaAvEkS5kCHleEQ==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>wxi32lt1AnvKwUxHdXhZT8+ncyUAfuZ5iwpOiCDr/JY=</t>
+          <t>4FVanXr2GOl93HPewLzlXcKz1VnW2YtY5Stvu/ZEoxw=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RjPA8ahPxwfss4/1KSDaRw==</t>
+          <t>tdgjAoe9sezSjhaOp7D75w==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Uyepq+Ju/VdDRloYfzQRtYPriX3rSVWBx7ni+nx4sLs=</t>
+          <t>fiXAJ9qlFGk8eXhlnlUZUD+EIjo58hXa4jwUCf/xohQ=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WT20M/5znsbrBlL41PdSLA==</t>
+          <t>wTicUZhZJ+Q2oZ8oozx92A==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>nkPNdtCtHTVgJJtOUiVNm5voOIgJSi47PiDiqvJnCJw=</t>
+          <t>e9UO63yKdqTDO8nR7qZErxw+F/AhjNBGLefZ0bSBSIc=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>7YZqF82LfOJko1VsnUhieQ==</t>
+          <t>FSHXHV7RFF+pgwT8vGQazg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>knLMvuSOL86Y5jegpzPFJZ3qnIi5KAuk+TUQkbf6wl0=</t>
+          <t>ct2KoYzkmDtUAdSOXcbjJ4kt1um/G2zoKcODjohWAi4=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>M8sS+px1CutYUHyj8Xplxw==</t>
+          <t>e+cKpiNOPKbm+NkkY8mznw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dlrQTngtBTmmCvhnrqOIYnzcMDLl8AieXVnsbcglcwg=</t>
+          <t>BrvrLl9krymEK3OdGBTnyrZb7hxII/U59lPyCrjGMek=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AOn4Skta3OpX93Oiak3/Qw==</t>
+          <t>CC9RifkqvBFluMF+TMkU3Q==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>+HFwJvQSUq6pxLmrmc+8HKtr4xJXfcwufdJa27/AHAs=</t>
+          <t>qHZiTUGjhfs1Ip4TPIHjeG6O3rsBjZqToOtRITM/LpY=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LsKdgm4RHoyPcUe6AV1sQg==</t>
+          <t>LstNxUu6S+J0wN9hFWV/OA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>yjiBzYDeelaO3+dmP9tnWr1q0hz63BXLvjR2yk8lBS4=</t>
+          <t>IiaHOBE8dg6P2a3FSHwKuF6Ap7PXKgw7hrQt/YY9hhs=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ei3hJrxigFBs2kVljGhaiQ==</t>
+          <t>AREhXf6EzKImAOXzBdOP+A==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>xcSHD7Nd8pW2xL71rRGaRhGCG4Y+RUSCfdRjobRleZc=</t>
+          <t>kRZvySVnQUVcZT0EwltRrNsRHOZQMlTBP2czi3axqmk=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>u81bdfC2BuHnjpU0f0Tppg==</t>
+          <t>Wfu2UDrxiZo2RCkxTACwyg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>hGfH4hSRiPCvXQ70qT8pZ3mvT8e0qRj8orCapS6yq5k=</t>
+          <t>fi+NFHE0waMaTY+YxIjsTBV7PX9/T8o9wzV3O/lR2DY=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>E7IAcTyrkv1sgGCdF8JBXw==</t>
+          <t>V2XvoX0HGvX4J/nlEhMvZQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>eqG3iAOz4dFuq/Z7z7Y4mplJL3yTTL7CyiHRcocvptQ=</t>
+          <t>vilUZfKhJzbFlshXVW1bN+sYeF26Oa8PIK8tjHiD/oE=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>vTwnXnyorYsvCpNL/SrgNw==</t>
+          <t>odlPezWNrW3y12i6/Ev4XA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>uQje4EbV9MlfKR7mTPq/xgi12TPelYw7+VGDKsjL6l8=</t>
+          <t>r2eZ87Mi3ybAm2EBb/w/sTWSmoMvJKfuLbl09qpDw4c=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-07 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="46">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="86">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="90">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>303</v>
+        <v>316</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>303</v>
+        <v>316</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="117">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="120">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="121">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="124">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="125">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="127">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14">
@@ -6450,7 +6450,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16">
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="97">
@@ -10746,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="98">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="106">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="108">
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="109">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="120">
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="125">
@@ -12026,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="126">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="132">
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="134">
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>281</v>
+        <v>288</v>
       </c>
     </row>
     <row r="152">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="156">
@@ -14554,7 +14554,7 @@
         </is>
       </c>
       <c r="L174" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="175">
@@ -14610,7 +14610,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176">
@@ -14698,7 +14698,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="178">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="181">
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="188">
@@ -17002,7 +17002,7 @@
         </is>
       </c>
       <c r="L220" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="221">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="222">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1rao27DsCJcz84rq34WbmQ==</t>
+          <t>5uaojDB/sVscCfcljaxdVg==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>67zVwlAHih3dvANwuYR+INzB0dYO3KTgT8Qo/rxzSAo=</t>
+          <t>SqpM3vC0qRz0I0SdQoDdJUfmSPLG6HTCpCsoHO68Byc=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>qBoJiubApTv/l3DnhrI7Ow==</t>
+          <t>4HsTuytPo3WDLLev7vrPDg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1gO7AUSN3XSwfCbeBBhu0gTPuAL78qKV6Lrhu4WXkhE=</t>
+          <t>bksEPyixj5ISKp+wUQTPUgs0Zhx1U8c7GzOn3lenfPo=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9NGOYWzjWbvapzWOkeq+Qw==</t>
+          <t>R4A1OOzhD0wMXRVwaV2URA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FizPmwbuVXcOaUngZHCt8zxGp0qHWbBoEOrw/nDAL6s=</t>
+          <t>1iypmbZD1JG+MHz6gsp/5FpWyyVfCpiOzu23RmYA6Pk=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>P/TUjpq8tpeTT53FCTfQtQ==</t>
+          <t>s02Infn/9cI6IwjcYYE9Gw==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>755Zt1wKCBzAOGj/jh6MdUEr0Vr8bsMD+VM73elpltk=</t>
+          <t>fQY5V6Tcl+DqHs/ufhCrEXSGkdLEKAuy5FUzCWrUZG0=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>dmAlD0zJHDnNICd5QNZomQ==</t>
+          <t>RRU58+C//xn/ZPkDwQPWuw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>fyH/8jvwsYYJj5H7z4m/ZskCXN/zG/jCUDS0OcIW7ME=</t>
+          <t>/fzEzAmymnGY/V9etjgiwTZNq9E9nvRqnz2JaC4txXM=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ptsGBLjLM9DLJi3rhpgxPg==</t>
+          <t>yEKBvtx5ifQ1yKShpYS1cg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6BpAeBaCDScr5RRpnN1mzfh0+QrakwQe3aXKHIQpbeo=</t>
+          <t>tqvyk4CYLfvvgO0iDKBEV9/Bl05gEXX3SyoGg+OEQuE=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8Gd5swA0qV1OH1ZKyOHMaQ==</t>
+          <t>BV0YTHPrEh9KCDcOvlwCdg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>FXlqAYZwhKEHCaG1AOwvgtV/MReX/DcUwp2i09gEX0Q=</t>
+          <t>TrCtg4cjVNhr7NTZ62pIWoY6hq6CO4lY10j6KbLxBCw=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ZvJ2NRL36pQpDzGvDBIyIw==</t>
+          <t>BcTLf6GCZ9Zxshv9xdTC+g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>KayMe7cFOB61FxsNxraQzDepKa0Dhts6+d4wUZd1/hE=</t>
+          <t>lTSRL99VBfJw+aqnYFIw21Jx58lhUIolm8iUB25X2OM=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OksomJqgkLuP/soxUjWr5Q==;566POo2ZZMEvPnuUhJGA1w==</t>
+          <t>PeA0UK0ClIswWV5ymJpF2w==;+YRjwrJX763EEKn5PbMYTA==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>pJyw4IOgQAf8WlboXNral4FGT53Q2C2s8RPhr1Q2Jgs=;XQDTV30zQCpTVNiKzpLgoyOaHwXM5/4zt5nVP5x2Ce0=</t>
+          <t>K1Qp58h/8h5xjaGolWZ9Rb5MtIxfjUY15lsB7fCyCdY=;4++zY6RG+/ttCjQ+K2w+7inlpk9A+v2piqaQ9oQES68=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tahyxi2ALInOUMZGqwShlw==</t>
+          <t>eyAe0BuQrRsQ7G74unecig==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SkPZj2+HtZCgm534eKxg5CJDsxuRWXqU5rQaGvBdjBM=</t>
+          <t>U+MmvnB2N+VnmmRVDmTrV6sl/DqsfpRMOqSL/C/VSGQ=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>b1ETZ8agKjepLgwXIzrRBw==</t>
+          <t>gKvzh/zPB4mEvC9KCIDbEg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C8d696vHiKKfETniM1PdaNAotvwTuHzgiK+w0f15Lgw=</t>
+          <t>CFp+3mF8PWhX3QqMacRveLN1llswhRjZzegMw4P9vU4=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>eBO1UsOAru6UB4hq8THkew==</t>
+          <t>l3zDGkywLkBcPkz/FZgYHw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>+WG57WE3dEYhRFI0D6Kg8RD9KxaVNMXzBZcQiWdcPkY=</t>
+          <t>jRTxLxRho8ijQCrHSP2DXx6UVJDm9/rXKz1crkw1RAE=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>XqgBoCUdnBhZh6pmy4+l0Q==</t>
+          <t>qMeRGpVjZOQkuqDl6lgaUg==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>9mr6hd7lCcdIVbDxOMeYJNQrF73ZluLO2fK/kxSog/0=</t>
+          <t>fTjPjKosObSJbEM5zDb1akQprSMInTsNrIzgYG3e4nk=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>wMP/1k31SgchhGfS+lAb0w==</t>
+          <t>1+1VZDL//OS8wDDewJkfGQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3M1+U9YSP4MRDQTNfkSkXeLkLPK80m+e2cg9Rbj9BLs=</t>
+          <t>RJlV5GTlj9F9xg2yRl5QFAxGf9cCKiQGgiji15OmPAg=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>++TzdZg5iLdiMFDQ/9aajA==</t>
+          <t>831MwHcmUHN27NjEe5AvfQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>NRbvkOnV6hab7+IKP/rCAeEhuTD0jufJsFh/26kpY1U=</t>
+          <t>41PCeBNJWG93nEgzIzz6LTXTbafcfaEKMMnb8JNhYfk=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>bUaNcuJPqK/ZrmRk5n7xSQ==</t>
+          <t>lSCoPdQLarmHWXIcK4uP5A==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ASUy8kCg5MCAmucFI3LvZG3oi5N8DxMTDXS9Vwg62cY=</t>
+          <t>Ht89Y5lTKpQ8vNHSAibn0hCjKTFQ9i72RuqYd8zFWNI=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nmv5yacL70zVJ1xcBJ2zeQ==</t>
+          <t>5uGCvfAOAMTulr57S6/4vw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>b/X1gVEHxtAco3DlJz1g2vaTvyGcRhGvdYJEw9jC+rQ=</t>
+          <t>0K8FDLbZq0n6lYDdUs+3TxODQISVMf3gqxRxGEBYEt4=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>xfVmy/iUWxmoild3iQRI2A==</t>
+          <t>P3jYxq7RFwkywjxB8dxinA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Rb0hFlH3gsoBaJtiLPsaVOUDMYuvQcTs3yJtmcJ/A98=</t>
+          <t>hb3+12ZNyXfaxEkPTdtcdJ7uTsds3NBofBATt0VsH+o=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SsTBFAZxnLas/mUezaqvmw==</t>
+          <t>Veb6HdEs9J4VG9pvZ+i1vA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>DZuXgagcNzfZ4pSupiTGKE6G3H/VGC2HCa3H4US16R8=</t>
+          <t>w9tbp6quMiGWX7FtJjEwt/bKotpwaczDUkqxKw3EtUc=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>zPP/yA+pal1hSxZFMVof1w==</t>
+          <t>hTe0rbFDWdQZOt1FgLVGdw==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4DxJ73X4M5qXSWZt6C88P11xTdkc2VAjaWYnAI9us1s=</t>
+          <t>DZBz2r0gxYZ+d+SUfb/HU9PNlSE0fBgr7CEA09ltIhg=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>N6Zk0ujRSLdnxk21u1jKlg==</t>
+          <t>0UYV2u90HFNIt7k1ArnjGQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>K3wR/AcFJDiHN8Gk4rOnhfArjT/LqotQ7iRNaOJXUno=</t>
+          <t>59Qz9K/OdPg2W0SN8U14Zw7E7oAVxEmV3eYCnKt9IBQ=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3HT2OGil7P/j5CS/VPW8NA==</t>
+          <t>4I7uRZJXEUZx8D+wLObQew==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>9DaLYgXrUgARnB+PddQTMizgti/TSCg/SAaDTkZGXmw=</t>
+          <t>s+El3R500zxKM/ETlw676OJ47Ap5WA8KIHGqF/ifuo4=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BIbjE3ZuTn6rIYfffE9dbA==</t>
+          <t>mWy/1aoXvo8ZKIozMIbpFg==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>KAfE3p5EV5A/D5GixMgPuT/p9AKwmv7/XpBgLmRMzqk=</t>
+          <t>pOYIUQ7uMX/zmP/O9KLBCk3ACdvUR2YTAvvaxuhlV/s=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>sQPPwYXIYoLXRPJ2K/HewA==</t>
+          <t>mous3dGOzigBHOnDbBYm5A==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>/ObHEhDtyiObkKLBN3xpjGH2b2z0MgaXCBwskplD1G0=</t>
+          <t>b6w9PWL/nOpTAfwKZsNeL6oo6Kj+y2WWxWeHEvIlxtU=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>F1w45Om7UlzL5FSwFv4YFw==</t>
+          <t>8OvoPltzA6FEM2fVjA/G5Q==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>8DCuzogtwfn+14d0YJeTGDjwmxGQaJHydfJZUSllyGA=</t>
+          <t>Ffv67MJV1UIy9fqiEfo8nB6IL+QZkqOoVLn6LIscc+A=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3rkTel7fhJmXP++FfYYH1g==</t>
+          <t>DaDzuJVmAgOUonKdpwTGPw==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>5Va5k2kFlwaMIu4R2BvWryQ95GbWF8+7vS9YN+goKU0=</t>
+          <t>WjRN8iGgNG5ZF2yWv6xRRPjchT2wbzn2aqRzTt31zKc=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>YZWCrZtFaAvEkS5kCHleEQ==</t>
+          <t>DJE8GV0GbSm4tJMF1KB/7w==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>4FVanXr2GOl93HPewLzlXcKz1VnW2YtY5Stvu/ZEoxw=</t>
+          <t>Eff7T8ri0Xg6rwOy21neDVm6cjSOv/3RDTWK/CyUoTQ=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>tdgjAoe9sezSjhaOp7D75w==</t>
+          <t>EONo4T7pIRILMWrA+y+HGQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>fiXAJ9qlFGk8eXhlnlUZUD+EIjo58hXa4jwUCf/xohQ=</t>
+          <t>+09TimDGGM0vyeuWvkLi5fuNuhAIZG1i3BR0LwtUhc8=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>wTicUZhZJ+Q2oZ8oozx92A==</t>
+          <t>x4AvdgjgoTh1GaQ0IieD0Q==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e9UO63yKdqTDO8nR7qZErxw+F/AhjNBGLefZ0bSBSIc=</t>
+          <t>aUL2JMqGeaSoHkjL+KpM1kTLho8ViNiSf1awkY5UFCE=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FSHXHV7RFF+pgwT8vGQazg==</t>
+          <t>/hNszvqojr0bxIIKaVFSxA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ct2KoYzkmDtUAdSOXcbjJ4kt1um/G2zoKcODjohWAi4=</t>
+          <t>jhsTU2RpGWczeyG1DC7ktkyz8aD2oZiUppATo5BPEmE=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>e+cKpiNOPKbm+NkkY8mznw==</t>
+          <t>e4EDbPId9WKlSQZHV+2Gjw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>BrvrLl9krymEK3OdGBTnyrZb7hxII/U59lPyCrjGMek=</t>
+          <t>++doUapiQOxlLvAKtxY9vdp4YRBtawDk17Zzh4+y5t0=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CC9RifkqvBFluMF+TMkU3Q==</t>
+          <t>w0MH9aRmsc3k+UIcVpKlhA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>qHZiTUGjhfs1Ip4TPIHjeG6O3rsBjZqToOtRITM/LpY=</t>
+          <t>LVswHb9Iw0kZnRdyme8ZD1MQTcZqaUStHcSkjEQ1JCY=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LstNxUu6S+J0wN9hFWV/OA==</t>
+          <t>DK4VWrz0XBHFW2gJHE5tJg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>IiaHOBE8dg6P2a3FSHwKuF6Ap7PXKgw7hrQt/YY9hhs=</t>
+          <t>xZqI1X/OtGNiaoSZtbUjaAdIe4wiAVVyLUsrk2d9Uw4=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AREhXf6EzKImAOXzBdOP+A==</t>
+          <t>Xx05c4F55qD24ZPtLsaiCQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>kRZvySVnQUVcZT0EwltRrNsRHOZQMlTBP2czi3axqmk=</t>
+          <t>fRdR/C4osIQTDVWmSqFyMzqiwHTECdSi1QQ0RaMjabw=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Wfu2UDrxiZo2RCkxTACwyg==</t>
+          <t>HntDDfrNecMx2IUQxOTd8Q==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>fi+NFHE0waMaTY+YxIjsTBV7PX9/T8o9wzV3O/lR2DY=</t>
+          <t>kXnLHJabAUuLBkPxHLtYHxQKPeA0ICKefAQ4xWUEhRE=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>V2XvoX0HGvX4J/nlEhMvZQ==</t>
+          <t>U+0RzA/pQXA3Hct0UBGIAg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>vilUZfKhJzbFlshXVW1bN+sYeF26Oa8PIK8tjHiD/oE=</t>
+          <t>S6OAVtPlJrz3JzNYpQU9l3LK9oyFeqnVsWQM6lKOwjg=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>odlPezWNrW3y12i6/Ev4XA==</t>
+          <t>70lfcQRRsE1S9w/8ZuAvxQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>r2eZ87Mi3ybAm2EBb/w/sTWSmoMvJKfuLbl09qpDw4c=</t>
+          <t>o14uaR8TGfUeGmSWR1swemkm0O30zoSiOa76jaQ/VsQ=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-08 07:39) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VENTAS MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>VENTAS MENOR COSTE</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -2007,12 +2007,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="91">
@@ -3751,12 +3751,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="117">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="121">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="124">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="125">
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="128">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=11cc3a84-a83e-4020-844d-43919a87f1b9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=11cc3a84-a83e-4020-844d-43919a87f1b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4">
@@ -6010,7 +6010,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
@@ -6318,7 +6318,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18">
@@ -10746,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="98">
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="104">
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="105">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="106">
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="107">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="108">
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="109">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="110">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="120">
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="125">
@@ -12026,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="126">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="132">
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="134">
@@ -12958,7 +12958,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="145">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="147">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="149">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>329</v>
+        <v>314</v>
       </c>
     </row>
     <row r="150">
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="152">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="156">
@@ -13626,7 +13626,7 @@
         </is>
       </c>
       <c r="L157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158">
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="173">
@@ -14610,7 +14610,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="176">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="181">
@@ -14874,7 +14874,7 @@
         </is>
       </c>
       <c r="L181" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="182">
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="188">
@@ -17002,7 +17002,7 @@
         </is>
       </c>
       <c r="L220" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="221">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="222">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5uaojDB/sVscCfcljaxdVg==</t>
+          <t>aKYzPx2vrpjQCFgQ5P76eA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SqpM3vC0qRz0I0SdQoDdJUfmSPLG6HTCpCsoHO68Byc=</t>
+          <t>vvU5RHpLof+APwQDvOgte5ItvGZgNvCdfrRMgmY50eo=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>4HsTuytPo3WDLLev7vrPDg==</t>
+          <t>vf2b8qQTxfuMZsOCyy/jEg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>bksEPyixj5ISKp+wUQTPUgs0Zhx1U8c7GzOn3lenfPo=</t>
+          <t>j/AC0fNMkQKwot2kRfQ7GlPzljerbkEYQ5yj5FL2jw8=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>R4A1OOzhD0wMXRVwaV2URA==</t>
+          <t>ZTdUxzPhBNlJOdF8loeORA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1iypmbZD1JG+MHz6gsp/5FpWyyVfCpiOzu23RmYA6Pk=</t>
+          <t>2Di+ITEtRIgZNlJDFXrxSmkzjHZBSWcfds7fNP4te0Y=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>s02Infn/9cI6IwjcYYE9Gw==</t>
+          <t>Gcu69P2PMaQT2EkDXpKLYA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>fQY5V6Tcl+DqHs/ufhCrEXSGkdLEKAuy5FUzCWrUZG0=</t>
+          <t>Jxo8J1hepAYTNgtRXk+w+D8J29psOqPn8Bp6SRcrS5I=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>RRU58+C//xn/ZPkDwQPWuw==</t>
+          <t>QDOsWMuZMjSc7q61fWelQQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>/fzEzAmymnGY/V9etjgiwTZNq9E9nvRqnz2JaC4txXM=</t>
+          <t>qxY7p1JRznr6ygvDgoQAl5v57n+KJF+kvkJqNPkWGzg=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>yEKBvtx5ifQ1yKShpYS1cg==</t>
+          <t>PYBnZtdnH3OArSUo7Jevig==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>tqvyk4CYLfvvgO0iDKBEV9/Bl05gEXX3SyoGg+OEQuE=</t>
+          <t>l2b7UMnQYqLzpTnmh0NPTHTa8VcOJctrdxnZKIPsMAU=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BV0YTHPrEh9KCDcOvlwCdg==</t>
+          <t>V3BjEvwQblJ3+7K54VwQTQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TrCtg4cjVNhr7NTZ62pIWoY6hq6CO4lY10j6KbLxBCw=</t>
+          <t>fL1HrFVwW0R7AqdzVsB44qy7ORSvgdN9FgIR1Z+khUs=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BcTLf6GCZ9Zxshv9xdTC+g==</t>
+          <t>6PZHkX+rIU7FUSF9rUn52w==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>lTSRL99VBfJw+aqnYFIw21Jx58lhUIolm8iUB25X2OM=</t>
+          <t>BcgvRdxLzz/kCDvkjoIzZHmwdAULa7ia61gnp2yDPPA=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PeA0UK0ClIswWV5ymJpF2w==;+YRjwrJX763EEKn5PbMYTA==</t>
+          <t>Xdb11ehlKzwUJkn3bCzC8A==;1C/WHdwHvOcx3YfQB9h4SQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>K1Qp58h/8h5xjaGolWZ9Rb5MtIxfjUY15lsB7fCyCdY=;4++zY6RG+/ttCjQ+K2w+7inlpk9A+v2piqaQ9oQES68=</t>
+          <t>WgkAz2RwA8wPsP+rvWkjJtZglc5exEzq+oRMr/y/Kb4=;+Zm9qsr5o6oea+xRpwrNZkMJFPqX6v8u43TtTep4Tfg=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>eyAe0BuQrRsQ7G74unecig==</t>
+          <t>UI8ohrnFBmk3LMEmQK8mWQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>U+MmvnB2N+VnmmRVDmTrV6sl/DqsfpRMOqSL/C/VSGQ=</t>
+          <t>bwNS8MxWOzSjORzG0xF5VT27hZcmz44nthABqDVuYEE=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>gKvzh/zPB4mEvC9KCIDbEg==</t>
+          <t>QeWbrwem4baF67xs3DtU5A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CFp+3mF8PWhX3QqMacRveLN1llswhRjZzegMw4P9vU4=</t>
+          <t>E52Je4K0feyP55rl7tlAjPaDHhKuBVENd95LfFtsF6s=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>l3zDGkywLkBcPkz/FZgYHw==</t>
+          <t>Ta5WMzMzolpstn7502rDCQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>jRTxLxRho8ijQCrHSP2DXx6UVJDm9/rXKz1crkw1RAE=</t>
+          <t>pUhf/KjqyBm8GsCLKF4GW6u16TqyE4sllqk5HOvMRrk=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>qMeRGpVjZOQkuqDl6lgaUg==</t>
+          <t>Y/wMqMaXraYcZwLYGO1Xiw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>fTjPjKosObSJbEM5zDb1akQprSMInTsNrIzgYG3e4nk=</t>
+          <t>LEPf1TSRePc4z8nJfeJlQNXJS0QlgiUqr/MbgkpxJfc=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1+1VZDL//OS8wDDewJkfGQ==</t>
+          <t>3o+C/wojPrrC0QHCkTUqzA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RJlV5GTlj9F9xg2yRl5QFAxGf9cCKiQGgiji15OmPAg=</t>
+          <t>67W3dNVQsHvqyBKMWVVWe+OUKxbg+ZMAwhJxbI0HaUo=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>831MwHcmUHN27NjEe5AvfQ==</t>
+          <t>+XaX55X7Tt5PpGnCdXxbWQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>41PCeBNJWG93nEgzIzz6LTXTbafcfaEKMMnb8JNhYfk=</t>
+          <t>O3rPj7CzgtIewigH2+B24QlFrnIfVIoBLAXQCjvT1qs=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>lSCoPdQLarmHWXIcK4uP5A==</t>
+          <t>2h4AvN1yxhZc5jtSWcuTgQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ht89Y5lTKpQ8vNHSAibn0hCjKTFQ9i72RuqYd8zFWNI=</t>
+          <t>uJgHRqnU7YOtLQkKvIWXECRW/NzlUWHG8rXPYUCk1bk=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5uGCvfAOAMTulr57S6/4vw==</t>
+          <t>gQh8wL+0G0K/ROZRmZXXHg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0K8FDLbZq0n6lYDdUs+3TxODQISVMf3gqxRxGEBYEt4=</t>
+          <t>aKrzL+E+CJ/v/DNhboakBtJme7xp8Vk/TjhYcsvxAT4=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>P3jYxq7RFwkywjxB8dxinA==</t>
+          <t>aXsFKyAPtdjfFWDWDVAJAA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>hb3+12ZNyXfaxEkPTdtcdJ7uTsds3NBofBATt0VsH+o=</t>
+          <t>UpLL1sefhJrVa6FUb3h+cNrKU+QgKVlvOty+w6ousog=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Veb6HdEs9J4VG9pvZ+i1vA==</t>
+          <t>B4uUp3b75Mm/9deczMV9Ew==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>w9tbp6quMiGWX7FtJjEwt/bKotpwaczDUkqxKw3EtUc=</t>
+          <t>xEOGt9NbYsgbe9pR9FxgTbCQSGlv+M6CE3LzVZl3pHk=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>hTe0rbFDWdQZOt1FgLVGdw==</t>
+          <t>IrrDZClE7FiezTICHN9D0g==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>DZBz2r0gxYZ+d+SUfb/HU9PNlSE0fBgr7CEA09ltIhg=</t>
+          <t>4sLpuJjNbm52X2pwL9/ECvStQAPAnaXn292QV8ywfvY=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0UYV2u90HFNIt7k1ArnjGQ==</t>
+          <t>XZuTC1e4fL4oJzrAlHU3rA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>59Qz9K/OdPg2W0SN8U14Zw7E7oAVxEmV3eYCnKt9IBQ=</t>
+          <t>liE+TPFIUYKAcOMkc+gywbGxowIy7HrlP8PFFN+axLw=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4I7uRZJXEUZx8D+wLObQew==</t>
+          <t>2zt0TLTCT4ENtwhCp4fa7A==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>s+El3R500zxKM/ETlw676OJ47Ap5WA8KIHGqF/ifuo4=</t>
+          <t>d8Ou52Jv2A5DKNxXEHUt/U/Kn3o5CPqJ6/ZHR2Gi9z8=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mWy/1aoXvo8ZKIozMIbpFg==</t>
+          <t>0MiGaiNq1gKwwAgY6sZArw==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>pOYIUQ7uMX/zmP/O9KLBCk3ACdvUR2YTAvvaxuhlV/s=</t>
+          <t>uw3WO0ZqcOEHE/8VV+0iYcrzVY49YSh2ulBSPUssyZg=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mous3dGOzigBHOnDbBYm5A==</t>
+          <t>ZKBeeLQ0nXs18hUxufOAEQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>b6w9PWL/nOpTAfwKZsNeL6oo6Kj+y2WWxWeHEvIlxtU=</t>
+          <t>Q/jbngR4mUuVHd8UXWt/gSeP+99XYQWZUD2xOmVrlSA=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>8OvoPltzA6FEM2fVjA/G5Q==</t>
+          <t>u1znovr5aSko3yvecCMLxQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Ffv67MJV1UIy9fqiEfo8nB6IL+QZkqOoVLn6LIscc+A=</t>
+          <t>iEt3Ir/tCZX2OmCSuvvIDI0SrgTCmLm8986Ul3EI13I=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DaDzuJVmAgOUonKdpwTGPw==</t>
+          <t>AfQ+zK6zM2riDXhDeQFPkg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>WjRN8iGgNG5ZF2yWv6xRRPjchT2wbzn2aqRzTt31zKc=</t>
+          <t>erkvqZtiWCB/0HydB9PQd9RoeuFdTCUN0haorxMI7QQ=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DJE8GV0GbSm4tJMF1KB/7w==</t>
+          <t>lSXDKqsx3JEup0MKL6BLKg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Eff7T8ri0Xg6rwOy21neDVm6cjSOv/3RDTWK/CyUoTQ=</t>
+          <t>3BRoOjGORUk9dbUvvIO90/t293IP/Yd6BO2jn+k4S1w=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>EONo4T7pIRILMWrA+y+HGQ==</t>
+          <t>E52fiPZgZfSkD9gTFeSrNQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>+09TimDGGM0vyeuWvkLi5fuNuhAIZG1i3BR0LwtUhc8=</t>
+          <t>jF5vEPMcU8cB0xAqFACBRM1PJR1LBl24BT7KfHUrFLI=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>x4AvdgjgoTh1GaQ0IieD0Q==</t>
+          <t>zUnfR2HUcYJZJtpBArDvqg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>aUL2JMqGeaSoHkjL+KpM1kTLho8ViNiSf1awkY5UFCE=</t>
+          <t>UzO6w5Y6inQxLD893N6NJcJgynPtQRTK8pJb90NToF4=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>/hNszvqojr0bxIIKaVFSxA==</t>
+          <t>l6/9xuPZpBmu3IYpO9zV5Q==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>jhsTU2RpGWczeyG1DC7ktkyz8aD2oZiUppATo5BPEmE=</t>
+          <t>AMfAurFz3P/TiXY7wOKXlNpz1muMjL/1rVkJwuIfSbM=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>e4EDbPId9WKlSQZHV+2Gjw==</t>
+          <t>OEo/cMyXXIoa97mB1hsiSw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>++doUapiQOxlLvAKtxY9vdp4YRBtawDk17Zzh4+y5t0=</t>
+          <t>fpPJZQYL8/S6iIJykPuLTYZop7sUmK8xU78HcWiNoMU=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>w0MH9aRmsc3k+UIcVpKlhA==</t>
+          <t>dZ5NMLTgvOT0Jw83hm5JDg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>LVswHb9Iw0kZnRdyme8ZD1MQTcZqaUStHcSkjEQ1JCY=</t>
+          <t>90Cum+KwMrORDU1hN1UKvh8nRiQa2PrF/YuHg4e8vvE=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>DK4VWrz0XBHFW2gJHE5tJg==</t>
+          <t>vqRhvlD66jJ4ipOZzplHFw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>xZqI1X/OtGNiaoSZtbUjaAdIe4wiAVVyLUsrk2d9Uw4=</t>
+          <t>F/ajVhUvm2lOv/jxbHm9FKA0ttwbLcM0O6sWRbV52/w=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Xx05c4F55qD24ZPtLsaiCQ==</t>
+          <t>/uWQO8/xkq0oEb+hVzsdwQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>fRdR/C4osIQTDVWmSqFyMzqiwHTECdSi1QQ0RaMjabw=</t>
+          <t>AXYR9hOlNKzfbv81P1cfw7vHm/iOM3pmohlhNZT9uEk=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>HntDDfrNecMx2IUQxOTd8Q==</t>
+          <t>NHt/3bqpNV5YmrKYeUvm6A==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>kXnLHJabAUuLBkPxHLtYHxQKPeA0ICKefAQ4xWUEhRE=</t>
+          <t>l9PY+SXYH4djlpMk/wvygnJq2ev21a3HAxluDFW/S2o=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>U+0RzA/pQXA3Hct0UBGIAg==</t>
+          <t>aHt4HHuvnq1g6wsgzmgq5Q==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>S6OAVtPlJrz3JzNYpQU9l3LK9oyFeqnVsWQM6lKOwjg=</t>
+          <t>+gTRneO1d01EikOe74PCEY5oL8T5qYmtVJ/n+SZtOtQ=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>70lfcQRRsE1S9w/8ZuAvxQ==</t>
+          <t>4JYsIATwIFrtCUZ2nGo1Cg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>o14uaR8TGfUeGmSWR1swemkm0O30zoSiOa76jaQ/VsQ=</t>
+          <t>dARE3qn6p/sX143kM6vXK/vNW+O4K3sEogcTx2m6XXw=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-08 10:40) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>aKYzPx2vrpjQCFgQ5P76eA==</t>
+          <t>vOroU8A1hWfVkFFuk7aK9Q==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>vvU5RHpLof+APwQDvOgte5ItvGZgNvCdfrRMgmY50eo=</t>
+          <t>KtGdj9UcIuL4wDLjB9iyBBdUGD7CbU1KIszcIwu/0m0=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>vf2b8qQTxfuMZsOCyy/jEg==</t>
+          <t>RfGojeu/GgEUq9gAjitfjQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>j/AC0fNMkQKwot2kRfQ7GlPzljerbkEYQ5yj5FL2jw8=</t>
+          <t>T4PKDLR730/LblErWQXxNj/qnDaSCbAgdrgreOkOX8E=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ZTdUxzPhBNlJOdF8loeORA==</t>
+          <t>f75lXX7SfSlHZRDx+Zah5g==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2Di+ITEtRIgZNlJDFXrxSmkzjHZBSWcfds7fNP4te0Y=</t>
+          <t>Akv8bOhAhgEG3AO+ovtHiaGY+DVbnpYU5B9Qwr9Yr2g=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Gcu69P2PMaQT2EkDXpKLYA==</t>
+          <t>ZF3tv56BXrEFrE0QQKo+LQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Jxo8J1hepAYTNgtRXk+w+D8J29psOqPn8Bp6SRcrS5I=</t>
+          <t>SpDadPJYuuw2lwkEtXsCADSB8y6bc7xjOn76Jlk4Q5Y=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>QDOsWMuZMjSc7q61fWelQQ==</t>
+          <t>1MOVmj1f46vPidlkP8vdPw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>qxY7p1JRznr6ygvDgoQAl5v57n+KJF+kvkJqNPkWGzg=</t>
+          <t>XJT7ldpo9Mj1akbYVuqf/CNF+/UhamZ1XkcpRWkUtLM=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PYBnZtdnH3OArSUo7Jevig==</t>
+          <t>L4x9t7fSBsMJ2rbcYTFDhw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>l2b7UMnQYqLzpTnmh0NPTHTa8VcOJctrdxnZKIPsMAU=</t>
+          <t>9qYLH6keIGlLMjFxY9YY99tzyS4QU7oNcMi+i78Kqx8=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>V3BjEvwQblJ3+7K54VwQTQ==</t>
+          <t>RrpRS6MSpblpWuvkWGucMA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>fL1HrFVwW0R7AqdzVsB44qy7ORSvgdN9FgIR1Z+khUs=</t>
+          <t>GYHbAArYncCe7mdxH1G8j9Au1+V+MtnnqLSb216mykk=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>6PZHkX+rIU7FUSF9rUn52w==</t>
+          <t>Eu/62BRmjNJZrt4fSC2WsQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>BcgvRdxLzz/kCDvkjoIzZHmwdAULa7ia61gnp2yDPPA=</t>
+          <t>rc4lQ3MyalfcDORGpPPNW4PDWC1TknHVPoyLBwgiB4o=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Xdb11ehlKzwUJkn3bCzC8A==;1C/WHdwHvOcx3YfQB9h4SQ==</t>
+          <t>iRN58DXvC39hObBaEebfXw==;8tW7lZ5WCEzyd7MhGnwQ+w==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>WgkAz2RwA8wPsP+rvWkjJtZglc5exEzq+oRMr/y/Kb4=;+Zm9qsr5o6oea+xRpwrNZkMJFPqX6v8u43TtTep4Tfg=</t>
+          <t>5N3YNeorrXHDZZ4duvZak13k3zUUCKCiaM986QaodNg=;wh4NQIVeyGbU1fpZDoRPdWnxh93zESEfLevoytV9Z7w=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>UI8ohrnFBmk3LMEmQK8mWQ==</t>
+          <t>6esm3RNqZXtnClxKKx1qFg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>bwNS8MxWOzSjORzG0xF5VT27hZcmz44nthABqDVuYEE=</t>
+          <t>IsbaSNFm5AsnRPtZCZytRfeJ10PozDw6/X7w1G2t5js=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>QeWbrwem4baF67xs3DtU5A==</t>
+          <t>m+Wi5BF6ur0U4aejM+7moQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>E52Je4K0feyP55rl7tlAjPaDHhKuBVENd95LfFtsF6s=</t>
+          <t>zbmxhMYW3u1JsGKW/oRidGouaOpyQTc4Bdx25HLLUEA=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ta5WMzMzolpstn7502rDCQ==</t>
+          <t>kF7S7i0+yIUPx6K9IxUkyQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>pUhf/KjqyBm8GsCLKF4GW6u16TqyE4sllqk5HOvMRrk=</t>
+          <t>s+LdfqU20uUAEYIreRN5ORZc+IvjbjOxF90O1BDOjic=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Y/wMqMaXraYcZwLYGO1Xiw==</t>
+          <t>NlpYAPpeNgSHUOk3JJDxlQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LEPf1TSRePc4z8nJfeJlQNXJS0QlgiUqr/MbgkpxJfc=</t>
+          <t>GTKsLFIa1Lt6mYc4O7hsy2JI0mXBtkrTJSWUCYAQYzw=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3o+C/wojPrrC0QHCkTUqzA==</t>
+          <t>dm9CnrdTXEgV3D/cnV7T4w==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>67W3dNVQsHvqyBKMWVVWe+OUKxbg+ZMAwhJxbI0HaUo=</t>
+          <t>y7oNYtZrX9B4HAKVSHML53zDOwIAPeS/bwYEE9Te1tQ=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>+XaX55X7Tt5PpGnCdXxbWQ==</t>
+          <t>EqBI/J8YD9/2Mcme2ngQuA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>O3rPj7CzgtIewigH2+B24QlFrnIfVIoBLAXQCjvT1qs=</t>
+          <t>FA0Iivsh4PkGvQWX4MPGEsVBZL4k5QZST4FQspT5PB8=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2h4AvN1yxhZc5jtSWcuTgQ==</t>
+          <t>9XCPp4U59j59IKmR3M2qWA==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>uJgHRqnU7YOtLQkKvIWXECRW/NzlUWHG8rXPYUCk1bk=</t>
+          <t>sY1ndRaOHOOz3GdA6NDQpZgyywoJ82T07j31onR1MuQ=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>gQh8wL+0G0K/ROZRmZXXHg==</t>
+          <t>UzImOOwaRFzhT5tTKb1shQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>aKrzL+E+CJ/v/DNhboakBtJme7xp8Vk/TjhYcsvxAT4=</t>
+          <t>mC07zZv1wGxOnIN9egqKagNKr1GLoe3Od895GmKphOI=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>aXsFKyAPtdjfFWDWDVAJAA==</t>
+          <t>XxPOcyqjBFLmt/LhAPKAog==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>UpLL1sefhJrVa6FUb3h+cNrKU+QgKVlvOty+w6ousog=</t>
+          <t>erkmt5HO9fY6crFzwVe3wCRMUwONdo3ZGrc0jmF4Lmw=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>B4uUp3b75Mm/9deczMV9Ew==</t>
+          <t>+t1lrKHwn7VsFmm8oFSl4w==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>xEOGt9NbYsgbe9pR9FxgTbCQSGlv+M6CE3LzVZl3pHk=</t>
+          <t>xMlVEkEUSELMLUr3/UIgwWkIvJdAXY5GByZKjhMC6os=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>IrrDZClE7FiezTICHN9D0g==</t>
+          <t>wnqSgHOliY+Qkc/X5SkiRg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4sLpuJjNbm52X2pwL9/ECvStQAPAnaXn292QV8ywfvY=</t>
+          <t>QU6nB/CR84ieONsnUyLKM5x7U2KsCHaK4EUsMqOpBIo=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>XZuTC1e4fL4oJzrAlHU3rA==</t>
+          <t>pZYwqFOkmtdgrV69EyTB/A==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>liE+TPFIUYKAcOMkc+gywbGxowIy7HrlP8PFFN+axLw=</t>
+          <t>k01QQWtPQ7bs+KhJMN+wfmnWMg0MPJ1PsHYRArF+nTs=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2zt0TLTCT4ENtwhCp4fa7A==</t>
+          <t>dzK14l4cFvbMaw3mhslAuQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d8Ou52Jv2A5DKNxXEHUt/U/Kn3o5CPqJ6/ZHR2Gi9z8=</t>
+          <t>5fX6cWG+qZjcMY8ksOnn/3cmDTCC6GOwTyH2HZQXIGA=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0MiGaiNq1gKwwAgY6sZArw==</t>
+          <t>RABYViRPNm3IUZ8VoP+FcA==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>uw3WO0ZqcOEHE/8VV+0iYcrzVY49YSh2ulBSPUssyZg=</t>
+          <t>XPA4ZkIINfYHAScBvrXSMxUD87/sqKGuyRwU3mLAWv8=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ZKBeeLQ0nXs18hUxufOAEQ==</t>
+          <t>E/+krLbJ+EgKFM+LxZPvPg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Q/jbngR4mUuVHd8UXWt/gSeP+99XYQWZUD2xOmVrlSA=</t>
+          <t>NEwwmtFBzT3+NMtAkojVYodD5VFHbwmt7azjcYlzVG4=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>u1znovr5aSko3yvecCMLxQ==</t>
+          <t>+c6ix/dI27tUccWOgpFaUQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>iEt3Ir/tCZX2OmCSuvvIDI0SrgTCmLm8986Ul3EI13I=</t>
+          <t>VIJk3Yw7CTOQId1/EZTDHzqnDkymdE7ePZcPuI2RdYg=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>AfQ+zK6zM2riDXhDeQFPkg==</t>
+          <t>hs7G2ZIV5Ugg+wJ34zVhxA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>erkvqZtiWCB/0HydB9PQd9RoeuFdTCUN0haorxMI7QQ=</t>
+          <t>clrlDLRaPhzzKcM6zCMSbrhtze8PRotiCJEZLQ5Iocw=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>lSXDKqsx3JEup0MKL6BLKg==</t>
+          <t>oItc1Bk5dwiGsZdC2cYuLg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3BRoOjGORUk9dbUvvIO90/t293IP/Yd6BO2jn+k4S1w=</t>
+          <t>tvtdLxmec9uzy+ZuklMDNZa2j1dBp4Lywq3Zk7WkyY4=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>E52fiPZgZfSkD9gTFeSrNQ==</t>
+          <t>QpjEgBrY7VgIq677gszkOQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>jF5vEPMcU8cB0xAqFACBRM1PJR1LBl24BT7KfHUrFLI=</t>
+          <t>LVXX/L2xRJzeKOaUbYjG+5orpt2wNyUXhrfZd8L4Ux0=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>zUnfR2HUcYJZJtpBArDvqg==</t>
+          <t>RABzntpDi8ps1kiXm8AKQg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UzO6w5Y6inQxLD893N6NJcJgynPtQRTK8pJb90NToF4=</t>
+          <t>+uCae/afGRmcsqLX03yEB5Yexsi7hzUiVCTTJvqyDEM=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>l6/9xuPZpBmu3IYpO9zV5Q==</t>
+          <t>g7lbqWqTCM4Jp/99C0vzhA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AMfAurFz3P/TiXY7wOKXlNpz1muMjL/1rVkJwuIfSbM=</t>
+          <t>/XWXBGegJVPEZjm6P+c6a9r90HAcfii+iw/umHYET1s=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OEo/cMyXXIoa97mB1hsiSw==</t>
+          <t>xUcoxLHBMCg3PHE+Qe3tdA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>fpPJZQYL8/S6iIJykPuLTYZop7sUmK8xU78HcWiNoMU=</t>
+          <t>j9p5BGpvFpos35UCSaRb5kFWQMxcbOoBBtIj8ElK5Do=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>dZ5NMLTgvOT0Jw83hm5JDg==</t>
+          <t>Zk6L8s1XBpzAXACpl0sb0g==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>90Cum+KwMrORDU1hN1UKvh8nRiQa2PrF/YuHg4e8vvE=</t>
+          <t>PPYMdmUew0IpvFem+ijb+oIpwmxduQMCEXx1TehBkP8=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>vqRhvlD66jJ4ipOZzplHFw==</t>
+          <t>FJPTbrzQuRxAen6elQRylg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>F/ajVhUvm2lOv/jxbHm9FKA0ttwbLcM0O6sWRbV52/w=</t>
+          <t>KgPtOi9QPuoIkYm4reCy0tV1+uhyT2TgX2ih4svGdTs=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/uWQO8/xkq0oEb+hVzsdwQ==</t>
+          <t>jIiEGZMMwUCuDAIPM4cYKg==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AXYR9hOlNKzfbv81P1cfw7vHm/iOM3pmohlhNZT9uEk=</t>
+          <t>MkNAye/fkUUQ9EDqvXTZiabloqu30vg9Rp3q1xvk99o=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NHt/3bqpNV5YmrKYeUvm6A==</t>
+          <t>A2JAU05znoYBUKSzqYF/Kg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>l9PY+SXYH4djlpMk/wvygnJq2ev21a3HAxluDFW/S2o=</t>
+          <t>FEnEtt5KrJ9fd51Y9ubpM1SIpvoThW5wePinzhzxCJM=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>aHt4HHuvnq1g6wsgzmgq5Q==</t>
+          <t>HN8t3/NlzV8jH+SmpLCKXA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>+gTRneO1d01EikOe74PCEY5oL8T5qYmtVJ/n+SZtOtQ=</t>
+          <t>szxjYNy6CHeh73D8jeGCYk+vGNTlRfaFE41aEvpbvck=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>4JYsIATwIFrtCUZ2nGo1Cg==</t>
+          <t>NCNuUFhJvtvUcCMadsm5pQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dARE3qn6p/sX143kM6vXK/vNW+O4K3sEogcTx2m6XXw=</t>
+          <t>CQyP7/0fcU9VyYZGKTtPMQ+xkp+Y8+U+OkF3FVEmBJw=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-09 07:39) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>VENTAS MENOR COSTE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VENTAS MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>269</v>
+        <v>278</v>
       </c>
     </row>
     <row r="86">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="96">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>328</v>
+        <v>341</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>328</v>
+        <v>341</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="118">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="121">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="97">
@@ -10746,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="98">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="106">
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="107">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="108">
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="109">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>269</v>
+        <v>278</v>
       </c>
     </row>
     <row r="110">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="120">
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="125">
@@ -12026,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="126">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="132">
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="134">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="147">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>314</v>
+        <v>306</v>
       </c>
     </row>
     <row r="150">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="153">
@@ -13494,7 +13494,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="155">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="156">
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="188">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="222">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>vOroU8A1hWfVkFFuk7aK9Q==</t>
+          <t>Pwn09WxfjK7k7/EqRMDuNQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>KtGdj9UcIuL4wDLjB9iyBBdUGD7CbU1KIszcIwu/0m0=</t>
+          <t>Whi+ejxh0XUUaIAfzTDHSgkb/4ZFDTe+EKMU+byULjU=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>RfGojeu/GgEUq9gAjitfjQ==</t>
+          <t>tcA0Rw1uhTJ6SdSRjSZgXA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>T4PKDLR730/LblErWQXxNj/qnDaSCbAgdrgreOkOX8E=</t>
+          <t>dJHg24JcSDB7spafQL+I0VqBvHvOjSBp5Yk65Iibliw=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>f75lXX7SfSlHZRDx+Zah5g==</t>
+          <t>aG3b9J9lNpsbFqT50cY2gA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Akv8bOhAhgEG3AO+ovtHiaGY+DVbnpYU5B9Qwr9Yr2g=</t>
+          <t>1r+2wedHEM9Hr06VDND3amTEZiCJuJV50h+db/GxtkU=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ZF3tv56BXrEFrE0QQKo+LQ==</t>
+          <t>x0qCHeX4EvhGhSeF6nOS9g==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SpDadPJYuuw2lwkEtXsCADSB8y6bc7xjOn76Jlk4Q5Y=</t>
+          <t>uNmgKXJ8ioEVVeneL5+ggxUkw5P05FtvJWkbvcJj06g=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1MOVmj1f46vPidlkP8vdPw==</t>
+          <t>C63tioEgbkQ0Ld3fcZF9pg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>XJT7ldpo9Mj1akbYVuqf/CNF+/UhamZ1XkcpRWkUtLM=</t>
+          <t>wVvp6yBuJOKY4CFngaoM/Lpyj+bWBg8Q92MMpuvpryU=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>L4x9t7fSBsMJ2rbcYTFDhw==</t>
+          <t>t/IeYQATKn35d/vtbpo1ZQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9qYLH6keIGlLMjFxY9YY99tzyS4QU7oNcMi+i78Kqx8=</t>
+          <t>ziRELLtF6HI5VbVwaFpiGscqPXQimV+dhbBICJfowEE=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>RrpRS6MSpblpWuvkWGucMA==</t>
+          <t>QHEC5wMmbiYsQwsSy+Hsgg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GYHbAArYncCe7mdxH1G8j9Au1+V+MtnnqLSb216mykk=</t>
+          <t>maDc864E60CUPZD8OX9H7r3VY32HZp1exhka1EawTt0=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Eu/62BRmjNJZrt4fSC2WsQ==</t>
+          <t>xsQnQpY4IS7xh1I8Sy1a6g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>rc4lQ3MyalfcDORGpPPNW4PDWC1TknHVPoyLBwgiB4o=</t>
+          <t>Z+8MkhUqbYdBveXG+Dsymq+h9Be9MnPRTDLue172IOo=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>iRN58DXvC39hObBaEebfXw==;8tW7lZ5WCEzyd7MhGnwQ+w==</t>
+          <t>tOEP8jAvomyQvWeJrMkXkA==;2Pq7WFK2hPbiLwoCmwpyQg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>5N3YNeorrXHDZZ4duvZak13k3zUUCKCiaM986QaodNg=;wh4NQIVeyGbU1fpZDoRPdWnxh93zESEfLevoytV9Z7w=</t>
+          <t>NMMic6mBkbKI9md8jGhA3uAyGumD4sgZS1q2QKJYbuc=;InQdzAC4bzx8LJK9S2hp1md2RhXaSnEPw0I7mr6YC6k=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>6esm3RNqZXtnClxKKx1qFg==</t>
+          <t>kvuzMfWuyu6j6+SArDqznw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>IsbaSNFm5AsnRPtZCZytRfeJ10PozDw6/X7w1G2t5js=</t>
+          <t>WDEMn19eVSTiw60oBny2LT74RuauT3eewrAJ4bffUjc=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>m+Wi5BF6ur0U4aejM+7moQ==</t>
+          <t>1QVG5Jj/S6f8tJXgG+1LeA==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>zbmxhMYW3u1JsGKW/oRidGouaOpyQTc4Bdx25HLLUEA=</t>
+          <t>oS9QoyDC+H11RUDBFNSdGrqR8UehcwGqe9s0KgTxpB4=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>kF7S7i0+yIUPx6K9IxUkyQ==</t>
+          <t>+ZBjWY2R7SYz51wMGEFHvw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>s+LdfqU20uUAEYIreRN5ORZc+IvjbjOxF90O1BDOjic=</t>
+          <t>Xi4jS3p7TB1tGuleaFyRhLP0capiDWXGDu9kdjib6P8=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NlpYAPpeNgSHUOk3JJDxlQ==</t>
+          <t>yb0hZaiJHyX5AqAe+uz9UA==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GTKsLFIa1Lt6mYc4O7hsy2JI0mXBtkrTJSWUCYAQYzw=</t>
+          <t>lTqGja8fwG92Q68CuUCMDRNXNKvz5L+A4PpLxGomxEg=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>dm9CnrdTXEgV3D/cnV7T4w==</t>
+          <t>oJhHoKdZtpK6Pfjlj+W7pQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>y7oNYtZrX9B4HAKVSHML53zDOwIAPeS/bwYEE9Te1tQ=</t>
+          <t>PcpXI5B0AifzlAKV7ZgT+AHluq16xZnQAGm9RqVsPtQ=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>EqBI/J8YD9/2Mcme2ngQuA==</t>
+          <t>RBjQVKiCZ/iwTpwd/tpjtg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>FA0Iivsh4PkGvQWX4MPGEsVBZL4k5QZST4FQspT5PB8=</t>
+          <t>D+obMY4x3s/nlpWdgyBI+cuJPFflip5l3wFB/n2ZRj0=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>9XCPp4U59j59IKmR3M2qWA==</t>
+          <t>mXPraIdWR9YE7tAOqqLvLw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>sY1ndRaOHOOz3GdA6NDQpZgyywoJ82T07j31onR1MuQ=</t>
+          <t>e9dclH7HyJVsrPojtoBBiQl8KZQgFNRaR7XcbuCpK38=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>UzImOOwaRFzhT5tTKb1shQ==</t>
+          <t>956+S2rVxp84g2CFqS5h5w==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>mC07zZv1wGxOnIN9egqKagNKr1GLoe3Od895GmKphOI=</t>
+          <t>97QzDccmZAr2OZxR3+z8INofGMe1k1XIcD4qP2ptt1Y=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>XxPOcyqjBFLmt/LhAPKAog==</t>
+          <t>DgJgC7zqr9d81n8P79fFJA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>erkmt5HO9fY6crFzwVe3wCRMUwONdo3ZGrc0jmF4Lmw=</t>
+          <t>9O4KRZ7gJL4T1Mk1pngrwqARCXwu81rpljPTJfGxKt0=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>+t1lrKHwn7VsFmm8oFSl4w==</t>
+          <t>JiQgYqIybM5K5Zf4W9wKFw==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>xMlVEkEUSELMLUr3/UIgwWkIvJdAXY5GByZKjhMC6os=</t>
+          <t>NUwfzjB4p0vyBOJlkyOxRxn7OgfWpWbY/icp+bu97CA=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>wnqSgHOliY+Qkc/X5SkiRg==</t>
+          <t>TxuLufri/IRh+mNRlVLZGA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>QU6nB/CR84ieONsnUyLKM5x7U2KsCHaK4EUsMqOpBIo=</t>
+          <t>KWS+0m0amz4uYvn5+57WRasbLwa2MjIsc4GcyMCr5g4=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>pZYwqFOkmtdgrV69EyTB/A==</t>
+          <t>GmR7FpcttZys4Ui1y5EvNA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>k01QQWtPQ7bs+KhJMN+wfmnWMg0MPJ1PsHYRArF+nTs=</t>
+          <t>vqBmHYEy/q/gr9o6V6ShcqwNiQSito4LwIoEs4xwwxU=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>dzK14l4cFvbMaw3mhslAuQ==</t>
+          <t>Qtay3h3IszVsflI4E8EzGg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>5fX6cWG+qZjcMY8ksOnn/3cmDTCC6GOwTyH2HZQXIGA=</t>
+          <t>yLYPJ4WZ+LJ8OBxBxrEZH2yi+X60WYZ/CeM04Yt/X3I=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RABYViRPNm3IUZ8VoP+FcA==</t>
+          <t>eJBLSQvpDNgQ6uBnKO+QtQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>XPA4ZkIINfYHAScBvrXSMxUD87/sqKGuyRwU3mLAWv8=</t>
+          <t>tT+OR/YKHSzmx09KnQ7TmuU9pCjxNWFfDhj4unfGtnk=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>E/+krLbJ+EgKFM+LxZPvPg==</t>
+          <t>ear6XPn+sfJ3JjOKUDjysw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>NEwwmtFBzT3+NMtAkojVYodD5VFHbwmt7azjcYlzVG4=</t>
+          <t>HX4QFFJq/qO1QwXPjlcVWrT3K++yPm9IrHVg9A0IatU=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>+c6ix/dI27tUccWOgpFaUQ==</t>
+          <t>Y/QFinnnFyFQBPghMMxzsg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>VIJk3Yw7CTOQId1/EZTDHzqnDkymdE7ePZcPuI2RdYg=</t>
+          <t>VFF8EaL2O4lSyNQCkPY8sIt8a6pA9YV7B7ANftFf0v4=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>hs7G2ZIV5Ugg+wJ34zVhxA==</t>
+          <t>hHREfv3eH9j088nxZN10yg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>clrlDLRaPhzzKcM6zCMSbrhtze8PRotiCJEZLQ5Iocw=</t>
+          <t>dNbqqsgzGDxaVjLk90yDviRuzx81pNmdbhee8uX9bSA=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>oItc1Bk5dwiGsZdC2cYuLg==</t>
+          <t>ghE1SqhaYYhGFdi/l0S/yA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>tvtdLxmec9uzy+ZuklMDNZa2j1dBp4Lywq3Zk7WkyY4=</t>
+          <t>DbvTAe5oFwCZ9vLsIboxiNetKNEsTL2L/ge/m8ih0Xc=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>QpjEgBrY7VgIq677gszkOQ==</t>
+          <t>UX25fx2cEImt7Z4of+VdVQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>LVXX/L2xRJzeKOaUbYjG+5orpt2wNyUXhrfZd8L4Ux0=</t>
+          <t>1ifAIInZKaxrudpnbrL4Zz3jBCeYnqyfWbE4PB12UaA=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>RABzntpDi8ps1kiXm8AKQg==</t>
+          <t>r5RczeQMELH/lXHm81KEsw==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>+uCae/afGRmcsqLX03yEB5Yexsi7hzUiVCTTJvqyDEM=</t>
+          <t>3sv+sPKsvXgJz9Cq3McK3BoFVN7Q9+xDT7dkOnJg7IE=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>g7lbqWqTCM4Jp/99C0vzhA==</t>
+          <t>queEUPHqVHq1k98FQ3t/wQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>/XWXBGegJVPEZjm6P+c6a9r90HAcfii+iw/umHYET1s=</t>
+          <t>0RxjUa3nMIdCAhr8mbpE0+juBiRRGLNGJQgCTGw2LgQ=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>xUcoxLHBMCg3PHE+Qe3tdA==</t>
+          <t>DxQsQKyA7H4Z0crLxInmbA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>j9p5BGpvFpos35UCSaRb5kFWQMxcbOoBBtIj8ElK5Do=</t>
+          <t>cG1C1Hqh4bhzGmJ6uyaxVIfR5+Osga8OqaXGPvdtfYk=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Zk6L8s1XBpzAXACpl0sb0g==</t>
+          <t>72Sx22mlDNjaANBC9nviFA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PPYMdmUew0IpvFem+ijb+oIpwmxduQMCEXx1TehBkP8=</t>
+          <t>Dh8fjAFvWAGhKaOqQpSasKlOAk9Vej+cpvTCdLasiGw=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FJPTbrzQuRxAen6elQRylg==</t>
+          <t>cB51hGq+IPfr7Evb2b277g==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>KgPtOi9QPuoIkYm4reCy0tV1+uhyT2TgX2ih4svGdTs=</t>
+          <t>U9zOtTnvJUbdlnVGkuCsDS/46gRk/yISM8358S8TYKI=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>jIiEGZMMwUCuDAIPM4cYKg==</t>
+          <t>GDstRzNgnEDnw4PhhnLTIg==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MkNAye/fkUUQ9EDqvXTZiabloqu30vg9Rp3q1xvk99o=</t>
+          <t>KJHyRMELuBMgy8EBib4wz66zj2yzC+jEub20AjSzf64=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>A2JAU05znoYBUKSzqYF/Kg==</t>
+          <t>hdL4Ntz66dl5zi7SbNCZZQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FEnEtt5KrJ9fd51Y9ubpM1SIpvoThW5wePinzhzxCJM=</t>
+          <t>0xRgoTPPJgQLxWGbx8GAzJVUWGuIfLGygAnIA+IXfZo=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HN8t3/NlzV8jH+SmpLCKXA==</t>
+          <t>m7UMbDeCtjwykT0MnQKJgQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>szxjYNy6CHeh73D8jeGCYk+vGNTlRfaFE41aEvpbvck=</t>
+          <t>f0C0/Nh37x9cJ0Rh4TjRKSFALgtPZ3ALYFg9n6QGuJ0=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>NCNuUFhJvtvUcCMadsm5pQ==</t>
+          <t>IYCxxIZlpHJqe+yoAagD4A==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CQyP7/0fcU9VyYZGKTtPMQ+xkp+Y8+U+OkF3FVEmBJw=</t>
+          <t>AWBbVJvdF4rOnRXLWfZAPgVbBxzfNX0isIpeRXldFuY=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-10 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="86">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="88">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="96">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>341</v>
+        <v>350</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>341</v>
+        <v>350</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="117">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="121">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14">
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="97">
@@ -10746,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="106">
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="109">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="110">
@@ -11326,7 +11326,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="111">
@@ -11370,7 +11370,7 @@
         </is>
       </c>
       <c r="L111" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="112">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="120">
@@ -12026,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="126">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="132">
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="152">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="156">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="181">
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="188">
@@ -16802,7 +16802,7 @@
         </is>
       </c>
       <c r="L216" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217">
@@ -17002,7 +17002,7 @@
         </is>
       </c>
       <c r="L220" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="221">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="222">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pwn09WxfjK7k7/EqRMDuNQ==</t>
+          <t>2mUJcPRNk6AjNCovXW4/Ug==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Whi+ejxh0XUUaIAfzTDHSgkb/4ZFDTe+EKMU+byULjU=</t>
+          <t>Tw1A3kZgLARf+/Dhi3eNlgTmvzrlPpYmuFiN9jCb1rs=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tcA0Rw1uhTJ6SdSRjSZgXA==</t>
+          <t>ziZthbSkVDC2UCDJOjXU1Q==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dJHg24JcSDB7spafQL+I0VqBvHvOjSBp5Yk65Iibliw=</t>
+          <t>Wx/LnIeF+NX6A6KcdVn1/2ZF6R7hp9/qDWk0sYoEXt8=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>aG3b9J9lNpsbFqT50cY2gA==</t>
+          <t>CBwIL5ccHAHmjBbSNwZPqA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1r+2wedHEM9Hr06VDND3amTEZiCJuJV50h+db/GxtkU=</t>
+          <t>eUjjS8fU8EzpDPINJjnq2t5Z0s4QGg/plIs4kUEkIkQ=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>x0qCHeX4EvhGhSeF6nOS9g==</t>
+          <t>PyjSqyVRmJw6adcDWfEgOg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>uNmgKXJ8ioEVVeneL5+ggxUkw5P05FtvJWkbvcJj06g=</t>
+          <t>4w3HQOsB94olzpll3zex5xfY0xuVcf0EtRSLEtMpYMk=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>C63tioEgbkQ0Ld3fcZF9pg==</t>
+          <t>zbANduHyxnoC0hoRSRC62A==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>wVvp6yBuJOKY4CFngaoM/Lpyj+bWBg8Q92MMpuvpryU=</t>
+          <t>j055V0ja6qmlXN/C3JiFRpAki4TpigRNiv/Xddau4EQ=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>t/IeYQATKn35d/vtbpo1ZQ==</t>
+          <t>aooHwpREbcmr53KaHQzu1w==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ziRELLtF6HI5VbVwaFpiGscqPXQimV+dhbBICJfowEE=</t>
+          <t>idOlC0Jf9TIN462MaTRloFdDrsIB/JQf+Mx6nVAVCUw=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>QHEC5wMmbiYsQwsSy+Hsgg==</t>
+          <t>8crvWytgf+WxyvoJlqspbw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>maDc864E60CUPZD8OX9H7r3VY32HZp1exhka1EawTt0=</t>
+          <t>z/yUSry7Z6n8n5PYqMmgpK4sVshCrkv6za/Nsm/Iuos=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>xsQnQpY4IS7xh1I8Sy1a6g==</t>
+          <t>bVQqR4G8ePQavf7pIuJe9g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Z+8MkhUqbYdBveXG+Dsymq+h9Be9MnPRTDLue172IOo=</t>
+          <t>zMImFdP10GMcYsiLd1j2eSMsnwJeqKctuNY14QOsWCg=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>tOEP8jAvomyQvWeJrMkXkA==;2Pq7WFK2hPbiLwoCmwpyQg==</t>
+          <t>Md0jpbBP7lsRg54ClpACrw==;LghFW6SCnR+YUr1/58+e+w==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>NMMic6mBkbKI9md8jGhA3uAyGumD4sgZS1q2QKJYbuc=;InQdzAC4bzx8LJK9S2hp1md2RhXaSnEPw0I7mr6YC6k=</t>
+          <t>uzhccWBxMTYI5YaSPAbGRdDNG0JYInB/T8lCBIlrhSc=;yrIkuvb3UO42P8h74+UTxSitelc8DSptY4k5e9rDNPc=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>kvuzMfWuyu6j6+SArDqznw==</t>
+          <t>045m/QyRrXYYG4gyICb+Ag==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>WDEMn19eVSTiw60oBny2LT74RuauT3eewrAJ4bffUjc=</t>
+          <t>RKRSWDiVhxXkyImOf/t36y3jF8bX0Pw413h+XgGSn+M=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1QVG5Jj/S6f8tJXgG+1LeA==</t>
+          <t>NZqv+5UUAY680vBSBf7IDA==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>oS9QoyDC+H11RUDBFNSdGrqR8UehcwGqe9s0KgTxpB4=</t>
+          <t>lDUZjm6i5r2NRkxrqfg1Rfad4JN+M4PjBaiR6IPMo+0=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+ZBjWY2R7SYz51wMGEFHvw==</t>
+          <t>3IVxAX6ogHxxUZf/Z71pdQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Xi4jS3p7TB1tGuleaFyRhLP0capiDWXGDu9kdjib6P8=</t>
+          <t>ukzjNBAVpyJBTtqbfyEJbjJSSZkCXnha4c1xjCh/PZA=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>yb0hZaiJHyX5AqAe+uz9UA==</t>
+          <t>ELH7e8n2QyMHB/29/OTFTQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>lTqGja8fwG92Q68CuUCMDRNXNKvz5L+A4PpLxGomxEg=</t>
+          <t>D5SmX2BP+E2VQxgX0ixS8uZoxWLbF95N1bb6In/nHzA=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>oJhHoKdZtpK6Pfjlj+W7pQ==</t>
+          <t>kaFdyfYhdIlKjslvq9V2/A==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PcpXI5B0AifzlAKV7ZgT+AHluq16xZnQAGm9RqVsPtQ=</t>
+          <t>76zie1EyjIN8fwBvGcq8VmQwQfkfxTIpXxKFx8SNzgI=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>RBjQVKiCZ/iwTpwd/tpjtg==</t>
+          <t>nT3k5GtkrkGShQwzubPVcA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>D+obMY4x3s/nlpWdgyBI+cuJPFflip5l3wFB/n2ZRj0=</t>
+          <t>Lh3bnkhlfTPEUq/+q1Ti5HCqXuSLSQRFD3bZyNgUK8Q=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>mXPraIdWR9YE7tAOqqLvLw==</t>
+          <t>ZFxtlab3QfN8W9kqsM5wSA==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>e9dclH7HyJVsrPojtoBBiQl8KZQgFNRaR7XcbuCpK38=</t>
+          <t>1ooTzt6q7g6ZiHRmgdvHzERZuw2LOAwAYOxSbBx3jvI=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>956+S2rVxp84g2CFqS5h5w==</t>
+          <t>6faJImtE2bZ8cAlT/8Nx7A==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>97QzDccmZAr2OZxR3+z8INofGMe1k1XIcD4qP2ptt1Y=</t>
+          <t>Z996KhtUDH6WYZ+SrEb+ifQDsfh75cT46Pl29MK6sx4=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>DgJgC7zqr9d81n8P79fFJA==</t>
+          <t>BYohSntgH9DDZdyQIm5zlg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>9O4KRZ7gJL4T1Mk1pngrwqARCXwu81rpljPTJfGxKt0=</t>
+          <t>aCwfk/HdcDa/1DEqSywBk8jgrjDc/JjPzclisdlRedw=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>JiQgYqIybM5K5Zf4W9wKFw==</t>
+          <t>WdKjlb7H0Ob3kv898VrRnA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>NUwfzjB4p0vyBOJlkyOxRxn7OgfWpWbY/icp+bu97CA=</t>
+          <t>0af9E/573YMcjzLzvjRxF1nghiwZDPxeOG+/YwWE5Ps=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TxuLufri/IRh+mNRlVLZGA==</t>
+          <t>oTGP9UkfPo061PzQvYGB6g==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>KWS+0m0amz4uYvn5+57WRasbLwa2MjIsc4GcyMCr5g4=</t>
+          <t>pi6AfgmS/7A79okmRZOAJcwu7mPmxF4GkcOPkZVFx9U=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GmR7FpcttZys4Ui1y5EvNA==</t>
+          <t>F9darz5xj7ctgfntk/P+jA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>vqBmHYEy/q/gr9o6V6ShcqwNiQSito4LwIoEs4xwwxU=</t>
+          <t>rHbl1iUe/ifQCkVRZxmKkdRElUe3m4lFT589YsrGIMY=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Qtay3h3IszVsflI4E8EzGg==</t>
+          <t>K9VFLD66MHR27GzM3rihqg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>yLYPJ4WZ+LJ8OBxBxrEZH2yi+X60WYZ/CeM04Yt/X3I=</t>
+          <t>b3aadSujdK/Eg5ZhcVxM059B0jsdpspF/xt8l5U2qCI=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>eJBLSQvpDNgQ6uBnKO+QtQ==</t>
+          <t>wyam0+Lz2O3l8ki1KvdJ5g==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>tT+OR/YKHSzmx09KnQ7TmuU9pCjxNWFfDhj4unfGtnk=</t>
+          <t>AnXYbhO+PRXU/+1Rbz2UG21uW6MH5EeqcGb3jw0qPkc=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ear6XPn+sfJ3JjOKUDjysw==</t>
+          <t>X/chuU/v8ivuXc9Vi9uyOg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>HX4QFFJq/qO1QwXPjlcVWrT3K++yPm9IrHVg9A0IatU=</t>
+          <t>Ko3E26FszVRPCf+TEKOQkv8/zghv1wsEdfizo+OfBx8=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Y/QFinnnFyFQBPghMMxzsg==</t>
+          <t>VGjesbzGd0vUBxTAUDzmQw==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>VFF8EaL2O4lSyNQCkPY8sIt8a6pA9YV7B7ANftFf0v4=</t>
+          <t>utMMA9bnf9kWsEP/b8oG4CjGwas1biiYkr1JbMJHOXk=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>hHREfv3eH9j088nxZN10yg==</t>
+          <t>OCv5gaJJtF/LASSjy+M+IQ==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dNbqqsgzGDxaVjLk90yDviRuzx81pNmdbhee8uX9bSA=</t>
+          <t>gJMyTqr6IS5J3TMr+WAgtfBN589Bp44BrLcbipzBQiQ=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ghE1SqhaYYhGFdi/l0S/yA==</t>
+          <t>SV6//rHsAM5C2D7wF/7z0Q==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>DbvTAe5oFwCZ9vLsIboxiNetKNEsTL2L/ge/m8ih0Xc=</t>
+          <t>9WoeKZMy1wTEtIDVUcsrLAuTfpGHRVjMy8SJzQwCgRw=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>UX25fx2cEImt7Z4of+VdVQ==</t>
+          <t>cC1A1RrKm7H3+czT7+RnLQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1ifAIInZKaxrudpnbrL4Zz3jBCeYnqyfWbE4PB12UaA=</t>
+          <t>BoBRzUac3FfAwE9hBC6zp0gg5Im+a0hSi7ohmjbp/nc=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>r5RczeQMELH/lXHm81KEsw==</t>
+          <t>PC0ohrwPm/I9WSJGyCayLA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3sv+sPKsvXgJz9Cq3McK3BoFVN7Q9+xDT7dkOnJg7IE=</t>
+          <t>FfnfA7CYBJJBHxd0ptJant6EC2tH2OCy/a6jGUJ3Z4Q=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>queEUPHqVHq1k98FQ3t/wQ==</t>
+          <t>9ROY8D+nYw90vd334DqvnQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0RxjUa3nMIdCAhr8mbpE0+juBiRRGLNGJQgCTGw2LgQ=</t>
+          <t>Y0BbvRzUBGv0C8DmRWPcHTydqSLWzyIt0dsByP6Jqro=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DxQsQKyA7H4Z0crLxInmbA==</t>
+          <t>U9SjFo8pTRZmL2ono2ahlg==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>cG1C1Hqh4bhzGmJ6uyaxVIfR5+Osga8OqaXGPvdtfYk=</t>
+          <t>9J0Id+0czq9B1QejT0Tr+jDhkEpivvMOHUx7iwYLb/M=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>72Sx22mlDNjaANBC9nviFA==</t>
+          <t>bQYkFp31MUAmx0vdx00wJg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Dh8fjAFvWAGhKaOqQpSasKlOAk9Vej+cpvTCdLasiGw=</t>
+          <t>Iop3jKJHlq5DFa8TXvv9K28hKaMAaBjkyt6jv4HuExA=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>cB51hGq+IPfr7Evb2b277g==</t>
+          <t>OI8kZ+e+MJKJgChW85Ym5w==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>U9zOtTnvJUbdlnVGkuCsDS/46gRk/yISM8358S8TYKI=</t>
+          <t>B8SW96Ci7lBvORsPPvvavN3syMffc2uKwEoCj1m2ro4=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>GDstRzNgnEDnw4PhhnLTIg==</t>
+          <t>OejCY35ywaaAHgKIxVttXQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>KJHyRMELuBMgy8EBib4wz66zj2yzC+jEub20AjSzf64=</t>
+          <t>xxHjbfFV1Yl78kfVTnCVWLKSFyS5VbDgzqEixM1QlCg=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>hdL4Ntz66dl5zi7SbNCZZQ==</t>
+          <t>Ipd3Hi+NwUD40C0Ziedgfg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0xRgoTPPJgQLxWGbx8GAzJVUWGuIfLGygAnIA+IXfZo=</t>
+          <t>uGyHGAzNTA2GNRn5oJ51DFNJNgmkfiNoK6hAz4o0k5A=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>m7UMbDeCtjwykT0MnQKJgQ==</t>
+          <t>ijyPHvfsx6Mqll/wwrGa8w==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>f0C0/Nh37x9cJ0Rh4TjRKSFALgtPZ3ALYFg9n6QGuJ0=</t>
+          <t>kfoGqNg17vVkkpV58ksE3UiwMRn5ZqcyTuIsG7YWnd8=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>IYCxxIZlpHJqe+yoAagD4A==</t>
+          <t>TDkyT4Dumz2UyO0GB2ygyQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AWBbVJvdF4rOnRXLWfZAPgVbBxzfNX0isIpeRXldFuY=</t>
+          <t>Z7aQKVXa1DCZpWnHIe5zzGhLWBzmQHapCn1908M/XrA=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-11 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="46">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="86">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="92">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="96">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>350</v>
+        <v>363</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>350</v>
+        <v>363</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="117">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="120">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="127">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="128">
@@ -5119,12 +5119,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="131">
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
@@ -6274,7 +6274,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -8846,7 +8846,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61">
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="97">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="106">
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="107">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="110">
@@ -11326,7 +11326,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="111">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="120">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="147">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>306</v>
+        <v>296</v>
       </c>
     </row>
     <row r="150">
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="152">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="156">
@@ -13582,7 +13582,7 @@
         </is>
       </c>
       <c r="L156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157">
@@ -13670,7 +13670,7 @@
         </is>
       </c>
       <c r="L158" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="159">
@@ -14386,7 +14386,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="172">
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="173">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="181">
@@ -14874,7 +14874,7 @@
         </is>
       </c>
       <c r="L181" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="182">
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="188">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="222">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2mUJcPRNk6AjNCovXW4/Ug==</t>
+          <t>ad7lnplyepsaF1fOMTi1WA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Tw1A3kZgLARf+/Dhi3eNlgTmvzrlPpYmuFiN9jCb1rs=</t>
+          <t>d4H3WmlQQBWvUyLz8mtZMwgq5ZUgMRRnf2cPgzkNhXo=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ziZthbSkVDC2UCDJOjXU1Q==</t>
+          <t>zJdlpseCwTQJoWg2erbaVQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Wx/LnIeF+NX6A6KcdVn1/2ZF6R7hp9/qDWk0sYoEXt8=</t>
+          <t>2Xu4O6eEcq7tVyuMHVMzFacuCabbFa8HXNbfM/M9NB0=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CBwIL5ccHAHmjBbSNwZPqA==</t>
+          <t>ESvkbA8lsLHz/FzH4U+ySA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>eUjjS8fU8EzpDPINJjnq2t5Z0s4QGg/plIs4kUEkIkQ=</t>
+          <t>P/98Pepg24hSjEKqp4k9p0HNh6+yDzDT2yFOzMlAo7M=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PyjSqyVRmJw6adcDWfEgOg==</t>
+          <t>P8B7CJsVcAECKgLsSYEDew==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4w3HQOsB94olzpll3zex5xfY0xuVcf0EtRSLEtMpYMk=</t>
+          <t>9dBmVHVgLeXuzSdz/nUeRIOvo6fL2n+IXTUcjCsWwhE=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>zbANduHyxnoC0hoRSRC62A==</t>
+          <t>wV2eeruMjjTa5eUbFHTq/A==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>j055V0ja6qmlXN/C3JiFRpAki4TpigRNiv/Xddau4EQ=</t>
+          <t>72pIUaY+SZp/czflvniktlhk/L07+jGXhpcSUEL0NK8=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>aooHwpREbcmr53KaHQzu1w==</t>
+          <t>zGPtuEPLJocpYALVYZRszQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>idOlC0Jf9TIN462MaTRloFdDrsIB/JQf+Mx6nVAVCUw=</t>
+          <t>lKxWHthGbqTlEmTU1kQxZPGeWJ7KB0coHwUrVOJv7as=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8crvWytgf+WxyvoJlqspbw==</t>
+          <t>9qWnUagG9xtp7vFAFDemgA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>z/yUSry7Z6n8n5PYqMmgpK4sVshCrkv6za/Nsm/Iuos=</t>
+          <t>45Frj6m0VUfWX0eFsSrOuc/o1JvpHQ9LAREFemNgVMI=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bVQqR4G8ePQavf7pIuJe9g==</t>
+          <t>eHYS6CODv+swlrTGmMV45g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>zMImFdP10GMcYsiLd1j2eSMsnwJeqKctuNY14QOsWCg=</t>
+          <t>9507sbocjIXCadupNFDDPJpf2iML6JOshTG64u4HERM=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Md0jpbBP7lsRg54ClpACrw==;LghFW6SCnR+YUr1/58+e+w==</t>
+          <t>K+gNSnpSoIrHg9nza4XDmQ==;5EzNx3FhE9YPAPAhvRgvcg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>uzhccWBxMTYI5YaSPAbGRdDNG0JYInB/T8lCBIlrhSc=;yrIkuvb3UO42P8h74+UTxSitelc8DSptY4k5e9rDNPc=</t>
+          <t>FzBA0IM3ZyXeCS+xkPuy4NTPM7B5FtZJ0LRMwQb3dUA=;YRDGLNVuwk2Pvbb7ZPRNXHJdFIkDfiM7Y5l1jWPghes=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>045m/QyRrXYYG4gyICb+Ag==</t>
+          <t>E4lz3C9ByhXqtQEpRjnS0Q==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RKRSWDiVhxXkyImOf/t36y3jF8bX0Pw413h+XgGSn+M=</t>
+          <t>Kkj59FSg2FZlwxBDFS/SR7nAWu8WEZpmY2IlGLKTGbA=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>NZqv+5UUAY680vBSBf7IDA==</t>
+          <t>4c8lF5wKiTo31VN6q9Ieaw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>lDUZjm6i5r2NRkxrqfg1Rfad4JN+M4PjBaiR6IPMo+0=</t>
+          <t>92vaKkWOrkdv3l/dz3uHXjJwCe1XwHi+vvtaGpe+TgM=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3IVxAX6ogHxxUZf/Z71pdQ==</t>
+          <t>NtfzraYjncEo+hx/8kwTSg==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ukzjNBAVpyJBTtqbfyEJbjJSSZkCXnha4c1xjCh/PZA=</t>
+          <t>guRNpNYO7QoRCs1O1OFy2WdAXLqC/USS3StFk5LFif8=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ELH7e8n2QyMHB/29/OTFTQ==</t>
+          <t>VyOdrRfqU67IHxE+Yghr5Q==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>D5SmX2BP+E2VQxgX0ixS8uZoxWLbF95N1bb6In/nHzA=</t>
+          <t>RHszodaRhNDEkbcxhe6cnU/x3t9aQQ5IQ+y9ERrDSB4=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>kaFdyfYhdIlKjslvq9V2/A==</t>
+          <t>yPKKDXBjyRROouyNXzT2ww==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>76zie1EyjIN8fwBvGcq8VmQwQfkfxTIpXxKFx8SNzgI=</t>
+          <t>rE9lFUDuVeSjfrBzsoiWYUBzRWedp/wcsV+7tgL+0kk=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>nT3k5GtkrkGShQwzubPVcA==</t>
+          <t>xO2HW8PPqgfj1qGw1m7XAg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Lh3bnkhlfTPEUq/+q1Ti5HCqXuSLSQRFD3bZyNgUK8Q=</t>
+          <t>nnjxevFWU2nN2iw1effagnLCSVzNFuFUEz5+AECXlkU=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ZFxtlab3QfN8W9kqsM5wSA==</t>
+          <t>Rw6MiQQ3WIvy31CXxOTR7Q==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1ooTzt6q7g6ZiHRmgdvHzERZuw2LOAwAYOxSbBx3jvI=</t>
+          <t>vXBG8IZSV6tpmVvRyQAjBaeGJVKo5wIi4ZROotSDyfI=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6faJImtE2bZ8cAlT/8Nx7A==</t>
+          <t>7ZvLEt0cHZz+ZAj0S8wAzw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Z996KhtUDH6WYZ+SrEb+ifQDsfh75cT46Pl29MK6sx4=</t>
+          <t>EKNwoZBgP5jwAbxHn+OhR0S32+swjVPZtZQ69xbdOfI=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BYohSntgH9DDZdyQIm5zlg==</t>
+          <t>Msi+n+Bb2ny8CFOwLsM9Qw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>aCwfk/HdcDa/1DEqSywBk8jgrjDc/JjPzclisdlRedw=</t>
+          <t>6zefmq9TbxQ/Im3K5ISXNpZ5F8Zq/5tIWTLzymZKco8=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WdKjlb7H0Ob3kv898VrRnA==</t>
+          <t>ycGADJ5eT7NiFmx19QIc5A==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0af9E/573YMcjzLzvjRxF1nghiwZDPxeOG+/YwWE5Ps=</t>
+          <t>mcAAsJYN6A62KA/7h2nJcydRGNlIG+A8PECJ6wSk/bo=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>oTGP9UkfPo061PzQvYGB6g==</t>
+          <t>aWZF6Vfo9YmJdgRRNmYdSA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>pi6AfgmS/7A79okmRZOAJcwu7mPmxF4GkcOPkZVFx9U=</t>
+          <t>BD8WbpEcrvQHPDzXDTuRG4IWJ7a9h6m3K27HCR0QeCM=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>F9darz5xj7ctgfntk/P+jA==</t>
+          <t>Bzpxjf7ZHmxHRBA0dg4odA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>rHbl1iUe/ifQCkVRZxmKkdRElUe3m4lFT589YsrGIMY=</t>
+          <t>7GQAFhXkKzcqOSXZ7aIPRBVldLHSRMA2MK9qLywNK74=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>K9VFLD66MHR27GzM3rihqg==</t>
+          <t>RQP5DLgZDXYcDNUOnxu9gQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>b3aadSujdK/Eg5ZhcVxM059B0jsdpspF/xt8l5U2qCI=</t>
+          <t>nWfOKiO9u6QQLy/oGt8h439GwdBuRaVQWDN5LvYWUBU=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>wyam0+Lz2O3l8ki1KvdJ5g==</t>
+          <t>QH9GB25GHf5QH+uuKTXmFQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AnXYbhO+PRXU/+1Rbz2UG21uW6MH5EeqcGb3jw0qPkc=</t>
+          <t>ma6SxsbjxnCeKylRiN/J/8SC8Qyp6HCzs4nC0POP+7Q=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>X/chuU/v8ivuXc9Vi9uyOg==</t>
+          <t>Kq+tcIi9rNWnsQGc9KovbA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Ko3E26FszVRPCf+TEKOQkv8/zghv1wsEdfizo+OfBx8=</t>
+          <t>C6A8WiuOmG0PGpKYvTBsGrAM0PLnUBV8TIUKiHqZjso=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>VGjesbzGd0vUBxTAUDzmQw==</t>
+          <t>JylKRzicmrf5YHnawa509A==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>utMMA9bnf9kWsEP/b8oG4CjGwas1biiYkr1JbMJHOXk=</t>
+          <t>p2E2NTPehUOEsO1yffGCwISwasJPvsPc0hsP4BIwNF8=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>OCv5gaJJtF/LASSjy+M+IQ==</t>
+          <t>CZqczhkddjxj6EsaJ/jR8A==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>gJMyTqr6IS5J3TMr+WAgtfBN589Bp44BrLcbipzBQiQ=</t>
+          <t>kHr2pn+E7TNjtvGFh8mXIzfxjLlAQ1ooNQPV1JKcDI0=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SV6//rHsAM5C2D7wF/7z0Q==</t>
+          <t>pAHJuMaz6V0QkyMEkp1jHg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>9WoeKZMy1wTEtIDVUcsrLAuTfpGHRVjMy8SJzQwCgRw=</t>
+          <t>MiDG2DUazDewAmjutkdst9aFhQgBMON9/+zqaizDgHs=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>cC1A1RrKm7H3+czT7+RnLQ==</t>
+          <t>PdSkQ9eyjTEUFxyNyk5A9g==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>BoBRzUac3FfAwE9hBC6zp0gg5Im+a0hSi7ohmjbp/nc=</t>
+          <t>i9+rF8R5qoq7zQEL5RA7mFRe3rydFNhqFMvCZTAosBk=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PC0ohrwPm/I9WSJGyCayLA==</t>
+          <t>OwfAno+r085azZ12NJHXVA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>FfnfA7CYBJJBHxd0ptJant6EC2tH2OCy/a6jGUJ3Z4Q=</t>
+          <t>Kh9kVCsia6IOV5YuUELZ6n1COo6uwBtzVoP3IQIMV0A=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>9ROY8D+nYw90vd334DqvnQ==</t>
+          <t>JgigoJ/3+2wMLHRNJrboDA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Y0BbvRzUBGv0C8DmRWPcHTydqSLWzyIt0dsByP6Jqro=</t>
+          <t>IXTPMrZHjViJ7gGsvFLUyGOXW4Hok+TszLM4LWQApIU=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>U9SjFo8pTRZmL2ono2ahlg==</t>
+          <t>aFigR0OMgxNyXwHpLkI5OA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>9J0Id+0czq9B1QejT0Tr+jDhkEpivvMOHUx7iwYLb/M=</t>
+          <t>eo1ujLkdfBP/MBwX6Ss3wXc6/c2kI95cVdYqeSGDsiI=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>bQYkFp31MUAmx0vdx00wJg==</t>
+          <t>v7x4P3cbIVb4QTjQCuarxA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Iop3jKJHlq5DFa8TXvv9K28hKaMAaBjkyt6jv4HuExA=</t>
+          <t>lRCHG1BdAI4XzL+g0UjadFRibDVhbsIknpJhVI1TCWM=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OI8kZ+e+MJKJgChW85Ym5w==</t>
+          <t>7RuOp2Fa1ZnzebetVkpnhw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>B8SW96Ci7lBvORsPPvvavN3syMffc2uKwEoCj1m2ro4=</t>
+          <t>Hd46Grpj52i8wGMTvqvfGZmlnOt1LaEFlOqnIsn/A2A=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OejCY35ywaaAHgKIxVttXQ==</t>
+          <t>DG8d+RQ81217Euc8XE83eA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>xxHjbfFV1Yl78kfVTnCVWLKSFyS5VbDgzqEixM1QlCg=</t>
+          <t>KUVsNndhl1j5zq4tM9ry+GaAFssn7u5c8Q6zr8xbIH4=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ipd3Hi+NwUD40C0Ziedgfg==</t>
+          <t>zJz6U8/nGL2PyQQWtKBtxg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>uGyHGAzNTA2GNRn5oJ51DFNJNgmkfiNoK6hAz4o0k5A=</t>
+          <t>nv+yehRIqSh4ECeieh2FtUNWo/X6qOH6imFTpxPfYMc=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ijyPHvfsx6Mqll/wwrGa8w==</t>
+          <t>yGCvfQ1qEtN+dDsH83BoUw==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>kfoGqNg17vVkkpV58ksE3UiwMRn5ZqcyTuIsG7YWnd8=</t>
+          <t>KnqUJch7TEgOOH6BYARyeO9L/uqdneLRkepiSf7nISU=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TDkyT4Dumz2UyO0GB2ygyQ==</t>
+          <t>1OxvuslmEAfncDFkTRacNQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Z7aQKVXa1DCZpWnHIe5zzGhLWBzmQHapCn1908M/XrA=</t>
+          <t>fxYh8ax5rBCIBwg+hJE8dbrNl/aRZlTL9VE9n7lTuB8=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-12 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="91">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="116">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="127">
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131">
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
@@ -9326,7 +9326,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -9370,7 +9370,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="72">
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="99">
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="107">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="147">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>296</v>
+        <v>289</v>
       </c>
     </row>
     <row r="150">
@@ -13670,7 +13670,7 @@
         </is>
       </c>
       <c r="L158" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="159">
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="173">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="181">
@@ -17090,7 +17090,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="223">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ad7lnplyepsaF1fOMTi1WA==</t>
+          <t>dVhgRv21hk+SqzREMZbliA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>d4H3WmlQQBWvUyLz8mtZMwgq5ZUgMRRnf2cPgzkNhXo=</t>
+          <t>QgdX2yppodSzUWemIn6Mo3WMPctAg1sbGKfJzNHHjFc=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>zJdlpseCwTQJoWg2erbaVQ==</t>
+          <t>pXoRS6IZ5EuCYqorjxPMGA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2Xu4O6eEcq7tVyuMHVMzFacuCabbFa8HXNbfM/M9NB0=</t>
+          <t>1NZxrUPMBZNWnQykzsLc3AxkvzlH+AllGBHX/ICGKH0=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ESvkbA8lsLHz/FzH4U+ySA==</t>
+          <t>1vB4XgzhLK8YbuchJ5p1qA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>P/98Pepg24hSjEKqp4k9p0HNh6+yDzDT2yFOzMlAo7M=</t>
+          <t>v+HapH9TbnMwEPJdpck6wt8+d65u5nhZigprCw9hX1c=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>P8B7CJsVcAECKgLsSYEDew==</t>
+          <t>QM1I+x0NFKV1qsdVw0cxMg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>9dBmVHVgLeXuzSdz/nUeRIOvo6fL2n+IXTUcjCsWwhE=</t>
+          <t>/O4r0nfQkopfK1HO/O3KM5lam15dVSyyfE7Ok7tBEsw=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>wV2eeruMjjTa5eUbFHTq/A==</t>
+          <t>XvgcC1hJFEByrqF1o/oJQA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>72pIUaY+SZp/czflvniktlhk/L07+jGXhpcSUEL0NK8=</t>
+          <t>8+AummikhmciNOdNE2kGT47qd8xJt7KZh54V/zMLzR8=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>zGPtuEPLJocpYALVYZRszQ==</t>
+          <t>JPrqw8hphWl0+V+55cyziA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>lKxWHthGbqTlEmTU1kQxZPGeWJ7KB0coHwUrVOJv7as=</t>
+          <t>NZphUl7v7oW6IlC5XQGEeM/kD+o3BIZNCoQi3kSuy9Y=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>9qWnUagG9xtp7vFAFDemgA==</t>
+          <t>dKelBD5Vg7EtB01jdOk4fg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>45Frj6m0VUfWX0eFsSrOuc/o1JvpHQ9LAREFemNgVMI=</t>
+          <t>XnHSPY2DctffTgzYO6qGyg/rgNvDxGp/+hCpdxqrsNA=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>eHYS6CODv+swlrTGmMV45g==</t>
+          <t>4VIw8A2qaVmNOQC8s/6lKg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9507sbocjIXCadupNFDDPJpf2iML6JOshTG64u4HERM=</t>
+          <t>16jYyZ7GLRx7G9AonNyXe9npFoI9NLz7a4lKFXCnA2E=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>K+gNSnpSoIrHg9nza4XDmQ==;5EzNx3FhE9YPAPAhvRgvcg==</t>
+          <t>ZUNmaTWFN7QYyhSljBOXXw==;rjMV56jfz6Q3kBYaMU4Utg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>FzBA0IM3ZyXeCS+xkPuy4NTPM7B5FtZJ0LRMwQb3dUA=;YRDGLNVuwk2Pvbb7ZPRNXHJdFIkDfiM7Y5l1jWPghes=</t>
+          <t>SGwH40jtlNsaj1lC7uRyX104EvbTqy5YATJbt0DagNU=;PfEEavhzBbSdqJzWipJO/TjJnzGun6fZCuRm8dJE41w=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>E4lz3C9ByhXqtQEpRjnS0Q==</t>
+          <t>ntMmPnkRPuDU5LYVAVJKUw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Kkj59FSg2FZlwxBDFS/SR7nAWu8WEZpmY2IlGLKTGbA=</t>
+          <t>FN2sPS0Zs2Un5WzCa3T8VJ3kdApSKoCzw+R1wwgYZd4=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4c8lF5wKiTo31VN6q9Ieaw==</t>
+          <t>BRgRTqKOLGB13nLDRLSJ6g==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>92vaKkWOrkdv3l/dz3uHXjJwCe1XwHi+vvtaGpe+TgM=</t>
+          <t>oLAuggDTI/JdTtKJ97SWRclk1/MegjOoKU1Ibb1HgX4=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NtfzraYjncEo+hx/8kwTSg==</t>
+          <t>+UOZVxcuK2GzQovyQ5nRUg==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>guRNpNYO7QoRCs1O1OFy2WdAXLqC/USS3StFk5LFif8=</t>
+          <t>ohxKkfsW1dRfqsiBufuQgEc+vWmUZo1VoAz1D0Ml1YQ=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>VyOdrRfqU67IHxE+Yghr5Q==</t>
+          <t>xQjrTglXIXq4SEku3OwXng==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RHszodaRhNDEkbcxhe6cnU/x3t9aQQ5IQ+y9ERrDSB4=</t>
+          <t>d+YCjP91lrHIS8OoxfCesZ8Xd32FNPIfGSvTmLIdzkc=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>yPKKDXBjyRROouyNXzT2ww==</t>
+          <t>Xh0Hm2Q00emVz0EutOvt5Q==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>rE9lFUDuVeSjfrBzsoiWYUBzRWedp/wcsV+7tgL+0kk=</t>
+          <t>yyayYAEFgJ2RmbyRv4OlhsIcm15hbdH6JDD2nhzj9sA=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>xO2HW8PPqgfj1qGw1m7XAg==</t>
+          <t>KtPAmQfii+ETfrfr+QkwXA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>nnjxevFWU2nN2iw1effagnLCSVzNFuFUEz5+AECXlkU=</t>
+          <t>7OflSsNtOvrmsmCvUIns7AZ2GmkcFWUCM4y0vJRa2cg=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Rw6MiQQ3WIvy31CXxOTR7Q==</t>
+          <t>n6Udszljm+aSUiPnv8F2kg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>vXBG8IZSV6tpmVvRyQAjBaeGJVKo5wIi4ZROotSDyfI=</t>
+          <t>CxriFYrJdiD/nn+jZBMGRSV6R5Hv5K5y1y0Ut3Tu0fI=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>7ZvLEt0cHZz+ZAj0S8wAzw==</t>
+          <t>cKkBU4abhTXo5IyQboyhIw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>EKNwoZBgP5jwAbxHn+OhR0S32+swjVPZtZQ69xbdOfI=</t>
+          <t>tNLXqgDpUDmsYM9ZDAYhWvsNUrM02oubxmr3iY//kMk=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Msi+n+Bb2ny8CFOwLsM9Qw==</t>
+          <t>5zcr9zvBZr3GZP2iudt8yQ==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6zefmq9TbxQ/Im3K5ISXNpZ5F8Zq/5tIWTLzymZKco8=</t>
+          <t>ui6u71NshMvL75uat647FtPLPQpIgv18kz1igwci9mE=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ycGADJ5eT7NiFmx19QIc5A==</t>
+          <t>obq1fbBridXdzbcNXEBtwA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>mcAAsJYN6A62KA/7h2nJcydRGNlIG+A8PECJ6wSk/bo=</t>
+          <t>cVdKivWAVEweafnRo1gjTT/cugGy7Aflf4FVp9dyFCM=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>aWZF6Vfo9YmJdgRRNmYdSA==</t>
+          <t>h7H2wcUBJnFYeL1zWyFnOQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BD8WbpEcrvQHPDzXDTuRG4IWJ7a9h6m3K27HCR0QeCM=</t>
+          <t>ucFdLJ27mM/jTQZ4HBnnZhZQ++UeIrCEZ0j8noqndZg=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bzpxjf7ZHmxHRBA0dg4odA==</t>
+          <t>b2rhZV3c2133V8wu8LIqLg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>7GQAFhXkKzcqOSXZ7aIPRBVldLHSRMA2MK9qLywNK74=</t>
+          <t>MbUoisuwfzrb/B9xoBk5zAokucX0vIOFn48LFCq+hBY=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RQP5DLgZDXYcDNUOnxu9gQ==</t>
+          <t>URQYvgEzVKLhwvjudGjtYQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>nWfOKiO9u6QQLy/oGt8h439GwdBuRaVQWDN5LvYWUBU=</t>
+          <t>SbX8a+BCBq61ED0KAv+qVwqgirRZ1yyzCXjwB65V/cY=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>QH9GB25GHf5QH+uuKTXmFQ==</t>
+          <t>K8mWik/ogMgKr/4mu+B+fQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ma6SxsbjxnCeKylRiN/J/8SC8Qyp6HCzs4nC0POP+7Q=</t>
+          <t>5SsOPYyBK5SNPHWGfCh23hbDVM74Mkk36Q5XY2ARAZU=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kq+tcIi9rNWnsQGc9KovbA==</t>
+          <t>Z02b6IxyoTo/JpQBq6lu8Q==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C6A8WiuOmG0PGpKYvTBsGrAM0PLnUBV8TIUKiHqZjso=</t>
+          <t>F0xqSfVTk5RjVI1o+DNC/hNnhSIcoTrmw9c2Yo97GDY=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>JylKRzicmrf5YHnawa509A==</t>
+          <t>Bweii/gA9gI12kIMQfM+OA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>p2E2NTPehUOEsO1yffGCwISwasJPvsPc0hsP4BIwNF8=</t>
+          <t>Vaid9lnMaVKs94td8X4mZxIdy898Vuc5bgV9kit6jVM=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CZqczhkddjxj6EsaJ/jR8A==</t>
+          <t>09mYoR8ipEJDd7/W3Z3iSA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>kHr2pn+E7TNjtvGFh8mXIzfxjLlAQ1ooNQPV1JKcDI0=</t>
+          <t>sykaiapT+iozbkY3Ro9QdlME6g/Q7tNMnNIvvL2T8gs=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>pAHJuMaz6V0QkyMEkp1jHg==</t>
+          <t>3KuXjqXb5QiB2ilmb+Unkw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>MiDG2DUazDewAmjutkdst9aFhQgBMON9/+zqaizDgHs=</t>
+          <t>3l6UIA5nlBYOSkPOQqB3RTweldghUSO3u4Cyf6hNYeQ=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PdSkQ9eyjTEUFxyNyk5A9g==</t>
+          <t>xjLjq0qVGyYTkCHpv4y8UQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>i9+rF8R5qoq7zQEL5RA7mFRe3rydFNhqFMvCZTAosBk=</t>
+          <t>ImZKXH0NcdSW1D91r08fCLrYlt+1Zi7CppxcU2uUaL4=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OwfAno+r085azZ12NJHXVA==</t>
+          <t>HwvIGJdqAajt+FRyaApBsQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Kh9kVCsia6IOV5YuUELZ6n1COo6uwBtzVoP3IQIMV0A=</t>
+          <t>leZzMLQSQRXg2jdQxzrr35R34cgRB7DnhRI+mXLIoac=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>JgigoJ/3+2wMLHRNJrboDA==</t>
+          <t>hZM//x815rIJ1/ApxNdxQA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>IXTPMrZHjViJ7gGsvFLUyGOXW4Hok+TszLM4LWQApIU=</t>
+          <t>hAhLtwT4p18+7mlEn2Gg9kXoljwu1b7+73lnbFicK94=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>aFigR0OMgxNyXwHpLkI5OA==</t>
+          <t>CiGTe6O5zNnkiLeYLPN1sg==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>eo1ujLkdfBP/MBwX6Ss3wXc6/c2kI95cVdYqeSGDsiI=</t>
+          <t>BnqKKs240T38ujGH3HmES6bw0L17JuFfkBJR450GpPY=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>v7x4P3cbIVb4QTjQCuarxA==</t>
+          <t>evUZFWDGyq01IPfHGmTVKw==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>lRCHG1BdAI4XzL+g0UjadFRibDVhbsIknpJhVI1TCWM=</t>
+          <t>U7qoT8sY2mHKs8XtudzWcUf7EkLIfR9Xuoak2fAZons=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>7RuOp2Fa1ZnzebetVkpnhw==</t>
+          <t>eQd1QzRi5NANJOZtS8GOmQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Hd46Grpj52i8wGMTvqvfGZmlnOt1LaEFlOqnIsn/A2A=</t>
+          <t>EKv8eZKV5lwLI7RV4+/2YPav3ihYSZU8NK/cH8WdWG0=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>DG8d+RQ81217Euc8XE83eA==</t>
+          <t>7A6bna+JcYZzzCpXjTCBzQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>KUVsNndhl1j5zq4tM9ry+GaAFssn7u5c8Q6zr8xbIH4=</t>
+          <t>BdTFQOmZSFWZHzSnmcwQ87tSBws9gF5zWqEiNEHPonc=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>zJz6U8/nGL2PyQQWtKBtxg==</t>
+          <t>qe/IjJ5C9kjudlSLj7pmDg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>nv+yehRIqSh4ECeieh2FtUNWo/X6qOH6imFTpxPfYMc=</t>
+          <t>RNzQsDPP3/gvuHLA2LFKFDxh0PBKOyTDXDW9A/ezmL8=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>yGCvfQ1qEtN+dDsH83BoUw==</t>
+          <t>CF5DMVEIniaFGAAaaZ1uBg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>KnqUJch7TEgOOH6BYARyeO9L/uqdneLRkepiSf7nISU=</t>
+          <t>laM6XCdg4liRkZ5bxcF/g4YF7EjHxxFHHjuZ0mjNaig=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1OxvuslmEAfncDFkTRacNQ==</t>
+          <t>mAnMPfxbBsfoLjRFphQmlw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>fxYh8ax5rBCIBwg+hJE8dbrNl/aRZlTL9VE9n7lTuB8=</t>
+          <t>ZvjE8k1jSnpGyRkmpPHCHbV5wBHO9vKjJRlaNeNfmzY=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-13 07:38) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="91">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="116">
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="107">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>289</v>
+        <v>263</v>
       </c>
     </row>
     <row r="150">
@@ -14330,7 +14330,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="171">
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="181">
@@ -17220,12 +17220,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>dVhgRv21hk+SqzREMZbliA==</t>
+          <t>ir0qB78gdEqBC2JQAXDngw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>QgdX2yppodSzUWemIn6Mo3WMPctAg1sbGKfJzNHHjFc=</t>
+          <t>bAZET2ptha+cpfX9CeHbYSjO6b5QFINShHImEmwikhs=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17252,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>pXoRS6IZ5EuCYqorjxPMGA==</t>
+          <t>dz64YCUFNNdPGFRmdRFzrQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1NZxrUPMBZNWnQykzsLc3AxkvzlH+AllGBHX/ICGKH0=</t>
+          <t>rI0R65tL3hKrBQJXud2B1bs5EPnax+5pmMuOyVsEWbw=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17284,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1vB4XgzhLK8YbuchJ5p1qA==</t>
+          <t>7DJQ0D2wjx/U8RcGR95txw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>v+HapH9TbnMwEPJdpck6wt8+d65u5nhZigprCw9hX1c=</t>
+          <t>RbhMyUwAHkRZ4A3at5qFXxABH9p2wWGogbyApXH6sUE=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17311,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>QM1I+x0NFKV1qsdVw0cxMg==</t>
+          <t>9Wc3zGA2XUoqdQU49UHzuw==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>/O4r0nfQkopfK1HO/O3KM5lam15dVSyyfE7Ok7tBEsw=</t>
+          <t>Iw36PTZfLcYcDFaVaiEcdgnhsHW5+UXv8U6lavOWJ9E=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>XvgcC1hJFEByrqF1o/oJQA==</t>
+          <t>67EkhcmTkGw/KUGu4vJisw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>8+AummikhmciNOdNE2kGT47qd8xJt7KZh54V/zMLzR8=</t>
+          <t>1WqCpMgoLgx56y8L4ieiqQZcexXxfJk0M+tn09vJTDQ=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17375,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>JPrqw8hphWl0+V+55cyziA==</t>
+          <t>kxvyIbQ9FAMuZHSmukQs3w==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>NZphUl7v7oW6IlC5XQGEeM/kD+o3BIZNCoQi3kSuy9Y=</t>
+          <t>3tJ/IsuAkAbm3WKtjuXEYqFp8i8/0NiuglAsVFEB0TE=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17407,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>dKelBD5Vg7EtB01jdOk4fg==</t>
+          <t>Cbtj4vkwtpRo51s7a5mCKg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>XnHSPY2DctffTgzYO6qGyg/rgNvDxGp/+hCpdxqrsNA=</t>
+          <t>rbE6VSMQqmFjMjoDiAQLoqiMiPWkDTn0KiYwzAPek1g=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17434,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4VIw8A2qaVmNOQC8s/6lKg==</t>
+          <t>wOBrppSZRrQRx17FTmFnAg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16jYyZ7GLRx7G9AonNyXe9npFoI9NLz7a4lKFXCnA2E=</t>
+          <t>oqXcB0pt7uSw3xT0AVKoxokTY84WhnVdK9gfiS4YHl0=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17466,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ZUNmaTWFN7QYyhSljBOXXw==;rjMV56jfz6Q3kBYaMU4Utg==</t>
+          <t>4s365Qc8W57Sf30LvX2hUQ==;9RjWFbi02Mg1I/QN0FeVLg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SGwH40jtlNsaj1lC7uRyX104EvbTqy5YATJbt0DagNU=;PfEEavhzBbSdqJzWipJO/TjJnzGun6fZCuRm8dJE41w=</t>
+          <t>MnB3ABsh+GVjXWtwuDR3ZM2pxvNV/SIirAJurjKDOp4=;0haysLHocZX0ly0ijFwCsHrC/+7hBw27w9duNhS/xHE=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ntMmPnkRPuDU5LYVAVJKUw==</t>
+          <t>sMAupca+v787jS+NTeXdoA==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>FN2sPS0Zs2Un5WzCa3T8VJ3kdApSKoCzw+R1wwgYZd4=</t>
+          <t>FVxIHVwNZmJlSxeZ/BISovR27jsrjorRBXeS0M3Jb9Y=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17530,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BRgRTqKOLGB13nLDRLSJ6g==</t>
+          <t>SclH8u2gWM9WbeLK19hA4w==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>oLAuggDTI/JdTtKJ97SWRclk1/MegjOoKU1Ibb1HgX4=</t>
+          <t>o+mXhm7urXDU2fr5b4xqUMhI23qGi4LXuTMxXIaCe+Q=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17562,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+UOZVxcuK2GzQovyQ5nRUg==</t>
+          <t>L0G7fpQdl+zc9JQf9LZ38w==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ohxKkfsW1dRfqsiBufuQgEc+vWmUZo1VoAz1D0Ml1YQ=</t>
+          <t>PXobr6zy8M00yiQOp+IGXKKxcTW0KTs9Vdskz1jx25c=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17594,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xQjrTglXIXq4SEku3OwXng==</t>
+          <t>+I5q+tidIq0WfVTpStfVyA==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d+YCjP91lrHIS8OoxfCesZ8Xd32FNPIfGSvTmLIdzkc=</t>
+          <t>/f6G9ycyJtITmoeIK8N7nxZMGEy3CoyoHIqyMsNc6/c=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17626,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Xh0Hm2Q00emVz0EutOvt5Q==</t>
+          <t>/nBK4MdWD14OCBS1L185Lw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>yyayYAEFgJ2RmbyRv4OlhsIcm15hbdH6JDD2nhzj9sA=</t>
+          <t>3iOSBY4zVCTT6cqCq7BW2Ni6lDpqK+SKwwr0RfNfxZE=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>KtPAmQfii+ETfrfr+QkwXA==</t>
+          <t>/w4b5TUGXyM73/cTpi1zZg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>7OflSsNtOvrmsmCvUIns7AZ2GmkcFWUCM4y0vJRa2cg=</t>
+          <t>ulMTCGx8PhbRh1uIFaTvLrIqMKTnHuvr3PX1iwSHWhw=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>n6Udszljm+aSUiPnv8F2kg==</t>
+          <t>cMBDNzUUr339lwWKDRx5Zg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CxriFYrJdiD/nn+jZBMGRSV6R5Hv5K5y1y0Ut3Tu0fI=</t>
+          <t>AS383zvX/ehyTM0EWUusz9Ljw4iQkJvBvKhKFGoi/Z8=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17722,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>cKkBU4abhTXo5IyQboyhIw==</t>
+          <t>vsQfJIe8HGHGFFmOAcw32A==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>tNLXqgDpUDmsYM9ZDAYhWvsNUrM02oubxmr3iY//kMk=</t>
+          <t>TV23cz9BtV2E6yQ294y41C3FHMdLOJQa16wBptuj16o=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17754,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5zcr9zvBZr3GZP2iudt8yQ==</t>
+          <t>8WiROceVwzoIyPP7woEa/A==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ui6u71NshMvL75uat647FtPLPQpIgv18kz1igwci9mE=</t>
+          <t>XAHKJdGM1DpdbN3qZkPKmjfrE7bjXcWMEw8tEM3wzsA=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17786,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>obq1fbBridXdzbcNXEBtwA==</t>
+          <t>ERRzvFqC//IRx3Wjfy8YbQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>cVdKivWAVEweafnRo1gjTT/cugGy7Aflf4FVp9dyFCM=</t>
+          <t>t2mnaHVAdug23wk5vgT79FSYj0V3AgWC0eZO1+w4o4E=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17818,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>h7H2wcUBJnFYeL1zWyFnOQ==</t>
+          <t>M0I1GwterysKHEAvWexmZQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ucFdLJ27mM/jTQZ4HBnnZhZQ++UeIrCEZ0j8noqndZg=</t>
+          <t>CO4LSHDrmYbPYHm/qHk5Al0u+cVk95grZ+y6j6RkX2U=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17850,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>b2rhZV3c2133V8wu8LIqLg==</t>
+          <t>2DEHWTDwK7H5djHup/xbEQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>MbUoisuwfzrb/B9xoBk5zAokucX0vIOFn48LFCq+hBY=</t>
+          <t>hjmpkLnMiR7FA13O39cl9bhlLR1qoRLe7UBJ/SMFKX4=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +17882,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>URQYvgEzVKLhwvjudGjtYQ==</t>
+          <t>tHgxCj8c6IRG0GdREgg/8g==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SbX8a+BCBq61ED0KAv+qVwqgirRZ1yyzCXjwB65V/cY=</t>
+          <t>txKXvibFVCVcJOR/+LwHwbEU96j+AX0DwS9CN0DFC3w=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17914,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>K8mWik/ogMgKr/4mu+B+fQ==</t>
+          <t>q/DHf7LvoqMSFnqF0jLl0A==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>5SsOPYyBK5SNPHWGfCh23hbDVM74Mkk36Q5XY2ARAZU=</t>
+          <t>hZ1mlB28cVuWfgjEI4Vihk7CFnTHbKYkJoR49bLL4Q4=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +17946,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Z02b6IxyoTo/JpQBq6lu8Q==</t>
+          <t>w/3u/kmIimlgjiuhFgxbSw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>F0xqSfVTk5RjVI1o+DNC/hNnhSIcoTrmw9c2Yo97GDY=</t>
+          <t>LVja/2N6qYlM8qpKufShx24Q3LzY4CqkeHLO8fVzDxQ=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +17978,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bweii/gA9gI12kIMQfM+OA==</t>
+          <t>sNA8GJIdbkAk9qk7HyJMkA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Vaid9lnMaVKs94td8X4mZxIdy898Vuc5bgV9kit6jVM=</t>
+          <t>NsA5ie/u88u5FiQCOcwjeXICM6K66fkgXMpV+CLewtQ=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18010,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>09mYoR8ipEJDd7/W3Z3iSA==</t>
+          <t>3ZIAUPHo8mvXkvmwqanbgg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>sykaiapT+iozbkY3Ro9QdlME6g/Q7tNMnNIvvL2T8gs=</t>
+          <t>F1WEQshuJaNp03QYdaXIZ9NqjGz9poE4N7Hl3sB3fow=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18042,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3KuXjqXb5QiB2ilmb+Unkw==</t>
+          <t>SN8A3lGn7AnOxPUgPzusSA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3l6UIA5nlBYOSkPOQqB3RTweldghUSO3u4Cyf6hNYeQ=</t>
+          <t>1cO6o7dtV1MVMNtZsruoHzWrfYMDGGYXsD74CgudcN4=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18074,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>xjLjq0qVGyYTkCHpv4y8UQ==</t>
+          <t>19sGreEj1jgxBxUpLzT4hQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ImZKXH0NcdSW1D91r08fCLrYlt+1Zi7CppxcU2uUaL4=</t>
+          <t>s2BVbmFBrolz5aA1suIzCwakLJCAw06lk04CzuFC+7g=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18106,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HwvIGJdqAajt+FRyaApBsQ==</t>
+          <t>g8PPkyMVrRAjZqWCrVk9Eg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>leZzMLQSQRXg2jdQxzrr35R34cgRB7DnhRI+mXLIoac=</t>
+          <t>6wVtvJpJ8nDO7j7fRZ3YwKTHj8pJi6LdS1evg+1JZ4k=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18138,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>hZM//x815rIJ1/ApxNdxQA==</t>
+          <t>+lDt4oGuonMQWrHvKwWtKQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>hAhLtwT4p18+7mlEn2Gg9kXoljwu1b7+73lnbFicK94=</t>
+          <t>ZGR7ipINNo2r14spLF96PRt8iHb48Wdy5V8CzmFAr8E=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18170,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CiGTe6O5zNnkiLeYLPN1sg==</t>
+          <t>+loD/RCuuuqr1C3xx8q8ZA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>BnqKKs240T38ujGH3HmES6bw0L17JuFfkBJR450GpPY=</t>
+          <t>Dzlw3KN3VsPP9404oD8qOSRDqR//ZWBlRs2irWmidaw=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18202,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>evUZFWDGyq01IPfHGmTVKw==</t>
+          <t>BO6VyBfAAPIK+cwC7jNZDg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>U7qoT8sY2mHKs8XtudzWcUf7EkLIfR9Xuoak2fAZons=</t>
+          <t>KUPu/oxA04Er3IBFMSKUwg56Pli3ySqJLsJHtKRH2x0=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18234,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>eQd1QzRi5NANJOZtS8GOmQ==</t>
+          <t>Qnq7HTq9/njspFtpBH8LWg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>EKv8eZKV5lwLI7RV4+/2YPav3ihYSZU8NK/cH8WdWG0=</t>
+          <t>cVdLIf0HHRl6jXSjeUn8EgsUE6eYc/R1EjXly8jDU44=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18266,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>7A6bna+JcYZzzCpXjTCBzQ==</t>
+          <t>/WtD7CLqFDKRz8BOWsFiCA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BdTFQOmZSFWZHzSnmcwQ87tSBws9gF5zWqEiNEHPonc=</t>
+          <t>U9f+lBV3YGKQ2BTeEON+YaZX7CdEevoBayK/n5lYzwU=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18298,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>qe/IjJ5C9kjudlSLj7pmDg==</t>
+          <t>ixoZluk5eDAfU04qPNc3EA==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>RNzQsDPP3/gvuHLA2LFKFDxh0PBKOyTDXDW9A/ezmL8=</t>
+          <t>2pX3FB2kYu9h98a+PVPQrlGh5GOc84MZqXzS1AiRVds=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18330,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CF5DMVEIniaFGAAaaZ1uBg==</t>
+          <t>daH0o3Nf0ov1+jMXa3/9jA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>laM6XCdg4liRkZ5bxcF/g4YF7EjHxxFHHjuZ0mjNaig=</t>
+          <t>b6M9aQdCwfulKXn98F4nvN9wJYE0mQe20EqJgsd/76g=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18362,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mAnMPfxbBsfoLjRFphQmlw==</t>
+          <t>Zj4dxeewddaUWqxUP71ltA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ZvjE8k1jSnpGyRkmpPHCHbV5wBHO9vKjJRlaNeNfmzY=</t>
+          <t>xp7Vy1zhTYeI6aiDwYklP3i+aPMo1a0a+TfT65qzVwY=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-14 07:38) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$147</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$223</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$225</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H147"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49">
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2799,12 +2799,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="81">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="90">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91">
@@ -3787,12 +3787,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cddfdfd9-8261-4403-9f7d-ede767a414ea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="95">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>363</v>
+        <v>378</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>363</v>
+        <v>378</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="117">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="119">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="120">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="121">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="123">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="126">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5427,7 +5427,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5623,12 +5623,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5659,12 +5659,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5695,12 +5695,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=17a76e1b-4a1d-4f00-88ee-66022635680c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5762,17 +5762,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5790,8 +5790,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>MENOR COSTE</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>INFORME</t>
+        </is>
+      </c>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H147"/>
+  <autoFilter ref="A1:H148"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5802,7 +5838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L223"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5966,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
@@ -6274,7 +6310,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -6406,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14">
@@ -6494,7 +6530,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16">
@@ -6582,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -7710,7 +7746,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -8018,7 +8054,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -9014,7 +9050,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -9326,7 +9362,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
@@ -10702,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="97">
@@ -10746,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="98">
@@ -10974,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="103">
@@ -11062,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="105">
@@ -11106,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="106">
@@ -11150,7 +11186,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="107">
@@ -11238,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="109">
@@ -11282,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="110">
@@ -12070,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="132">
@@ -12466,7 +12502,7 @@
         </is>
       </c>
       <c r="L135" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="136">
@@ -13182,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="149">
@@ -13238,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>263</v>
+        <v>237</v>
       </c>
     </row>
     <row r="150">
@@ -13406,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="156">
@@ -14442,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="173">
@@ -14698,7 +14734,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="178">
@@ -14830,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="181">
@@ -15178,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="188">
@@ -16039,30 +16075,26 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
+          <t>SEGUIMIENTO DE MARCAS</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 26</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr"/>
       <c r="J203" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16070,11 +16102,11 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>17a76e1b-4a1d-4f00-88ee-66022635680c</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204">
@@ -16095,7 +16127,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16106,17 +16138,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16126,11 +16158,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="205">
@@ -16151,7 +16183,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16162,17 +16194,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16182,11 +16214,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206">
@@ -16207,7 +16239,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16218,17 +16250,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16238,11 +16270,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
@@ -16263,7 +16295,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
@@ -16274,17 +16306,17 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16294,7 +16326,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L207" t="n">
@@ -16319,7 +16351,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -16330,17 +16362,17 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -16350,7 +16382,7 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L208" t="n">
@@ -16375,7 +16407,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16386,17 +16418,17 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -16406,7 +16438,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L209" t="n">
@@ -16431,7 +16463,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16442,17 +16474,17 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -16462,7 +16494,7 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L210" t="n">
@@ -16487,7 +16519,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16498,17 +16530,17 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -16518,7 +16550,7 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L211" t="n">
@@ -16543,7 +16575,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16554,17 +16586,17 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -16574,11 +16606,11 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213">
@@ -16599,7 +16631,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16610,17 +16642,17 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -16630,11 +16662,11 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="214">
@@ -16655,7 +16687,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E214" t="inlineStr"/>
@@ -16666,17 +16698,17 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -16686,11 +16718,11 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L214" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215">
@@ -16711,7 +16743,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -16722,17 +16754,17 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -16742,11 +16774,11 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L215" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="216">
@@ -16767,7 +16799,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -16778,17 +16810,17 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -16798,11 +16830,11 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L216" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="217">
@@ -16823,7 +16855,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -16834,17 +16866,17 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -16854,11 +16886,11 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L217" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="218">
@@ -16879,7 +16911,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -16890,17 +16922,17 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Octubre - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -16910,11 +16942,11 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>1ddf1ffb-0655-4b37-96ee-4ee69ebd5764</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="219">
@@ -16935,18 +16967,30 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 26</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Octubre - 26</t>
+        </is>
+      </c>
       <c r="J219" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16954,7 +16998,7 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>1ddf1ffb-0655-4b37-96ee-4ee69ebd5764</t>
         </is>
       </c>
       <c r="L219" t="n">
@@ -16979,7 +17023,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -16987,7 +17031,7 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>Sin cargo CFH</t>
         </is>
       </c>
       <c r="I220" t="inlineStr"/>
@@ -16998,11 +17042,11 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>46395ec1-f0ac-4b34-9a0c-40fe1322db9f</t>
         </is>
       </c>
       <c r="L220" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
@@ -17023,7 +17067,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -17031,7 +17075,7 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I221" t="inlineStr"/>
@@ -17042,11 +17086,11 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L221" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222">
@@ -17067,7 +17111,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -17075,7 +17119,7 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I222" t="inlineStr"/>
@@ -17086,11 +17130,11 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L222" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
     </row>
     <row r="223">
@@ -17111,7 +17155,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -17119,7 +17163,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -17130,17 +17174,105 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+        </is>
+      </c>
+      <c r="L223" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>HERGO - DISTRIBUCION</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>VENTAS SMK</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>VENTAS SMK</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Grupo Hergo - Jefes</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+        </is>
+      </c>
+      <c r="L224" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>HERGO - DISTRIBUCION</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>VENTA MAYORISTA DETALLE</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Venta Mayorista Detalle</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Grupo Hergo - Jefes</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
           <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
-      <c r="L223" t="n">
-        <v>53</v>
+      <c r="L225" t="n">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L223"/>
+  <autoFilter ref="A1:L225"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17220,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ir0qB78gdEqBC2JQAXDngw==</t>
+          <t>MMfYRNognDKOPgmz4A4sGw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>bAZET2ptha+cpfX9CeHbYSjO6b5QFINShHImEmwikhs=</t>
+          <t>S5WawbTHTk1pdfOGDQqwWBYtFbhAgMwrT5uORBK5l/s=</t>
         </is>
       </c>
     </row>
@@ -17252,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>dz64YCUFNNdPGFRmdRFzrQ==</t>
+          <t>h4+fNSVJcbWN1G5YLSbc6A==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>rI0R65tL3hKrBQJXud2B1bs5EPnax+5pmMuOyVsEWbw=</t>
+          <t>lLcOqRsk+JFTD/7k+Le7xtz1Gd8ThJWIJZwyFzczcos=</t>
         </is>
       </c>
     </row>
@@ -17284,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7DJQ0D2wjx/U8RcGR95txw==</t>
+          <t>Jlr5LQDzjhRuQhsuLDKDOQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>RbhMyUwAHkRZ4A3at5qFXxABH9p2wWGogbyApXH6sUE=</t>
+          <t>Qx19SgKc0hNpHWGgKNPGZ0QPJ8yEgv63cLz/QbHqxYo=</t>
         </is>
       </c>
     </row>
@@ -17311,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9Wc3zGA2XUoqdQU49UHzuw==</t>
+          <t>2vtu/V/uAL1jP2ie74w8tg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Iw36PTZfLcYcDFaVaiEcdgnhsHW5+UXv8U6lavOWJ9E=</t>
+          <t>FeFd4lqLzhrU5fP0h1nAvI6xj4AZ+QInfsdICbqwS9M=</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>67EkhcmTkGw/KUGu4vJisw==</t>
+          <t>nlqiF4Nj/soXBDGS45IDqw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1WqCpMgoLgx56y8L4ieiqQZcexXxfJk0M+tn09vJTDQ=</t>
+          <t>PuZI2CGegVvHeJy6HsVrprrzxhY+EcpZV577diou+Uw=</t>
         </is>
       </c>
     </row>
@@ -17375,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>kxvyIbQ9FAMuZHSmukQs3w==</t>
+          <t>LTIzsrlkHBkvW0l8IovsBg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3tJ/IsuAkAbm3WKtjuXEYqFp8i8/0NiuglAsVFEB0TE=</t>
+          <t>j3tSlFphBsRCAXsv5yGyrMAuGyq75tmDneknyTUBwL0=</t>
         </is>
       </c>
     </row>
@@ -17407,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Cbtj4vkwtpRo51s7a5mCKg==</t>
+          <t>oUSpnp3ZSwpQjZ39ZVEsEw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>rbE6VSMQqmFjMjoDiAQLoqiMiPWkDTn0KiYwzAPek1g=</t>
+          <t>TIVs75s6A7jZJsAVZGp35/o1gFreTf9LjrVK7ehSqNI=</t>
         </is>
       </c>
     </row>
@@ -17434,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>wOBrppSZRrQRx17FTmFnAg==</t>
+          <t>xvNrBY2Ug6eyt6Y/vceshA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>oqXcB0pt7uSw3xT0AVKoxokTY84WhnVdK9gfiS4YHl0=</t>
+          <t>6OWUcOpVOq+PswTl3bBcinFfZHRgBBZeBCossbDdZU0=</t>
         </is>
       </c>
     </row>
@@ -17466,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4s365Qc8W57Sf30LvX2hUQ==;9RjWFbi02Mg1I/QN0FeVLg==</t>
+          <t>sh0SeQyllOSQVcTQ63ohWg==;lrosInhylvlbkJk412qgaQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MnB3ABsh+GVjXWtwuDR3ZM2pxvNV/SIirAJurjKDOp4=;0haysLHocZX0ly0ijFwCsHrC/+7hBw27w9duNhS/xHE=</t>
+          <t>TmyQRFR5JUMzk1mOlrEg+ijlo7hvaeMB1wnbzIvlX5Q=;yM/t4kb7YqF3FnKwPf0BNOAVZlRf/oMcJviVlinCuf8=</t>
         </is>
       </c>
     </row>
@@ -17498,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sMAupca+v787jS+NTeXdoA==</t>
+          <t>KNXyrzLhtxj+xH7rdaV4hw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>FVxIHVwNZmJlSxeZ/BISovR27jsrjorRBXeS0M3Jb9Y=</t>
+          <t>/AcsOluJfdyLOfpcOSBWkIHEdj3upLqTmCD8yDd1+UA=</t>
         </is>
       </c>
     </row>
@@ -17530,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SclH8u2gWM9WbeLK19hA4w==</t>
+          <t>0XN+1BB4ohyv5XZpU5n2Jg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>o+mXhm7urXDU2fr5b4xqUMhI23qGi4LXuTMxXIaCe+Q=</t>
+          <t>cK60LrdhFiWU3YwELQ4JgbtRI+LhLX1dsN0AR1h/9QQ=</t>
         </is>
       </c>
     </row>
@@ -17562,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L0G7fpQdl+zc9JQf9LZ38w==</t>
+          <t>VLre2aTVVQZyoSEluRknRA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PXobr6zy8M00yiQOp+IGXKKxcTW0KTs9Vdskz1jx25c=</t>
+          <t>FqraElTn7JiyEMjELx7gA9Npc9MdS3XSy2lMQGIsdN4=</t>
         </is>
       </c>
     </row>
@@ -17594,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+I5q+tidIq0WfVTpStfVyA==</t>
+          <t>adR1cTMKkZTrWk4wo1Pg7A==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>/f6G9ycyJtITmoeIK8N7nxZMGEy3CoyoHIqyMsNc6/c=</t>
+          <t>MX6atKYlR001rfvxJ4iOeb5yxgrtqPDp96KMBB7hoRw=</t>
         </is>
       </c>
     </row>
@@ -17626,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>/nBK4MdWD14OCBS1L185Lw==</t>
+          <t>V3LEIGag2dfBWzj+J8JKcg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3iOSBY4zVCTT6cqCq7BW2Ni6lDpqK+SKwwr0RfNfxZE=</t>
+          <t>SXjbTH0v3JUbnhjXXooeCIYXz0GLHUZXfAerDMpj4KQ=</t>
         </is>
       </c>
     </row>
@@ -17658,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>/w4b5TUGXyM73/cTpi1zZg==</t>
+          <t>/TBlpCCZdcR/AWp3O0gKyg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ulMTCGx8PhbRh1uIFaTvLrIqMKTnHuvr3PX1iwSHWhw=</t>
+          <t>LrDn9YRR8OBoZHgSCjZM3WDH/NlE4QZxg0dR/lBX8Ks=</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>cMBDNzUUr339lwWKDRx5Zg==</t>
+          <t>YyZ+Dc+9kX/AXgDnw/+wGw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AS383zvX/ehyTM0EWUusz9Ljw4iQkJvBvKhKFGoi/Z8=</t>
+          <t>FpzuvYwCZjl0mfNbXHeFq14HF2LZ3kGI3v4RafqhSms=</t>
         </is>
       </c>
     </row>
@@ -17722,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vsQfJIe8HGHGFFmOAcw32A==</t>
+          <t>iCjSNRdP+R+AjU3G6saHSA==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TV23cz9BtV2E6yQ294y41C3FHMdLOJQa16wBptuj16o=</t>
+          <t>u+uBed1cqCxlZdtKoOpdN+JK9i5QtUtFdJj5kzaM/tY=</t>
         </is>
       </c>
     </row>
@@ -17754,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>8WiROceVwzoIyPP7woEa/A==</t>
+          <t>B0imQp54K6qZ3yjXC+nOKA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>XAHKJdGM1DpdbN3qZkPKmjfrE7bjXcWMEw8tEM3wzsA=</t>
+          <t>MRFGUIXRE8tJJWnM3DtZTs6Kk/Bv6C3+yIGGVw/Btk4=</t>
         </is>
       </c>
     </row>
@@ -17786,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ERRzvFqC//IRx3Wjfy8YbQ==</t>
+          <t>VWfz3G1OlIHxVGyPaPEPOA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>t2mnaHVAdug23wk5vgT79FSYj0V3AgWC0eZO1+w4o4E=</t>
+          <t>Zw3c13fyZPXiv9AbC+sZoimBAgCH4o/Y+JGD4IFh0i4=</t>
         </is>
       </c>
     </row>
@@ -17818,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>M0I1GwterysKHEAvWexmZQ==</t>
+          <t>UEyyli7BZGuESMHvu21E1Q==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CO4LSHDrmYbPYHm/qHk5Al0u+cVk95grZ+y6j6RkX2U=</t>
+          <t>wXkGL72NUSJ9aNE1QYqGSfXgbbvUSDwPUW3IfkQDAGs=</t>
         </is>
       </c>
     </row>
@@ -17850,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2DEHWTDwK7H5djHup/xbEQ==</t>
+          <t>Qwu2+KZe1yALhnjWb5yVQg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>hjmpkLnMiR7FA13O39cl9bhlLR1qoRLe7UBJ/SMFKX4=</t>
+          <t>F1x4E8sJ3dvMSbW9ey9GrqJOkjFx2a6D9o9fBWABY8Q=</t>
         </is>
       </c>
     </row>
@@ -17882,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>tHgxCj8c6IRG0GdREgg/8g==</t>
+          <t>OKWNfeAzOaPJfnzKPfSh6A==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>txKXvibFVCVcJOR/+LwHwbEU96j+AX0DwS9CN0DFC3w=</t>
+          <t>ZIHoBFbPYxdH2fGpwLZmvzCjNeObO9ojFpfqlaUSypU=</t>
         </is>
       </c>
     </row>
@@ -17914,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>q/DHf7LvoqMSFnqF0jLl0A==</t>
+          <t>6+LJYI0CSD3OoOPdHdgsOQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>hZ1mlB28cVuWfgjEI4Vihk7CFnTHbKYkJoR49bLL4Q4=</t>
+          <t>PAp4BfBWW/8Ri1nkPj9eMOpPD2JX6Vy2DXWdLgssqM8=</t>
         </is>
       </c>
     </row>
@@ -17946,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>w/3u/kmIimlgjiuhFgxbSw==</t>
+          <t>jnHaX7zxG2plu6Rbn6X+Ew==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>LVja/2N6qYlM8qpKufShx24Q3LzY4CqkeHLO8fVzDxQ=</t>
+          <t>lHuB21zpUz7hAkj3be7JDo35S2uCo5P5ZW4VdJ51kZ4=</t>
         </is>
       </c>
     </row>
@@ -17978,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>sNA8GJIdbkAk9qk7HyJMkA==</t>
+          <t>AroTs5Q1x+Hd8XqmBYHXMA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NsA5ie/u88u5FiQCOcwjeXICM6K66fkgXMpV+CLewtQ=</t>
+          <t>s5EwSkD5AHw0Q0eZTdWQeH83Viev/cjwHOgv+LXD6gA=</t>
         </is>
       </c>
     </row>
@@ -18010,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3ZIAUPHo8mvXkvmwqanbgg==</t>
+          <t>o2yzpu1vqrHRC5o883VTAA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>F1WEQshuJaNp03QYdaXIZ9NqjGz9poE4N7Hl3sB3fow=</t>
+          <t>zPSTQUwOrsbVpuRuN7I/SFbS2N+WmneMdXRHFuN56Ic=</t>
         </is>
       </c>
     </row>
@@ -18042,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SN8A3lGn7AnOxPUgPzusSA==</t>
+          <t>hHzzWi9CC9EqB1Hl/0zhgw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1cO6o7dtV1MVMNtZsruoHzWrfYMDGGYXsD74CgudcN4=</t>
+          <t>pygI7iz3eMDn50e4Gggesff9Eb1ZWR/IpUaTVPpbXbw=</t>
         </is>
       </c>
     </row>
@@ -18074,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>19sGreEj1jgxBxUpLzT4hQ==</t>
+          <t>I6B+LA0IVkpFJeG8AOgKUA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>s2BVbmFBrolz5aA1suIzCwakLJCAw06lk04CzuFC+7g=</t>
+          <t>ED4oz28OBOm9+fEeXhMSR7cR+ctATYXxPspA1NJckGU=</t>
         </is>
       </c>
     </row>
@@ -18106,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>g8PPkyMVrRAjZqWCrVk9Eg==</t>
+          <t>jRy4CFlw5qOP8mn6xVUloA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>6wVtvJpJ8nDO7j7fRZ3YwKTHj8pJi6LdS1evg+1JZ4k=</t>
+          <t>91eIEpLXKGjHzv7pKXGZCUwcT3DWcmClL7QEP63TfSU=</t>
         </is>
       </c>
     </row>
@@ -18138,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>+lDt4oGuonMQWrHvKwWtKQ==</t>
+          <t>7aJ/iADkkRdAK8GGijZaPQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ZGR7ipINNo2r14spLF96PRt8iHb48Wdy5V8CzmFAr8E=</t>
+          <t>UTUCioLmYRvWrg3GN+qn+LT9rDpKv0C3A/BNOKyESBY=</t>
         </is>
       </c>
     </row>
@@ -18170,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>+loD/RCuuuqr1C3xx8q8ZA==</t>
+          <t>eF9eKCJFVz+aIsz/HOMSkQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Dzlw3KN3VsPP9404oD8qOSRDqR//ZWBlRs2irWmidaw=</t>
+          <t>lYf9Eo/MZHiYxxHA+8Ox4DNt03FOCQWoKoMJPI6pw5Q=</t>
         </is>
       </c>
     </row>
@@ -18202,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BO6VyBfAAPIK+cwC7jNZDg==</t>
+          <t>A5RXlILPINcgrH90XbjHeg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>KUPu/oxA04Er3IBFMSKUwg56Pli3ySqJLsJHtKRH2x0=</t>
+          <t>MjU6jcfGairn3aOdxb6N9ABFt1AiUGLbJSJ8Aq7GEh4=</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Qnq7HTq9/njspFtpBH8LWg==</t>
+          <t>Xuh73dwLLsoJQCU2EtRpXQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>cVdLIf0HHRl6jXSjeUn8EgsUE6eYc/R1EjXly8jDU44=</t>
+          <t>f4QV3U9xm02zGdj/8vI8ghiRMK7wZRhIxGWsK9vkhoc=</t>
         </is>
       </c>
     </row>
@@ -18266,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/WtD7CLqFDKRz8BOWsFiCA==</t>
+          <t>Tm/iMbNbp/hqWhv2ydeGtg==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>U9f+lBV3YGKQ2BTeEON+YaZX7CdEevoBayK/n5lYzwU=</t>
+          <t>P6sGbK/8vyHtb+Rgh7bJ6N8eV7w7aBT/di2KWqW4Lqg=</t>
         </is>
       </c>
     </row>
@@ -18298,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ixoZluk5eDAfU04qPNc3EA==</t>
+          <t>Up5JqJlcy1+AQCVUiK9x/g==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2pX3FB2kYu9h98a+PVPQrlGh5GOc84MZqXzS1AiRVds=</t>
+          <t>o6SnANZsXu6IVGGeME7CMzeCUehPQcH8SoZ5oU+/DcA=</t>
         </is>
       </c>
     </row>
@@ -18330,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>daH0o3Nf0ov1+jMXa3/9jA==</t>
+          <t>ej8Rg6OEDhoIs8Os3TbCMg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>b6M9aQdCwfulKXn98F4nvN9wJYE0mQe20EqJgsd/76g=</t>
+          <t>fs2FU1s4sZ5FEoFJYbs5QL8ffBPTS2iwnEf4tn+/EXE=</t>
         </is>
       </c>
     </row>
@@ -18362,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Zj4dxeewddaUWqxUP71ltA==</t>
+          <t>STp30NPQw/ILDCTt93m+/w==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>xp7Vy1zhTYeI6aiDwYklP3i+aPMo1a0a+TfT65qzVwY=</t>
+          <t>1/6TEOnnZuis+6erIsMxxhLWu86NT4OKhudFbnmObn4=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-15 07:39) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VENTAS MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>VENTAS MENOR COSTE</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55">
@@ -2655,12 +2655,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -2691,12 +2691,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -2799,12 +2799,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2871,12 +2871,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="81">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>292</v>
+        <v>303</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="87">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="88">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f6b3105-24e6-4d67-a983-097bd5e40d58&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="89">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="90">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="97">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="99">
@@ -4131,7 +4131,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="109">
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="110">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="117">
@@ -4687,12 +4687,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="119">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="120">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="122">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="126">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="128">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10">
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18">
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -7922,7 +7922,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -9138,7 +9138,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="97">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="98">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="103">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="104">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="106">
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="107">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>292</v>
+        <v>303</v>
       </c>
     </row>
     <row r="110">
@@ -11362,7 +11362,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="111">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="L115" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="116">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="120">
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="132">
@@ -12370,7 +12370,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="134">
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="140">
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="147">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>237</v>
+        <v>214</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="156">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="173">
@@ -14866,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="181">
@@ -14910,7 +14910,7 @@
         </is>
       </c>
       <c r="L181" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MMfYRNognDKOPgmz4A4sGw==</t>
+          <t>ESxBOD/r9FLQ9g+xtwuF3A==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>S5WawbTHTk1pdfOGDQqwWBYtFbhAgMwrT5uORBK5l/s=</t>
+          <t>MJZl09u1qJJsP8Bgpi78iyzel0XdMOxTeKcVozATLb8=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>h4+fNSVJcbWN1G5YLSbc6A==</t>
+          <t>XoKQiJhf+a4ihrnRi3tstA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>lLcOqRsk+JFTD/7k+Le7xtz1Gd8ThJWIJZwyFzczcos=</t>
+          <t>lFnS0Lo97QAAbw2CRMKEJMrVEdVYwdXyasdfjRwMxq8=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Jlr5LQDzjhRuQhsuLDKDOQ==</t>
+          <t>f8WH4MEWuyG2Shqm9cr9iQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Qx19SgKc0hNpHWGgKNPGZ0QPJ8yEgv63cLz/QbHqxYo=</t>
+          <t>r4+Hhp9Ml3Ttg6JorwbMCgO1PXEXGb8SwSAIt7cUCb4=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2vtu/V/uAL1jP2ie74w8tg==</t>
+          <t>VZBP07iHawHcoyCv3btg5w==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>FeFd4lqLzhrU5fP0h1nAvI6xj4AZ+QInfsdICbqwS9M=</t>
+          <t>jOwMT1VPM8SJ+3zDX9AirLC678WsB+gKcnxIFJLiaPU=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>nlqiF4Nj/soXBDGS45IDqw==</t>
+          <t>+3PSwFdbmH9lIXyNLmH7/g==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PuZI2CGegVvHeJy6HsVrprrzxhY+EcpZV577diou+Uw=</t>
+          <t>K9mn5iYuZFg3b39gdx3BZy+yRANWCvV0IBuP0GFwTLI=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LTIzsrlkHBkvW0l8IovsBg==</t>
+          <t>pDbna2YO2Mx0D/DTNSeF0g==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>j3tSlFphBsRCAXsv5yGyrMAuGyq75tmDneknyTUBwL0=</t>
+          <t>iKadgYor9uhTIC+ndyscDFdJaUroCdzlj8dSJ/RNCQs=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>oUSpnp3ZSwpQjZ39ZVEsEw==</t>
+          <t>1aBGQX+mO7aK33Ww6QNqmg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TIVs75s6A7jZJsAVZGp35/o1gFreTf9LjrVK7ehSqNI=</t>
+          <t>/E0Lxiss2wnZ1lXTUGZZn97Gh6sDxlGwWFzzLY2hQ+g=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>xvNrBY2Ug6eyt6Y/vceshA==</t>
+          <t>eqkgR2QBYMVnUZzKWXqL4Q==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>6OWUcOpVOq+PswTl3bBcinFfZHRgBBZeBCossbDdZU0=</t>
+          <t>SlgigWfFCV+LvudiAkzc4zbgLnQHpQ24CHL5dcXUkrs=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>sh0SeQyllOSQVcTQ63ohWg==;lrosInhylvlbkJk412qgaQ==</t>
+          <t>JcjnMMwRhlZic3CBA2QLXQ==;gAutnIcqQxkXwM3FqGIY1A==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TmyQRFR5JUMzk1mOlrEg+ijlo7hvaeMB1wnbzIvlX5Q=;yM/t4kb7YqF3FnKwPf0BNOAVZlRf/oMcJviVlinCuf8=</t>
+          <t>eBolrsRbpIG6ikir3KNnI2lBG1tvfBUpTRwGOb4xTgw=;M8XzCU3dMXTyfKPNPso7IZx6QGCjPpXbny0MGiHVTKk=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>KNXyrzLhtxj+xH7rdaV4hw==</t>
+          <t>4aU4tTLPfMOzicRdgfhboQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>/AcsOluJfdyLOfpcOSBWkIHEdj3upLqTmCD8yDd1+UA=</t>
+          <t>GH98rxQQiC3KmGTw+B4z5oudQZx4NKraVz9P7fP24E4=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0XN+1BB4ohyv5XZpU5n2Jg==</t>
+          <t>K0Z2C+rsyF+epNTYWbWtYw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>cK60LrdhFiWU3YwELQ4JgbtRI+LhLX1dsN0AR1h/9QQ=</t>
+          <t>Klx2fCh+IY0QvPL1tS4Ty/Bz1Q30WpRuI4dLgWRFUDw=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VLre2aTVVQZyoSEluRknRA==</t>
+          <t>s18h0hwp4o+Pe+4AOr3j/A==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FqraElTn7JiyEMjELx7gA9Npc9MdS3XSy2lMQGIsdN4=</t>
+          <t>lO2TZzlEluSoDlj71w7OzWG9GWae2GOOa6fxh3Py9U4=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>adR1cTMKkZTrWk4wo1Pg7A==</t>
+          <t>nllhKYlrnzddD3YzLUfKag==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MX6atKYlR001rfvxJ4iOeb5yxgrtqPDp96KMBB7hoRw=</t>
+          <t>lqnYiU530rP66PWt5VROPO2+jjtgwQGNes8p6GB7yrw=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>V3LEIGag2dfBWzj+J8JKcg==</t>
+          <t>1ZuC7anANpT6TMFpj++rcg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SXjbTH0v3JUbnhjXXooeCIYXz0GLHUZXfAerDMpj4KQ=</t>
+          <t>e/Gc4rtuuDmf1nZDNkrNNgkNS55pOgzHXcZX9gDXqtg=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>/TBlpCCZdcR/AWp3O0gKyg==</t>
+          <t>u4QSp/mkVSId2MYM1VBHRw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>LrDn9YRR8OBoZHgSCjZM3WDH/NlE4QZxg0dR/lBX8Ks=</t>
+          <t>bqITxVM696POgqPtT+mEfFwlKxEBZONXgPI85Ab4Vl8=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YyZ+Dc+9kX/AXgDnw/+wGw==</t>
+          <t>UFTqchBvoTB+5kqdiEXa5w==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>FpzuvYwCZjl0mfNbXHeFq14HF2LZ3kGI3v4RafqhSms=</t>
+          <t>qLP+X9cOnocLHB7OrQ0RW2pcoGjK+dXPuLJ/QxzCuxo=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>iCjSNRdP+R+AjU3G6saHSA==</t>
+          <t>zSxwAKOUyUkPazXokU1OBQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>u+uBed1cqCxlZdtKoOpdN+JK9i5QtUtFdJj5kzaM/tY=</t>
+          <t>Ry5DJJjzB1vMZkn1xtd2zFt8PLqSDJJD2Nb6SWsbpcA=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>B0imQp54K6qZ3yjXC+nOKA==</t>
+          <t>nl9R1T4fMbL9hch2ELe+rw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MRFGUIXRE8tJJWnM3DtZTs6Kk/Bv6C3+yIGGVw/Btk4=</t>
+          <t>23dt3trMDWcJMzWStyM9gKozXTdJOKTlRL6gaB7BN+o=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>VWfz3G1OlIHxVGyPaPEPOA==</t>
+          <t>RTS2U0+hhf06M/F/oC+yRQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Zw3c13fyZPXiv9AbC+sZoimBAgCH4o/Y+JGD4IFh0i4=</t>
+          <t>nF220X/oRwjJJy7jWvJ3R0yhPGP326QI0IZBtHaiqEg=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>UEyyli7BZGuESMHvu21E1Q==</t>
+          <t>2CSRrRbDRqeKemhlkO1ICw==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>wXkGL72NUSJ9aNE1QYqGSfXgbbvUSDwPUW3IfkQDAGs=</t>
+          <t>Iv+VJwRDRAgoG7YwGm1EaPgHZRyQaT+LyeFDol1MAkk=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Qwu2+KZe1yALhnjWb5yVQg==</t>
+          <t>CjPQGSKWTRIOGtImBoXsQQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>F1x4E8sJ3dvMSbW9ey9GrqJOkjFx2a6D9o9fBWABY8Q=</t>
+          <t>6tar797UgxfvE0W/UB8fJ5iiGDjzQwXgi6B0PxSDyvw=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OKWNfeAzOaPJfnzKPfSh6A==</t>
+          <t>9yu8bLb6PviATXtbY96nZQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>ZIHoBFbPYxdH2fGpwLZmvzCjNeObO9ojFpfqlaUSypU=</t>
+          <t>1Sk96Q93FlWI93kZj/WzGQoZKuH0yaG2b5bTdM1mtMI=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>6+LJYI0CSD3OoOPdHdgsOQ==</t>
+          <t>b3DvmfiPfFly2Hklldv6kA==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>PAp4BfBWW/8Ri1nkPj9eMOpPD2JX6Vy2DXWdLgssqM8=</t>
+          <t>xRF8vmCJT90ejdlSbVntH46gcQ+oeuFCv5D+UYk95VE=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>jnHaX7zxG2plu6Rbn6X+Ew==</t>
+          <t>k7f520FP8VGjbhhLEh9r6A==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>lHuB21zpUz7hAkj3be7JDo35S2uCo5P5ZW4VdJ51kZ4=</t>
+          <t>RPhATdSq2s1mxQkExbmtAQvvU00Gih2Z+QZH4ADbeD8=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AroTs5Q1x+Hd8XqmBYHXMA==</t>
+          <t>fTlHK7O+Pa+2xioxh73cuA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>s5EwSkD5AHw0Q0eZTdWQeH83Viev/cjwHOgv+LXD6gA=</t>
+          <t>9xgB1cJgMn7t0U4B0+WzFCzKc17wyG1gTrLu8r7glKM=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>o2yzpu1vqrHRC5o883VTAA==</t>
+          <t>A7Sn+m6U79h8zRZ0OxLjHw==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>zPSTQUwOrsbVpuRuN7I/SFbS2N+WmneMdXRHFuN56Ic=</t>
+          <t>IEhYSnBv4acdGVKOmhzZ/IfXv0bFZjWEDcl6Awyv+Aw=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>hHzzWi9CC9EqB1Hl/0zhgw==</t>
+          <t>/SSHD9bMnvOu9obOmnvy7w==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>pygI7iz3eMDn50e4Gggesff9Eb1ZWR/IpUaTVPpbXbw=</t>
+          <t>vcopz/EaY9Hh38M0DxxW1KaN+F8cdiZVBgRssSJbIxk=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>I6B+LA0IVkpFJeG8AOgKUA==</t>
+          <t>izu4WXGK50OUd4jLbB5Ogg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ED4oz28OBOm9+fEeXhMSR7cR+ctATYXxPspA1NJckGU=</t>
+          <t>YCkZ3dj2KKCaIjXX+VoJ/p9GDC+rT/4pSHsDyxz3yZE=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>jRy4CFlw5qOP8mn6xVUloA==</t>
+          <t>5QvTui0Fhb+yT2NIcfAamA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>91eIEpLXKGjHzv7pKXGZCUwcT3DWcmClL7QEP63TfSU=</t>
+          <t>NcFM8c9YXBx+fMofYK2T+bc0kPGYvcyACDZIwYDY5Rc=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>7aJ/iADkkRdAK8GGijZaPQ==</t>
+          <t>9NzuZft8QIz72rs/HUJGdw==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>UTUCioLmYRvWrg3GN+qn+LT9rDpKv0C3A/BNOKyESBY=</t>
+          <t>3wYJ3DT0vIJvgprAmSxfQ4cyNgMgEP5MyRMJmdJx4dk=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>eF9eKCJFVz+aIsz/HOMSkQ==</t>
+          <t>svGiyCSjAy13g9v1pWcOcw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>lYf9Eo/MZHiYxxHA+8Ox4DNt03FOCQWoKoMJPI6pw5Q=</t>
+          <t>7A0eCCPslbhV0dTssK1xf4Ko14IFFCt8O6Tgk09co0M=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A5RXlILPINcgrH90XbjHeg==</t>
+          <t>ntyhJANCJPRpucHqb1e3Wg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MjU6jcfGairn3aOdxb6N9ABFt1AiUGLbJSJ8Aq7GEh4=</t>
+          <t>ICdfEYnPOqBARAePJQ8fBfQD1htLHAPKREK1ot1YjPI=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Xuh73dwLLsoJQCU2EtRpXQ==</t>
+          <t>/agqlzEYWvNHQ53B7CaL4A==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>f4QV3U9xm02zGdj/8vI8ghiRMK7wZRhIxGWsK9vkhoc=</t>
+          <t>efdlwT1UXM/DGD731cyPySVu3STNo/j7TnOeRO8n97Y=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Tm/iMbNbp/hqWhv2ydeGtg==</t>
+          <t>RgcoDmnCUhAp041AxDVkOQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>P6sGbK/8vyHtb+Rgh7bJ6N8eV7w7aBT/di2KWqW4Lqg=</t>
+          <t>QbSPI5Vaxe9p8PjpzooqOkatOykAaw4S9GXgJq4NYqo=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Up5JqJlcy1+AQCVUiK9x/g==</t>
+          <t>3RqeLtwYq7EC2EVocM9Abg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>o6SnANZsXu6IVGGeME7CMzeCUehPQcH8SoZ5oU+/DcA=</t>
+          <t>q18m+GawjTvWDPA1D3kEAysaMkCT82ii3TGPZmzlTa0=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ej8Rg6OEDhoIs8Os3TbCMg==</t>
+          <t>bxjh+qzlXF00oWnbe782nw==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>fs2FU1s4sZ5FEoFJYbs5QL8ffBPTS2iwnEf4tn+/EXE=</t>
+          <t>OmjlKnJqDkTONQb70G1S5GOJXbrTOtbGES1wV6Hl4SY=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>STp30NPQw/ILDCTt93m+/w==</t>
+          <t>MJGrzESUMNtLgGxOynHmJQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1/6TEOnnZuis+6erIsMxxhLWu86NT4OKhudFbnmObn4=</t>
+          <t>Ekl4wZENTmmF38aZIQQkQNC5spHfK+J6LTgz90RHId8=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-16 07:38) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>VENTAS MENOR COSTE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VENTAS MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6d8bba6a-0f85-418a-a3de-a46559c081dd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>164</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="49">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DASHBOARD FINANCIERO</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>DASHBOARD FINANCIERO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ab000668-c7ee-4c12-8689-e4afdbe23b96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=266c62e3-af8c-40b2-adb7-0b725d7b15b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2511,12 +2511,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>HECTOLITROS 10-2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=266c62e3-af8c-40b2-adb7-0b725d7b15b9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2619,12 +2619,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -2655,12 +2655,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2799,12 +2799,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c81e4915-018b-44c6-a93d-efe70059b2ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2871,12 +2871,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -2943,12 +2943,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>303</v>
+        <v>317</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="89">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="109">
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="110">
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>386</v>
+        <v>398</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>386</v>
+        <v>398</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="118">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="120">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="124">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="125">
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="126">
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=11cc3a84-a83e-4020-844d-43919a87f1b9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=11cc3a84-a83e-4020-844d-43919a87f1b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5355,7 +5355,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="136">
@@ -5958,7 +5958,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
@@ -6310,7 +6310,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14">
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18">
@@ -7922,7 +7922,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43">
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="65">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>164</v>
+        <v>182</v>
       </c>
     </row>
     <row r="97">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="98">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="106">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>303</v>
+        <v>317</v>
       </c>
     </row>
     <row r="110">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="120">
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="126">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="132">
@@ -12370,7 +12370,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="133">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="134">
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="140">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>214</v>
+        <v>204</v>
       </c>
     </row>
     <row r="150">
@@ -13386,7 +13386,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="152">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="156">
@@ -13662,7 +13662,7 @@
         </is>
       </c>
       <c r="L157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158">
@@ -14366,7 +14366,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="173">
@@ -14646,7 +14646,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="224">
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ESxBOD/r9FLQ9g+xtwuF3A==</t>
+          <t>jSzLQkWV92B8LKjt3onctA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MJZl09u1qJJsP8Bgpi78iyzel0XdMOxTeKcVozATLb8=</t>
+          <t>Gm15seQsU9ANgwqMwRJ34Y//EF45znzAtfrenY4BwSk=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XoKQiJhf+a4ihrnRi3tstA==</t>
+          <t>Mdrwmm7c3de8ivHkC5FtTQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>lFnS0Lo97QAAbw2CRMKEJMrVEdVYwdXyasdfjRwMxq8=</t>
+          <t>FumtCgVpWXFXw4vzYa3BaRr/R1J51rKmukGWOZRFBac=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>f8WH4MEWuyG2Shqm9cr9iQ==</t>
+          <t>IyD9rhPR0VCpVmFx5t6Frw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>r4+Hhp9Ml3Ttg6JorwbMCgO1PXEXGb8SwSAIt7cUCb4=</t>
+          <t>iXgVfffY7301ZO8VKP/x45dbCLY7FdcAmcGRnq6yWhE=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VZBP07iHawHcoyCv3btg5w==</t>
+          <t>2LiPO+FNGxcur7fuXZyGjA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>jOwMT1VPM8SJ+3zDX9AirLC678WsB+gKcnxIFJLiaPU=</t>
+          <t>Egk4zeS8budMZmeUVStklBM564WeFU4TpOrpohwcPP0=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+3PSwFdbmH9lIXyNLmH7/g==</t>
+          <t>EP8lvFcrBPQVUWuQjRPYww==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>K9mn5iYuZFg3b39gdx3BZy+yRANWCvV0IBuP0GFwTLI=</t>
+          <t>S4y4L8rLVGTixHdxAEj9o+9joDhBX/oeqFrlC2ki/pY=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>pDbna2YO2Mx0D/DTNSeF0g==</t>
+          <t>3NFx/Q6r1BHQgj18yE9TGA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>iKadgYor9uhTIC+ndyscDFdJaUroCdzlj8dSJ/RNCQs=</t>
+          <t>H14lqwjEG9rCApwNX1tPDJXKmrzoNHL/yzcrkr3c6Mc=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1aBGQX+mO7aK33Ww6QNqmg==</t>
+          <t>C2SkxFnqyMt6vYA2/IphZw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>/E0Lxiss2wnZ1lXTUGZZn97Gh6sDxlGwWFzzLY2hQ+g=</t>
+          <t>An7GR5O/n3FQ92wTqB5O+u/Autz5iet2KSAwyA7PBcg=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>eqkgR2QBYMVnUZzKWXqL4Q==</t>
+          <t>84hItCF2De3f7EG/EzSxTQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SlgigWfFCV+LvudiAkzc4zbgLnQHpQ24CHL5dcXUkrs=</t>
+          <t>uvIohNCUScT3iopQrP2Udnp299jaxpWpaXOfcwR5Y/I=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>JcjnMMwRhlZic3CBA2QLXQ==;gAutnIcqQxkXwM3FqGIY1A==</t>
+          <t>wsCwx4ALiKHPiLggbFNRsQ==;2BhRDXZuXYUBhmcQ+vmkZg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>eBolrsRbpIG6ikir3KNnI2lBG1tvfBUpTRwGOb4xTgw=;M8XzCU3dMXTyfKPNPso7IZx6QGCjPpXbny0MGiHVTKk=</t>
+          <t>k/SQMWqrbggRGYtrYDe0qBwE3FrllYzoAb3CD5sXMg8=;yT37xnqoGjt01l++SGZYRoOIz6BMbyHs3OyuCURGSts=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4aU4tTLPfMOzicRdgfhboQ==</t>
+          <t>Ab9NgggsspLTqT8LFdMK2w==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GH98rxQQiC3KmGTw+B4z5oudQZx4NKraVz9P7fP24E4=</t>
+          <t>5EArzkCUQ3EwwSPpwSyVV2d9dCs8ekh5lbGZY1BdrXw=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>K0Z2C+rsyF+epNTYWbWtYw==</t>
+          <t>iiwQCq5SMkmwol2KwtuKDQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Klx2fCh+IY0QvPL1tS4Ty/Bz1Q30WpRuI4dLgWRFUDw=</t>
+          <t>TV1zYQb6ujFU+f22w45mhGsynav9X009vCOdSCeJLW0=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>s18h0hwp4o+Pe+4AOr3j/A==</t>
+          <t>UymCqLydWpkSOEvjSX12Cw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>lO2TZzlEluSoDlj71w7OzWG9GWae2GOOa6fxh3Py9U4=</t>
+          <t>K1Zuf3bm287Y7hkdck3i1ynEOFhWrk4RjuycT6qHWaY=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>nllhKYlrnzddD3YzLUfKag==</t>
+          <t>YZtirkMzBMeKDIa5WPkLHg==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>lqnYiU530rP66PWt5VROPO2+jjtgwQGNes8p6GB7yrw=</t>
+          <t>TTH8ZmzvC75/17EzuRmOYhslS5V+zPhZr7FPF3ZkAug=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1ZuC7anANpT6TMFpj++rcg==</t>
+          <t>QuLKv2wirC818q6iynQYVA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>e/Gc4rtuuDmf1nZDNkrNNgkNS55pOgzHXcZX9gDXqtg=</t>
+          <t>AdcfWbhCrlb/WxUd5Y6fNnFs+a0S+a+EKU7O9ZZiUF4=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>u4QSp/mkVSId2MYM1VBHRw==</t>
+          <t>Ce1CVFHwqpFic8d5uxlebg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>bqITxVM696POgqPtT+mEfFwlKxEBZONXgPI85Ab4Vl8=</t>
+          <t>T/7yv4TgOWmOtG4H7Rk67u9q/3EWsZfxglTRMZhEpdc=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>UFTqchBvoTB+5kqdiEXa5w==</t>
+          <t>veDvmuKSLeORchQhSJ/bXg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>qLP+X9cOnocLHB7OrQ0RW2pcoGjK+dXPuLJ/QxzCuxo=</t>
+          <t>NTPYGwLVElKpvCN9Y88XFm1MIFc2mhMCynU0nJkVXT8=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>zSxwAKOUyUkPazXokU1OBQ==</t>
+          <t>ZkKUXk0XvzD0KS7jUWRbIQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ry5DJJjzB1vMZkn1xtd2zFt8PLqSDJJD2Nb6SWsbpcA=</t>
+          <t>BHx3PC9I5LeukihHyGbJfP2BhrPUpFGMj2wXdCjiU88=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>nl9R1T4fMbL9hch2ELe+rw==</t>
+          <t>Xm/TbVNlDZSnLF5TeD7vQg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>23dt3trMDWcJMzWStyM9gKozXTdJOKTlRL6gaB7BN+o=</t>
+          <t>aiRtT0kqdXJnqHPWtbtf4lpDHt7rqyNcUxcnt6B8Wa8=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RTS2U0+hhf06M/F/oC+yRQ==</t>
+          <t>PC0wIh5WfwKZtUyNm7F1hA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>nF220X/oRwjJJy7jWvJ3R0yhPGP326QI0IZBtHaiqEg=</t>
+          <t>4N81E7knPqrgrRIx56Kpn8Ff++dy/d03wf82M1+uqmE=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2CSRrRbDRqeKemhlkO1ICw==</t>
+          <t>GHw9JyxZEmlKtQW9Nv+W1Q==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Iv+VJwRDRAgoG7YwGm1EaPgHZRyQaT+LyeFDol1MAkk=</t>
+          <t>29vMDVUce8QoGlCy6W6A+oXvhBr5nJqRnIPDvAWU1SI=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CjPQGSKWTRIOGtImBoXsQQ==</t>
+          <t>hHPRo2cuRt1QnTDus12WtA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>6tar797UgxfvE0W/UB8fJ5iiGDjzQwXgi6B0PxSDyvw=</t>
+          <t>kcwiPiADRTFEAzONS8P82CFg15DhJ7Klp23esFrRS+8=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>9yu8bLb6PviATXtbY96nZQ==</t>
+          <t>kgXxkNTp5udyHQUMxCW/Qg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1Sk96Q93FlWI93kZj/WzGQoZKuH0yaG2b5bTdM1mtMI=</t>
+          <t>XhhSMG8Bv+t9j4RYF5pN1dL4/ZaB8sAOWkZI6GIamLs=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>b3DvmfiPfFly2Hklldv6kA==</t>
+          <t>x4GzeGOdcPjTH/3s3fDEig==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>xRF8vmCJT90ejdlSbVntH46gcQ+oeuFCv5D+UYk95VE=</t>
+          <t>z0PVtyBEZe2x4rjQUha0lVdY9eRlROefEDYQWlKlpbc=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>k7f520FP8VGjbhhLEh9r6A==</t>
+          <t>RlE90moL+6Ti6gykthbCwg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RPhATdSq2s1mxQkExbmtAQvvU00Gih2Z+QZH4ADbeD8=</t>
+          <t>U/7XkUo9esxxoDbXKRyXR/SlfLEyPdVhu7UljbDnh/4=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>fTlHK7O+Pa+2xioxh73cuA==</t>
+          <t>ySbVAXxO1U1sQLRERql2rg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>9xgB1cJgMn7t0U4B0+WzFCzKc17wyG1gTrLu8r7glKM=</t>
+          <t>qkJYzTzv6IlDdZSq+R2556mGbSN+CYU44ff6RDMok+g=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>A7Sn+m6U79h8zRZ0OxLjHw==</t>
+          <t>nfrcDNxI970jNFzOGOF7iQ==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>IEhYSnBv4acdGVKOmhzZ/IfXv0bFZjWEDcl6Awyv+Aw=</t>
+          <t>zAdzKIrEtqiVpI1nt6F67LYzvHm945CH6P1Qlzka9WY=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>/SSHD9bMnvOu9obOmnvy7w==</t>
+          <t>z2+QlsspIZVPK6w3Wfq8MA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>vcopz/EaY9Hh38M0DxxW1KaN+F8cdiZVBgRssSJbIxk=</t>
+          <t>N1bMTw0mv6/ww7Lo6M77DtF01hdlN5WZVlVF6oFG0ks=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>izu4WXGK50OUd4jLbB5Ogg==</t>
+          <t>cvpcgUlluP4TO9Gtc6Pj0w==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>YCkZ3dj2KKCaIjXX+VoJ/p9GDC+rT/4pSHsDyxz3yZE=</t>
+          <t>T0nuCiBqKFSlLKw2rPzvYlm7fTFZfK0An0MQIXtfgTA=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5QvTui0Fhb+yT2NIcfAamA==</t>
+          <t>U/bcKCROEh+wuWWWUFXFOQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>NcFM8c9YXBx+fMofYK2T+bc0kPGYvcyACDZIwYDY5Rc=</t>
+          <t>ND39iwRc6xy3DeqpyBEfrzGlF1s72SrgZyKMI36BbqY=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>9NzuZft8QIz72rs/HUJGdw==</t>
+          <t>CkB3gRra8kaNxlR3eQ9oIg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3wYJ3DT0vIJvgprAmSxfQ4cyNgMgEP5MyRMJmdJx4dk=</t>
+          <t>QnkpXuZcpaLXoUQq7mHI2DQBlJmUHbQBecPnieX1eA4=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>svGiyCSjAy13g9v1pWcOcw==</t>
+          <t>J7W5VyNN+HlLxBQEMwBBrA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>7A0eCCPslbhV0dTssK1xf4Ko14IFFCt8O6Tgk09co0M=</t>
+          <t>GPnkMmihOvnLXE1Z0C2ZaEktfZRURDGV0mKgrDZQBFQ=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ntyhJANCJPRpucHqb1e3Wg==</t>
+          <t>ExwuNL74jryle/4B17KaaA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ICdfEYnPOqBARAePJQ8fBfQD1htLHAPKREK1ot1YjPI=</t>
+          <t>MJjcTtSecwMGQkAFJJVnH+wMDPEN+5BLHJ7Hpwi0EGQ=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>/agqlzEYWvNHQ53B7CaL4A==</t>
+          <t>9peXWToT3yoLBy0XCB7gYw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>efdlwT1UXM/DGD731cyPySVu3STNo/j7TnOeRO8n97Y=</t>
+          <t>OV/pGHD2E6UTa5RxPRa3Qc9UYSrbW/z3dlK6n+RN4Bk=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RgcoDmnCUhAp041AxDVkOQ==</t>
+          <t>BsgkKA92bgdgWfAfCz93XA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>QbSPI5Vaxe9p8PjpzooqOkatOykAaw4S9GXgJq4NYqo=</t>
+          <t>VDOaS8mse9FlTVxebSsX6k6wi0fDV6BIEJcEsKC2eQI=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>3RqeLtwYq7EC2EVocM9Abg==</t>
+          <t>6a2AbAYaMhY3Mlsq9nTwSA==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>q18m+GawjTvWDPA1D3kEAysaMkCT82ii3TGPZmzlTa0=</t>
+          <t>7OJLiZ9hBAHdILy6eZ3fJnHQ3dFOrzXsbmuLHG/d7AM=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>bxjh+qzlXF00oWnbe782nw==</t>
+          <t>YnzWQSxHLTM5ETvbktNCUA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>OmjlKnJqDkTONQb70G1S5GOJXbrTOtbGES1wV6Hl4SY=</t>
+          <t>ZZ/TeH/T1Ui7US3MV4KSmkQhvvfzySdPh9kVbhzgXzI=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MJGrzESUMNtLgGxOynHmJQ==</t>
+          <t>1OJT5ztGiUlwPTCDZMahwg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Ekl4wZENTmmF38aZIQQkQNC5spHfK+J6LTgz90RHId8=</t>
+          <t>35vhssiANGXyfed+DlmO62XG4H1tiuXMhc8Sm2C2I5M=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-17 08:38) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55">
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="56">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="86">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="89">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="96">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="97">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>398</v>
+        <v>408</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>398</v>
+        <v>408</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="118">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="120">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="122">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="123">
@@ -4903,12 +4903,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="124">
@@ -4939,12 +4939,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b56bb142-8685-433a-bd0c-b8969d964151&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>HECTOLITROS 10-2026</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b56bb142-8685-433a-bd0c-b8969d964151&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="126">
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -7922,7 +7922,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43">
@@ -8010,7 +8010,7 @@
         </is>
       </c>
       <c r="L44" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45">
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="98">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="106">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="110">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="120">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="126">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="132">
@@ -12502,7 +12502,7 @@
         </is>
       </c>
       <c r="L135" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="136">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="156">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>jSzLQkWV92B8LKjt3onctA==</t>
+          <t>NvjhJ/p4c3DO0OpoXckoPw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Gm15seQsU9ANgwqMwRJ34Y//EF45znzAtfrenY4BwSk=</t>
+          <t>tNbsbzfkDVWrWv4rou7H+Vc+21WXyMLsSx3Q0h/Zl78=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mdrwmm7c3de8ivHkC5FtTQ==</t>
+          <t>0XieV1GhgsHBUJ9YkMa9eg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FumtCgVpWXFXw4vzYa3BaRr/R1J51rKmukGWOZRFBac=</t>
+          <t>lMK/D1yTmL1Ftzw/X+jBKG2IDRaqIosxWu7rRHFro44=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>IyD9rhPR0VCpVmFx5t6Frw==</t>
+          <t>ncYjw1VRvCjsy7NTDGS7TA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>iXgVfffY7301ZO8VKP/x45dbCLY7FdcAmcGRnq6yWhE=</t>
+          <t>O3N+BfTy/Zy5sS7cQW0pOxaqZuIbnj72A631bqx2JTo=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2LiPO+FNGxcur7fuXZyGjA==</t>
+          <t>VLdPjpBH6MQnqP51rbS23Q==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Egk4zeS8budMZmeUVStklBM564WeFU4TpOrpohwcPP0=</t>
+          <t>lWRvuDSYfIqEzqU4RiLE6Gp28GyybEj9k/tiLCIRe+Y=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EP8lvFcrBPQVUWuQjRPYww==</t>
+          <t>g6JqfR/T5vo0g4gDg/QRhg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>S4y4L8rLVGTixHdxAEj9o+9joDhBX/oeqFrlC2ki/pY=</t>
+          <t>p+3aY021qaNRalWBVkfLLrJ5GqLVsAPVuwJWZjh+5Lw=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3NFx/Q6r1BHQgj18yE9TGA==</t>
+          <t>XHIVcHl6SlT+qkf7oNKYuw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>H14lqwjEG9rCApwNX1tPDJXKmrzoNHL/yzcrkr3c6Mc=</t>
+          <t>uX1KrNRNoNhfkho1F4nRyKxp0zbql7WmRFIx0vDdbDA=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>C2SkxFnqyMt6vYA2/IphZw==</t>
+          <t>bkm9B7bDiB0xz1GnFOSDxw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>An7GR5O/n3FQ92wTqB5O+u/Autz5iet2KSAwyA7PBcg=</t>
+          <t>Gbnl01JEY3zToy/rObQcgsfUrEzyhA92S2soqWiA4hM=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>84hItCF2De3f7EG/EzSxTQ==</t>
+          <t>Ninr0cT5HXDlBYS/Bv3CQA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>uvIohNCUScT3iopQrP2Udnp299jaxpWpaXOfcwR5Y/I=</t>
+          <t>TRna2FBjcP/DxZgRJT2wJCy5Fk/OgyL1pWmzfNdkai4=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>wsCwx4ALiKHPiLggbFNRsQ==;2BhRDXZuXYUBhmcQ+vmkZg==</t>
+          <t>lbSspM54Y9R3p5RWkWXYyw==;icKhrFpl85rJlivR0Fooog==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>k/SQMWqrbggRGYtrYDe0qBwE3FrllYzoAb3CD5sXMg8=;yT37xnqoGjt01l++SGZYRoOIz6BMbyHs3OyuCURGSts=</t>
+          <t>G6IgbJf52peZ4le40YUpVeXrw+LGtlBjqMzFM6rYKCE=;OVAACF/VicD2BNp5fV+9uSPhHGwYqnPVFkqe6WNycV4=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ab9NgggsspLTqT8LFdMK2w==</t>
+          <t>P14ipVfU5Q+kK5AzC1/MVg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5EArzkCUQ3EwwSPpwSyVV2d9dCs8ekh5lbGZY1BdrXw=</t>
+          <t>DH6WRwZIBlfCGUNafz+X50MfsIFgW65cqHcqMvulYDw=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>iiwQCq5SMkmwol2KwtuKDQ==</t>
+          <t>akiV6vl4dK7AHYXyRoWItw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TV1zYQb6ujFU+f22w45mhGsynav9X009vCOdSCeJLW0=</t>
+          <t>x1VxDsNW/lDY+ROAsK1sSSYvniNt9F4rQP1HDwd6CMM=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>UymCqLydWpkSOEvjSX12Cw==</t>
+          <t>WvvcGcca9XPg9R8JGIluaA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>K1Zuf3bm287Y7hkdck3i1ynEOFhWrk4RjuycT6qHWaY=</t>
+          <t>egvGI1KTwIhoVr/nDg1dRhBf60F4QGrTZxRBJSDkQHE=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>YZtirkMzBMeKDIa5WPkLHg==</t>
+          <t>hq/QOx9zWk2DfVOKC/JmbA==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TTH8ZmzvC75/17EzuRmOYhslS5V+zPhZr7FPF3ZkAug=</t>
+          <t>AHp+Aj8otEG6a0Y6MccNksFJblxnodlWZaswNvIGPcg=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>QuLKv2wirC818q6iynQYVA==</t>
+          <t>3Nru7mxY/Rzx+4UfHDCmHA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AdcfWbhCrlb/WxUd5Y6fNnFs+a0S+a+EKU7O9ZZiUF4=</t>
+          <t>Q9cHV+/O/9M4xsb0kuU17ettVaCoZdTBorngwy3aqvk=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ce1CVFHwqpFic8d5uxlebg==</t>
+          <t>ZL5kXdGhqtaDpGYlzW9D/A==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>T/7yv4TgOWmOtG4H7Rk67u9q/3EWsZfxglTRMZhEpdc=</t>
+          <t>Bd8vjUvb1mSD6XVe3jZ8iUZysBicXinGEGUrdHM3UPw=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>veDvmuKSLeORchQhSJ/bXg==</t>
+          <t>flTog6ucoXQWZbEOFiNepQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>NTPYGwLVElKpvCN9Y88XFm1MIFc2mhMCynU0nJkVXT8=</t>
+          <t>JM0oKHbzy6Vd0e03WsDwuRSPLrd6bYcS48660JOhv8w=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ZkKUXk0XvzD0KS7jUWRbIQ==</t>
+          <t>X6PsbZwf/PE6dg3bW5hb3Q==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>BHx3PC9I5LeukihHyGbJfP2BhrPUpFGMj2wXdCjiU88=</t>
+          <t>2CrZ2SY4Td/d9i8L6M0y55dXtQYcZUb5v634zSUxnkw=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Xm/TbVNlDZSnLF5TeD7vQg==</t>
+          <t>RaU7tS4Woop4M7BSpME3kg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>aiRtT0kqdXJnqHPWtbtf4lpDHt7rqyNcUxcnt6B8Wa8=</t>
+          <t>NqBlPJ+erF1JR3yu9EKtER12btEXE3RM7NLMrT/Cpn0=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PC0wIh5WfwKZtUyNm7F1hA==</t>
+          <t>rWxsKasaXRbC16ZO4LkG8g==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>4N81E7knPqrgrRIx56Kpn8Ff++dy/d03wf82M1+uqmE=</t>
+          <t>ORGBQC+d2heC71yTZ30mkFWbVOlM410dVJKM1mjgauc=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>GHw9JyxZEmlKtQW9Nv+W1Q==</t>
+          <t>cvk7MQ88x/hw9IVkLeNwEA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>29vMDVUce8QoGlCy6W6A+oXvhBr5nJqRnIPDvAWU1SI=</t>
+          <t>2mOCjMXwuKMVogfq5eO14/HZxh6ZwxGpQAkBR70E0B8=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>hHPRo2cuRt1QnTDus12WtA==</t>
+          <t>p8fBEHNVD5SquYeYauV61Q==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>kcwiPiADRTFEAzONS8P82CFg15DhJ7Klp23esFrRS+8=</t>
+          <t>r5Y4B52TAUtl/MixJLkN4ZBJpaPWYv9nyLZYqqeGe3U=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>kgXxkNTp5udyHQUMxCW/Qg==</t>
+          <t>1cfei+Sh/q/F1YfsyCtieA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>XhhSMG8Bv+t9j4RYF5pN1dL4/ZaB8sAOWkZI6GIamLs=</t>
+          <t>CfPhRjC79C1cMZtQUrXJ9NHJLnSZh08WXF1cLquPPcc=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>x4GzeGOdcPjTH/3s3fDEig==</t>
+          <t>mOGlkjaQ4Fd4Qp2K61548w==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>z0PVtyBEZe2x4rjQUha0lVdY9eRlROefEDYQWlKlpbc=</t>
+          <t>Wzh4GRB53rFSYWlHFJa1bnNCQH53zWHPYubGQ+e3PUM=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RlE90moL+6Ti6gykthbCwg==</t>
+          <t>WKsaCiq3TDa/OJnFA8tKlw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>U/7XkUo9esxxoDbXKRyXR/SlfLEyPdVhu7UljbDnh/4=</t>
+          <t>0+lcU8264dogIMIFqx+20cqa7eBOFBGFBPQLtsz/7rk=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ySbVAXxO1U1sQLRERql2rg==</t>
+          <t>4BcxuZtveimhAMM5IPYv0Q==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>qkJYzTzv6IlDdZSq+R2556mGbSN+CYU44ff6RDMok+g=</t>
+          <t>T7q6Afdeh3BxhGfWyws4Cy8JVoRNvWsaCrhBsZIQbYg=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>nfrcDNxI970jNFzOGOF7iQ==</t>
+          <t>IodJC9RIZe0DAJdw8c7fKQ==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>zAdzKIrEtqiVpI1nt6F67LYzvHm945CH6P1Qlzka9WY=</t>
+          <t>ncnkGuqm3Y+BGB80Qjgs4Ahvt8/mb7vC8D4AWFAc1WE=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>z2+QlsspIZVPK6w3Wfq8MA==</t>
+          <t>PmTO3l5UxqfHjsI1QvFbfw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>N1bMTw0mv6/ww7Lo6M77DtF01hdlN5WZVlVF6oFG0ks=</t>
+          <t>/UUDt5IaJdcrMdpCakLnEBTPHRraDPaXo0FEyDyMsng=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>cvpcgUlluP4TO9Gtc6Pj0w==</t>
+          <t>SemLuExp8+0mQbvKRqdBeg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>T0nuCiBqKFSlLKw2rPzvYlm7fTFZfK0An0MQIXtfgTA=</t>
+          <t>KUVFhJnHBj0Sv6MA8SZd6jvdQc6Jaop5K4tOVEvpESk=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>U/bcKCROEh+wuWWWUFXFOQ==</t>
+          <t>JW37RD7J3zty7SYCcaK5dQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>ND39iwRc6xy3DeqpyBEfrzGlF1s72SrgZyKMI36BbqY=</t>
+          <t>v//LIiljZummQVdk7kDvNOBVHpLwFIlhYugfDacmidQ=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CkB3gRra8kaNxlR3eQ9oIg==</t>
+          <t>LhhiQ7Q65jCmFtjiFyyJxg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>QnkpXuZcpaLXoUQq7mHI2DQBlJmUHbQBecPnieX1eA4=</t>
+          <t>OK8Yf8Pjq8lHAAY2lsJh8ij2kBDDci0Jd+nXukj1wQM=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>J7W5VyNN+HlLxBQEMwBBrA==</t>
+          <t>P4QufN+yct2rvEEMEGGbpA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>GPnkMmihOvnLXE1Z0C2ZaEktfZRURDGV0mKgrDZQBFQ=</t>
+          <t>p1ui2BN18vmZyeNUSaHh+NATKDLuWd1uTEErpyvEAWw=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ExwuNL74jryle/4B17KaaA==</t>
+          <t>VgoF4Oceq1GWaL5ujRX4Og==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MJjcTtSecwMGQkAFJJVnH+wMDPEN+5BLHJ7Hpwi0EGQ=</t>
+          <t>N32HJRGXLfHgap9uf+PhJOxXjOxRggrSidcGxGuI2fE=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>9peXWToT3yoLBy0XCB7gYw==</t>
+          <t>VVRGEigH3nU1nP54dC4Oxw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>OV/pGHD2E6UTa5RxPRa3Qc9UYSrbW/z3dlK6n+RN4Bk=</t>
+          <t>mUTS8umX+X7uc4avsdrFWcoI0Jpa7fStWwuJYXtMsCw=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BsgkKA92bgdgWfAfCz93XA==</t>
+          <t>CZiIPSXn/laqFYP/62vkvQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VDOaS8mse9FlTVxebSsX6k6wi0fDV6BIEJcEsKC2eQI=</t>
+          <t>SnBHC2PIgnxx59Fl0YcHdq9fOnB2cZcMKqhQi7Vbq2I=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>6a2AbAYaMhY3Mlsq9nTwSA==</t>
+          <t>qkdFiDCGEWe0Xorw+8RzKw==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>7OJLiZ9hBAHdILy6eZ3fJnHQ3dFOrzXsbmuLHG/d7AM=</t>
+          <t>j0mMdoC7R+SXtogCQteqj14RcKZDUcPtpZHVPDjkL4M=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>YnzWQSxHLTM5ETvbktNCUA==</t>
+          <t>Xe/C5xqLYnq8O3D8ly/jTQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ZZ/TeH/T1Ui7US3MV4KSmkQhvvfzySdPh9kVbhzgXzI=</t>
+          <t>tEHSD0H8EqlqbYc3KBrjm10lbg+p5M3UdZaR0EoX61E=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1OJT5ztGiUlwPTCDZMahwg==</t>
+          <t>Rw+8aRsre0DZtFvNG56w3A==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>35vhssiANGXyfed+DlmO62XG4H1tiuXMhc8Sm2C2I5M=</t>
+          <t>LS/kwKugsVVZ1p/S6x2xquqBZ2JV8RweNUIEMq3ZWSE=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-18 07:39) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="81">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="86">
@@ -3571,12 +3571,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="87">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=21258af6-7c9d-434c-b296-8bda0eb9806f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18668d79-2a2c-47bf-b666-33ac22fe1b6f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="88">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="90">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="94">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="97">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>408</v>
+        <v>417</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>408</v>
+        <v>417</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="118">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="120">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="122">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="124">
@@ -5958,7 +5958,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18">
@@ -8882,7 +8882,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="97">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="103">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105">
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="107">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="110">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="120">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="127">
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="139">
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="140">
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="147">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>204</v>
+        <v>191</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="156">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="173">
@@ -14866,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="181">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NvjhJ/p4c3DO0OpoXckoPw==</t>
+          <t>ujkTkhsOpCyCWTUdrKKRjg==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>tNbsbzfkDVWrWv4rou7H+Vc+21WXyMLsSx3Q0h/Zl78=</t>
+          <t>dVGLCnJwFoA9/5CZnTnReZFt/1DQ+FX202Aq+PEo1ps=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0XieV1GhgsHBUJ9YkMa9eg==</t>
+          <t>sC7UCuuQNuskzQTHifaPSg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>lMK/D1yTmL1Ftzw/X+jBKG2IDRaqIosxWu7rRHFro44=</t>
+          <t>TKST1qKC6Qn/0AB89Ywg7XfkDoN/Q0FAnT7lshxy4BQ=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ncYjw1VRvCjsy7NTDGS7TA==</t>
+          <t>FdeoATesyVUPmiPgYwC8tQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>O3N+BfTy/Zy5sS7cQW0pOxaqZuIbnj72A631bqx2JTo=</t>
+          <t>fpMSB+gseT6ybdAUP56W7J6ymK78A00hsZRb/XxKlpQ=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VLdPjpBH6MQnqP51rbS23Q==</t>
+          <t>B5or5Qg5kY1uYfX2LFJo5w==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>lWRvuDSYfIqEzqU4RiLE6Gp28GyybEj9k/tiLCIRe+Y=</t>
+          <t>rKZVqoPPLDW+pcRbfbh7MxY7UndntrHNjhz7AMMyJG4=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>g6JqfR/T5vo0g4gDg/QRhg==</t>
+          <t>6KAlQZ9rXGUqYP7ubiCTNQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>p+3aY021qaNRalWBVkfLLrJ5GqLVsAPVuwJWZjh+5Lw=</t>
+          <t>A9ROz9+eJal1f6NUjjMCAuswPfj4lEK+sDk67ksm99g=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>XHIVcHl6SlT+qkf7oNKYuw==</t>
+          <t>ng1IVtzdwWB/lF3m2zj6DA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>uX1KrNRNoNhfkho1F4nRyKxp0zbql7WmRFIx0vDdbDA=</t>
+          <t>cqZH/T9MIvh+LemzoFgCNnj737gBPa0ZVOTQhZ/k7VM=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bkm9B7bDiB0xz1GnFOSDxw==</t>
+          <t>SPxm4OI4Jci5z7F8/UbzrA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Gbnl01JEY3zToy/rObQcgsfUrEzyhA92S2soqWiA4hM=</t>
+          <t>9Hp/pazCc23Cr9abWxTeAFXvZ3l7IcHW5Dxg/lXl3jQ=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ninr0cT5HXDlBYS/Bv3CQA==</t>
+          <t>rYq5uH2/aKnN5czhNBKIaQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TRna2FBjcP/DxZgRJT2wJCy5Fk/OgyL1pWmzfNdkai4=</t>
+          <t>31TiyytxmvRSi4/nG/YvVNq3ToXST9oWJo5toMp3KJw=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>lbSspM54Y9R3p5RWkWXYyw==;icKhrFpl85rJlivR0Fooog==</t>
+          <t>AC6ZdaQ9xkjFwJAcamy1tQ==;Y+wKspWVHWrtXFN6pYVK+Q==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>G6IgbJf52peZ4le40YUpVeXrw+LGtlBjqMzFM6rYKCE=;OVAACF/VicD2BNp5fV+9uSPhHGwYqnPVFkqe6WNycV4=</t>
+          <t>k/TZPz5px11FLxc4FhDmrLfGj4PNOnvNLGPqkzGitYg=;q/sela0lTLPf7r+R+OiQHLd/aYuO4xM/Mo8I5pnhyt8=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>P14ipVfU5Q+kK5AzC1/MVg==</t>
+          <t>bNvxRtUI5eEF0p3xOB+fYw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DH6WRwZIBlfCGUNafz+X50MfsIFgW65cqHcqMvulYDw=</t>
+          <t>4ItWRiGX/BekIGzCAn98o44pnZ9W4jW0n1WVp+jWKkI=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>akiV6vl4dK7AHYXyRoWItw==</t>
+          <t>c72Dgu+UBAj2OlQcE6efDQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>x1VxDsNW/lDY+ROAsK1sSSYvniNt9F4rQP1HDwd6CMM=</t>
+          <t>HCSe2oQR8Uhap7CWVs4PtRufLyZhtjkM2j+h6Nai/sY=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>WvvcGcca9XPg9R8JGIluaA==</t>
+          <t>4RnOp4JBA/q5+J2iINskOw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>egvGI1KTwIhoVr/nDg1dRhBf60F4QGrTZxRBJSDkQHE=</t>
+          <t>pspYaySx0Ex3Q3ynYJE8aW+z9oVoXxQj7Cz2qYn+KpI=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>hq/QOx9zWk2DfVOKC/JmbA==</t>
+          <t>0NPerFv65sBvnEaZOn/w6w==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AHp+Aj8otEG6a0Y6MccNksFJblxnodlWZaswNvIGPcg=</t>
+          <t>3Dl8hR2CGlNu7vIXXr3Gw//MBNrgX2ppGGwGn+mfrBs=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3Nru7mxY/Rzx+4UfHDCmHA==</t>
+          <t>R25nFqUIxsNoNrmFhn0aAQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Q9cHV+/O/9M4xsb0kuU17ettVaCoZdTBorngwy3aqvk=</t>
+          <t>uhtDFYeN/t8ZMQup/Ja76LiUCPdsISwcM73TeWktSHw=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ZL5kXdGhqtaDpGYlzW9D/A==</t>
+          <t>yE4XBY3jqQ9lD7JDk0D2WA==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bd8vjUvb1mSD6XVe3jZ8iUZysBicXinGEGUrdHM3UPw=</t>
+          <t>lsAe6b/z/h5yVHMsvwTq8p3QI8JuEDtMjhWsG31MxIE=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>flTog6ucoXQWZbEOFiNepQ==</t>
+          <t>ESR9Cj+YLm63y9J8WY6xLw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>JM0oKHbzy6Vd0e03WsDwuRSPLrd6bYcS48660JOhv8w=</t>
+          <t>ml9R/XMBYEsmr14m0ycystMl2AmQsRAoOZlTaUPdE7A=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>X6PsbZwf/PE6dg3bW5hb3Q==</t>
+          <t>PgitorGbqv+q6cl6pyjjdw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2CrZ2SY4Td/d9i8L6M0y55dXtQYcZUb5v634zSUxnkw=</t>
+          <t>DixkAdzBGSp1H32Cp1a+MYqIDLQt/jJSJuPsZDwgy1g=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RaU7tS4Woop4M7BSpME3kg==</t>
+          <t>gfxnm2UzDrkhIyPQ/AybEQ==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>NqBlPJ+erF1JR3yu9EKtER12btEXE3RM7NLMrT/Cpn0=</t>
+          <t>2fO0+FajkkKwBkTrmdPdebouZnRxH9SRKzPHJAiya9A=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>rWxsKasaXRbC16ZO4LkG8g==</t>
+          <t>lwYNZiHLlMcMszWOZtVIHA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ORGBQC+d2heC71yTZ30mkFWbVOlM410dVJKM1mjgauc=</t>
+          <t>BemMGMDVf6L0+KKUoZq4VtpCNyUZkTHh7ZOas9tKYc8=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>cvk7MQ88x/hw9IVkLeNwEA==</t>
+          <t>vd3JTVv+aoL6iMMBnzWcxQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2mOCjMXwuKMVogfq5eO14/HZxh6ZwxGpQAkBR70E0B8=</t>
+          <t>WyHG7yk7DBbK59ZoYnyiL20xTEuPu7qFfkP/Pd9q55Y=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>p8fBEHNVD5SquYeYauV61Q==</t>
+          <t>5OLE+7cQWQDdT1oSp0OPOQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>r5Y4B52TAUtl/MixJLkN4ZBJpaPWYv9nyLZYqqeGe3U=</t>
+          <t>c2jycUCDusQvaJG+Z0Ss0lCgFdhWPRLZNgZVTeWj3wo=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1cfei+Sh/q/F1YfsyCtieA==</t>
+          <t>0GJFFE/i7GHsqIcqJqKk4g==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CfPhRjC79C1cMZtQUrXJ9NHJLnSZh08WXF1cLquPPcc=</t>
+          <t>eZG3thFP/CDx5TRUVk+hyxOkrgQT0RQCRG/PE/MRqS4=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mOGlkjaQ4Fd4Qp2K61548w==</t>
+          <t>Zt890CwLF7C1RC5y/co0dg==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Wzh4GRB53rFSYWlHFJa1bnNCQH53zWHPYubGQ+e3PUM=</t>
+          <t>GH+GGNSQnRGBNkrrasgrKT8UOJ2oLMmzsiHFrr4vnr0=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WKsaCiq3TDa/OJnFA8tKlw==</t>
+          <t>sNStms3YxVe4CIT72O5oAw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0+lcU8264dogIMIFqx+20cqa7eBOFBGFBPQLtsz/7rk=</t>
+          <t>RyH0luZAqirRHgOFe4KtH4JbJVhiBQt7JLuSDZGxXAU=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4BcxuZtveimhAMM5IPYv0Q==</t>
+          <t>7Iom3xlO75bEhloPzuPiqw==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>T7q6Afdeh3BxhGfWyws4Cy8JVoRNvWsaCrhBsZIQbYg=</t>
+          <t>UdYNjr3jkL9H34FJUudx2FaBJ4bFgysUFpOmoV+isbY=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IodJC9RIZe0DAJdw8c7fKQ==</t>
+          <t>TPHJDV+ojOdFZW/o5Aul5g==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ncnkGuqm3Y+BGB80Qjgs4Ahvt8/mb7vC8D4AWFAc1WE=</t>
+          <t>CkmSJ2IZTlTc6ho5q/JWn/WboJsM5ys0Me0g8YcE5QE=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PmTO3l5UxqfHjsI1QvFbfw==</t>
+          <t>7VVBAQ8v4khRWrzYvhxO1A==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>/UUDt5IaJdcrMdpCakLnEBTPHRraDPaXo0FEyDyMsng=</t>
+          <t>/my448WlX8+lVFEFI/STXIEDAQdol/RjvCJQMN7i6JY=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SemLuExp8+0mQbvKRqdBeg==</t>
+          <t>DsTqhrYQoMxEx37xKSUNkg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>KUVFhJnHBj0Sv6MA8SZd6jvdQc6Jaop5K4tOVEvpESk=</t>
+          <t>OJy0GCWRYomQ05WV2mNYpquP9JcFWZidt7gT33KFa9g=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>JW37RD7J3zty7SYCcaK5dQ==</t>
+          <t>kUI4SgegUDBV95YdjDDxtQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>v//LIiljZummQVdk7kDvNOBVHpLwFIlhYugfDacmidQ=</t>
+          <t>v3BJyiyIheO9QD3gNRApmbtmOgCMHHLwOCSLBaZM8ko=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LhhiQ7Q65jCmFtjiFyyJxg==</t>
+          <t>CTeUuco6cua0ivLkGaWUjA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>OK8Yf8Pjq8lHAAY2lsJh8ij2kBDDci0Jd+nXukj1wQM=</t>
+          <t>kpMtBnU+s+gRKeEwPfPeMzjgZO2yw0j1ISOXOFw0mw0=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>P4QufN+yct2rvEEMEGGbpA==</t>
+          <t>11iQogr5GaZndiGTbDKPMA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>p1ui2BN18vmZyeNUSaHh+NATKDLuWd1uTEErpyvEAWw=</t>
+          <t>UoVIzgxBhCjFYz7p241ehkE6MmuvZvh9x1ZtjcT5S9A=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>VgoF4Oceq1GWaL5ujRX4Og==</t>
+          <t>bj3GoGylRy83AbRzF/kyNg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>N32HJRGXLfHgap9uf+PhJOxXjOxRggrSidcGxGuI2fE=</t>
+          <t>wRowk32oIDoOol5/NsndzNvYjeU72xRTf8nmuDR2u6M=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VVRGEigH3nU1nP54dC4Oxw==</t>
+          <t>CvsRsbi4T/xKA+vubp+zxg==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>mUTS8umX+X7uc4avsdrFWcoI0Jpa7fStWwuJYXtMsCw=</t>
+          <t>p6M8IUhbEf/EW6SLe48ydVgCkXOLgOA7mhaR96i91GQ=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CZiIPSXn/laqFYP/62vkvQ==</t>
+          <t>fqQfjOYwnqhKtEpr0NFeYA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SnBHC2PIgnxx59Fl0YcHdq9fOnB2cZcMKqhQi7Vbq2I=</t>
+          <t>FF//sBeuydB5xoQvZXiJfIYPiNqm09qo5SEopYiUOJE=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>qkdFiDCGEWe0Xorw+8RzKw==</t>
+          <t>o6D88l1ZFAyjxvEqE0u3wA==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>j0mMdoC7R+SXtogCQteqj14RcKZDUcPtpZHVPDjkL4M=</t>
+          <t>UdDRF8EZ73D3Y9A07q5OUBqKf/hpiKTxghUQ2zIpaMQ=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Xe/C5xqLYnq8O3D8ly/jTQ==</t>
+          <t>qiF34sk7j/0nheGR4KN/nQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tEHSD0H8EqlqbYc3KBrjm10lbg+p5M3UdZaR0EoX61E=</t>
+          <t>TweP1CM0l4/azCQJWvUjvVmBVLV0I0Rv89mY3xPXNBc=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Rw+8aRsre0DZtFvNG56w3A==</t>
+          <t>ZBoTPPxTppBRgwySf2SdRw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>LS/kwKugsVVZ1p/S6x2xquqBZ2JV8RweNUIEMq3ZWSE=</t>
+          <t>1keQlkXCzWUzwnWdT+fFlaWehG6v2OS3hWicidFZ4FE=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-20 07:40) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CONTROL DE COSTOS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>CONTROL DE COSTOS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=362f0557-5f53-45e4-a162-67584d13a444&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COMPARATIVO 10-2026</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0698e4be-cdc5-444c-af18-f7fb4a3b733f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2331,12 +2331,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>COMPARATIVO 10-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0698e4be-cdc5-444c-af18-f7fb4a3b733f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55">
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="81">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="89">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="90">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93">
@@ -3823,12 +3823,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8bdb45d1-c1c9-4ee3-9658-d4ab30fb67b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f04b41aa-2bd1-4166-8005-a78fcad04720&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="94">
@@ -3859,12 +3859,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f04b41aa-2bd1-4166-8005-a78fcad04720&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8bdb45d1-c1c9-4ee3-9658-d4ab30fb67b9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>417</v>
+        <v>430</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>417</v>
+        <v>430</v>
       </c>
     </row>
     <row r="115">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="119">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="120">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="122">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="124">
@@ -5958,7 +5958,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -6090,7 +6090,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
@@ -6310,7 +6310,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14">
@@ -6486,7 +6486,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -7922,7 +7922,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43">
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
     </row>
     <row r="65">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="98">
@@ -10830,7 +10830,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="103">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="104">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="106">
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="107">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="110">
@@ -11362,7 +11362,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="111">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="120">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="132">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="134">
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="139">
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="140">
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="147">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>191</v>
+        <v>163</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>121</v>
+        <v>134</v>
       </c>
     </row>
     <row r="153">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="173">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ujkTkhsOpCyCWTUdrKKRjg==</t>
+          <t>SVOrpxZmn3crXNZEA6rtWw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dVGLCnJwFoA9/5CZnTnReZFt/1DQ+FX202Aq+PEo1ps=</t>
+          <t>b+MBVwJkLEYNAXVlXximtNMNjqZCCMrkNauZh/D3Vk4=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sC7UCuuQNuskzQTHifaPSg==</t>
+          <t>XyH8alN1JvJSeLfNj97z0A==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TKST1qKC6Qn/0AB89Ywg7XfkDoN/Q0FAnT7lshxy4BQ=</t>
+          <t>3R15MN5+1q/M0VvPDYofzrwRJWSIK0cA23oFuekiGFo=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FdeoATesyVUPmiPgYwC8tQ==</t>
+          <t>Faze7NYA51u2SbbTYu2MAw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>fpMSB+gseT6ybdAUP56W7J6ymK78A00hsZRb/XxKlpQ=</t>
+          <t>J1MfFe159ZIGiCZOih0pBnHdUJdB4prZvQkHWPRHjmc=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>B5or5Qg5kY1uYfX2LFJo5w==</t>
+          <t>13hnNkSlALi6n93j3QMI/g==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>rKZVqoPPLDW+pcRbfbh7MxY7UndntrHNjhz7AMMyJG4=</t>
+          <t>aUtXCLfr5skaBf/6yLJbDYkXW7SV6UKKVRX5eSnhoAA=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6KAlQZ9rXGUqYP7ubiCTNQ==</t>
+          <t>478ROW58zbv/T/A06HF4Vg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>A9ROz9+eJal1f6NUjjMCAuswPfj4lEK+sDk67ksm99g=</t>
+          <t>byM3XmGElFyOrABo+bROSD02IqPjpMR0GU6smupt10k=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ng1IVtzdwWB/lF3m2zj6DA==</t>
+          <t>R28s2HV2IMT8rCV4c0PCqg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>cqZH/T9MIvh+LemzoFgCNnj737gBPa0ZVOTQhZ/k7VM=</t>
+          <t>CWuWFxcqEkW43Ki6HvVFT6sOu22hHHogLSVWi/KB1S0=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SPxm4OI4Jci5z7F8/UbzrA==</t>
+          <t>0iBOd0LRZvw4sOU6fCpV7Q==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9Hp/pazCc23Cr9abWxTeAFXvZ3l7IcHW5Dxg/lXl3jQ=</t>
+          <t>iWBqJbysH7vVaoqgwoNHnX6GLqs9b8GlM0P9qmhp6Fs=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>rYq5uH2/aKnN5czhNBKIaQ==</t>
+          <t>5Cm8mTURFpsPd1fI9MKNgg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>31TiyytxmvRSi4/nG/YvVNq3ToXST9oWJo5toMp3KJw=</t>
+          <t>CRGJ7OF7GwxkZxvdEueez2cXgNIZP8gdJcVjMKCf2xI=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AC6ZdaQ9xkjFwJAcamy1tQ==;Y+wKspWVHWrtXFN6pYVK+Q==</t>
+          <t>DIBPlR6dkkAjMJ8UkQPKMQ==;GgZo+dxvYU8qKtkGnH3lyg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>k/TZPz5px11FLxc4FhDmrLfGj4PNOnvNLGPqkzGitYg=;q/sela0lTLPf7r+R+OiQHLd/aYuO4xM/Mo8I5pnhyt8=</t>
+          <t>x7Oxn0bV49NvOtVpPNcs9jz1RFhI22Zi3T4Vm4WUso0=;7TT6LqjHo5hk9SBKmYvsP7tY1NA860EPoQ1yGNSOdlE=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>bNvxRtUI5eEF0p3xOB+fYw==</t>
+          <t>O5U8m9PJ9t3Ido1ESJjF3A==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4ItWRiGX/BekIGzCAn98o44pnZ9W4jW0n1WVp+jWKkI=</t>
+          <t>RK3ru4jdNXz59mdhkGYYbjOwomOVIjM8+nBofijtvn0=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>c72Dgu+UBAj2OlQcE6efDQ==</t>
+          <t>hzIzBrjHVdvcAD0RPTuhww==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HCSe2oQR8Uhap7CWVs4PtRufLyZhtjkM2j+h6Nai/sY=</t>
+          <t>V56ZnKGu0FU61w2UwyQSfJ9a558MJFpx6LLO5PRuMZE=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4RnOp4JBA/q5+J2iINskOw==</t>
+          <t>fZ4XzN3DJlNFCK0jhJZOWA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>pspYaySx0Ex3Q3ynYJE8aW+z9oVoXxQj7Cz2qYn+KpI=</t>
+          <t>tX76yDegWewPgknOHWWzM3G9dBQz38L20/FqXsGatTQ=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0NPerFv65sBvnEaZOn/w6w==</t>
+          <t>XoyrY4Afabf091+fhmrDWw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3Dl8hR2CGlNu7vIXXr3Gw//MBNrgX2ppGGwGn+mfrBs=</t>
+          <t>UoOWXJYQRgUYfUOLq+74M0yWmqgBQpF5P+JCy48HPms=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R25nFqUIxsNoNrmFhn0aAQ==</t>
+          <t>lD5wdHr+eNDy6RIR6gWaZQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>uhtDFYeN/t8ZMQup/Ja76LiUCPdsISwcM73TeWktSHw=</t>
+          <t>6z1tfz0eiRdFVcmsNwwfBSyxJRZ7CodJA19U2Flfksk=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>yE4XBY3jqQ9lD7JDk0D2WA==</t>
+          <t>3WaCCZZ62Xz0nquzjq3hng==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>lsAe6b/z/h5yVHMsvwTq8p3QI8JuEDtMjhWsG31MxIE=</t>
+          <t>ngy15Bq1ko9aE+bD1xIsjRCNvTLYIBmu2/6qAbjqac0=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ESR9Cj+YLm63y9J8WY6xLw==</t>
+          <t>NVg0Pn0wWla0LucPnOTPsg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ml9R/XMBYEsmr14m0ycystMl2AmQsRAoOZlTaUPdE7A=</t>
+          <t>VseeQhXRJZ97a8L1aDerZf217IfHs0LbPA8nT0q9iDs=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PgitorGbqv+q6cl6pyjjdw==</t>
+          <t>BrFF6zYfBrb8v/a3JiIkGQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>DixkAdzBGSp1H32Cp1a+MYqIDLQt/jJSJuPsZDwgy1g=</t>
+          <t>Sy4bp72vlfrpfBJlzp70hJq6u4di17M2UDPMk40YeVA=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>gfxnm2UzDrkhIyPQ/AybEQ==</t>
+          <t>WIkfEoAjbSBPh2wypsnF+A==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2fO0+FajkkKwBkTrmdPdebouZnRxH9SRKzPHJAiya9A=</t>
+          <t>flxnNTiTE9vfA1vwxObfOjbe2M0kOOVjHWXyqpYu+FY=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>lwYNZiHLlMcMszWOZtVIHA==</t>
+          <t>XUR7npLO3spA9qmSRhYoJA==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>BemMGMDVf6L0+KKUoZq4VtpCNyUZkTHh7ZOas9tKYc8=</t>
+          <t>9f6JIymIhuTlyqX6t50EzP48UEPPpxo7FsDTYgfKcMo=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>vd3JTVv+aoL6iMMBnzWcxQ==</t>
+          <t>EeQv327bqCjiRpnCF3Xbkw==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>WyHG7yk7DBbK59ZoYnyiL20xTEuPu7qFfkP/Pd9q55Y=</t>
+          <t>gR01RL+I32Dpu0Y/j7PF3Jp/CZ3Lqk5T8+x8CRSAv7s=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5OLE+7cQWQDdT1oSp0OPOQ==</t>
+          <t>7eQqX7QR7pubprjkbj6kdA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>c2jycUCDusQvaJG+Z0Ss0lCgFdhWPRLZNgZVTeWj3wo=</t>
+          <t>cRy7/Kr9GrPKlIE1Jql2Ohmh4w9w0AivWlUzk20/goY=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0GJFFE/i7GHsqIcqJqKk4g==</t>
+          <t>ViPNYUvk/qoWj12/E84OaQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>eZG3thFP/CDx5TRUVk+hyxOkrgQT0RQCRG/PE/MRqS4=</t>
+          <t>aaXf4ei7cIseTwSX1GBdKwA5TpF77NeDsWxbrLfv37I=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Zt890CwLF7C1RC5y/co0dg==</t>
+          <t>JYpK7cF0es3NjQd00Co+7w==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>GH+GGNSQnRGBNkrrasgrKT8UOJ2oLMmzsiHFrr4vnr0=</t>
+          <t>qv9Z1B+kImRLgEzd+npGi/9dZLGqjxlJFaDHYUl04HA=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>sNStms3YxVe4CIT72O5oAw==</t>
+          <t>rSFBacscYZcn1N77iuaYFQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RyH0luZAqirRHgOFe4KtH4JbJVhiBQt7JLuSDZGxXAU=</t>
+          <t>pt6p2WZRxOJfaZoNHbrnsupLYjgWwBZ258c7nkr2eNU=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>7Iom3xlO75bEhloPzuPiqw==</t>
+          <t>VHBvg2eslQkKay7gdoViMg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>UdYNjr3jkL9H34FJUudx2FaBJ4bFgysUFpOmoV+isbY=</t>
+          <t>tJ+Q/liYRyouU3cjdKKbjvEIUDjBbkh5RN/JbiP2K68=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TPHJDV+ojOdFZW/o5Aul5g==</t>
+          <t>F+k1XFGQGNQUsHVWYxbu4w==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CkmSJ2IZTlTc6ho5q/JWn/WboJsM5ys0Me0g8YcE5QE=</t>
+          <t>GQ3gwCm7osQnRRJzP0hmCgg4AV7KwLJjPBcOoP2V++I=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>7VVBAQ8v4khRWrzYvhxO1A==</t>
+          <t>+7e1kXU55Sb+J5LVqch96A==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>/my448WlX8+lVFEFI/STXIEDAQdol/RjvCJQMN7i6JY=</t>
+          <t>upyB1S+3NgWPwdnbUq2lyIfzq0zMii1mmieFn1O/3HE=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DsTqhrYQoMxEx37xKSUNkg==</t>
+          <t>+/vqJnlisgo47cYbXsMbNg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>OJy0GCWRYomQ05WV2mNYpquP9JcFWZidt7gT33KFa9g=</t>
+          <t>ZpSpDWxvuIhpcQwW7p6vSTXUngRtBjWwXWGsplHEbsQ=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>kUI4SgegUDBV95YdjDDxtQ==</t>
+          <t>KuimfutJiOIimHaPVVfbuw==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>v3BJyiyIheO9QD3gNRApmbtmOgCMHHLwOCSLBaZM8ko=</t>
+          <t>hr81Z67f37qVq3sXpveQSMyP20VOFVTyppOrbANy+as=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CTeUuco6cua0ivLkGaWUjA==</t>
+          <t>s73viZo7akVbab5v1cP7cg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>kpMtBnU+s+gRKeEwPfPeMzjgZO2yw0j1ISOXOFw0mw0=</t>
+          <t>/9LAsF0zE40v8aRlBQTST6sH5HK488z+0fbpmHXH1ko=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>11iQogr5GaZndiGTbDKPMA==</t>
+          <t>tmr047KJtvEWqbh0WQDk4w==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>UoVIzgxBhCjFYz7p241ehkE6MmuvZvh9x1ZtjcT5S9A=</t>
+          <t>yxbpRyd30hHePIpEyHwguFuqpA8UYO+IgbH2iCNa3Yo=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>bj3GoGylRy83AbRzF/kyNg==</t>
+          <t>SQN9+PRWKm+akQKCwKuXfg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>wRowk32oIDoOol5/NsndzNvYjeU72xRTf8nmuDR2u6M=</t>
+          <t>ybcFPKMgyrluwdkgZy7Ri0+URsW7RK0f3I93dR6xrV4=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CvsRsbi4T/xKA+vubp+zxg==</t>
+          <t>lhpdepcEvz59YFK7p/S+sA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>p6M8IUhbEf/EW6SLe48ydVgCkXOLgOA7mhaR96i91GQ=</t>
+          <t>nkpDK11b06KC6lmsPxaPcPnJrNa5ZB+36/3oYh3J5xE=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>fqQfjOYwnqhKtEpr0NFeYA==</t>
+          <t>03SpcXhD7lsboB6iD0GY8A==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>FF//sBeuydB5xoQvZXiJfIYPiNqm09qo5SEopYiUOJE=</t>
+          <t>dII8ss3sqII7r74Hbu/Kucq8AKOfbvgw04DLHYQfBtE=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>o6D88l1ZFAyjxvEqE0u3wA==</t>
+          <t>RVSFru/iS8I4g2gjq77PTg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>UdDRF8EZ73D3Y9A07q5OUBqKf/hpiKTxghUQ2zIpaMQ=</t>
+          <t>bEUVJvu1Aw5ehLNX6Sb2j8pzrEoDzhRIDM6wtxo+ArQ=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>qiF34sk7j/0nheGR4KN/nQ==</t>
+          <t>0fxIyLkD2LLREPEwReQNgA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TweP1CM0l4/azCQJWvUjvVmBVLV0I0Rv89mY3xPXNBc=</t>
+          <t>hrmVrQtnWTmfiCCMafgKdKW52TjGV/+2Q657WjtASpk=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ZBoTPPxTppBRgwySf2SdRw==</t>
+          <t>pBBEqZUXPHCnTvjcfi1hUA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1keQlkXCzWUzwnWdT+fFlaWehG6v2OS3hWicidFZ4FE=</t>
+          <t>Ug7fZbO0KpnoIxZRWA5WA2UJ2ylB5CVOT/8iohK11XI=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-21 07:40) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="53">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="55">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="81">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="89">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="91">
@@ -3751,12 +3751,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="97">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="99">
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="100">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>430</v>
+        <v>444</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>430</v>
+        <v>444</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="119">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="124">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="137">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5427,7 +5427,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138">
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5623,12 +5623,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5659,12 +5659,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5695,12 +5695,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=17a76e1b-4a1d-4f00-88ee-66022635680c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=17a76e1b-4a1d-4f00-88ee-66022635680c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14">
@@ -7746,7 +7746,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="72">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="97">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="98">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="106">
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="L106" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="109">
@@ -11362,7 +11362,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="111">
@@ -11666,7 +11666,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="120">
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="124">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="132">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="134">
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="139">
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="147">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>163</v>
+        <v>137</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="156">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="173">
@@ -14866,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="181">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="188">
@@ -17046,7 +17046,7 @@
         </is>
       </c>
       <c r="L220" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="221">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="224">
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SVOrpxZmn3crXNZEA6rtWw==</t>
+          <t>a30IGSqCfV+SpNnal4hx3Q==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>b+MBVwJkLEYNAXVlXximtNMNjqZCCMrkNauZh/D3Vk4=</t>
+          <t>UJUEIL98h/H1nN5fREdWRgmtToGVFT40p46vaIcux4M=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XyH8alN1JvJSeLfNj97z0A==</t>
+          <t>z/3uLCz0HD23PUYcg5sX1w==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3R15MN5+1q/M0VvPDYofzrwRJWSIK0cA23oFuekiGFo=</t>
+          <t>r7ecaAU6b6BS65CsDghxS1aM07sYVGDbFV+OzHr6KjQ=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Faze7NYA51u2SbbTYu2MAw==</t>
+          <t>J3/D7ck0a6g4xExg2hDjKA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>J1MfFe159ZIGiCZOih0pBnHdUJdB4prZvQkHWPRHjmc=</t>
+          <t>X+QpNn9ghYzgaQKaT3ZSD6SmQHt7H3LnbT1VOhKYIz8=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13hnNkSlALi6n93j3QMI/g==</t>
+          <t>sgBLbqiJWKAZPQGMMB49CA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>aUtXCLfr5skaBf/6yLJbDYkXW7SV6UKKVRX5eSnhoAA=</t>
+          <t>k6w0RFUlF3BQZjCKXeLmWDYcHIumwYaYsxjI1MbZDo8=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>478ROW58zbv/T/A06HF4Vg==</t>
+          <t>m4wdyCCmfzQLue4Y86mqjw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>byM3XmGElFyOrABo+bROSD02IqPjpMR0GU6smupt10k=</t>
+          <t>4ga3NFt8dytXb1XOqh/pNRZgtB2mGRBlJJ/0k2czELs=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>R28s2HV2IMT8rCV4c0PCqg==</t>
+          <t>cnd8xKMQGk/4RJ1ZwZs+FA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CWuWFxcqEkW43Ki6HvVFT6sOu22hHHogLSVWi/KB1S0=</t>
+          <t>wdOS2KaAhS+02BuT2dUvb7kLzI1tZsEXzxjBh2u7ric=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0iBOd0LRZvw4sOU6fCpV7Q==</t>
+          <t>71mQwHLtZJXUUeFOo0/Lqg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>iWBqJbysH7vVaoqgwoNHnX6GLqs9b8GlM0P9qmhp6Fs=</t>
+          <t>hXZz2kxi59Wr1p2M5shmK1c5rnQy5+FEnasy2vBCZU8=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5Cm8mTURFpsPd1fI9MKNgg==</t>
+          <t>HvEv4dxmNiRP1uYaVhNd0g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CRGJ7OF7GwxkZxvdEueez2cXgNIZP8gdJcVjMKCf2xI=</t>
+          <t>/utY2FDGLVXqoCYixpU1Rk/Qg7am03zvkbg2oSrLPmg=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DIBPlR6dkkAjMJ8UkQPKMQ==;GgZo+dxvYU8qKtkGnH3lyg==</t>
+          <t>336k1nJ6t0p2QSR3A52dbA==;YIrrxMk6GohwJYpA+R1mAw==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>x7Oxn0bV49NvOtVpPNcs9jz1RFhI22Zi3T4Vm4WUso0=;7TT6LqjHo5hk9SBKmYvsP7tY1NA860EPoQ1yGNSOdlE=</t>
+          <t>SHYZx/YPG9sCawasSCx6KCzHrq4p0ELdb8byYE/62vM=;rtq0LMhbcGhPxEG3SO3Y/Krg9fJiPC6646YcAR24Kyk=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>O5U8m9PJ9t3Ido1ESJjF3A==</t>
+          <t>2Gz5ZSSTKZnEVy/CGTAlmQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RK3ru4jdNXz59mdhkGYYbjOwomOVIjM8+nBofijtvn0=</t>
+          <t>OEhReB7rPk7gouQarlDDQO9RhjorYmZQpkxHhfMhvQc=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>hzIzBrjHVdvcAD0RPTuhww==</t>
+          <t>nvOAYqHVHCBvRXB9Usi6hQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>V56ZnKGu0FU61w2UwyQSfJ9a558MJFpx6LLO5PRuMZE=</t>
+          <t>43e7MztnBnlcWXAhWJZXphebJuyCHjul7Idn82MiW/4=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>fZ4XzN3DJlNFCK0jhJZOWA==</t>
+          <t>GE9EihophMH2kelkFA70JA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>tX76yDegWewPgknOHWWzM3G9dBQz38L20/FqXsGatTQ=</t>
+          <t>/lhrYzNh12eoC4+1fw6UDYdiE7qT+tWkE3x+oDlS7io=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>XoyrY4Afabf091+fhmrDWw==</t>
+          <t>1zRdGmF7rHv1mcRWDgmzXw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>UoOWXJYQRgUYfUOLq+74M0yWmqgBQpF5P+JCy48HPms=</t>
+          <t>G0vR+bvCyR4pxggbG2ZcwM33nPoTBCkY6aqyKxSrPwU=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>lD5wdHr+eNDy6RIR6gWaZQ==</t>
+          <t>mhWEHLix3DRbfBHpX3UXrA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6z1tfz0eiRdFVcmsNwwfBSyxJRZ7CodJA19U2Flfksk=</t>
+          <t>Ar+1liyUPD/tMjqDWReS4jTFmLS5SO2vKGguPzXyVO8=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3WaCCZZ62Xz0nquzjq3hng==</t>
+          <t>1PzVqO19crMrJHsOf1zwqQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ngy15Bq1ko9aE+bD1xIsjRCNvTLYIBmu2/6qAbjqac0=</t>
+          <t>R9dwzWPpnX5aigMcQtcdbLRHfz+U+BRi8Gr4wdw2Uk0=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NVg0Pn0wWla0LucPnOTPsg==</t>
+          <t>Bxr3A+HBMYixttn2lpYPHw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>VseeQhXRJZ97a8L1aDerZf217IfHs0LbPA8nT0q9iDs=</t>
+          <t>koUbnUIaIOTVQ/x80KejkiLIOSwtEAhhDQrUit6KjHI=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BrFF6zYfBrb8v/a3JiIkGQ==</t>
+          <t>OftAI9N2437nFdTFembBOg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sy4bp72vlfrpfBJlzp70hJq6u4di17M2UDPMk40YeVA=</t>
+          <t>D3O9jLKIximjH0LdFmJv3btVdvBhp9QaO9SGv4WNyeY=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>WIkfEoAjbSBPh2wypsnF+A==</t>
+          <t>P3LItdoXAYNAvS+4JfC2KQ==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>flxnNTiTE9vfA1vwxObfOjbe2M0kOOVjHWXyqpYu+FY=</t>
+          <t>OA3Zr/uJOGQkU3xJ58JmOWfsjm9gYvKwe2pOMLVVnZY=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>XUR7npLO3spA9qmSRhYoJA==</t>
+          <t>nevrTRvHK4FRrcmx7svE2Q==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>9f6JIymIhuTlyqX6t50EzP48UEPPpxo7FsDTYgfKcMo=</t>
+          <t>yyJCwjNwmz8Yumk0NihavL8BzMOwGUx8pOFnKX6vyDs=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>EeQv327bqCjiRpnCF3Xbkw==</t>
+          <t>ua20eSnw8SAypJ4dT6xFMg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>gR01RL+I32Dpu0Y/j7PF3Jp/CZ3Lqk5T8+x8CRSAv7s=</t>
+          <t>VYoR46kgO3mfNbbawwPvIexfv3JMs2dkP/787m+4hwU=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>7eQqX7QR7pubprjkbj6kdA==</t>
+          <t>7xWi87RO5+6J4RyJfsRNmA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>cRy7/Kr9GrPKlIE1Jql2Ohmh4w9w0AivWlUzk20/goY=</t>
+          <t>uZzY7OzMro6MjiGRb3tNzvZD2sOkPFUHqjYvRiO1NaM=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ViPNYUvk/qoWj12/E84OaQ==</t>
+          <t>n0+REq3DfCSyo8lvFu29Lg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>aaXf4ei7cIseTwSX1GBdKwA5TpF77NeDsWxbrLfv37I=</t>
+          <t>OdjjRkeCzzyC3Y4RzRoiE919zhukax+7huI0a6cq34w=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>JYpK7cF0es3NjQd00Co+7w==</t>
+          <t>D7+SKaONXfkLkaErsmY6rw==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>qv9Z1B+kImRLgEzd+npGi/9dZLGqjxlJFaDHYUl04HA=</t>
+          <t>YvBrlW8i7v3v6E6EcHERJ88VG2rH55HMV9/CyOwJJmw=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>rSFBacscYZcn1N77iuaYFQ==</t>
+          <t>5ODbqkx7/sZJOus+0J9h8Q==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>pt6p2WZRxOJfaZoNHbrnsupLYjgWwBZ258c7nkr2eNU=</t>
+          <t>dfaLfXSM08eseWfE/16t40J/t3fysMV5bhcm6SRBrtQ=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>VHBvg2eslQkKay7gdoViMg==</t>
+          <t>r9IA9QeXsPKbGABTrc2RmQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>tJ+Q/liYRyouU3cjdKKbjvEIUDjBbkh5RN/JbiP2K68=</t>
+          <t>qsN26C11SJ7pTM68rffZCNzt/vBee+s3k4OhlUYx6fI=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>F+k1XFGQGNQUsHVWYxbu4w==</t>
+          <t>1ojRp3vJAAlbrcSr+aFiRA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>GQ3gwCm7osQnRRJzP0hmCgg4AV7KwLJjPBcOoP2V++I=</t>
+          <t>pCJqjUoX2om0bERYG+0rOiu+ZKjZ5FgubOVpcxiIVtw=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>+7e1kXU55Sb+J5LVqch96A==</t>
+          <t>n0zfEySpuUsGnjtQsjlnYg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>upyB1S+3NgWPwdnbUq2lyIfzq0zMii1mmieFn1O/3HE=</t>
+          <t>4hXCzCVC+8N+Qy1JwkReYlG+/BC54RzeXLD6q6CW3ww=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>+/vqJnlisgo47cYbXsMbNg==</t>
+          <t>ZrzjxngGkN2+hOOyhvesEg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ZpSpDWxvuIhpcQwW7p6vSTXUngRtBjWwXWGsplHEbsQ=</t>
+          <t>nen6+mbuo6bMuHVWdEKOGvE8ONYoLB3z6CcwcT5kckc=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KuimfutJiOIimHaPVVfbuw==</t>
+          <t>X6sDEXQqjeWQKLIESlDuXg==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>hr81Z67f37qVq3sXpveQSMyP20VOFVTyppOrbANy+as=</t>
+          <t>+PQIg8gjQUc1ObpTx/ubNPzUaFqauD0tB9E5MCglAwI=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>s73viZo7akVbab5v1cP7cg==</t>
+          <t>JKmqrPHppreDYg3dj0Or4w==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>/9LAsF0zE40v8aRlBQTST6sH5HK488z+0fbpmHXH1ko=</t>
+          <t>5ewExYEHDp6zSrO/Lyj970NFEfyetasQKywY7jw/6U8=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>tmr047KJtvEWqbh0WQDk4w==</t>
+          <t>NBbZCrHSU5aS/PMuUc/WHA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>yxbpRyd30hHePIpEyHwguFuqpA8UYO+IgbH2iCNa3Yo=</t>
+          <t>MXBtgCVotNYHZOLiiRV51J2m8ODDbfCebzYc2EkalEI=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SQN9+PRWKm+akQKCwKuXfg==</t>
+          <t>FY06iTEZY1j3qOqEF2xxmg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ybcFPKMgyrluwdkgZy7Ri0+URsW7RK0f3I93dR6xrV4=</t>
+          <t>SHLIMa+ReImnozURu7lvX76qWJKQozlqUQ+9mmzWe3s=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>lhpdepcEvz59YFK7p/S+sA==</t>
+          <t>UNbVHphywF/BA0vSHPYsGA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nkpDK11b06KC6lmsPxaPcPnJrNa5ZB+36/3oYh3J5xE=</t>
+          <t>s8weVOCgX5FF3Wa0Y2vBSivl7NsLCcw1WuxKKnSeX3Q=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>03SpcXhD7lsboB6iD0GY8A==</t>
+          <t>BjdCJd+pYISiYzVTBvw9/g==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>dII8ss3sqII7r74Hbu/Kucq8AKOfbvgw04DLHYQfBtE=</t>
+          <t>afKV5tH/S3FVeacLTNxj5cU86NFqtCFXFLihAVKzuT8=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>RVSFru/iS8I4g2gjq77PTg==</t>
+          <t>xe8uko+m9dwctJr7sSWRVQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>bEUVJvu1Aw5ehLNX6Sb2j8pzrEoDzhRIDM6wtxo+ArQ=</t>
+          <t>7uEsGKWElzIQLACj6r+N9LRy8UhkW6L4CMjeMc6Nh04=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>0fxIyLkD2LLREPEwReQNgA==</t>
+          <t>hlrQCRlg+WwvQTJEmFJGtw==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>hrmVrQtnWTmfiCCMafgKdKW52TjGV/+2Q657WjtASpk=</t>
+          <t>ws+aBmc9wyxEtsySDoezf3w260MvpRnUWjBKnYlfUYE=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>pBBEqZUXPHCnTvjcfi1hUA==</t>
+          <t>TGaCrfEPBAP3DQIuX6P1oQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Ug7fZbO0KpnoIxZRWA5WA2UJ2ylB5CVOT/8iohK11XI=</t>
+          <t>FUw+fki0ZAKuxclsMX9/LqW5UL+F0L8PzSDQtPdKric=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-22 07:40) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="46">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="81">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>336</v>
+        <v>347</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="89">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fc182951-77ad-488d-8feb-5acc78e0c7e9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="97">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="98">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="99">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="109">
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>444</v>
+        <v>494</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>444</v>
+        <v>494</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="119">
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="120">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="124">
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14">
@@ -6486,7 +6486,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65">
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="97">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="98">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="103">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="106">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>336</v>
+        <v>347</v>
       </c>
     </row>
     <row r="110">
@@ -11666,7 +11666,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="117">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="120">
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="132">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="134">
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="139">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>148</v>
+        <v>198</v>
       </c>
     </row>
     <row r="153">
@@ -13530,7 +13530,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="155">
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="156">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="173">
@@ -14866,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="181">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="188">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>a30IGSqCfV+SpNnal4hx3Q==</t>
+          <t>O4cvVP9/Xx58ML4tZrzOZw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>UJUEIL98h/H1nN5fREdWRgmtToGVFT40p46vaIcux4M=</t>
+          <t>eMYWBZPt0KxXUTcXhXS0Zk0DYWgfOHEd/k9r8ZPXyUw=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>z/3uLCz0HD23PUYcg5sX1w==</t>
+          <t>Pmi7nj60bdw+rMIx5jmFTg==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>r7ecaAU6b6BS65CsDghxS1aM07sYVGDbFV+OzHr6KjQ=</t>
+          <t>VrLqBkt5BeGDYro7bSrtHrOo59ceSIq7ph36xGJ87yw=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>J3/D7ck0a6g4xExg2hDjKA==</t>
+          <t>QXn899yoSB5l2rqtROCL+A==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>X+QpNn9ghYzgaQKaT3ZSD6SmQHt7H3LnbT1VOhKYIz8=</t>
+          <t>FSx3E5DsmEMRjpawlwPly3CmvOghHto66fePzNbC5mo=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sgBLbqiJWKAZPQGMMB49CA==</t>
+          <t>BJV/qASEuG1BXgKmX/d3xQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>k6w0RFUlF3BQZjCKXeLmWDYcHIumwYaYsxjI1MbZDo8=</t>
+          <t>JMHiAG4MPlf9d41m4GFSqcndqqd6s4rNrfDpLCtD1dI=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>m4wdyCCmfzQLue4Y86mqjw==</t>
+          <t>Dg1bKRYag2aABe3XKcRK3A==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4ga3NFt8dytXb1XOqh/pNRZgtB2mGRBlJJ/0k2czELs=</t>
+          <t>gIZCwi9Zcs/gaTZ3i/fBhZlGpKdxirYeTqaZ5gnM9LM=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>cnd8xKMQGk/4RJ1ZwZs+FA==</t>
+          <t>D0jh/907CqYy2aZA6pvYPA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>wdOS2KaAhS+02BuT2dUvb7kLzI1tZsEXzxjBh2u7ric=</t>
+          <t>oQJHzS9r/gSkr6FIzuYS7ZJ0j2DM15nDgGvYjE9d4Ps=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>71mQwHLtZJXUUeFOo0/Lqg==</t>
+          <t>IxQsk4717oNdhSL3zbJskQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>hXZz2kxi59Wr1p2M5shmK1c5rnQy5+FEnasy2vBCZU8=</t>
+          <t>HtwSsN1YKUvJ5j64CPMXcYCJatw4t4dgwXkncYcg1co=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HvEv4dxmNiRP1uYaVhNd0g==</t>
+          <t>xreDgD+InyzW5qGR6ABrpQ==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>/utY2FDGLVXqoCYixpU1Rk/Qg7am03zvkbg2oSrLPmg=</t>
+          <t>Rn2plG6EFJbLQspMYaWV1ZG+baoCmDR9q/gOFCIqI5Y=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>336k1nJ6t0p2QSR3A52dbA==;YIrrxMk6GohwJYpA+R1mAw==</t>
+          <t>AhvJRiokyfDaA2xO+XRsCQ==;oenNyZEnKRHb8yMxbjR6dQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SHYZx/YPG9sCawasSCx6KCzHrq4p0ELdb8byYE/62vM=;rtq0LMhbcGhPxEG3SO3Y/Krg9fJiPC6646YcAR24Kyk=</t>
+          <t>xPKu//NxY6Xs+osMlt92NUmD8DmpchTtGvAaVpk5bAk=;RrZKrpnMGDT0/yy5kMtz4BfQcxw8RxpvUErk0AOYMFU=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2Gz5ZSSTKZnEVy/CGTAlmQ==</t>
+          <t>rcF6JnDpoAkv4tNwjwg2Kg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>OEhReB7rPk7gouQarlDDQO9RhjorYmZQpkxHhfMhvQc=</t>
+          <t>HYGlcCxscFFqIk9ZORr5S0PhjeL+AeNMjDZGxnYE9EA=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>nvOAYqHVHCBvRXB9Usi6hQ==</t>
+          <t>742H14bSbrO7FOqRS8nPWw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>43e7MztnBnlcWXAhWJZXphebJuyCHjul7Idn82MiW/4=</t>
+          <t>XcD0gQvwqvBuY0m2HmEri4CYbPftDdYVME34enWCkr8=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GE9EihophMH2kelkFA70JA==</t>
+          <t>fX9A2x/3QudaK9uAVjpNXQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>/lhrYzNh12eoC4+1fw6UDYdiE7qT+tWkE3x+oDlS7io=</t>
+          <t>5beYJzMObkxtLZeyafsgJq586dCKgYaL1QkSQdznAa0=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1zRdGmF7rHv1mcRWDgmzXw==</t>
+          <t>+OWngrsREjaEmGCz/xbc/Q==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>G0vR+bvCyR4pxggbG2ZcwM33nPoTBCkY6aqyKxSrPwU=</t>
+          <t>kF4XtyJKTWz4vC5oM3/QkxxGtUegm/frUP7l9y8Gtx4=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>mhWEHLix3DRbfBHpX3UXrA==</t>
+          <t>Yt7p2jMc51AwKZ4VrUBqfw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ar+1liyUPD/tMjqDWReS4jTFmLS5SO2vKGguPzXyVO8=</t>
+          <t>QPFIod8DRb1qK9Ac9VjVZ+zd8oskxsk7gcDzlxOVWLg=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1PzVqO19crMrJHsOf1zwqQ==</t>
+          <t>7vXHbLviy0ohfTDVmYJa7A==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>R9dwzWPpnX5aigMcQtcdbLRHfz+U+BRi8Gr4wdw2Uk0=</t>
+          <t>er+ya3qP0zn7JEugSaSA4MdaJYr3dyye6BiFhPRYisk=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bxr3A+HBMYixttn2lpYPHw==</t>
+          <t>9GXsbO1lK28f5JFoalsXCg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>koUbnUIaIOTVQ/x80KejkiLIOSwtEAhhDQrUit6KjHI=</t>
+          <t>mpQJJrA/sdnr6KkqWrmfT3JuFh0K8jZTxp3kyQMpl04=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OftAI9N2437nFdTFembBOg==</t>
+          <t>p39GXVK7N4qA+/ulB20khg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D3O9jLKIximjH0LdFmJv3btVdvBhp9QaO9SGv4WNyeY=</t>
+          <t>09a9HPIITIBlTJDkYy5aw6TvgD48pNrxwVmSil8nvBw=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>P3LItdoXAYNAvS+4JfC2KQ==</t>
+          <t>XznRNMLRbWh8SHApEsN4vw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>OA3Zr/uJOGQkU3xJ58JmOWfsjm9gYvKwe2pOMLVVnZY=</t>
+          <t>lY+jvshCrRn0rJ6gbMwDJ1v5QbpgTEOpBRy0DKbLGs8=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>nevrTRvHK4FRrcmx7svE2Q==</t>
+          <t>DgvpG8OpRBihjDO0oAV0tQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>yyJCwjNwmz8Yumk0NihavL8BzMOwGUx8pOFnKX6vyDs=</t>
+          <t>Sx7XD11nu+BdExnraiszCoK0JM6IjKuwdjosYUb+yFg=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ua20eSnw8SAypJ4dT6xFMg==</t>
+          <t>+7mMDh7zxKCiZbwQG8IiWw==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>VYoR46kgO3mfNbbawwPvIexfv3JMs2dkP/787m+4hwU=</t>
+          <t>MrKuvoMl1eOn7kY/Unwl68ofqMyh9nLLtbUIMvwKGwo=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>7xWi87RO5+6J4RyJfsRNmA==</t>
+          <t>UC/LL5F16KFVPUThAqOwHg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>uZzY7OzMro6MjiGRb3tNzvZD2sOkPFUHqjYvRiO1NaM=</t>
+          <t>DgTKr2gL3IrWQe5r8gxKivllDBRrxiRW8nw2jno0W0U=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>n0+REq3DfCSyo8lvFu29Lg==</t>
+          <t>EhbCIn6aN0dd1aEZ6EnD2Q==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>OdjjRkeCzzyC3Y4RzRoiE919zhukax+7huI0a6cq34w=</t>
+          <t>OVgiV5yYUCNC9ACmwzMt62sPAJENv9vkIoVf0ldbYK0=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>D7+SKaONXfkLkaErsmY6rw==</t>
+          <t>3god9D91mBEbfl+7QpDGog==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>YvBrlW8i7v3v6E6EcHERJ88VG2rH55HMV9/CyOwJJmw=</t>
+          <t>luiLpaNd/9oY4lS4yhJi78wDTQeBOvh+QbzKIf86q/A=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>5ODbqkx7/sZJOus+0J9h8Q==</t>
+          <t>374zRE9aRSy2zuc10Y2BaQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dfaLfXSM08eseWfE/16t40J/t3fysMV5bhcm6SRBrtQ=</t>
+          <t>zLcSzcdMfbTB4wfPdNrYMng7FrsjCVtU73ydwnj2d+c=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>r9IA9QeXsPKbGABTrc2RmQ==</t>
+          <t>zo7fqAasbAK+tE/JA2j4aA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>qsN26C11SJ7pTM68rffZCNzt/vBee+s3k4OhlUYx6fI=</t>
+          <t>q+v48XnPUQFUu6CPD4BtsGVWixFegnfiSsdg09YdfHY=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1ojRp3vJAAlbrcSr+aFiRA==</t>
+          <t>2+6RaUd4MGK9TgQuAmDlSg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>pCJqjUoX2om0bERYG+0rOiu+ZKjZ5FgubOVpcxiIVtw=</t>
+          <t>kk7JB0OsYyXt1/UEkAo4r4Wj7a2jTpN2VX1Eo/wPuZo=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>n0zfEySpuUsGnjtQsjlnYg==</t>
+          <t>0zRFc0TehUJWwldwCyEcmQ==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>4hXCzCVC+8N+Qy1JwkReYlG+/BC54RzeXLD6q6CW3ww=</t>
+          <t>Oo+fB6HETo/+mR1fi+KAXZ2S3LCGqm7fu5z4OFdqGc0=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ZrzjxngGkN2+hOOyhvesEg==</t>
+          <t>+zZGK1ZauiGRcxLrh5eI5w==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>nen6+mbuo6bMuHVWdEKOGvE8ONYoLB3z6CcwcT5kckc=</t>
+          <t>cqZ2hYwltzN4KXkZTHmsyqDSAvAcSHFQB98IT56D4P0=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>X6sDEXQqjeWQKLIESlDuXg==</t>
+          <t>2RmI+Kjkhg42oEjaam3p3A==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>+PQIg8gjQUc1ObpTx/ubNPzUaFqauD0tB9E5MCglAwI=</t>
+          <t>amV9yH0PnxRSRIEG69Qb1rH5/18sfMSIOU0PPN0ZACY=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>JKmqrPHppreDYg3dj0Or4w==</t>
+          <t>v9L2ZDYSa6hDbQxyjLhJIg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>5ewExYEHDp6zSrO/Lyj970NFEfyetasQKywY7jw/6U8=</t>
+          <t>UBIkumGy7Dg/iRbvtQH8b7OZVBCQdLjraUPovoGE9C8=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NBbZCrHSU5aS/PMuUc/WHA==</t>
+          <t>yDuvyPfoxM4nRYmuDSK/IQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MXBtgCVotNYHZOLiiRV51J2m8ODDbfCebzYc2EkalEI=</t>
+          <t>DnjxsMXC4cX7toATlKcIDzxlMOzPegiVo4rx2h59sVs=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FY06iTEZY1j3qOqEF2xxmg==</t>
+          <t>GaRcKgG+SUi92e/y/qWmkQ==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SHLIMa+ReImnozURu7lvX76qWJKQozlqUQ+9mmzWe3s=</t>
+          <t>cs3bXej4mY/FbfgKWzBdTzKIZKyfSWsNnvED6+E1HDI=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>UNbVHphywF/BA0vSHPYsGA==</t>
+          <t>19U61Aa8WgXn77hQnPrfSA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>s8weVOCgX5FF3Wa0Y2vBSivl7NsLCcw1WuxKKnSeX3Q=</t>
+          <t>PjQ1Q9YZlpUeQF8Ea+gpUEZmMky1g0A4RRxLaAX0ve0=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BjdCJd+pYISiYzVTBvw9/g==</t>
+          <t>IjP7EhelOC21jfvtXYyi8g==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>afKV5tH/S3FVeacLTNxj5cU86NFqtCFXFLihAVKzuT8=</t>
+          <t>sEaZ6FPBlyg3NU+go/GLNxvkH4He35dsC/NOV6213/s=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>xe8uko+m9dwctJr7sSWRVQ==</t>
+          <t>a52XR0Lta77KywGyY9NsRg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>7uEsGKWElzIQLACj6r+N9LRy8UhkW6L4CMjeMc6Nh04=</t>
+          <t>t4tMzcS3SYO+d9nT81oSN2hTPUMicbLUYk/Oz4x+Gg0=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>hlrQCRlg+WwvQTJEmFJGtw==</t>
+          <t>aGQoKSXImmFKxGa54ZkpAg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ws+aBmc9wyxEtsySDoezf3w260MvpRnUWjBKnYlfUYE=</t>
+          <t>kragnLIJZJtyE8LVa2LOWMwJgz37BO731nvTCTvLUrM=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TGaCrfEPBAP3DQIuX6P1oQ==</t>
+          <t>9NhhQPd92VqhwOVdAqbnog==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>FUw+fki0ZAKuxclsMX9/LqW5UL+F0L8PzSDQtPdKric=</t>
+          <t>6fk1P7UWpydsV30BBRKIKEQQ7Bu/2N3eKu1pFwP8bqE=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-23 07:40) - 120 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -1791,12 +1791,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>CASH FLOW</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6339ca7-bf01-48b1-a5ce-930d679671a2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CASH FLOW</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6339ca7-bf01-48b1-a5ce-930d679671a2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>INVERSION FINANCIERA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>INVERSION FINANCIERA</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=adc9bc9c-d24d-44ee-b04b-e4050a68027e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>46</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="55">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57">
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -2619,12 +2619,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2655,12 +2655,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
@@ -2691,12 +2691,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="81">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="86">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="87">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="89">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=785ded3c-9ed4-4463-8373-7992a07cc40c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c4fb5d8-ccf7-4e0a-8361-362399f22c0c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="95">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="97">
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="100">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>494</v>
+        <v>507</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>494</v>
+        <v>507</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="116">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="119">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="124">
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -6222,7 +6222,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14">
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16">
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -7746,7 +7746,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
@@ -7878,7 +7878,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
@@ -9050,7 +9050,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>46</v>
+        <v>93</v>
       </c>
     </row>
     <row r="65">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="72">
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="97">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="98">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="103">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="104">
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="105">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="106">
@@ -11274,7 +11274,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="109">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="110">
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124">
@@ -12018,7 +12018,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12062,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="132">
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="134">
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="139">
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="140">
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="149">
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13442,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>198</v>
+        <v>211</v>
       </c>
     </row>
     <row r="153">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="173">
@@ -14866,7 +14866,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="181">
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="L187" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="188">
@@ -16666,7 +16666,7 @@
         </is>
       </c>
       <c r="L213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -16834,7 +16834,7 @@
         </is>
       </c>
       <c r="L216" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="217">
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="223">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="224">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="L225" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -17352,12 +17352,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>O4cvVP9/Xx58ML4tZrzOZw==</t>
+          <t>TJDTJytBapUscCxqxdISgQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>eMYWBZPt0KxXUTcXhXS0Zk0DYWgfOHEd/k9r8ZPXyUw=</t>
+          <t>9Xac61Ub9or6SNCyrlHB+4kZEpDPopEdGh36PYq9uU4=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17384,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pmi7nj60bdw+rMIx5jmFTg==</t>
+          <t>YfUdVZIPrWxfkqPO2ClYHw==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>VrLqBkt5BeGDYro7bSrtHrOo59ceSIq7ph36xGJ87yw=</t>
+          <t>wsgImwBHStrY/7zIPpBFilhzSf88fv0w4eshuiGO2aE=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17416,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>QXn899yoSB5l2rqtROCL+A==</t>
+          <t>F9TgyTbnsA47EbGrSWnDzA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FSx3E5DsmEMRjpawlwPly3CmvOghHto66fePzNbC5mo=</t>
+          <t>yWR+BmUI6cn/ep7DdU01tZxiNQ4CQ0iBnqQloN9jKg4=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17443,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BJV/qASEuG1BXgKmX/d3xQ==</t>
+          <t>ljtBXyOKexuTB4EgraLH6w==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>JMHiAG4MPlf9d41m4GFSqcndqqd6s4rNrfDpLCtD1dI=</t>
+          <t>OYwFFVBPMiInY3iPPj4Q3l5EtJAH77HACsvGMi6HsIo=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17475,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dg1bKRYag2aABe3XKcRK3A==</t>
+          <t>05gSo2QiLDWTR4Izsdf9mw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>gIZCwi9Zcs/gaTZ3i/fBhZlGpKdxirYeTqaZ5gnM9LM=</t>
+          <t>FcmXTpdBxK8MvpRk9VdieJ/ovGBXmBU63waYkfZ/CiE=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17507,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>D0jh/907CqYy2aZA6pvYPA==</t>
+          <t>/IF3rvYgptXvKqxLl//RjA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>oQJHzS9r/gSkr6FIzuYS7ZJ0j2DM15nDgGvYjE9d4Ps=</t>
+          <t>sJbBTPLSTQATwkbWL5n7HxbqV+cgOSzVYkfSk48QDO8=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17539,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IxQsk4717oNdhSL3zbJskQ==</t>
+          <t>3p9YJcS3pQrWCQvPYq/PvA==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>HtwSsN1YKUvJ5j64CPMXcYCJatw4t4dgwXkncYcg1co=</t>
+          <t>fyoWCgwDpTGosr9zaD+WIgOgtNvaKxhmX2tYM5liYDY=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17566,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>xreDgD+InyzW5qGR6ABrpQ==</t>
+          <t>979Wi1WgILCHm9j4pMomMg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rn2plG6EFJbLQspMYaWV1ZG+baoCmDR9q/gOFCIqI5Y=</t>
+          <t>JDJvV8ekxMic6Kbxz86WabhZed5brUMtuVu6pAb4GEQ=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17598,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AhvJRiokyfDaA2xO+XRsCQ==;oenNyZEnKRHb8yMxbjR6dQ==</t>
+          <t>hR6miHFVEw+lg0jc2G0hxw==;WBxtZT6RUk3Fh71BNTRZ1g==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>xPKu//NxY6Xs+osMlt92NUmD8DmpchTtGvAaVpk5bAk=;RrZKrpnMGDT0/yy5kMtz4BfQcxw8RxpvUErk0AOYMFU=</t>
+          <t>G0DqAZdKoBow36aCcRzEQ4hXFjECUPpYVTOwQs6Wh+M=;LaKG0atUxPnk7mnHjXkk/cIBtC2VPRA+C8mooWDHdWg=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17630,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>rcF6JnDpoAkv4tNwjwg2Kg==</t>
+          <t>h8GC+74fUHaJR6WQWM1Ohg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>HYGlcCxscFFqIk9ZORr5S0PhjeL+AeNMjDZGxnYE9EA=</t>
+          <t>fizfvwDvac6K0ZkpKwzmS+mmf5cYWAFCxWpmU28qt5o=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17662,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>742H14bSbrO7FOqRS8nPWw==</t>
+          <t>jniFg6orowYkVNdQgsvu1A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>XcD0gQvwqvBuY0m2HmEri4CYbPftDdYVME34enWCkr8=</t>
+          <t>7MQomKrSS7kF63a52lIP+CUqt5bEcty8VRjQ50lUFXw=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17694,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>fX9A2x/3QudaK9uAVjpNXQ==</t>
+          <t>gTKiFCx/RLszCD+bQw/HSw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>5beYJzMObkxtLZeyafsgJq586dCKgYaL1QkSQdznAa0=</t>
+          <t>bqk1lTVwABV0L1uPWACfaPB+0ryB26FtLyf/WgjAay8=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+OWngrsREjaEmGCz/xbc/Q==</t>
+          <t>NXkpjRJkSQe/E3QREz5Cxg==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>kF4XtyJKTWz4vC5oM3/QkxxGtUegm/frUP7l9y8Gtx4=</t>
+          <t>skIsLT3Sij1MLWwP5XEG0236XggaV3VfwXvm1Pz/seI=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17758,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Yt7p2jMc51AwKZ4VrUBqfw==</t>
+          <t>7ptTQBO2T/4UV6s6vmQUng==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>QPFIod8DRb1qK9Ac9VjVZ+zd8oskxsk7gcDzlxOVWLg=</t>
+          <t>0fvRXWLE40O02pS3sEab+qsi2EplsBaKc6FgAoyLt+k=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17790,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7vXHbLviy0ohfTDVmYJa7A==</t>
+          <t>GnsB0Kb30hIgb4SshbGw6w==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>er+ya3qP0zn7JEugSaSA4MdaJYr3dyye6BiFhPRYisk=</t>
+          <t>olXFf13rO9Pqb9Og07ZC12Nru8CzrQe+mVP8sDMtqxE=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>9GXsbO1lK28f5JFoalsXCg==</t>
+          <t>XQVPOYPXFL3+921V3z2vjw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>mpQJJrA/sdnr6KkqWrmfT3JuFh0K8jZTxp3kyQMpl04=</t>
+          <t>+HvTInlmkUCVHIhEcUGbNqRayzjClMRjjU5H3Y6iEuM=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17854,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>p39GXVK7N4qA+/ulB20khg==</t>
+          <t>LpvxKtTBT9aK62bCEQ5hQg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>09a9HPIITIBlTJDkYy5aw6TvgD48pNrxwVmSil8nvBw=</t>
+          <t>NFskpy3GMq/fxu0L2UIKVsougV60Dq8vqhdQCVPhFnU=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17886,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>XznRNMLRbWh8SHApEsN4vw==</t>
+          <t>m4XBWnYG1XxQx/zSnxkb+w==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>lY+jvshCrRn0rJ6gbMwDJ1v5QbpgTEOpBRy0DKbLGs8=</t>
+          <t>FQCFnl3KUbf2LHZi8S3AYY6cIfo9pLrccImKMG5IgYE=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17918,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DgvpG8OpRBihjDO0oAV0tQ==</t>
+          <t>vhAU5A167a1sx0iqB7nSgw==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sx7XD11nu+BdExnraiszCoK0JM6IjKuwdjosYUb+yFg=</t>
+          <t>oKRyWsUFNItifCslkDIQV/wdgjFbOB5JB/m0IgUdvGM=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17950,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+7mMDh7zxKCiZbwQG8IiWw==</t>
+          <t>hn1xDsE4mh8OQPJcFJ1sUA==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>MrKuvoMl1eOn7kY/Unwl68ofqMyh9nLLtbUIMvwKGwo=</t>
+          <t>JBUxtBwmzm3g5nwo9N7pSjyxWmc1i3lvKD0ze9TF6Fo=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17982,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>UC/LL5F16KFVPUThAqOwHg==</t>
+          <t>VQLG1zMR24sVoyNjgr7YIA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>DgTKr2gL3IrWQe5r8gxKivllDBRrxiRW8nw2jno0W0U=</t>
+          <t>tlvCydDKLZJqKBLyoYHhSjaCWubSM5tO/BOydGX2qKg=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +18014,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>EhbCIn6aN0dd1aEZ6EnD2Q==</t>
+          <t>Thnj+LmVCOCRUH3nk57KRg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>OVgiV5yYUCNC9ACmwzMt62sPAJENv9vkIoVf0ldbYK0=</t>
+          <t>ViAJP7X0QchHgdZv73lmrC9zX3glOUp7tmWuTaOAFhI=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +18046,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3god9D91mBEbfl+7QpDGog==</t>
+          <t>L/9LzXuh97xQRdiZbsNr3w==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>luiLpaNd/9oY4lS4yhJi78wDTQeBOvh+QbzKIf86q/A=</t>
+          <t>joli6RO3cvKlLNxPtWTWmXCQmXWjTrSSfBa627/8zYE=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +18078,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>374zRE9aRSy2zuc10Y2BaQ==</t>
+          <t>7VslR3sgoWQ7hSpfBVqeFg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>zLcSzcdMfbTB4wfPdNrYMng7FrsjCVtU73ydwnj2d+c=</t>
+          <t>1GHvdeUZlr0aPlzQw65+hpf8GwQXqTexBuzx+Xn6Qas=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18110,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>zo7fqAasbAK+tE/JA2j4aA==</t>
+          <t>NU+YPBLhzSIpwe98x3Lkeg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>q+v48XnPUQFUu6CPD4BtsGVWixFegnfiSsdg09YdfHY=</t>
+          <t>EQoIm5yijZx3PGlvvRjLUy/mW64D7SAmyG21PwvsdkY=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18142,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2+6RaUd4MGK9TgQuAmDlSg==</t>
+          <t>SmVgLO9DHCdUonFWpoQYKg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>kk7JB0OsYyXt1/UEkAo4r4Wj7a2jTpN2VX1Eo/wPuZo=</t>
+          <t>cdUFyE/GiKxRF3SjEc4YAfbBBvq0l/s6aWizQhaDWTM=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18174,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0zRFc0TehUJWwldwCyEcmQ==</t>
+          <t>KvVMR5qWW3ncG0H1LANOKA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Oo+fB6HETo/+mR1fi+KAXZ2S3LCGqm7fu5z4OFdqGc0=</t>
+          <t>JT7YY00X9daqu0qNqXl9UnnD3oQ7Nv2OF/I9YnqWW+k=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18206,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>+zZGK1ZauiGRcxLrh5eI5w==</t>
+          <t>3GP+KnaCOohCuDoGJ+8isA==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>cqZ2hYwltzN4KXkZTHmsyqDSAvAcSHFQB98IT56D4P0=</t>
+          <t>MqQhkz8CUkuS3AVQQquU2eF5GHjjvp50CZmCe7lpF9o=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18238,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2RmI+Kjkhg42oEjaam3p3A==</t>
+          <t>rbZwcQ+BLk9mWY/LvflTNA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>amV9yH0PnxRSRIEG69Qb1rH5/18sfMSIOU0PPN0ZACY=</t>
+          <t>tFMiA/k0WurDTrFZcNTq1xAQlhiPN39z0PoLxLUR9Sg=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18270,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>v9L2ZDYSa6hDbQxyjLhJIg==</t>
+          <t>WHyFfzPOGFj2DNC3ZS57Dg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>UBIkumGy7Dg/iRbvtQH8b7OZVBCQdLjraUPovoGE9C8=</t>
+          <t>lTErwbVmQZ+8a8hErOPXzm4f+O376xNcwr0TIj0GoWc=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18302,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>yDuvyPfoxM4nRYmuDSK/IQ==</t>
+          <t>S0yPBB4tw6NQSSu96atfng==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>DnjxsMXC4cX7toATlKcIDzxlMOzPegiVo4rx2h59sVs=</t>
+          <t>i4ZO/tOhPzYQ2whUFp7oC565IwwF3C3FBfcAMj/8sPo=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18334,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>GaRcKgG+SUi92e/y/qWmkQ==</t>
+          <t>txXNFGUSXUKOeWOeAGCXfA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>cs3bXej4mY/FbfgKWzBdTzKIZKyfSWsNnvED6+E1HDI=</t>
+          <t>chsVhPsWsFIKAfadyPmPuQoiCEErFkCluvQNrYipYnM=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>19U61Aa8WgXn77hQnPrfSA==</t>
+          <t>kWBTBR5GiRr8xY7YN/nqOQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PjQ1Q9YZlpUeQF8Ea+gpUEZmMky1g0A4RRxLaAX0ve0=</t>
+          <t>rF/pZOWPGgaHtyg9G4n5r6LGwVjeyyIKfblxDiFiDXY=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18398,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>IjP7EhelOC21jfvtXYyi8g==</t>
+          <t>tCv2t/o8ckZrS6sulF4/2A==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>sEaZ6FPBlyg3NU+go/GLNxvkH4He35dsC/NOV6213/s=</t>
+          <t>orzGHtB7/LI0IY6DxcqnSnARu3KpgQGmbUTqjBM0+cE=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>a52XR0Lta77KywGyY9NsRg==</t>
+          <t>kVv0ef341YpVjPNJjQs1vQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>t4tMzcS3SYO+d9nT81oSN2hTPUMicbLUYk/Oz4x+Gg0=</t>
+          <t>WOuTucb994pC2bIwMObYT5gd2FxasozSEh5BDaHCeTE=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18462,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>aGQoKSXImmFKxGa54ZkpAg==</t>
+          <t>9wAls07AImfePTmATS+00g==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>kragnLIJZJtyE8LVa2LOWMwJgz37BO731nvTCTvLUrM=</t>
+          <t>J4NGRVLEalbDrxUUgXfPq512A7o4Pf9AgHZHuIDsiuo=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18494,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>9NhhQPd92VqhwOVdAqbnog==</t>
+          <t>hELaQlinsO7a/qZM/XTwnA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6fk1P7UWpydsV30BBRKIKEQQ7Bu/2N3eKu1pFwP8bqE=</t>
+          <t>WBH/IPmhB12H/lfZvteV/a4TdZCghY+nE1PgzDOa0OY=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-24 07:40) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$148</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$225</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$224</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H148"/>
+  <dimension ref="A1:H147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d0552e68-9c0f-4d49-839f-f22fdc6c6f8e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57">
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="86">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="89">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="90">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="91">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="95">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="96">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="97">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="108">
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="109">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>507</v>
+        <v>516</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>507</v>
+        <v>516</v>
       </c>
     </row>
     <row r="115">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="119">
@@ -4867,12 +4867,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4903,12 +4903,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="124">
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=11cc3a84-a83e-4020-844d-43919a87f1b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5427,7 +5427,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5623,12 +5623,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5659,12 +5659,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5695,12 +5695,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=17a76e1b-4a1d-4f00-88ee-66022635680c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=17a76e1b-4a1d-4f00-88ee-66022635680c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5762,17 +5762,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5790,44 +5790,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>MENOR COSTE</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>INFORME</t>
-        </is>
-      </c>
-      <c r="H148" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H148"/>
+  <autoFilter ref="A1:H147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5838,7 +5802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5958,7 +5922,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -6002,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
@@ -6134,7 +6098,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -6178,7 +6142,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -6222,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9">
@@ -6266,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -6442,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14">
@@ -6486,7 +6450,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -6530,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -7746,7 +7710,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39">
@@ -9050,7 +9014,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -9406,7 +9370,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="72">
@@ -10782,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="98">
@@ -11142,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="106">
@@ -11230,7 +11194,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="108">
@@ -11318,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="110">
@@ -11362,7 +11326,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="111">
@@ -11798,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="120">
@@ -12018,7 +11982,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="125">
@@ -12062,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="126">
@@ -12106,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="127">
@@ -12326,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="132">
@@ -12414,7 +12378,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="134">
@@ -13274,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="150">
@@ -13442,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>211</v>
+        <v>220</v>
       </c>
     </row>
     <row r="153">
@@ -13574,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="156">
@@ -13639,7 +13603,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -13647,7 +13611,7 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -13658,11 +13622,11 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>11cc3a84-a83e-4020-844d-43919a87f1b9</t>
+          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
         </is>
       </c>
       <c r="L157" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="158">
@@ -13683,7 +13647,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -13691,7 +13655,7 @@
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>Grupo Clientes BLACK 2026</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -13702,11 +13666,11 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
+          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
         </is>
       </c>
       <c r="L158" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="159">
@@ -13727,18 +13691,30 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>HECTOLITROS 07-2025</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>HECTOLITROS</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Grupo Clientes BLACK 2026</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr"/>
+          <t>Informe Hctos - Julio 25</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J159" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -13746,11 +13722,11 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
+          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
         </is>
       </c>
       <c r="L159" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -13771,7 +13747,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2025</t>
+          <t>HECTOLITROS 08-2025</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -13782,17 +13758,17 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 25</t>
+          <t>Informe Hctos - Agosto 25</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -13802,7 +13778,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
+          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -13827,7 +13803,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2025</t>
+          <t>HECTOLITROS 09-2025</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -13838,17 +13814,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 25</t>
+          <t>Informe Hctos - Septiembre 25</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -13858,7 +13834,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
+          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -13883,7 +13859,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2025</t>
+          <t>HECTOLITROS 10-2025</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -13894,17 +13870,17 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 25</t>
+          <t>Informe Hctos - Octubre 25</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -13914,7 +13890,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
+          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -13939,7 +13915,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2025</t>
+          <t>HECTOLITROS 11-2025</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -13950,17 +13926,17 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 25</t>
+          <t>Informe Hctos - Noviembre 25</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -13970,7 +13946,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
+          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -13995,7 +13971,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>HECTOLITROS 11-2025</t>
+          <t>HECTOLITROS 12-2025</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -14006,17 +13982,17 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Informe Hctos - Noviembre 25</t>
+          <t>Informe Hctos - Diciembre 25</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -14026,7 +14002,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
+          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -14051,7 +14027,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>HECTOLITROS 12-2025</t>
+          <t>HECTOLITROS 01-2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -14062,17 +14038,17 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Informe Hctos - Diciembre 25</t>
+          <t>Informe Hctos - Enero 26</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -14082,7 +14058,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
+          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -14107,7 +14083,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>HECTOLITROS 01-2026</t>
+          <t>HECTOLITROS 02-2026</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
@@ -14118,17 +14094,17 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Informe Hctos - Enero 26</t>
+          <t>Informe Hctos - Febrero 26</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -14138,7 +14114,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
+          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -14163,7 +14139,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>HECTOLITROS 02-2026</t>
+          <t>HECTOLITROS 03-2026</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -14174,17 +14150,17 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Informe Hctos - Febrero 26</t>
+          <t>Informe Hctos - Marzo 26</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -14194,7 +14170,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
+          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -14219,7 +14195,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>HECTOLITROS 03-2026</t>
+          <t>HECTOLITROS 04-2026</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
@@ -14230,17 +14206,17 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Informe Hctos - Marzo 26</t>
+          <t>Informe Hctos - Abril 26</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -14250,7 +14226,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
+          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -14275,7 +14251,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>HECTOLITROS 04-2026</t>
+          <t>HECTOLITROS 05-2026</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
@@ -14286,17 +14262,17 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Informe Hctos - Abril 26</t>
+          <t>Informe Hctos - Mayo 26</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -14306,11 +14282,11 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
+          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
         </is>
       </c>
       <c r="L169" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
@@ -14331,7 +14307,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>HECTOLITROS 05-2026</t>
+          <t>HECTOLITROS 06-2026</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
@@ -14342,17 +14318,17 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Informe Hctos - Mayo 26</t>
+          <t>Informe Hctos - Junio 26</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -14362,7 +14338,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
+          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -14387,7 +14363,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -14398,17 +14374,17 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 26</t>
+          <t>Informe Hctos - Julio 26</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -14418,11 +14394,11 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
+          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
         </is>
       </c>
       <c r="L171" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="172">
@@ -14443,7 +14419,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="E172" t="inlineStr"/>
@@ -14454,17 +14430,17 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 26</t>
+          <t>Informe Hctos - Agosto 26</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -14474,11 +14450,11 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
+          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
         </is>
       </c>
       <c r="L172" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="173">
@@ -14499,7 +14475,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
@@ -14510,17 +14486,17 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 26</t>
+          <t>Informe Hctos - Septiembre 26</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -14530,11 +14506,11 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
+          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
         </is>
       </c>
       <c r="L173" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="174">
@@ -14555,7 +14531,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 10-2026</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
@@ -14566,17 +14542,17 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 26</t>
+          <t>Informe Hctos - Octubre 26</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Octubre - 26</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -14586,11 +14562,11 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
+          <t>b56bb142-8685-433a-bd0c-b8969d964151</t>
         </is>
       </c>
       <c r="L174" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
     </row>
     <row r="175">
@@ -14611,30 +14587,18 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2026</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>HECTOLITROS</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 26</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>Octubre - 26</t>
-        </is>
-      </c>
+          <t>INFO MARCA CORE CCU</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14642,11 +14606,11 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>b56bb142-8685-433a-bd0c-b8969d964151</t>
+          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
         </is>
       </c>
       <c r="L175" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">
@@ -14667,7 +14631,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
@@ -14675,7 +14639,7 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -14686,11 +14650,11 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
+          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
     </row>
     <row r="177">
@@ -14711,7 +14675,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
@@ -14719,7 +14683,7 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -14730,11 +14694,11 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
+          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -14755,7 +14719,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
@@ -14763,7 +14727,7 @@
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -14774,7 +14738,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
+          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -14799,7 +14763,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -14807,7 +14771,7 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -14818,11 +14782,11 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
+          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
         </is>
       </c>
       <c r="L179" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
     </row>
     <row r="180">
@@ -14843,7 +14807,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -14851,7 +14815,7 @@
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -14862,11 +14826,11 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L180" t="n">
-        <v>210</v>
+        <v>12</v>
       </c>
     </row>
     <row r="181">
@@ -14887,18 +14851,30 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>PARTICIPACION VENTAS CCU</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr"/>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J181" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14906,11 +14882,11 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
+          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
       </c>
       <c r="L181" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182">
@@ -14931,28 +14907,28 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -14962,11 +14938,11 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
+          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
       </c>
       <c r="L182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -14987,13 +14963,13 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -15003,7 +14979,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
+          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -15018,11 +14994,11 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
+          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
       </c>
       <c r="L183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184">
@@ -15043,28 +15019,20 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP COSTA</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Octubre - 26</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -15074,11 +15042,11 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
+          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
         </is>
       </c>
       <c r="L184" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185">
@@ -15094,12 +15062,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -15107,14 +15075,10 @@
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>Octubre - 26</t>
-        </is>
-      </c>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15122,11 +15086,11 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
+          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
       <c r="L185" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186">
@@ -15142,12 +15106,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -15155,7 +15119,7 @@
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>RECHAZOS ago 26</t>
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
@@ -15166,11 +15130,11 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
+          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
         </is>
       </c>
       <c r="L186" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
     </row>
     <row r="187">
@@ -15191,18 +15155,30 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO DE MARCAS</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>RECHAZOS ago 26</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr"/>
+          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J187" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15210,11 +15186,11 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
+          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
       <c r="L187" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188">
@@ -15235,7 +15211,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -15246,17 +15222,17 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -15266,7 +15242,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
+          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
       <c r="L188" t="n">
@@ -15291,7 +15267,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
@@ -15302,17 +15278,17 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -15322,7 +15298,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
+          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
       <c r="L189" t="n">
@@ -15347,7 +15323,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -15358,17 +15334,17 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -15378,7 +15354,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
+          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
       <c r="L190" t="n">
@@ -15403,7 +15379,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -15414,17 +15390,17 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -15434,7 +15410,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
+          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
       <c r="L191" t="n">
@@ -15459,7 +15435,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
@@ -15470,17 +15446,17 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -15490,7 +15466,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
+          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
       <c r="L192" t="n">
@@ -15515,7 +15491,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -15526,17 +15502,17 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -15546,7 +15522,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
+          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
       <c r="L193" t="n">
@@ -15571,7 +15547,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -15582,17 +15558,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15602,7 +15578,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
+          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
       <c r="L194" t="n">
@@ -15627,7 +15603,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -15638,17 +15614,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15658,7 +15634,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
+          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
       <c r="L195" t="n">
@@ -15683,7 +15659,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -15694,17 +15670,17 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -15714,7 +15690,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
+          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
       <c r="L196" t="n">
@@ -15739,7 +15715,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -15750,17 +15726,17 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -15770,7 +15746,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
+          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
       <c r="L197" t="n">
@@ -15795,7 +15771,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -15806,17 +15782,17 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -15826,7 +15802,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
+          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
       <c r="L198" t="n">
@@ -15851,7 +15827,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -15862,17 +15838,17 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -15882,7 +15858,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
+          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
       <c r="L199" t="n">
@@ -15907,7 +15883,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -15918,17 +15894,17 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15938,11 +15914,11 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
+          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
       <c r="L200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -15963,7 +15939,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -15974,17 +15950,17 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15994,11 +15970,11 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
+          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
         </is>
       </c>
       <c r="L201" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="202">
@@ -16019,7 +15995,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
@@ -16030,19 +16006,15 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
-        </is>
-      </c>
-      <c r="I202" t="inlineStr">
-        <is>
-          <t>Septiembre - 26</t>
-        </is>
-      </c>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 26</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr"/>
       <c r="J202" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16050,7 +16022,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
+          <t>17a76e1b-4a1d-4f00-88ee-66022635680c</t>
         </is>
       </c>
       <c r="L202" t="n">
@@ -16075,26 +16047,30 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 26</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J203" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16102,11 +16078,11 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>17a76e1b-4a1d-4f00-88ee-66022635680c</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204">
@@ -16127,7 +16103,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16138,17 +16114,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16158,11 +16134,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
@@ -16183,7 +16159,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16194,17 +16170,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16214,11 +16190,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206">
@@ -16239,7 +16215,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16250,17 +16226,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16270,11 +16246,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="207">
@@ -16295,7 +16271,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
@@ -16306,17 +16282,17 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16326,7 +16302,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L207" t="n">
@@ -16351,7 +16327,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -16362,17 +16338,17 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -16382,7 +16358,7 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L208" t="n">
@@ -16407,7 +16383,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16418,17 +16394,17 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -16438,7 +16414,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L209" t="n">
@@ -16463,7 +16439,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16474,17 +16450,17 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -16494,7 +16470,7 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L210" t="n">
@@ -16519,7 +16495,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16530,17 +16506,17 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -16550,7 +16526,7 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L211" t="n">
@@ -16575,7 +16551,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16586,17 +16562,17 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -16606,7 +16582,7 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L212" t="n">
@@ -16631,7 +16607,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16642,17 +16618,17 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -16662,11 +16638,11 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -16687,7 +16663,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E214" t="inlineStr"/>
@@ -16698,17 +16674,17 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -16718,11 +16694,11 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L214" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215">
@@ -16743,7 +16719,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -16754,17 +16730,17 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -16774,11 +16750,11 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L215" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="216">
@@ -16799,7 +16775,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -16810,17 +16786,17 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -16830,11 +16806,11 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L216" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217">
@@ -16855,7 +16831,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -16866,17 +16842,17 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -16886,11 +16862,11 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L217" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218">
@@ -16911,7 +16887,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -16922,17 +16898,17 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 26</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Octubre - 26</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -16942,11 +16918,11 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>1ddf1ffb-0655-4b37-96ee-4ee69ebd5764</t>
         </is>
       </c>
       <c r="L218" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
@@ -16967,30 +16943,18 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 26</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr">
-        <is>
-          <t>Octubre - 26</t>
-        </is>
-      </c>
+          <t>Sin cargo CFH</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr"/>
       <c r="J219" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16998,11 +16962,11 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>1ddf1ffb-0655-4b37-96ee-4ee69ebd5764</t>
+          <t>46395ec1-f0ac-4b34-9a0c-40fe1322db9f</t>
         </is>
       </c>
       <c r="L219" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="220">
@@ -17023,7 +16987,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -17031,7 +16995,7 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Sin cargo CFH</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I220" t="inlineStr"/>
@@ -17042,11 +17006,11 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>46395ec1-f0ac-4b34-9a0c-40fe1322db9f</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L220" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
@@ -17067,7 +17031,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -17075,7 +17039,7 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I221" t="inlineStr"/>
@@ -17086,11 +17050,11 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L221" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="222">
@@ -17111,7 +17075,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -17119,7 +17083,7 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I222" t="inlineStr"/>
@@ -17130,11 +17094,11 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
         </is>
       </c>
       <c r="L222" t="n">
-        <v>48</v>
+        <v>81</v>
       </c>
     </row>
     <row r="223">
@@ -17155,7 +17119,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -17163,7 +17127,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -17174,11 +17138,11 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L223" t="n">
-        <v>79</v>
+        <v>2</v>
       </c>
     </row>
     <row r="224">
@@ -17199,7 +17163,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
@@ -17207,7 +17171,7 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -17218,61 +17182,17 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
       <c r="L224" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>HERGO - DISTRIBUCION</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>VENTA MAYORISTA DETALLE</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>Venta Mayorista Detalle</t>
-        </is>
-      </c>
-      <c r="I225" t="inlineStr"/>
-      <c r="J225" t="inlineStr">
-        <is>
-          <t>Grupo Hergo - Jefes</t>
-        </is>
-      </c>
-      <c r="K225" t="inlineStr">
-        <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
-        </is>
-      </c>
-      <c r="L225" t="n">
         <v>50</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L225"/>
+  <autoFilter ref="A1:L224"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A224" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17352,12 +17272,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TJDTJytBapUscCxqxdISgQ==</t>
+          <t>j8eboO+iauOb/PrhZpYpoA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>9Xac61Ub9or6SNCyrlHB+4kZEpDPopEdGh36PYq9uU4=</t>
+          <t>dvY1c3x7iFbSMC9cexB0aZ2eYJ73B2wjBC0jspV4IPw=</t>
         </is>
       </c>
     </row>
@@ -17384,12 +17304,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>YfUdVZIPrWxfkqPO2ClYHw==</t>
+          <t>zRn2wiinIoA3SKU9BJyl5A==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>wsgImwBHStrY/7zIPpBFilhzSf88fv0w4eshuiGO2aE=</t>
+          <t>2za7EQy9AFRvcNzjJWQNILhGmjno9Cu4li5QzMEzFos=</t>
         </is>
       </c>
     </row>
@@ -17416,12 +17336,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>F9TgyTbnsA47EbGrSWnDzA==</t>
+          <t>gK98WGsPFIhOjqXGtkZNww==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>yWR+BmUI6cn/ep7DdU01tZxiNQ4CQ0iBnqQloN9jKg4=</t>
+          <t>Fa7JLw+9VBwn/+pAD0etLWvcinhINO4LiZyjsXgVep4=</t>
         </is>
       </c>
     </row>
@@ -17443,12 +17363,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ljtBXyOKexuTB4EgraLH6w==</t>
+          <t>bDw9KiyeFYsMAzUbVPpkUQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>OYwFFVBPMiInY3iPPj4Q3l5EtJAH77HACsvGMi6HsIo=</t>
+          <t>bxsRN1Vt5lxECM7y3OGIa3VqY5XSKicsNjUbvllMf1E=</t>
         </is>
       </c>
     </row>
@@ -17475,12 +17395,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>05gSo2QiLDWTR4Izsdf9mw==</t>
+          <t>fVmaMKaCHnVnzhjrvYiQOg==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>FcmXTpdBxK8MvpRk9VdieJ/ovGBXmBU63waYkfZ/CiE=</t>
+          <t>jXKEYQXBXs+AX3XthW5h4jLGY46dD1KwnwZ2taRzkYc=</t>
         </is>
       </c>
     </row>
@@ -17507,12 +17427,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>/IF3rvYgptXvKqxLl//RjA==</t>
+          <t>igFneKgeC5pk8fs/2GUtoA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>sJbBTPLSTQATwkbWL5n7HxbqV+cgOSzVYkfSk48QDO8=</t>
+          <t>mpx2Ot4E/XRk7hOacYhaSsF6XFOw81cI7QVSlblSO9g=</t>
         </is>
       </c>
     </row>
@@ -17539,12 +17459,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3p9YJcS3pQrWCQvPYq/PvA==</t>
+          <t>lN53Nb4QGdRlSIouBtuIsg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>fyoWCgwDpTGosr9zaD+WIgOgtNvaKxhmX2tYM5liYDY=</t>
+          <t>l1AWknEaaG57At7FUZBw0LPULPMxkRHrV1wHj1n3pYQ=</t>
         </is>
       </c>
     </row>
@@ -17566,12 +17486,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>979Wi1WgILCHm9j4pMomMg==</t>
+          <t>sxCP5O4v49iY6yVyDC//pw==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>JDJvV8ekxMic6Kbxz86WabhZed5brUMtuVu6pAb4GEQ=</t>
+          <t>UAKmE3Fh+r7rikEabkZMCTPRwzJdjnuxGPQTDiNpALU=</t>
         </is>
       </c>
     </row>
@@ -17598,12 +17518,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>hR6miHFVEw+lg0jc2G0hxw==;WBxtZT6RUk3Fh71BNTRZ1g==</t>
+          <t>o7NmT7LQMnulFw+MnJ0Vcw==;Ah3c6e4Ri4+vl1b4WK6icQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>G0DqAZdKoBow36aCcRzEQ4hXFjECUPpYVTOwQs6Wh+M=;LaKG0atUxPnk7mnHjXkk/cIBtC2VPRA+C8mooWDHdWg=</t>
+          <t>WXtTQZqyXE4DA1Pa8L2mzgecbXG1ahW/Nw/ZGTYENAk=;+ESmF2FhbZu5ALV2YktZisYJ3etGjYPav5uS5zPYKTE=</t>
         </is>
       </c>
     </row>
@@ -17630,12 +17550,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>h8GC+74fUHaJR6WQWM1Ohg==</t>
+          <t>aYibzIXvOItOc98nUPgORw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>fizfvwDvac6K0ZkpKwzmS+mmf5cYWAFCxWpmU28qt5o=</t>
+          <t>uobc5utBXQ4yF34cgVUOGCXVX23spSyDeOjSuFJQ6dk=</t>
         </is>
       </c>
     </row>
@@ -17662,12 +17582,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>jniFg6orowYkVNdQgsvu1A==</t>
+          <t>1Vl0Gaae/LaLwg5wcgcSOw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>7MQomKrSS7kF63a52lIP+CUqt5bEcty8VRjQ50lUFXw=</t>
+          <t>ZGFoICiPYaLGsA5ODsYLG5ksUIEhqBwNVf7TmDrO/RA=</t>
         </is>
       </c>
     </row>
@@ -17694,12 +17614,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>gTKiFCx/RLszCD+bQw/HSw==</t>
+          <t>GU+FP1sq/PeWqLHW47SBFg==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>bqk1lTVwABV0L1uPWACfaPB+0ryB26FtLyf/WgjAay8=</t>
+          <t>EJ/PCI/QQkIUQc/DLmXSxWUnBv/U3E34kzEcKjjR1pY=</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17646,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NXkpjRJkSQe/E3QREz5Cxg==</t>
+          <t>bgeVOk/I6xLJG343sOiV4w==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>skIsLT3Sij1MLWwP5XEG0236XggaV3VfwXvm1Pz/seI=</t>
+          <t>gYAdJ1buRF1b9SV/c0IBGbDcRpB0Ft9noE33LlP/8rM=</t>
         </is>
       </c>
     </row>
@@ -17758,12 +17678,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7ptTQBO2T/4UV6s6vmQUng==</t>
+          <t>q3lmBhsFz8xMg3MWP2CRCg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0fvRXWLE40O02pS3sEab+qsi2EplsBaKc6FgAoyLt+k=</t>
+          <t>EWpukGWdluXIwSyonRCK724WMNfzJUFvnzSpMnPIk0Y=</t>
         </is>
       </c>
     </row>
@@ -17790,12 +17710,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GnsB0Kb30hIgb4SshbGw6w==</t>
+          <t>l2wJYNAmBuZANgTRX3uxaw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>olXFf13rO9Pqb9Og07ZC12Nru8CzrQe+mVP8sDMtqxE=</t>
+          <t>XoAiS5LGWKKq3U+XmxhScroZxwQ68qn+obf4gXmmmBI=</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17742,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>XQVPOYPXFL3+921V3z2vjw==</t>
+          <t>C4azEe+m64ZUPis9y5eaIw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>+HvTInlmkUCVHIhEcUGbNqRayzjClMRjjU5H3Y6iEuM=</t>
+          <t>oO5YabUHKRrYAHO0Fbtg0wYatxHHgMBPAuYv3VJ0n48=</t>
         </is>
       </c>
     </row>
@@ -17854,12 +17774,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LpvxKtTBT9aK62bCEQ5hQg==</t>
+          <t>iShfhSPoHk0QyFLd0HaMOw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>NFskpy3GMq/fxu0L2UIKVsougV60Dq8vqhdQCVPhFnU=</t>
+          <t>J7MqZ4IP8F48NndnP9J5n5bQy4jJ2Ix1asVHFKWDOQ8=</t>
         </is>
       </c>
     </row>
@@ -17886,12 +17806,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>m4XBWnYG1XxQx/zSnxkb+w==</t>
+          <t>DVg5rjI9wbXLwrmlXK/Hpg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>FQCFnl3KUbf2LHZi8S3AYY6cIfo9pLrccImKMG5IgYE=</t>
+          <t>D67V4OhDX6fj4GAwkHvsKUzs/X5/YMPQrg0e8hF0izQ=</t>
         </is>
       </c>
     </row>
@@ -17918,12 +17838,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vhAU5A167a1sx0iqB7nSgw==</t>
+          <t>4GJfLQqMNN7OKxRIQSuiag==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>oKRyWsUFNItifCslkDIQV/wdgjFbOB5JB/m0IgUdvGM=</t>
+          <t>jDfSIPztlIFsinHIWUH72md9ixfF0SjTkwgllEMjJQ0=</t>
         </is>
       </c>
     </row>
@@ -17950,12 +17870,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>hn1xDsE4mh8OQPJcFJ1sUA==</t>
+          <t>7f0zBhw5oJRWVWSOqU9I6w==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>JBUxtBwmzm3g5nwo9N7pSjyxWmc1i3lvKD0ze9TF6Fo=</t>
+          <t>95l6BtodKaqLQnOmjpLW20CA4DjrejfBjR5kmY9i+PM=</t>
         </is>
       </c>
     </row>
@@ -17982,12 +17902,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VQLG1zMR24sVoyNjgr7YIA==</t>
+          <t>tSgKjYj8xcf8yqBDj5whsQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>tlvCydDKLZJqKBLyoYHhSjaCWubSM5tO/BOydGX2qKg=</t>
+          <t>KL1P4/78J8lfB6O3hyvG+e3FVkLTiBotr8WGJHATfcI=</t>
         </is>
       </c>
     </row>
@@ -18014,12 +17934,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Thnj+LmVCOCRUH3nk57KRg==</t>
+          <t>jMRALTyVuGG+mgBJSG42MA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>ViAJP7X0QchHgdZv73lmrC9zX3glOUp7tmWuTaOAFhI=</t>
+          <t>4Pt32u8fCxVHpapb3tRd4BB6qrYeiX757gzRy4eNZwU=</t>
         </is>
       </c>
     </row>
@@ -18046,12 +17966,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>L/9LzXuh97xQRdiZbsNr3w==</t>
+          <t>GvRCWG9h0cOAG//+wf617A==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>joli6RO3cvKlLNxPtWTWmXCQmXWjTrSSfBa627/8zYE=</t>
+          <t>y1ocOwZCP15TNvm+NweiqNiSQv+OHg4q4bkQF8cC5BI=</t>
         </is>
       </c>
     </row>
@@ -18078,12 +17998,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7VslR3sgoWQ7hSpfBVqeFg==</t>
+          <t>z8Y0K4s7hq3BBTZt0ZW4BQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1GHvdeUZlr0aPlzQw65+hpf8GwQXqTexBuzx+Xn6Qas=</t>
+          <t>65ljYhkTk8TOa2n4Ir4PNLz7TO8dExvR8qdT0wvRbaQ=</t>
         </is>
       </c>
     </row>
@@ -18110,12 +18030,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NU+YPBLhzSIpwe98x3Lkeg==</t>
+          <t>Ywy9BW/d+0Yvz5W4ZK54rA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>EQoIm5yijZx3PGlvvRjLUy/mW64D7SAmyG21PwvsdkY=</t>
+          <t>w3jw/kmvG7RJM59zcuFX82CPgY9WHZDL4hLMqfwgDsg=</t>
         </is>
       </c>
     </row>
@@ -18142,12 +18062,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SmVgLO9DHCdUonFWpoQYKg==</t>
+          <t>f2kKJKCchFmaq4WM53rhOA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>cdUFyE/GiKxRF3SjEc4YAfbBBvq0l/s6aWizQhaDWTM=</t>
+          <t>gnAj/drdIcT+mSfSeZKjT0RUqVvvR7pUINA2yq5qPwg=</t>
         </is>
       </c>
     </row>
@@ -18174,12 +18094,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>KvVMR5qWW3ncG0H1LANOKA==</t>
+          <t>hF1nn4Ny+IFtEDyHbkDMgw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>JT7YY00X9daqu0qNqXl9UnnD3oQ7Nv2OF/I9YnqWW+k=</t>
+          <t>Dre9aU0WmLSvz76rmpiT/Ta2/XGnSLuRl5yaLOkd0rg=</t>
         </is>
       </c>
     </row>
@@ -18206,12 +18126,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3GP+KnaCOohCuDoGJ+8isA==</t>
+          <t>2V6rv8y4mpoU/YCtKepHxQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>MqQhkz8CUkuS3AVQQquU2eF5GHjjvp50CZmCe7lpF9o=</t>
+          <t>ZnWfykwJy2CCtLeg8sDo9+5ImpNiidvRr5iwAO2y0xY=</t>
         </is>
       </c>
     </row>
@@ -18238,12 +18158,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>rbZwcQ+BLk9mWY/LvflTNA==</t>
+          <t>v/rS1S64lukqlibjp5JgTQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>tFMiA/k0WurDTrFZcNTq1xAQlhiPN39z0PoLxLUR9Sg=</t>
+          <t>5A85q+H8l1ilYqIqT2is/hTsGFQfePuf382D5du7uXo=</t>
         </is>
       </c>
     </row>
@@ -18270,12 +18190,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WHyFfzPOGFj2DNC3ZS57Dg==</t>
+          <t>AWvTj3bSfcVOPqhsqONbwQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>lTErwbVmQZ+8a8hErOPXzm4f+O376xNcwr0TIj0GoWc=</t>
+          <t>N/APm+WGLuRFMUmusjzlvD8sbaMLcr+jbNXBm5sTzuA=</t>
         </is>
       </c>
     </row>
@@ -18302,12 +18222,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>S0yPBB4tw6NQSSu96atfng==</t>
+          <t>sY0U4H4KDvNmKnW2wCYbWA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>i4ZO/tOhPzYQ2whUFp7oC565IwwF3C3FBfcAMj/8sPo=</t>
+          <t>s8k8nIqBBFEv7+0c55zRX+E/iDtiY7skBjCum1tiApk=</t>
         </is>
       </c>
     </row>
@@ -18334,12 +18254,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>txXNFGUSXUKOeWOeAGCXfA==</t>
+          <t>MibTNruOrgYcyrFJ5EYhWg==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>chsVhPsWsFIKAfadyPmPuQoiCEErFkCluvQNrYipYnM=</t>
+          <t>L58Sd0HRjSxLjbczhB1fWjOK1paj2BymcUIpHjS6Njg=</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18286,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>kWBTBR5GiRr8xY7YN/nqOQ==</t>
+          <t>h4tNXCqbmy9vuvcu54vDNA==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>rF/pZOWPGgaHtyg9G4n5r6LGwVjeyyIKfblxDiFiDXY=</t>
+          <t>+i27jZcWtg8rVspP3ZRhXQdAEtviAZe67l5X5QCQ/Po=</t>
         </is>
       </c>
     </row>
@@ -18398,12 +18318,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>tCv2t/o8ckZrS6sulF4/2A==</t>
+          <t>0XXtlk6I/hdlfSqCxNAlRQ==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>orzGHtB7/LI0IY6DxcqnSnARu3KpgQGmbUTqjBM0+cE=</t>
+          <t>0tWKoR4g4sY1ug6N+dfHYY/lh40o8DNiexSbBsNcVao=</t>
         </is>
       </c>
     </row>
@@ -18430,12 +18350,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>kVv0ef341YpVjPNJjQs1vQ==</t>
+          <t>zayIxoqu1KSu+QPSVFdy5w==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>WOuTucb994pC2bIwMObYT5gd2FxasozSEh5BDaHCeTE=</t>
+          <t>gSEiIQGiuuGXDHLksTh58NracnPQt484s9rYLVgsYUQ=</t>
         </is>
       </c>
     </row>
@@ -18462,12 +18382,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>9wAls07AImfePTmATS+00g==</t>
+          <t>bYQfixQ78hlIlGINue7BSQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>J4NGRVLEalbDrxUUgXfPq512A7o4Pf9AgHZHuIDsiuo=</t>
+          <t>/kPGlGQxUA0qcTjRDhWSSJmgqTW6OYP8bitdSiIxIto=</t>
         </is>
       </c>
     </row>
@@ -18494,12 +18414,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>hELaQlinsO7a/qZM/XTwnA==</t>
+          <t>2vZySjKepWnnbJ3rFOw63g==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>WBH/IPmhB12H/lfZvteV/a4TdZCghY+nE1PgzDOa0OY=</t>
+          <t>ZWCAeoUdebJBSmaZhoF4JM4ShmKpmpkjA6/6UvFtm9A=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-25 07:40) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="81">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>356</v>
+        <v>363</v>
       </c>
     </row>
     <row r="86">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="89">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="91">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="92">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="95">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="96">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f47ca5f4-a334-4064-94a1-564f810c0b7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5454cf95-0660-40a2-8768-67b20b4a707a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="97">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="98">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="99">
@@ -4147,12 +4147,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103">
@@ -4183,12 +4183,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a698bdc2-d8e9-45f8-b668-1d321e44a201&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="109">
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="110">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>516</v>
+        <v>526</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>516</v>
+        <v>526</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="119">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="123">
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="124">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5355,7 +5355,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136">
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5922,7 +5922,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9">
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14">
@@ -6758,7 +6758,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -7542,7 +7542,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -7974,7 +7974,7 @@
         </is>
       </c>
       <c r="L44" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45">
@@ -8018,7 +8018,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46">
@@ -8846,7 +8846,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65">
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="97">
@@ -10746,7 +10746,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98">
@@ -10974,7 +10974,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="103">
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="104">
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="105">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="106">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="108">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>356</v>
+        <v>363</v>
       </c>
     </row>
     <row r="110">
@@ -11630,7 +11630,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="120">
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="125">
@@ -12026,7 +12026,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="126">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="127">
@@ -12202,7 +12202,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130">
@@ -12334,7 +12334,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133">
@@ -12622,7 +12622,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="139">
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="149">
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>114</v>
+        <v>100</v>
       </c>
     </row>
     <row r="150">
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
     </row>
     <row r="153">
@@ -13538,7 +13538,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="156">
@@ -14398,7 +14398,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172">
@@ -14786,7 +14786,7 @@
         </is>
       </c>
       <c r="L179" t="n">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="180">
@@ -15134,7 +15134,7 @@
         </is>
       </c>
       <c r="L186" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="187">
@@ -17054,7 +17054,7 @@
         </is>
       </c>
       <c r="L221" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="222">
@@ -17098,7 +17098,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="223">
@@ -17142,7 +17142,7 @@
         </is>
       </c>
       <c r="L223" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="224">
@@ -17186,7 +17186,7 @@
         </is>
       </c>
       <c r="L224" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -17272,12 +17272,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>j8eboO+iauOb/PrhZpYpoA==</t>
+          <t>8xEcUKsFe74ZVePLv19Z8w==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dvY1c3x7iFbSMC9cexB0aZ2eYJ73B2wjBC0jspV4IPw=</t>
+          <t>hQZySSIPa9PEX5Zn+jyOQ7W8F6ZMLt8rcTCrRakYExc=</t>
         </is>
       </c>
     </row>
@@ -17304,12 +17304,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>zRn2wiinIoA3SKU9BJyl5A==</t>
+          <t>hzcuRpa1WW5wA9BEy7f4CA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2za7EQy9AFRvcNzjJWQNILhGmjno9Cu4li5QzMEzFos=</t>
+          <t>iG660XCBKIxDfPlfuNou7kA3IK8eCvGT6uLJzURN9U0=</t>
         </is>
       </c>
     </row>
@@ -17336,12 +17336,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>gK98WGsPFIhOjqXGtkZNww==</t>
+          <t>nt+9eRN9YNG+pwQS85mSGw==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Fa7JLw+9VBwn/+pAD0etLWvcinhINO4LiZyjsXgVep4=</t>
+          <t>vmKziK/PolLdaaRJ+ZwBz0LVSxD+LWrQ3WgGUJygpuY=</t>
         </is>
       </c>
     </row>
@@ -17363,12 +17363,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>bDw9KiyeFYsMAzUbVPpkUQ==</t>
+          <t>KgaLOd1D27NA1mWUaiyjfg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>bxsRN1Vt5lxECM7y3OGIa3VqY5XSKicsNjUbvllMf1E=</t>
+          <t>RKNj9iHc5h0UmQHYGv1+OHbPST6ilU+2YmPoCTh2YBA=</t>
         </is>
       </c>
     </row>
@@ -17395,12 +17395,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>fVmaMKaCHnVnzhjrvYiQOg==</t>
+          <t>DSkdotymuLR7lCFG4zGt+g==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>jXKEYQXBXs+AX3XthW5h4jLGY46dD1KwnwZ2taRzkYc=</t>
+          <t>iZk+A5C2hgRUcp8GWy2bG55JIoGv0dT9onvyLMqctWQ=</t>
         </is>
       </c>
     </row>
@@ -17427,12 +17427,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>igFneKgeC5pk8fs/2GUtoA==</t>
+          <t>CiI3hzhkX3aYJQ+pWnmeLw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>mpx2Ot4E/XRk7hOacYhaSsF6XFOw81cI7QVSlblSO9g=</t>
+          <t>FjlkiY2a5X+lrE+V3UAkF1LlbupyFJqSsAWuah6wFio=</t>
         </is>
       </c>
     </row>
@@ -17459,12 +17459,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>lN53Nb4QGdRlSIouBtuIsg==</t>
+          <t>0JJ3OpvNYqnbZCL72Rle4A==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>l1AWknEaaG57At7FUZBw0LPULPMxkRHrV1wHj1n3pYQ=</t>
+          <t>QFp9QRvbXEY1URrMZwea1DOWyzHA2LHb1dXskzWMD7E=</t>
         </is>
       </c>
     </row>
@@ -17486,12 +17486,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>sxCP5O4v49iY6yVyDC//pw==</t>
+          <t>bBdqFNTtZ0Ll91ZJL0ES5g==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UAKmE3Fh+r7rikEabkZMCTPRwzJdjnuxGPQTDiNpALU=</t>
+          <t>eEx016+LwZJOG5SVBhohWM0PGl7BpHfklrQIT1WB1Rs=</t>
         </is>
       </c>
     </row>
@@ -17518,12 +17518,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>o7NmT7LQMnulFw+MnJ0Vcw==;Ah3c6e4Ri4+vl1b4WK6icQ==</t>
+          <t>V1xEFybs/zQqXbXGkmXemw==;jHsjNKqpI4QkmXbrIOa2jg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>WXtTQZqyXE4DA1Pa8L2mzgecbXG1ahW/Nw/ZGTYENAk=;+ESmF2FhbZu5ALV2YktZisYJ3etGjYPav5uS5zPYKTE=</t>
+          <t>ocY72Jnb7sEd/wfO2Z4EALrvfbQ2LwkJy7XvdLBSQXQ=;CwMFqszHKkq5V08uIPOnXMcBL0e+t4svTcdvsDTmM1Q=</t>
         </is>
       </c>
     </row>
@@ -17550,12 +17550,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>aYibzIXvOItOc98nUPgORw==</t>
+          <t>N3qcAvOcAYvr6vGFVaH/Bg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>uobc5utBXQ4yF34cgVUOGCXVX23spSyDeOjSuFJQ6dk=</t>
+          <t>hRFnzIy/Qt3sILP40RcgAcX5amaznUn7s2/eE4I7u/s=</t>
         </is>
       </c>
     </row>
@@ -17582,12 +17582,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1Vl0Gaae/LaLwg5wcgcSOw==</t>
+          <t>w2P4vMP65OwEOvnZt4+Flw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ZGFoICiPYaLGsA5ODsYLG5ksUIEhqBwNVf7TmDrO/RA=</t>
+          <t>MElr2ud4uW2WM4g0u+7jxsmZkvmerOcKNgyq1vKhm0w=</t>
         </is>
       </c>
     </row>
@@ -17614,12 +17614,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GU+FP1sq/PeWqLHW47SBFg==</t>
+          <t>j3WbvxNXYprmekqGjZHGkQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>EJ/PCI/QQkIUQc/DLmXSxWUnBv/U3E34kzEcKjjR1pY=</t>
+          <t>qV4FlQ/rmNsojPNn4zu1DVHz4PkzCHxHiK1FZJuXQP4=</t>
         </is>
       </c>
     </row>
@@ -17646,12 +17646,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>bgeVOk/I6xLJG343sOiV4w==</t>
+          <t>iC2qzdQPUd0qPZybQzjpyw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>gYAdJ1buRF1b9SV/c0IBGbDcRpB0Ft9noE33LlP/8rM=</t>
+          <t>fk4ZBXXq50afUf1CnQyeo9oeW6VQ+NVqcOzi3QOBxWg=</t>
         </is>
       </c>
     </row>
@@ -17678,12 +17678,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>q3lmBhsFz8xMg3MWP2CRCg==</t>
+          <t>emI3BGDpu7MJt9oy75OLRQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>EWpukGWdluXIwSyonRCK724WMNfzJUFvnzSpMnPIk0Y=</t>
+          <t>JyZ+mLnOMr4LBUkrnEcO9OCOGKSbznk6hAy4ScCGCEU=</t>
         </is>
       </c>
     </row>
@@ -17710,12 +17710,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>l2wJYNAmBuZANgTRX3uxaw==</t>
+          <t>Vj1+EJooUtgr9O/6x8Wv3g==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>XoAiS5LGWKKq3U+XmxhScroZxwQ68qn+obf4gXmmmBI=</t>
+          <t>J27hj7vufJ64Y7gjRvRFMPbf6IYWN1RppirPFsBkI3k=</t>
         </is>
       </c>
     </row>
@@ -17742,12 +17742,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>C4azEe+m64ZUPis9y5eaIw==</t>
+          <t>tpb0cDBrYYZ+k5ZzcUp4lw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>oO5YabUHKRrYAHO0Fbtg0wYatxHHgMBPAuYv3VJ0n48=</t>
+          <t>KJnE7uGjlULJucxXtYE8u4wzHoOCKPxZgu8OVoBPvBo=</t>
         </is>
       </c>
     </row>
@@ -17774,12 +17774,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>iShfhSPoHk0QyFLd0HaMOw==</t>
+          <t>XofEs3SwD1BQ3WjsHofFxg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>J7MqZ4IP8F48NndnP9J5n5bQy4jJ2Ix1asVHFKWDOQ8=</t>
+          <t>nPd6HTP4EY2ux6SS5idwvkJjJWRcxt+8OeGYmLDm+EI=</t>
         </is>
       </c>
     </row>
@@ -17806,12 +17806,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>DVg5rjI9wbXLwrmlXK/Hpg==</t>
+          <t>qI4ajdiihBx7j4D80uqbtg==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>D67V4OhDX6fj4GAwkHvsKUzs/X5/YMPQrg0e8hF0izQ=</t>
+          <t>v6pT09ckHFmfjj8p8SruvO50WMaIvHSXD6sZriIdlAo=</t>
         </is>
       </c>
     </row>
@@ -17838,12 +17838,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4GJfLQqMNN7OKxRIQSuiag==</t>
+          <t>a5sETYAXZ8l/RDmNIp2tjQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>jDfSIPztlIFsinHIWUH72md9ixfF0SjTkwgllEMjJQ0=</t>
+          <t>kMJIWCgoC1a3zWodONTh7nicdaTsGL/uL60oriDPnOM=</t>
         </is>
       </c>
     </row>
@@ -17870,12 +17870,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7f0zBhw5oJRWVWSOqU9I6w==</t>
+          <t>4yEefvpZhZkE/hVKk5vJlQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>95l6BtodKaqLQnOmjpLW20CA4DjrejfBjR5kmY9i+PM=</t>
+          <t>BKk2RoNJ3SdImDRgK/GJQ8PlUk3bhcsvFnRYDUEDsq0=</t>
         </is>
       </c>
     </row>
@@ -17902,12 +17902,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>tSgKjYj8xcf8yqBDj5whsQ==</t>
+          <t>BrCe31/bzHxKi2p+GWxW5w==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>KL1P4/78J8lfB6O3hyvG+e3FVkLTiBotr8WGJHATfcI=</t>
+          <t>3zkLJKx0Rm/6xqMl0kijnXt88pC7kCDV3pVUmSzXDmo=</t>
         </is>
       </c>
     </row>
@@ -17934,12 +17934,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>jMRALTyVuGG+mgBJSG42MA==</t>
+          <t>mIJK+9egkNx1IhKS5mIIvg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>4Pt32u8fCxVHpapb3tRd4BB6qrYeiX757gzRy4eNZwU=</t>
+          <t>mcG+6tXaf/xgyo04pydhv/xv1VC+rwxN6eLJxTYOhP8=</t>
         </is>
       </c>
     </row>
@@ -17966,12 +17966,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GvRCWG9h0cOAG//+wf617A==</t>
+          <t>4JqcftGX/mhY/mcThgTf7g==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>y1ocOwZCP15TNvm+NweiqNiSQv+OHg4q4bkQF8cC5BI=</t>
+          <t>taSnvijzib5v7tnw+0TuXIOQwTSXHh+vYcsCNBswads=</t>
         </is>
       </c>
     </row>
@@ -17998,12 +17998,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>z8Y0K4s7hq3BBTZt0ZW4BQ==</t>
+          <t>ey+4Ml4aKo7/X1kgrovreA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>65ljYhkTk8TOa2n4Ir4PNLz7TO8dExvR8qdT0wvRbaQ=</t>
+          <t>zGcPA5qDiRQfmKLJbthaU9F070GZiSWaCRd2BthR4zg=</t>
         </is>
       </c>
     </row>
@@ -18030,12 +18030,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ywy9BW/d+0Yvz5W4ZK54rA==</t>
+          <t>Dt+o2jkpfKbhOf+JP48fEA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>w3jw/kmvG7RJM59zcuFX82CPgY9WHZDL4hLMqfwgDsg=</t>
+          <t>UcYAwYhMziWZqeGVj6uHjk1RZjQiHHp35uENcuSVKH8=</t>
         </is>
       </c>
     </row>
@@ -18062,12 +18062,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>f2kKJKCchFmaq4WM53rhOA==</t>
+          <t>BvqlUgXGbaeR2G+iljPtpA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>gnAj/drdIcT+mSfSeZKjT0RUqVvvR7pUINA2yq5qPwg=</t>
+          <t>Nr94LOoWdc71i6lpZtcA0k1mnqALSZdFPxVPrkIRo/U=</t>
         </is>
       </c>
     </row>
@@ -18094,12 +18094,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>hF1nn4Ny+IFtEDyHbkDMgw==</t>
+          <t>Si3g8my4VyFVWXOltlS1oA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Dre9aU0WmLSvz76rmpiT/Ta2/XGnSLuRl5yaLOkd0rg=</t>
+          <t>GrZjV59Wpq4wxetdlc5KpFT8QmJgpsrVuFQjO+GoryE=</t>
         </is>
       </c>
     </row>
@@ -18126,12 +18126,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2V6rv8y4mpoU/YCtKepHxQ==</t>
+          <t>2POafq6jxSTjJhzwWCQ3hg==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ZnWfykwJy2CCtLeg8sDo9+5ImpNiidvRr5iwAO2y0xY=</t>
+          <t>1+uettmDsPA245BZH8AW2Yhm3eIlQkoBWTZOiNUJdx4=</t>
         </is>
       </c>
     </row>
@@ -18158,12 +18158,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>v/rS1S64lukqlibjp5JgTQ==</t>
+          <t>M56NTJT5LT78XpOP/FvR2w==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>5A85q+H8l1ilYqIqT2is/hTsGFQfePuf382D5du7uXo=</t>
+          <t>/enKdCm/tADTK+ce+1vlNmpY9aMaTBrbLa+D4E7bkZY=</t>
         </is>
       </c>
     </row>
@@ -18190,12 +18190,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AWvTj3bSfcVOPqhsqONbwQ==</t>
+          <t>MYYAFVIDb/oAPiK5jcHmmA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>N/APm+WGLuRFMUmusjzlvD8sbaMLcr+jbNXBm5sTzuA=</t>
+          <t>uRueaeabKzKZ7R1d3FLmBAnZXdO48CsHWiFDydfM4vE=</t>
         </is>
       </c>
     </row>
@@ -18222,12 +18222,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>sY0U4H4KDvNmKnW2wCYbWA==</t>
+          <t>Ljxdf6E4oNAdCHYG3yfrzw==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>s8k8nIqBBFEv7+0c55zRX+E/iDtiY7skBjCum1tiApk=</t>
+          <t>iK1GOmCiHWzIrjLWybwjNd/q1zv1ef9cmZhTjo2NuAI=</t>
         </is>
       </c>
     </row>
@@ -18254,12 +18254,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>MibTNruOrgYcyrFJ5EYhWg==</t>
+          <t>xZdICbOyHitjLEWmfy5E9A==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>L58Sd0HRjSxLjbczhB1fWjOK1paj2BymcUIpHjS6Njg=</t>
+          <t>W/penPz8oMIqDhBhjeqE8qhdJ2rHCqzHs1xKZAbQ1d8=</t>
         </is>
       </c>
     </row>
@@ -18286,12 +18286,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>h4tNXCqbmy9vuvcu54vDNA==</t>
+          <t>oDkDY/sJC3JQoDzpyDgqPQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>+i27jZcWtg8rVspP3ZRhXQdAEtviAZe67l5X5QCQ/Po=</t>
+          <t>DFfXEIFKDy0Qd6aErVq/I6d7I5i23D0Xq4lGvKkmG1g=</t>
         </is>
       </c>
     </row>
@@ -18318,12 +18318,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0XXtlk6I/hdlfSqCxNAlRQ==</t>
+          <t>2X4LPqLAGDT3tu96uJ7r3Q==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0tWKoR4g4sY1ug6N+dfHYY/lh40o8DNiexSbBsNcVao=</t>
+          <t>3HGhEkGwTWYyLdwRX2cJgr0lPzUtxsm+J0gxbtPo3O0=</t>
         </is>
       </c>
     </row>
@@ -18350,12 +18350,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>zayIxoqu1KSu+QPSVFdy5w==</t>
+          <t>qi9cygrH1dr06s0JGx335g==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>gSEiIQGiuuGXDHLksTh58NracnPQt484s9rYLVgsYUQ=</t>
+          <t>5nErgohydaIJtRUnd4jHKv1+hh/mjPK9jEf04WWlun8=</t>
         </is>
       </c>
     </row>
@@ -18382,12 +18382,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>bYQfixQ78hlIlGINue7BSQ==</t>
+          <t>zCVM7XVoYSP3jL8uG0wF/w==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>/kPGlGQxUA0qcTjRDhWSSJmgqTW6OYP8bitdSiIxIto=</t>
+          <t>0wY2LmRCG0NJvSZWl+4fPUeXDGn2jlDQd1rri50YQ4Q=</t>
         </is>
       </c>
     </row>
@@ -18414,12 +18414,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2vZySjKepWnnbJ3rFOw63g==</t>
+          <t>eR2x9cpRZNdIlf4UTzCFhw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ZWCAeoUdebJBSmaZhoF4JM4ShmKpmpkjA6/6UvFtm9A=</t>
+          <t>oPFypAlVQGbZZ3lxThPr4PUz/9pDbXrBwtjPXr76Bg4=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-26 07:39) - 119 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40">
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="86">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="88">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="92">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="95">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="97">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="116">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="127">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128">
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
@@ -5119,12 +5119,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130">
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5263,12 +5263,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2026</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1ddf1ffb-0655-4b37-96ee-4ee69ebd5764&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5319,7 +5319,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f81dd4b4-8d4e-4a57-a673-eff19a270837&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -7486,7 +7486,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -8734,7 +8734,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -8846,7 +8846,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -9326,7 +9326,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104">
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="110">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="120">
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="127">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="132">
@@ -12622,7 +12622,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="139">
@@ -12678,7 +12678,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="140">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="149">
@@ -13626,7 +13626,7 @@
         </is>
       </c>
       <c r="L157" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
@@ -14398,7 +14398,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="172">
@@ -14786,7 +14786,7 @@
         </is>
       </c>
       <c r="L179" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="180">
@@ -17272,12 +17272,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>8xEcUKsFe74ZVePLv19Z8w==</t>
+          <t>lcgozS+n/AnCcXJrZMkQIw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>hQZySSIPa9PEX5Zn+jyOQ7W8F6ZMLt8rcTCrRakYExc=</t>
+          <t>RY68LWPMRWCs8VsFIWichl1LeQh3itkawwkl9i0RTkc=</t>
         </is>
       </c>
     </row>
@@ -17304,12 +17304,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>hzcuRpa1WW5wA9BEy7f4CA==</t>
+          <t>SiC9efeiZpQD5lbmhPDAUw==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>iG660XCBKIxDfPlfuNou7kA3IK8eCvGT6uLJzURN9U0=</t>
+          <t>6esIF0NU9mbG/kR/4zHkxTN9FGWT8IDk6A9x1V7UEAo=</t>
         </is>
       </c>
     </row>
@@ -17336,12 +17336,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>nt+9eRN9YNG+pwQS85mSGw==</t>
+          <t>2vL0Xe1A2Ff3DrbIsLgUcA==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>vmKziK/PolLdaaRJ+ZwBz0LVSxD+LWrQ3WgGUJygpuY=</t>
+          <t>dqHpFvkBQI4dyYj7pM3ty1SjR/ZbCOyrvjn9sD0meUc=</t>
         </is>
       </c>
     </row>
@@ -17363,12 +17363,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>KgaLOd1D27NA1mWUaiyjfg==</t>
+          <t>mkbVxYFH3y7JPuR11Mj+qQ==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>RKNj9iHc5h0UmQHYGv1+OHbPST6ilU+2YmPoCTh2YBA=</t>
+          <t>QUAj+kX2ZAttsOYI5NPy68tobJVpkJrqQOLL5ZphK7k=</t>
         </is>
       </c>
     </row>
@@ -17395,12 +17395,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DSkdotymuLR7lCFG4zGt+g==</t>
+          <t>gD4KyJe7HJhOiOJswrKuoA==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>iZk+A5C2hgRUcp8GWy2bG55JIoGv0dT9onvyLMqctWQ=</t>
+          <t>SrvVQCbMR8eNAaeMZiQdidsRNsm65r4KNfoiX/cY8lU=</t>
         </is>
       </c>
     </row>
@@ -17427,12 +17427,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CiI3hzhkX3aYJQ+pWnmeLw==</t>
+          <t>VnrTFGQX5AZFGAue9OSYeg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>FjlkiY2a5X+lrE+V3UAkF1LlbupyFJqSsAWuah6wFio=</t>
+          <t>uSayJk4fJmJxivkKKSj8RTgt0SzO0U2miNACAqiU+Jc=</t>
         </is>
       </c>
     </row>
@@ -17459,12 +17459,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0JJ3OpvNYqnbZCL72Rle4A==</t>
+          <t>kbhjcVlZR+hiK4VaXKql3Q==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>QFp9QRvbXEY1URrMZwea1DOWyzHA2LHb1dXskzWMD7E=</t>
+          <t>MXxlTrI3CyQTpBbNxPPaMg5bniDDnC/xdHijYDpntVE=</t>
         </is>
       </c>
     </row>
@@ -17486,12 +17486,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bBdqFNTtZ0Ll91ZJL0ES5g==</t>
+          <t>CrDyWhpOt9USPRQ6plTsLw==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>eEx016+LwZJOG5SVBhohWM0PGl7BpHfklrQIT1WB1Rs=</t>
+          <t>3zD9QHt3CsmQK1zh4e5AbkywB/g473EI5kimishaWdc=</t>
         </is>
       </c>
     </row>
@@ -17518,12 +17518,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>V1xEFybs/zQqXbXGkmXemw==;jHsjNKqpI4QkmXbrIOa2jg==</t>
+          <t>QHW2KWftnu5mF9202z4w7w==;Bwv6kF35MLZ6Z0GFPRWfYw==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ocY72Jnb7sEd/wfO2Z4EALrvfbQ2LwkJy7XvdLBSQXQ=;CwMFqszHKkq5V08uIPOnXMcBL0e+t4svTcdvsDTmM1Q=</t>
+          <t>RCePSzN07Baxl7MayJVN4sxDMf23k26h2tKuBD9vP2k=;iRN/dFZXP5FSkTUYGRJXoQv+CfIARuWq0aSH+KysHqA=</t>
         </is>
       </c>
     </row>
@@ -17550,12 +17550,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>N3qcAvOcAYvr6vGFVaH/Bg==</t>
+          <t>7WXfidJy1vBXOmXnbYrmJw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>hRFnzIy/Qt3sILP40RcgAcX5amaznUn7s2/eE4I7u/s=</t>
+          <t>gtYsb44q65MZyhokR75xRddmn1qA8e4fDWK7H1x/d5k=</t>
         </is>
       </c>
     </row>
@@ -17582,12 +17582,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>w2P4vMP65OwEOvnZt4+Flw==</t>
+          <t>dYfnxk6Pu37v7oY3l/QQOQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>MElr2ud4uW2WM4g0u+7jxsmZkvmerOcKNgyq1vKhm0w=</t>
+          <t>rsuy5MSmEGRCFRe8cci5p/+ik5FW+D628GNuFqgOoFo=</t>
         </is>
       </c>
     </row>
@@ -17614,12 +17614,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>j3WbvxNXYprmekqGjZHGkQ==</t>
+          <t>HPFrzFhSvnGigGeiz6Kp3g==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>qV4FlQ/rmNsojPNn4zu1DVHz4PkzCHxHiK1FZJuXQP4=</t>
+          <t>KUVJIxXRc7oMvGMWHiGI3n9qjRCMXqxlYQty0V2GKgE=</t>
         </is>
       </c>
     </row>
@@ -17646,12 +17646,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>iC2qzdQPUd0qPZybQzjpyw==</t>
+          <t>aQ5LAZPMiCOoQIFg852cog==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>fk4ZBXXq50afUf1CnQyeo9oeW6VQ+NVqcOzi3QOBxWg=</t>
+          <t>jlvnuxpbtco948OvNo5XjPaBF56wPRIs0RRK5nQQy+s=</t>
         </is>
       </c>
     </row>
@@ -17678,12 +17678,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>emI3BGDpu7MJt9oy75OLRQ==</t>
+          <t>GT7WW9bcLOb6W/G2SyHXmQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>JyZ+mLnOMr4LBUkrnEcO9OCOGKSbznk6hAy4ScCGCEU=</t>
+          <t>1reUhhckevH0cHkrPEexdy1xTKyYyo0U7yskMpu8Cu8=</t>
         </is>
       </c>
     </row>
@@ -17710,12 +17710,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Vj1+EJooUtgr9O/6x8Wv3g==</t>
+          <t>8Pa5TXc9dxe3IkL1E+JLRw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>J27hj7vufJ64Y7gjRvRFMPbf6IYWN1RppirPFsBkI3k=</t>
+          <t>gpwTWiYRu72cLdpNbwhI4NinY65RbKdMfAA+LxTEh6Q=</t>
         </is>
       </c>
     </row>
@@ -17742,12 +17742,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>tpb0cDBrYYZ+k5ZzcUp4lw==</t>
+          <t>1jnKeqfjRNHdoG0NJ7bOLw==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>KJnE7uGjlULJucxXtYE8u4wzHoOCKPxZgu8OVoBPvBo=</t>
+          <t>Edw2f3U0eKwLa7pTryFhvMuvdaMtttzKgR2E+SDJWWY=</t>
         </is>
       </c>
     </row>
@@ -17774,12 +17774,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>XofEs3SwD1BQ3WjsHofFxg==</t>
+          <t>gEIdzVTOh7BAdLtlGZG/Bg==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>nPd6HTP4EY2ux6SS5idwvkJjJWRcxt+8OeGYmLDm+EI=</t>
+          <t>rx96uJFxTSfaK42NHDEim9wXPU6DLw3gwAtCubny3b4=</t>
         </is>
       </c>
     </row>
@@ -17806,12 +17806,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>qI4ajdiihBx7j4D80uqbtg==</t>
+          <t>1glnVV6D/MMtvft1cRBZrQ==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>v6pT09ckHFmfjj8p8SruvO50WMaIvHSXD6sZriIdlAo=</t>
+          <t>rSb/tOR5XuKbW5ZeMOP4mzINvQa2dWrtoA1AoMilgXc=</t>
         </is>
       </c>
     </row>
@@ -17838,12 +17838,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>a5sETYAXZ8l/RDmNIp2tjQ==</t>
+          <t>JC3rEExLmqQEy0rZQzCpUQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>kMJIWCgoC1a3zWodONTh7nicdaTsGL/uL60oriDPnOM=</t>
+          <t>3BSDq2bGAWQGqpOl0ZzmlL7jwzM7+fke9GHl15yfcig=</t>
         </is>
       </c>
     </row>
@@ -17870,12 +17870,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4yEefvpZhZkE/hVKk5vJlQ==</t>
+          <t>Xpc+srtL+CDMiFCbxdn/ng==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BKk2RoNJ3SdImDRgK/GJQ8PlUk3bhcsvFnRYDUEDsq0=</t>
+          <t>k+LGrsyegnZPm3js3u9+V6SIEvmPmIzKUv+nsygvMHU=</t>
         </is>
       </c>
     </row>
@@ -17902,12 +17902,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BrCe31/bzHxKi2p+GWxW5w==</t>
+          <t>kd1H6HOXdvEF3dDjkfu6IQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3zkLJKx0Rm/6xqMl0kijnXt88pC7kCDV3pVUmSzXDmo=</t>
+          <t>EkPv3fCzNnjAcYRnYnV6fEcIyh3yW7tZo5ePELH7d6w=</t>
         </is>
       </c>
     </row>
@@ -17934,12 +17934,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mIJK+9egkNx1IhKS5mIIvg==</t>
+          <t>GhpD0iBguiLitvajJ5S6OQ==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>mcG+6tXaf/xgyo04pydhv/xv1VC+rwxN6eLJxTYOhP8=</t>
+          <t>jH/rllGH+40YXqNe0whIy3FCOUXCRURenID+92zXRHA=</t>
         </is>
       </c>
     </row>
@@ -17966,12 +17966,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>4JqcftGX/mhY/mcThgTf7g==</t>
+          <t>FPCRCXi+dumOcy2NUPxADw==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>taSnvijzib5v7tnw+0TuXIOQwTSXHh+vYcsCNBswads=</t>
+          <t>M3ena4VZbS/UALSrVT7ZzCQ3tYDusib9DrDlxUS9vAE=</t>
         </is>
       </c>
     </row>
@@ -17998,12 +17998,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ey+4Ml4aKo7/X1kgrovreA==</t>
+          <t>EhMnOpDHahPrqQUB5YmazQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>zGcPA5qDiRQfmKLJbthaU9F070GZiSWaCRd2BthR4zg=</t>
+          <t>BZtlZZY2HrVlNV7crKUgVOdZlf9CKVWQu0j3ET/jdL0=</t>
         </is>
       </c>
     </row>
@@ -18030,12 +18030,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Dt+o2jkpfKbhOf+JP48fEA==</t>
+          <t>0PzNXB5jgA5CFAkm+uFjIQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>UcYAwYhMziWZqeGVj6uHjk1RZjQiHHp35uENcuSVKH8=</t>
+          <t>ATLDjSGvkiPmd8O13xFJDGi3+rN7cCXetgvSzvq4F5M=</t>
         </is>
       </c>
     </row>
@@ -18062,12 +18062,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BvqlUgXGbaeR2G+iljPtpA==</t>
+          <t>FrxMTFcZdpl6mR77i0PZNg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Nr94LOoWdc71i6lpZtcA0k1mnqALSZdFPxVPrkIRo/U=</t>
+          <t>CYFiwXBsc7MCOAAz575sB5lnV7ML2QZNeWS1Y05ZPvg=</t>
         </is>
       </c>
     </row>
@@ -18094,12 +18094,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Si3g8my4VyFVWXOltlS1oA==</t>
+          <t>H59QFKhurXwPDJ9T8amLnA==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>GrZjV59Wpq4wxetdlc5KpFT8QmJgpsrVuFQjO+GoryE=</t>
+          <t>VoVAn3ZceA/e6Hk0yVn6erWuXgsqjG0Jc7zANohz/LU=</t>
         </is>
       </c>
     </row>
@@ -18126,12 +18126,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2POafq6jxSTjJhzwWCQ3hg==</t>
+          <t>JwKKs6GIlX1wIHdkZKQWyQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1+uettmDsPA245BZH8AW2Yhm3eIlQkoBWTZOiNUJdx4=</t>
+          <t>RYsPvJctuYNn5QkwqFdljQWEkl2iVgD0Zy/JkkjCAyo=</t>
         </is>
       </c>
     </row>
@@ -18158,12 +18158,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>M56NTJT5LT78XpOP/FvR2w==</t>
+          <t>OSoy/NjZ3mnGPb6rASMEZA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>/enKdCm/tADTK+ce+1vlNmpY9aMaTBrbLa+D4E7bkZY=</t>
+          <t>Xe4MrPY8wN0qjaKBTfAaIE9Fkvi1CyOU1wXWtmWKzGc=</t>
         </is>
       </c>
     </row>
@@ -18190,12 +18190,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MYYAFVIDb/oAPiK5jcHmmA==</t>
+          <t>adacpKwQimP4kb35tiptPw==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>uRueaeabKzKZ7R1d3FLmBAnZXdO48CsHWiFDydfM4vE=</t>
+          <t>E8FyktVzYpOwtwZTQZDtAhYtzC5z6fsZPmAlbUB8Gko=</t>
         </is>
       </c>
     </row>
@@ -18222,12 +18222,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ljxdf6E4oNAdCHYG3yfrzw==</t>
+          <t>UOWsyvyRpG+q5wkuJEaHLQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>iK1GOmCiHWzIrjLWybwjNd/q1zv1ef9cmZhTjo2NuAI=</t>
+          <t>KuNejcu/5GiIsFnmAtRWCjDEytGGwl1uw1FD47f19gI=</t>
         </is>
       </c>
     </row>
@@ -18254,12 +18254,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>xZdICbOyHitjLEWmfy5E9A==</t>
+          <t>3VtuGm/ONcgTnK6FXxpgog==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>W/penPz8oMIqDhBhjeqE8qhdJ2rHCqzHs1xKZAbQ1d8=</t>
+          <t>uJ2DtIVrF3Jhkl6aatHJzSb/o65CwWQE6fQDBSuYS+k=</t>
         </is>
       </c>
     </row>
@@ -18286,12 +18286,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>oDkDY/sJC3JQoDzpyDgqPQ==</t>
+          <t>6NAG8An/egXq8zmYTLLYrQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>DFfXEIFKDy0Qd6aErVq/I6d7I5i23D0Xq4lGvKkmG1g=</t>
+          <t>QP7LC3P/ZhzOvCR8C20wjX9eCZ//lGtEhkSS1cwcFQE=</t>
         </is>
       </c>
     </row>
@@ -18318,12 +18318,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2X4LPqLAGDT3tu96uJ7r3Q==</t>
+          <t>IaPvkZY54Sjit6DNNB8asA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3HGhEkGwTWYyLdwRX2cJgr0lPzUtxsm+J0gxbtPo3O0=</t>
+          <t>XalYWpwIcvPW1VKgSjTfvGYI2REUIzyCLKxPMIM65Ek=</t>
         </is>
       </c>
     </row>
@@ -18350,12 +18350,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>qi9cygrH1dr06s0JGx335g==</t>
+          <t>wsbxV4oFt0VZ5IrqFzsYBQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>5nErgohydaIJtRUnd4jHKv1+hh/mjPK9jEf04WWlun8=</t>
+          <t>QmYjw19X1EkYlC+cFn6QFwRszv0rKhR80+zJopZlCPo=</t>
         </is>
       </c>
     </row>
@@ -18382,12 +18382,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>zCVM7XVoYSP3jL8uG0wF/w==</t>
+          <t>ApjGE8K7b1xtHyjsb6XusQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0wY2LmRCG0NJvSZWl+4fPUeXDGn2jlDQd1rri50YQ4Q=</t>
+          <t>sCFHt2XnzrSyOdtnvDdBPdx0dvphRwWX/Jmxk5fXEXw=</t>
         </is>
       </c>
     </row>
@@ -18414,12 +18414,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>eR2x9cpRZNdIlf4UTzCFhw==</t>
+          <t>Ulqb46OD5wp/ala9qjwlMw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>oPFypAlVQGbZZ3lxThPr4PUz/9pDbXrBwtjPXr76Bg4=</t>
+          <t>tH5WQMlfNJc/LpdUOqxL/wNxL2HGUYcFTCs9+H5P+M8=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-28 07:40) - 105 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="39">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40">
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="44">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="47">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55">
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56">
@@ -3219,7 +3219,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="77">
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="78">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="80">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="82">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="83">
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86">
@@ -3623,7 +3623,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="88">
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="89">
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90">
@@ -3731,7 +3731,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="91">
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94">
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="101">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="102">
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="103">
@@ -4235,7 +4235,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>535</v>
+        <v>546</v>
       </c>
     </row>
     <row r="105">
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>535</v>
+        <v>546</v>
       </c>
     </row>
     <row r="106">
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="107">
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="108">
@@ -4379,7 +4379,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="109">
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="110">
@@ -4559,7 +4559,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="114">
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="115">
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9">
@@ -5722,7 +5722,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10">
@@ -5854,7 +5854,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13">
@@ -5898,7 +5898,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60">
@@ -8374,7 +8374,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="61">
@@ -8642,7 +8642,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67">
@@ -9974,7 +9974,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="92">
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="93">
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="97">
@@ -10242,7 +10242,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98">
@@ -10286,7 +10286,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="99">
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="100">
@@ -10506,7 +10506,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="104">
@@ -10986,7 +10986,7 @@
         </is>
       </c>
       <c r="L113" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="114">
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="115">
@@ -11162,7 +11162,7 @@
         </is>
       </c>
       <c r="L117" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -11206,7 +11206,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="119">
@@ -11250,7 +11250,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="120">
@@ -11294,7 +11294,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="121">
@@ -11426,7 +11426,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="124">
@@ -11470,7 +11470,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="125">
@@ -11726,7 +11726,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="130">
@@ -12230,7 +12230,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="139">
@@ -12286,7 +12286,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
     </row>
     <row r="140">
@@ -12454,7 +12454,7 @@
         </is>
       </c>
       <c r="L142" t="n">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="143">
@@ -12542,7 +12542,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="145">
@@ -13358,7 +13358,7 @@
         </is>
       </c>
       <c r="L159" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="160">
@@ -13746,7 +13746,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="168">
@@ -14002,7 +14002,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="173">
@@ -15922,7 +15922,7 @@
         </is>
       </c>
       <c r="L207" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="208">
@@ -15966,7 +15966,7 @@
         </is>
       </c>
       <c r="L208" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="209">
@@ -16054,7 +16054,7 @@
         </is>
       </c>
       <c r="L210" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -16140,12 +16140,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>iqOvTiLti/zKbt3mc7+/7w==</t>
+          <t>V//ZseinJqu5VhMooUT+LA==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>+pXtyV/NlxMqoVLTshk1xuFyc0gsiTPNL2HamXQXOHI=</t>
+          <t>QyePwSQgcTAqBCnFXIIrro9nmDqSJajXrTX/mW+pYGM=</t>
         </is>
       </c>
     </row>
@@ -16172,12 +16172,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0dXZiQ4nj+Y0z6TKM0eDoA==</t>
+          <t>nk57NnuYnwd3hHsbIIekIA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>aSkSi01PuCXP9VkW16yw7Gh8wDZWlxYQVuYzD8Z2bps=</t>
+          <t>dQfDPux/8EAe8AjxofYt/Jy4rrM5bQS0JjSVzEvbfXM=</t>
         </is>
       </c>
     </row>
@@ -16204,12 +16204,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5MERFX7mn4qrfFZmVdw2hg==</t>
+          <t>TVm2ebeXl6Qq/Sc5b21V9Q==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>jZn7TNgS2UaoCMeg/WzfS0SKHDdv0xO8CznXwzITOR8=</t>
+          <t>7D40of60B7vmQnArovrrpo3TfEISZ1g6v/UdM9CYIZc=</t>
         </is>
       </c>
     </row>
@@ -16231,12 +16231,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ph7P2juva/eR7MwG7ROH6Q==</t>
+          <t>oV/wQ/E3iBqTUO2pjmPGnA==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Vr5sFMja7XbD4ShHfUXpdR4vGM1/Rf8OcZFzV34Xq/s=</t>
+          <t>trJSggjnVemZ/liVmPn12hFL6KX/RCVoDH1YxHFBKyg=</t>
         </is>
       </c>
     </row>
@@ -16263,12 +16263,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>/bSicem4YZJwypx9lwsD2g==</t>
+          <t>1wIoyXnc8R6xri3dfsIAZQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WsV57gluQxfYc5cQDm4Z8Su2PPjefzkph2yQUHuWPm4=</t>
+          <t>KJm14uLaFOXC+pFH08ljtshcdylsbsyIu1f/fYHZxLk=</t>
         </is>
       </c>
     </row>
@@ -16295,12 +16295,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>YXGUNp88AJzqjv6uoKw38Q==</t>
+          <t>am3X9viG4zOvzp22/xlI3A==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>96lvU+EHaVf7ln8n4SbneF5qNjeW/FT0EMiccmJlCQ8=</t>
+          <t>bfOpY2+epSNEC6WaKKUafSUcRWRi4KTMNPoKIEHfp5s=</t>
         </is>
       </c>
     </row>
@@ -16327,12 +16327,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bEMixLVYYTQFjHj0RRITnA==</t>
+          <t>E6b87GSND9HsS/+0vPBN9A==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>NcdUc/H4pvM3qZfDDsbnXIhVfneYvpz1jatfvva44+4=</t>
+          <t>oJqP7V3KCV4WuoK2m0bElVT3IHfGt6nT3Oq6yKPtba4=</t>
         </is>
       </c>
     </row>
@@ -16354,12 +16354,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>T9VwSlirKL/d4t7oSHZaQg==</t>
+          <t>bu8Qf2HtvOm8TYOt6D//HA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>mX9SVxIoyxltFjeqLmAZ5vLCFhSCL9FSol9KHGUSvpk=</t>
+          <t>owm2YINTb71ZcBoAN1rI84n+QsH+R6QohqlqsPyyTRQ=</t>
         </is>
       </c>
     </row>
@@ -16386,12 +16386,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0LNd/bbzBc74z/DrYsldqQ==;beDzbfNmNn1uS/2Rlgnaxw==</t>
+          <t>XzWQ920ISqKHlwHfXFt5Gg==;egOXso7+9P5kFbdFRbUYwg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>qJme7PnQ2HrV821B6i3GaeEhXq21OGZ9OAnEX14SBQE=;GNjxZGPdWJRC1JdVjKlJMEQe1+vSSx7IMir60eyWQnE=</t>
+          <t>3AYGW3CLDBlNjT1+l7+iO6QLHDjJbO26sB7q6yszlxo=;RKeQZfAc8DweK7+jGf95reTe31C9xVweMPQYtJeEKMQ=</t>
         </is>
       </c>
     </row>
@@ -16418,12 +16418,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TRYAr/RIYBTtLC6BInfiTw==</t>
+          <t>sPVp0+f1qs6D5HpAbek2sQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>xBTgtcDmERNG0iY7+lc39SCmRNR2N2b8cFjgM4z2E9g=</t>
+          <t>XC3D0n2LAbPCbfEJgRFWi2pxMgv38qKtuGUwRL5TPx4=</t>
         </is>
       </c>
     </row>
@@ -16450,12 +16450,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13m7cyVd/DjOWp+OT/NR7g==</t>
+          <t>TezL2E8UvJ5H6iOFISvkIA==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A7PQ4jDy7wvINZrEcfRIOOTzRMIMvufej5lO7z+fEUs=</t>
+          <t>Z1RTYYapja7N3sWU0rMp8VRn61+U/a7PnRuOeajR+a0=</t>
         </is>
       </c>
     </row>
@@ -16482,12 +16482,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>eG0BY1ZrQ9bvHylXuAgUWA==</t>
+          <t>9z+EzuZzUhoAId5CdrNnwg==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>hAY67KO2WiLUb1QE6AtPI4FyCPHEX3v+jbcMuxsPppw=</t>
+          <t>aq/vY49QYedl7lVLXnncXS5PSmi815Z9l/3dsoniQ8c=</t>
         </is>
       </c>
     </row>
@@ -16514,12 +16514,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xtRwqYlsfvBZOmWHIhwLtg==</t>
+          <t>03m15DnDP/XcSyHrAmbmfQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>j01+VEkY0NxF1h/2RSkPzWrVt6Y8QUZtoxWhnPkTChI=</t>
+          <t>ARrwy0tPiN7XDvugRqFjkcE754Zr/+KxfFk68kmiqPw=</t>
         </is>
       </c>
     </row>
@@ -16546,12 +16546,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>uei+Dm4UueKu7Smh3ws2EQ==</t>
+          <t>QiTHsBHExsVD1L0yaqT0Qw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>jyocO+sho65aqgMBgihkRy7oKTObtPC3oPHC74hZM8Q=</t>
+          <t>9L7DQw4kg4zFvAq6mZebahbIyFBfl6SMQ4MPtathKFg=</t>
         </is>
       </c>
     </row>
@@ -16578,12 +16578,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>kj6elwHdBt3U6caryZvkqA==</t>
+          <t>oqKxYOH4cz8bUdmCDzkCwg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dPBU7PO9GI1afRcANxw6ZnXqfk3xwyBEFKVqFK58WTs=</t>
+          <t>IKHkbMRv7oSzfN/Fq9GJZrag8K7SOu+mFbTTev5C8YY=</t>
         </is>
       </c>
     </row>
@@ -16610,12 +16610,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>LAT4tg+H/kvh/QASrkaEeQ==</t>
+          <t>K+Pqlx/ehKFqg/KEZNmq9Q==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0UkwFhi437MmfSia7gLRP+y2kBRCelT/7OYt9t5STuk=</t>
+          <t>mr7fkJfh4YibADSl73HIYKKnWkTNsZALnUaDoTcQX54=</t>
         </is>
       </c>
     </row>
@@ -16642,12 +16642,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5xK7b0tVmb7AedBb4zdfLA==</t>
+          <t>ePXdadrbBeHZAKKLKetbAA==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SE8a8mw/nySOg+rhq8bYepw0bw5uS+acIpwH0nWgFQI=</t>
+          <t>S3cfinxJk/PH3IZ+3G2xyu/q4DyetzuR1m5F/SjMMXo=</t>
         </is>
       </c>
     </row>
@@ -16674,12 +16674,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Imf9B7Mwgyc8dAC4wTzlaw==</t>
+          <t>KRJ4hhg3NDpqYVzhlE90ow==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>QEFvJEXGCx5EjXM3/+KGE9FKOgCGde2yVHP5lYPcwpI=</t>
+          <t>WBju6X1SzEW5Dfju7JA2p3lGiHXcjyiQ07Vfvv9KPFY=</t>
         </is>
       </c>
     </row>
@@ -16706,12 +16706,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>pv33RUUi7AYUSvdokhRljQ==</t>
+          <t>2xdfIgLgcN9GPpditGKKRQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>X1d7PPObW/llsn2fa3ICO/NO8WONdeX1SFWEL83+uYA=</t>
+          <t>HBfnJdDZNRZeaoEzPasIgettEL3gXe0hzB5OvvKDdxQ=</t>
         </is>
       </c>
     </row>
@@ -16738,12 +16738,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YOCbwiyOaImXfVXHemfV0g==</t>
+          <t>VW6cj7tZzdg8vch/O8WoaQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PrHJMLrsWYgr5xvPQt/1dF2iwYShWFsRZykW8YbPPMc=</t>
+          <t>BfSbmgnZMqr9aYOb/eBnxCQchsAWnNw8C37sJR3xT+4=</t>
         </is>
       </c>
     </row>
@@ -16770,12 +16770,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0XXreE1PKIuqPjwtWiNOCw==</t>
+          <t>5Bs6f+v5/w8OcnAAqsEmyQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>LOL1puOVnBJGHbVEX1I84bzvieZa0klU/FNSJkPsfzc=</t>
+          <t>678cyenGt5JzjLVBzNy51otgb+zd70+qaK+u4M2nB78=</t>
         </is>
       </c>
     </row>
@@ -16802,12 +16802,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>eohsJ2MrYA6R5W7NbhmfCQ==</t>
+          <t>sUy2E6OuGywIONCitGH80Q==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>9b/k/poipczp7k4NiyALoEGz/hDZovMAhV9raDSeuyw=</t>
+          <t>YLVwaVVU88fr3rJsmkbpmcZo6LJD5DRJ5oAZ9+uSPQM=</t>
         </is>
       </c>
     </row>
@@ -16834,12 +16834,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Rn3lz27WZio2CKT3jgCjcA==</t>
+          <t>GDjgLYQAcHCtT6as/uFwig==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>5QzL2YmqpDMPVFcZHJmY5DSHdF0kOFX/FKglGEvwm+c=</t>
+          <t>VHQLDIgsS5DwlBD8dpdfTmtU7toR3PBM3KujSJm4Kho=</t>
         </is>
       </c>
     </row>
@@ -16866,12 +16866,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7Bo5Q6k828f0403yV4ZZYA==</t>
+          <t>UfrqZIr5NMu+o3SgyM7jEQ==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>EvPjjks7y2fySiFOXa885ONPVhE9IyuELcZkb7DMAsA=</t>
+          <t>VRDAcCSidGaduIQUUgzsscl0oAIQel2UPlMLE5JmRR8=</t>
         </is>
       </c>
     </row>
@@ -16898,12 +16898,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>e+Ru74gpRinxHM4vsNthYQ==</t>
+          <t>ba3WcLEYmnMRHkbMW4a5tQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>baVBWMjN9iGxgmKY5B3MTnZUQMOjseWpHtraOIqPZdw=</t>
+          <t>VIylgHNhQGzYLjkoipJzCuzD+C0D4XMUwbkOOxiSfgc=</t>
         </is>
       </c>
     </row>
@@ -16930,12 +16930,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>pHweZrdQY/3nKmr6Qf+VOQ==</t>
+          <t>/QR3osWso0mYXKCAGkFItw==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>YKT3Exw1tp4ijKf6/ZSVTCqiGCIUsP40rz0/HcgYVXA=</t>
+          <t>c3TCkfYl5MBCLCzmjoS5DSpEfe2FaPy4k9hZdH7cjls=</t>
         </is>
       </c>
     </row>
@@ -16962,12 +16962,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SE1oJAIVXoBz3WlacbGlqQ==</t>
+          <t>qQ/BKBCyuVyJ/rK3Xnc1GQ==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>LW/ms13wOazmpnncyIkfRRFSiIqXXSrOHUYx/ywtVI4=</t>
+          <t>VcyIKvLmDcpPwSHXp+e+bX2SC6kkcdMKKR8eQQxH8I0=</t>
         </is>
       </c>
     </row>
@@ -16994,12 +16994,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>nXzROOc88H2wWdlwO3aO9g==</t>
+          <t>DRnFqTgrduI+jQ/8SWpmkw==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>VCgkVT5KN2uaFYzGq4wy+yriDqYntzCFqNBgV5sBvLQ=</t>
+          <t>BnGNdi6SZ577WiCIQarqWKQF/2tkBxWco5oSjS+vaW0=</t>
         </is>
       </c>
     </row>
@@ -17026,12 +17026,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HEF4y+OZd9NhrWfHEaZYfQ==</t>
+          <t>IZCwSHfPisrpZakami10iA==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>hRZSZD+Ihfuq5QwsIAtHbRbsSEDdmecswJBAMUFhgrM=</t>
+          <t>sWG2pJPGQUjbwkwSAikv770C/kFN+HKeBuIDWd9utkg=</t>
         </is>
       </c>
     </row>
@@ -17058,12 +17058,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>GErLUya/Lw4/mnKL6QhAbg==</t>
+          <t>OYbZZMiwxDfs+rvYafUHcg==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>qTjzgFnMo1pFF/X9ghs3Nn2SqXpkYSYT17eDGeCynyI=</t>
+          <t>KS6dKpP3Kqnkj/wrz74ZBvkZkQhznKzBFZa3x1VxUQI=</t>
         </is>
       </c>
     </row>
@@ -17090,12 +17090,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PPNDfpOpf5HsG+sm8x3NyQ==</t>
+          <t>9IX396O7/IeCi/sFJO5CZg==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>NcebA6OCdYOgqAaZGSSsQtcgexxJ7fwt/fOQa+pGlq4=</t>
+          <t>fAdv5HbA91GXVdolwS5nUPmg20TTdtelhlU6zSAmnUk=</t>
         </is>
       </c>
     </row>
@@ -17122,12 +17122,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0BFmpMozrQdoEAcI5l/q0w==</t>
+          <t>RA+k8brlto87EjAP5QDS4g==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>LbjIebQgC5dTOb66itcrhCcRZ364NwPPOf5AVPMmWLI=</t>
+          <t>zTIgZ/hy7JRfiCZmt3KPysDFkLx4CADan9PTsCXje1o=</t>
         </is>
       </c>
     </row>
@@ -17154,12 +17154,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>hZKIDpKnvtba0kWL3zzbwQ==</t>
+          <t>N5fQiQ/A2NmZOGIhtg7C3A==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>9n+WtmpbK/lnw1Xk0vULc4UxFB965Q7P7CtpmiGr2iU=</t>
+          <t>IcGeekVxg+xw4fhMrfbA20rqFd/xQpapyoUHyPeVrHE=</t>
         </is>
       </c>
     </row>
@@ -17186,12 +17186,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>KDnB8kt0RvbFVWlGx6xuYw==</t>
+          <t>6mXntvmkNGCUQE2/fLVJBA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AvOx+vT9gaV3tjnfBHvB3+GiQREdO8Xzeahi5Pfxslk=</t>
+          <t>Mf3o7NIoIDuPqYFEx7N/yfKK1vFLPtQ4PmeVYnwywi8=</t>
         </is>
       </c>
     </row>
@@ -17218,12 +17218,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>mIJYkMzUenLEa/fp+APw+A==</t>
+          <t>gPM3CVM4TcLwpVIaS2a9fg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>OT+9wL4QYf4n0Yrl7W6izxf+dBsj3FdA5gRDGa9/AYQ=</t>
+          <t>m4Ve9QUlp2hTyPrINM3P1hbYBBxoTzjMSl1jUA5eeBc=</t>
         </is>
       </c>
     </row>
@@ -17250,12 +17250,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>VxKLInF6CVh9PNINzbb1Tg==</t>
+          <t>k83Cp1snnaDWIlSQz+tziQ==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>LGd8TyZlvtxBNWfWRPLMvQv/xCiZ4F+B/YYxNBpMwMw=</t>
+          <t>S6BcjY7rcOn276c6qBVD24RYpj/km2SlsZqBFgBm21o=</t>
         </is>
       </c>
     </row>
@@ -17282,12 +17282,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>d69l9Yl6G55LBs3VnMATDQ==</t>
+          <t>ronWm0tytHhcMSqSLha3aw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>lftcEhi2ddaMiiDEVFu7SZ8kYyyZNftwUYNuo1HmENc=</t>
+          <t>VtSKKlbmsm9x0Nhxm7YYB3iMXpxzJJuHiCFs6N1fmDk=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-28 14:48) - 88 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -2777,7 +2777,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>COMPARATIVO VIGENTE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>COMPARATIVO VIGENTE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -9193,12 +9193,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DE06CfH4kBE7shg5Ao+2Yw==</t>
+          <t>/ABBGqtqXXIEAUv/r3aB3Q==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>kBu77Pue4NEzJQvdnL21uxr051s9JMPmTnTCj26rqlY=</t>
+          <t>lFIiYOfgUMxI1qtlli4+yqwH6pHuLuOtd791X2NtxE8=</t>
         </is>
       </c>
     </row>
@@ -9225,12 +9225,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>mrlr3XDAhUegxijJ1pbWLQ==</t>
+          <t>yBhfwCqbkW2SXmVBy+2LWA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>bPBWpDdnTEPW5lrROH7NmFfUD7VOGDIwx/dnN+MrOQQ=</t>
+          <t>viWV1L56wrfa7gFgJXdUDVXjiibzRGQgQnBab7wzoys=</t>
         </is>
       </c>
     </row>
@@ -9257,12 +9257,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DJZZxAU2DpC18zRF3uHvrg==</t>
+          <t>jT+AVR2HTNZkD5Hog+uJJg==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>8LOBA+WA4/3dDznYaUsB6MRHj/mOom7195j07Ok4Byg=</t>
+          <t>dmGKgxT6J9ou/BtA2SVFZByYLpobz+lBLJfhjLG40s8=</t>
         </is>
       </c>
     </row>
@@ -9284,12 +9284,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>gtLq49+yZ/jWhk32ykeEog==</t>
+          <t>3xgQu1LJWnuC7swcM6zUqg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IFcDu3nkRfYBwp+XvRv4dv5cMyp2OGsz2OPJl7nztwU=</t>
+          <t>vB/Lgo+VyIHb3hQXvKbgyqgQ1bZonrvoQCbbE0rylHo=</t>
         </is>
       </c>
     </row>
@@ -9316,12 +9316,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>kVLgriv92w62qZBLmzmpSw==</t>
+          <t>6cYiMflI+ZM8Va9aSq3w7w==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WJ7ZeN3LDN6Mh14KwQJwS6ZAACvgKrXNVU94CIUPOkk=</t>
+          <t>RECiGmB5hoyIdWuAIgQ2Bo/RBL3bltpsAiKrl6DQGns=</t>
         </is>
       </c>
     </row>
@@ -9348,12 +9348,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PE6uXawWhUz4ZR6wVeyePw==</t>
+          <t>9AoxAuGKzEmKyCnQPVG7cw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>L16Kvf6myoBwVmfdeDb0wnQF3yJ5Eb+hq9IqkiSZpX8=</t>
+          <t>+4sN1aUhSvNfBV1qNpSjH5Vo3cNUjOMJ+sWsrwfQeuQ=</t>
         </is>
       </c>
     </row>
@@ -9380,12 +9380,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>UxK91f6lPOQgfBsbB0V1dA==</t>
+          <t>PJ00Qlb3el8uxuWxNdqF+A==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>t7zqhNtnfHiG6gtvjZ2TUTNEK1uErAZM+rh3RN0YkH0=</t>
+          <t>7iru5ahtgNHbHEPXDXYdaWO3+Zq/sMXzmh+W5YTpgtg=</t>
         </is>
       </c>
     </row>
@@ -9407,12 +9407,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2gASM2S7lAicd55vu5jbjw==</t>
+          <t>o08t0xZCdcK/8xsdF4wKag==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>u17QmT1f6Jn394vYp0XjYmD1M4y28hzJ7lgPpIuycRI=</t>
+          <t>tshHazoBdSU/b3adXvmFtfSUfziRWnQZ2mqSi7/4hZQ=</t>
         </is>
       </c>
     </row>
@@ -9439,12 +9439,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>QCts1TtRRv9uwOIPni+//Q==;T9P/8O/c36wQ8JOj8+dp1g==</t>
+          <t>1Sp0dHaYgNSRNBEiHsBASQ==;hZ0nJoJpqeDGEnLk9aMGSQ==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3LF97gHP1mZvVSVws9I2iqfVT3BA+HrnF5CDazsToig=;UkfMCqCwSGBBiLdG/uClU6QW6DzsTJBUiXFujC9Als4=</t>
+          <t>e8AMvnepYdNnjvOlb9gp/bGQp3vDGT31dQZODjOR2wE=;5WhMyd1lZ7XBVx3m2IqLuGGI00A/wmDMQ444jeC82rM=</t>
         </is>
       </c>
     </row>
@@ -9471,12 +9471,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>M7HPKrm82c9VYKDs2UpEjQ==</t>
+          <t>aAR3rpYPHJZYbuG3lt2ujQ==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>321q5pS339dXop9FvJPq0D/GFK9SDsErjIxR90wTOzM=</t>
+          <t>nURfJSsMWKYOvF4H/v+859DUPNX392bavpNi6GEYfk4=</t>
         </is>
       </c>
     </row>
@@ -9503,12 +9503,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AFWdK1wSv/aD+ZcBd5V5Ww==</t>
+          <t>z/PzffwmmvLkiFeKPm4T1A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>5lxSTeiFYAZeD19TEVwhVOTrUk9BEnLZdpMf/f/7TMU=</t>
+          <t>n58R+qy5Z9yU5Dgc5uL6R6n6v2BLp0n/+najsO1I/BE=</t>
         </is>
       </c>
     </row>
@@ -9535,12 +9535,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>tQkyR8asi/4G+7tQwc1drw==</t>
+          <t>irUqUIyVXC5rtKvXJp5sVg==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>gCEB0e7SFRgDgphlH/ipyO5peN7e9v6JIofILX3vMbM=</t>
+          <t>R2IDfDQ7mAZkSG+sE3ThDzGgPxxVl1qQfn3Abv5I/Fg=</t>
         </is>
       </c>
     </row>
@@ -9567,12 +9567,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ELkAFa3fW9snQcoEejq6Eg==</t>
+          <t>CjCAHU9iOQXARmoGVIYQFw==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MRm4ocWmazEEA/A0MgAJ2+jM/zCoT2ApMU+Ld/96Szk=</t>
+          <t>1+9jUiof6euQwf/OgcovS3j7qS3TKnAZ71ATj+L52qQ=</t>
         </is>
       </c>
     </row>
@@ -9599,12 +9599,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7lkll/eYtxN7zSZyDK1KuA==</t>
+          <t>Sp/e7B3/+6PrRRfHf/2LhA==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>rgHwN+T60yey67tqvl94bLnWkqaEKyHPLBrwWMj8Lh4=</t>
+          <t>teT3rq/nvnZfm8hgGCkCZ0eXASRUWbHY9o75y8KprC8=</t>
         </is>
       </c>
     </row>
@@ -9631,12 +9631,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>bhOlvwF6ybclslrM5dQWGw==</t>
+          <t>VvrWm0ZR4fBAGLYT3zPvjg==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mc16gRditozlupaO8M8wW+Y9i8AmsMQcwAXEr2Weu7E=</t>
+          <t>u3yb0mvKThiJTbzbRBjD0+gvvx1JNz61Db2TCkB3N/s=</t>
         </is>
       </c>
     </row>
@@ -9663,12 +9663,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>S6ZHNjVlr+1g0ApsmfuU2g==</t>
+          <t>Uh46UG76ep4pxRrIgOJ1EQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Y4mJFBrOJdcsJEeHUq8Wjsb6jAUeeAVA4B1AY5EQvbw=</t>
+          <t>fdV+2mnPn9aoKJZrVyoLU/Sy0bD1C3rr5NzhQT26dzs=</t>
         </is>
       </c>
     </row>
@@ -9695,12 +9695,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>I/vR2tCU2U8oTTNEvrtbvQ==</t>
+          <t>cSUt3He/MJrErnpiQguQXQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>cBDCRjOOuKv1AmZDbAQckzncyD0JKStbwB+RFc3R+k8=</t>
+          <t>aloEzA9j3FZHCY1i1eje0ZLcYC+wBjG//T9Dw7asZ0k=</t>
         </is>
       </c>
     </row>
@@ -9727,12 +9727,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>UNkaalOqmywwRvOrTcEAmA==</t>
+          <t>ume1N3yjRkcxMqzXzkNFDQ==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>hjXaE+TrWd5Fic92DZ+4QVy33i+s+H3Gr8pbT5uNP80=</t>
+          <t>JhQlOCjXWdn/8EnNm6pAyD/XjjAsMfgT/s8nC/dejf0=</t>
         </is>
       </c>
     </row>
@@ -9759,12 +9759,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LIsidH/lViHo0oLa22P2fg==</t>
+          <t>iJ4aJGJdod1ObEJZim14Ng==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>uTlvOIF/wmX3ycOxc0nFmqrG2vbYVec+Fq1sV2QzFtk=</t>
+          <t>c12xELOSxeSOAN2+UCiYKqs5TMIxfUDk/8RaLD1/uY8=</t>
         </is>
       </c>
     </row>
@@ -9791,12 +9791,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>f/SxANk7Y+bdn/pZm5worg==</t>
+          <t>YON5gvKxfwK8VyNPzYNXMg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AnUDB0397O3DkCwsahvZVQ+r493MTPEP3y9y/eirSec=</t>
+          <t>0plLUYd2m+sJKTdsCFs0KoplIau6ryhD5WH2PORUhsQ=</t>
         </is>
       </c>
     </row>
@@ -9823,12 +9823,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ktpgf741p2RROWK8ShLPaw==</t>
+          <t>ylaWUSmX5c7HZIShOBRmHg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>uAFk50hsrXEIysQ3EnW/xWXHIR5wLEhdvqtGZ/sL034=</t>
+          <t>nvlFA/xOvFxQYvU57Ds3PeVl2xqbkifeBZbDl1PIUEo=</t>
         </is>
       </c>
     </row>
@@ -9855,12 +9855,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TDD6AAn6S1UxhVMI7nvfUg==</t>
+          <t>dn56p6E9W+wTr3CbM6zqgw==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>jvgkpLutbxXgR8Pqrt/EB+hMEHT7UwaDD1W9G3lXv0U=</t>
+          <t>I6GMvktPENQwvtcmro9aA6xXoU83ig0H9kwWl4F4Ipk=</t>
         </is>
       </c>
     </row>
@@ -9887,12 +9887,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>nApi4BSriNQ52LlztQfYhg==</t>
+          <t>q3jrIN8755uztra/bWMQLQ==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>yQDuGUz2N5+j2S7fd56I/VZojkX90p9D8EoOi4qnWm0=</t>
+          <t>gij0dEs+iyq3FiSZK6edp3+49fiELCvQAwE1O/a91wI=</t>
         </is>
       </c>
     </row>
@@ -9919,12 +9919,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>27TuJex3N5Lse/dSUqfDeQ==</t>
+          <t>F7+XBRZiqQAQtSGkZNBJNw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>QGTyAfAsy1o9V8YgNR8oMRVXNU3AawTTb6x2MGDO2h4=</t>
+          <t>mhaAHGHs50minpsCZQl5arfGz9AnS8lqnZ942Y/MZb8=</t>
         </is>
       </c>
     </row>
@@ -9951,12 +9951,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PBssIvWC9SoRuuFYx6/Jeg==</t>
+          <t>DZmr6U4vYx+x9oKo2/LcNg==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>9mgidsNRX0iPqJUIMiPV6FvfCmNklJdwgC25W1YC0r8=</t>
+          <t>s8FaGyKijAuxKnETuGywKkBC/fK+w6gqaI2kDL8TAfw=</t>
         </is>
       </c>
     </row>
@@ -9983,12 +9983,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>32KKvbWk4OCSrFx6JR4f1Q==</t>
+          <t>79UZLYm4BEg1ao25TYsPiw==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CU6JrmnYqnsw/hz1QWxVYB7HWADcSYGrMGzzUWiyQD4=</t>
+          <t>wnOK2no3zx4br3VcoJIW6wc2N+z1uUCz5sS2AXzGv2w=</t>
         </is>
       </c>
     </row>
@@ -10015,12 +10015,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>26m9BTsVawGP3wSIvbVIaw==</t>
+          <t>FCtEt3naMjiPHDb6Yxzeqw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3xv/LL30SZWi2rFsL6Cx6N3o45XiwelWCruCBcAFR18=</t>
+          <t>yXOFsXOqYwVq14t43F4V/kkZdZO7u7GvPWDPhscV0lE=</t>
         </is>
       </c>
     </row>
@@ -10047,12 +10047,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FNKS0kAMTrF7Zqy0+GuxPg==</t>
+          <t>K7kCaZP1fwM4K03YbcrV/Q==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>eSO+70NZe8YygpvOz4yNRbovJdoWerUzVkaiWbazVb0=</t>
+          <t>qnZbLn8032VKs8GCC9FPEXFW/4s0v7tWr55mw68WRc0=</t>
         </is>
       </c>
     </row>
@@ -10079,12 +10079,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>lgrmgPE4fYgc2ddYEIvznQ==</t>
+          <t>Wpvj02tZLeaQ0YPmfmpX6A==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>wU0r/oZ/8eIRkZkengtIEdODeqd7OjWEz8LDDM87XEI=</t>
+          <t>UInOmQekh7rdatepfDHEhckY7qMCdrCgSb6L26dYIiM=</t>
         </is>
       </c>
     </row>
@@ -10111,12 +10111,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Xb+IE362+CsiafqGHtPfFg==</t>
+          <t>3VDZQw4h3U8w0IHD72+Law==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>x4+qc8lBDxjZZipoia/8vgmIfzlax3lOKfbwiVh5/Ns=</t>
+          <t>qaz82p512e5tSn8jvdVMg4bxNHYXKmdYbCHBCkkYmOI=</t>
         </is>
       </c>
     </row>
@@ -10143,12 +10143,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2ga1auwzk811xm5JutH0fg==</t>
+          <t>gmHvWYCj5AYbP3WqqVQ5hg==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Ooj+0cscwAwBYziZrW3k8ye0I4Gn/feH1n5t0L4b3T8=</t>
+          <t>pFPrrWLwBnycrmTWd/P71diLiUm4+Y4UXxQA/NCOSKs=</t>
         </is>
       </c>
     </row>
@@ -10175,12 +10175,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>gBhZOpX1BjY4+aV56cUBCw==</t>
+          <t>vfAyB7VU+OyuN6PlQvn32g==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>NTv7zvKPmXCJBl2So0nwTGA2gMCq0uw5+6KZXdgdHdo=</t>
+          <t>FvarUq5BLfq436Rc24gwKQYFnC1kXAlOcON+NjntWQI=</t>
         </is>
       </c>
     </row>
@@ -10207,12 +10207,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SpOzLbiOTuVT4SyZFNdF5w==</t>
+          <t>UMG4VavVlWtvSMMhflE9tQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dvPFq2FB9gy7q1scOjO9wtSPB3B9HoFybNOry7+uy10=</t>
+          <t>CZzUXfMbKeqOLh4ZjHbpwfUJKj1zrTypancuX4TZVwc=</t>
         </is>
       </c>
     </row>
@@ -10239,12 +10239,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>YBXl2GOsFLOtXAbPOK8oKg==</t>
+          <t>xf8mganqIM/3eFOMwl4enw==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ADfBtLGq2w1n26QsEy2J55r972UqpcIKJibO1vUQRUo=</t>
+          <t>lmzTd7anJ4w6qKHF4//Rx4O3kcLJgfdWoAwT/HDaSOk=</t>
         </is>
       </c>
     </row>
@@ -10271,12 +10271,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>pFlnJ26dict9w5pz4vv4OA==</t>
+          <t>SrTaaiQkROe//NBFUZXbiQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>4RcvSgU7pdpNwYJDs04E0QVmgfRZyp9KevYW2DWXjEI=</t>
+          <t>cPoTQ1oNUwfqmvqtkVu2SGREk4JzDLUXj0gKtHESxps=</t>
         </is>
       </c>
     </row>
@@ -10303,12 +10303,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>XCN5I2O4fPvUbLkpXbF7dw==</t>
+          <t>FlgV7IxzIRkRaeti0RQRuw==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>iPsgk1Z/WHSLMmd+mavF5SuobrpUY+Pe7oIdq5/mzgU=</t>
+          <t>LBSeosPQnBNezo3ce+HT8v8bqz9BNBIVNljP4tBXyio=</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>xED36l3O6e41puN3ctVDeg==</t>
+          <t>FpgXsnGa5ewUl4UjqZR5sg==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>8SDOsf82Ov5WqWu30VvWIYEjnZV2iVCFJ6cNZ07pPVI=</t>
+          <t>LhaxTXUi9QgxlQgW8Uk4y6ywuGeRc1hku079bqU+s5s=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-28 14:58) - 88 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Categorias'!$A$1:$B$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Categorias'!$A$1:$B$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -502,7 +502,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -6052,7 +6052,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8088,7 +8088,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8176,7 +8176,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8572,7 +8572,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8616,7 +8616,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8664,7 +8664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -8691,7 +8691,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8703,7 +8703,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8775,7 +8775,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8811,7 +8811,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8835,7 +8835,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8847,7 +8847,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -8859,7 +8859,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VENTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
     </row>
@@ -9115,8 +9115,92 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REPORTE DE VENTAS</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO DE OBJETIVOS</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>RELEVAMIENTO DE PRECIOS</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PRECIOS Y OFERTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>APP Ventas (Principal)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>APP Ventas (Backup)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>APP Ventas Mayorista</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Portal Autogestion Clientes</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B37"/>
+  <autoFilter ref="A1:B44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9193,12 +9277,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/ABBGqtqXXIEAUv/r3aB3Q==</t>
+          <t>/hG9HEYMYiYCgnkMTVtXpQ==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>lFIiYOfgUMxI1qtlli4+yqwH6pHuLuOtd791X2NtxE8=</t>
+          <t>J0lAOmhNZWmw3P74MPJlMCRC7E8sjLH1wFuvrYjPdFU=</t>
         </is>
       </c>
     </row>
@@ -9225,12 +9309,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>yBhfwCqbkW2SXmVBy+2LWA==</t>
+          <t>KuBKtKZFWZU5BzOYKzaNMw==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>viWV1L56wrfa7gFgJXdUDVXjiibzRGQgQnBab7wzoys=</t>
+          <t>ceTQNsRKNkFyq4cNJGvW5yf+yjXgBJsIloUx6Xw+sLI=</t>
         </is>
       </c>
     </row>
@@ -9257,12 +9341,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>jT+AVR2HTNZkD5Hog+uJJg==</t>
+          <t>egpoC3ik5kg0lJmsZka5Qg==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dmGKgxT6J9ou/BtA2SVFZByYLpobz+lBLJfhjLG40s8=</t>
+          <t>VfgOXdvx6sSOI6PUJswDVYYm9rHbICJqCtb8BTHkII8=</t>
         </is>
       </c>
     </row>
@@ -9284,12 +9368,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3xgQu1LJWnuC7swcM6zUqg==</t>
+          <t>w0INkPSqtF6Kf7iiANbuew==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>vB/Lgo+VyIHb3hQXvKbgyqgQ1bZonrvoQCbbE0rylHo=</t>
+          <t>vRu0YrhKLmJckCdzfJoxL89YS/CyEsAndB7GHgODFfw=</t>
         </is>
       </c>
     </row>
@@ -9316,12 +9400,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6cYiMflI+ZM8Va9aSq3w7w==</t>
+          <t>zfyUdHMLbtj7358HHAdknw==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>RECiGmB5hoyIdWuAIgQ2Bo/RBL3bltpsAiKrl6DQGns=</t>
+          <t>t6+EuFeXGsC8bF5EpIR+PdcR20GxDpDAxm2nBz+Y0X4=</t>
         </is>
       </c>
     </row>
@@ -9348,12 +9432,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9AoxAuGKzEmKyCnQPVG7cw==</t>
+          <t>odQK0N31Z+jpuB3uonTFDQ==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>+4sN1aUhSvNfBV1qNpSjH5Vo3cNUjOMJ+sWsrwfQeuQ=</t>
+          <t>eM+UUH1ts9jeXWcNBUtxZAQvwMGBe8JDE8ReIgU9x2s=</t>
         </is>
       </c>
     </row>
@@ -9380,12 +9464,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PJ00Qlb3el8uxuWxNdqF+A==</t>
+          <t>lcbmMJgj/Xje5zbJhWB3tQ==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7iru5ahtgNHbHEPXDXYdaWO3+Zq/sMXzmh+W5YTpgtg=</t>
+          <t>wZDwXOeg5ELNjVyHh0knOckvT5Sp5UINAw1hDFBpumU=</t>
         </is>
       </c>
     </row>
@@ -9407,12 +9491,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>o08t0xZCdcK/8xsdF4wKag==</t>
+          <t>h4tSRGjfzFxxiFCj9acOhg==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>tshHazoBdSU/b3adXvmFtfSUfziRWnQZ2mqSi7/4hZQ=</t>
+          <t>VhhMnJvENEdFIE48Km7NpPcpjXdGTevomxFMMigZCO8=</t>
         </is>
       </c>
     </row>
@@ -9439,12 +9523,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1Sp0dHaYgNSRNBEiHsBASQ==;hZ0nJoJpqeDGEnLk9aMGSQ==</t>
+          <t>q3T9RjMIDYpLSlhxJEhHOQ==;Ngo454r19zrJtCuLWhyioA==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>e8AMvnepYdNnjvOlb9gp/bGQp3vDGT31dQZODjOR2wE=;5WhMyd1lZ7XBVx3m2IqLuGGI00A/wmDMQ444jeC82rM=</t>
+          <t>wQFo08T16Ijwtkb5okHYkvJVBK9f044g8DPuZIOPIy0=;9V4HGfe/XEYltQFolzd/mHgmsIpNR2bw19N4qCXLqVQ=</t>
         </is>
       </c>
     </row>
@@ -9471,12 +9555,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>aAR3rpYPHJZYbuG3lt2ujQ==</t>
+          <t>8NV/9XufmNChW0uy2A3acA==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>nURfJSsMWKYOvF4H/v+859DUPNX392bavpNi6GEYfk4=</t>
+          <t>KymTnxgPrY5uAOI/7Uah68a7hjcn2LIsU87VrlTfAjY=</t>
         </is>
       </c>
     </row>
@@ -9503,12 +9587,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>z/PzffwmmvLkiFeKPm4T1A==</t>
+          <t>ciMkZiJCC7FnykR8U6yOjw==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>n58R+qy5Z9yU5Dgc5uL6R6n6v2BLp0n/+najsO1I/BE=</t>
+          <t>ZOfc4Z64DVv0MDFxOp12BKcGunnKqf3/L7b0c0jDlFQ=</t>
         </is>
       </c>
     </row>
@@ -9535,12 +9619,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>irUqUIyVXC5rtKvXJp5sVg==</t>
+          <t>wq5GU97vWMu9TJoYdS3w9Q==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>R2IDfDQ7mAZkSG+sE3ThDzGgPxxVl1qQfn3Abv5I/Fg=</t>
+          <t>vX6dvzawoBfZst2w1zlRKG7cPSdlcSJwdrDVU/g4QQ0=</t>
         </is>
       </c>
     </row>
@@ -9567,12 +9651,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CjCAHU9iOQXARmoGVIYQFw==</t>
+          <t>hBNL/xfQTGgisr9n2jRjdQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1+9jUiof6euQwf/OgcovS3j7qS3TKnAZ71ATj+L52qQ=</t>
+          <t>YAlwmIEB5UA/wKvxHZ38TcaetUly2l2joqLp5093cyo=</t>
         </is>
       </c>
     </row>
@@ -9599,12 +9683,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sp/e7B3/+6PrRRfHf/2LhA==</t>
+          <t>uGSGrwjViwj/DBzH8ZvqHw==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>teT3rq/nvnZfm8hgGCkCZ0eXASRUWbHY9o75y8KprC8=</t>
+          <t>cc5+ug9Ppe3RwWgssGBcyzavmvQgrPZTxZVakNNZH00=</t>
         </is>
       </c>
     </row>
@@ -9631,12 +9715,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>VvrWm0ZR4fBAGLYT3zPvjg==</t>
+          <t>pSvQqaNidgzR1PePX7wjvw==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>u3yb0mvKThiJTbzbRBjD0+gvvx1JNz61Db2TCkB3N/s=</t>
+          <t>dbuCqFnq3u36lfSCNG8ZJ4eazwJC4xTpehTdyFlgWLM=</t>
         </is>
       </c>
     </row>
@@ -9663,12 +9747,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Uh46UG76ep4pxRrIgOJ1EQ==</t>
+          <t>2j5JRQwn6qvFvZyHyO9lWQ==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>fdV+2mnPn9aoKJZrVyoLU/Sy0bD1C3rr5NzhQT26dzs=</t>
+          <t>KIWoKVUc+vXZ6B3fQEOH+zj6TSv+daLd/R6rHsmhbhk=</t>
         </is>
       </c>
     </row>
@@ -9695,12 +9779,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>cSUt3He/MJrErnpiQguQXQ==</t>
+          <t>oaoGOPWx6FjExSGtj1ehkQ==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>aloEzA9j3FZHCY1i1eje0ZLcYC+wBjG//T9Dw7asZ0k=</t>
+          <t>mVk4QaW2q64TzWpj7zX15ZxDr0gI1OXVfGnX39j+dPk=</t>
         </is>
       </c>
     </row>
@@ -9727,12 +9811,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ume1N3yjRkcxMqzXzkNFDQ==</t>
+          <t>2u0vipAmg0eSN7UFvpuFkw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>JhQlOCjXWdn/8EnNm6pAyD/XjjAsMfgT/s8nC/dejf0=</t>
+          <t>KYRz3eEe7fI62flWYlpBIE76afm5Mgqb0yt8HUoYOWc=</t>
         </is>
       </c>
     </row>
@@ -9759,12 +9843,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>iJ4aJGJdod1ObEJZim14Ng==</t>
+          <t>df8WQifwrFhvsl3PcMYB5g==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>c12xELOSxeSOAN2+UCiYKqs5TMIxfUDk/8RaLD1/uY8=</t>
+          <t>RZUdctN8sb+9O8p55pmKRaQ0eWPTDKO8fEJgJRGpItI=</t>
         </is>
       </c>
     </row>
@@ -9791,12 +9875,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YON5gvKxfwK8VyNPzYNXMg==</t>
+          <t>our7ZLcrFIrvt7qxXiBuLQ==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0plLUYd2m+sJKTdsCFs0KoplIau6ryhD5WH2PORUhsQ=</t>
+          <t>T5dv1yCGUsGGHSEaAspfuQc4gxJ+77nRgv8GhTefXYE=</t>
         </is>
       </c>
     </row>
@@ -9823,12 +9907,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ylaWUSmX5c7HZIShOBRmHg==</t>
+          <t>nQEo9GVDtE26JXTvDm6ppA==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nvlFA/xOvFxQYvU57Ds3PeVl2xqbkifeBZbDl1PIUEo=</t>
+          <t>umIcTjAA6hB4YgEQ0vOIzyglUJkHHIMs2ZRhwkHMk44=</t>
         </is>
       </c>
     </row>
@@ -9855,12 +9939,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>dn56p6E9W+wTr3CbM6zqgw==</t>
+          <t>1emADvboG9KOT6SWq4gjGw==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>I6GMvktPENQwvtcmro9aA6xXoU83ig0H9kwWl4F4Ipk=</t>
+          <t>+YcpWVnz716x0jbrodxj1DSW1q736NcXlGO0KORsTAw=</t>
         </is>
       </c>
     </row>
@@ -9887,12 +9971,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>q3jrIN8755uztra/bWMQLQ==</t>
+          <t>UfYd17/D2Rj5YibWhLRH0Q==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>gij0dEs+iyq3FiSZK6edp3+49fiELCvQAwE1O/a91wI=</t>
+          <t>xbq708nGEHyM4U2HzsA+8LNUYL9Cq53d/zPa3zhFPM0=</t>
         </is>
       </c>
     </row>
@@ -9919,12 +10003,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>F7+XBRZiqQAQtSGkZNBJNw==</t>
+          <t>Z2WzhNDJhv54SvEfaMQnJA==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>mhaAHGHs50minpsCZQl5arfGz9AnS8lqnZ942Y/MZb8=</t>
+          <t>sYU59zndtgjHtfF6tokf2lrb4wI3kBK0F0i5+cYMZAY=</t>
         </is>
       </c>
     </row>
@@ -9951,12 +10035,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>DZmr6U4vYx+x9oKo2/LcNg==</t>
+          <t>mSn/8daxqNaTjLgCN8o8PA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>s8FaGyKijAuxKnETuGywKkBC/fK+w6gqaI2kDL8TAfw=</t>
+          <t>SdBD602yiJUHsiifOCc1rW5fc9PPybrNLfZTXAVKTeg=</t>
         </is>
       </c>
     </row>
@@ -9983,12 +10067,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>79UZLYm4BEg1ao25TYsPiw==</t>
+          <t>/KkSHbryEQTDSyKuzLUWNg==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>wnOK2no3zx4br3VcoJIW6wc2N+z1uUCz5sS2AXzGv2w=</t>
+          <t>1t0mXUt4t1mBj5R2448B+NVvCmwNxL0rkgYN8IdyW2I=</t>
         </is>
       </c>
     </row>
@@ -10015,12 +10099,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FCtEt3naMjiPHDb6Yxzeqw==</t>
+          <t>u0NXeN14ll6Lu/HlZX9ysw==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>yXOFsXOqYwVq14t43F4V/kkZdZO7u7GvPWDPhscV0lE=</t>
+          <t>3dbjsR+iKmXL3z0Z2cFkHtX20AJivSYB5E2ArF2rLio=</t>
         </is>
       </c>
     </row>
@@ -10047,12 +10131,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>K7kCaZP1fwM4K03YbcrV/Q==</t>
+          <t>5VkVrZXqF3G2shfkbrSD9w==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>qnZbLn8032VKs8GCC9FPEXFW/4s0v7tWr55mw68WRc0=</t>
+          <t>awuxBADzJhtc/wRp/mrMyCsH8vSARbAUkdc0yMN52r0=</t>
         </is>
       </c>
     </row>
@@ -10079,12 +10163,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wpvj02tZLeaQ0YPmfmpX6A==</t>
+          <t>DglaGu/LBo6vnwM23y7NYQ==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UInOmQekh7rdatepfDHEhckY7qMCdrCgSb6L26dYIiM=</t>
+          <t>bKUh8Dw/XCMeqVfQwUn+5sJ9U7XDw5hUOvYFMqe7kLw=</t>
         </is>
       </c>
     </row>
@@ -10111,12 +10195,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>3VDZQw4h3U8w0IHD72+Law==</t>
+          <t>zKeA2AV81IHpQ0wCXnKwaQ==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>qaz82p512e5tSn8jvdVMg4bxNHYXKmdYbCHBCkkYmOI=</t>
+          <t>LePCb/ZsLWRp3onwN/stRYlzSRE7sMl/i3M9pG82hoE=</t>
         </is>
       </c>
     </row>
@@ -10143,12 +10227,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>gmHvWYCj5AYbP3WqqVQ5hg==</t>
+          <t>fh7/eotskNRV7WwIf7N/XQ==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>pFPrrWLwBnycrmTWd/P71diLiUm4+Y4UXxQA/NCOSKs=</t>
+          <t>RzweF0eWnJI8vCupYfyycA6yn2ozF9XwrFSAxHYt2zM=</t>
         </is>
       </c>
     </row>
@@ -10175,12 +10259,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>vfAyB7VU+OyuN6PlQvn32g==</t>
+          <t>zfJQ+V0xGDwmiHxEmSodug==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>FvarUq5BLfq436Rc24gwKQYFnC1kXAlOcON+NjntWQI=</t>
+          <t>Bkq1Dpw5scpWFsRM4UKr9Jl7l/8CeWNpWqvGR1yquDw=</t>
         </is>
       </c>
     </row>
@@ -10207,12 +10291,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>UMG4VavVlWtvSMMhflE9tQ==</t>
+          <t>HTiwy4GJcnqQImzhtWWEnw==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CZzUXfMbKeqOLh4ZjHbpwfUJKj1zrTypancuX4TZVwc=</t>
+          <t>F35uHkaqWJfaFpM27jZJxl8IU/x8I5NWS5W+nHFVGBI=</t>
         </is>
       </c>
     </row>
@@ -10239,12 +10323,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>xf8mganqIM/3eFOMwl4enw==</t>
+          <t>RVxyqRvGJepYwqHxvfOOwg==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>lmzTd7anJ4w6qKHF4//Rx4O3kcLJgfdWoAwT/HDaSOk=</t>
+          <t>MwZzp92NBIhjk0AH9jqPVC20RETYRF4REnw7guSZcVE=</t>
         </is>
       </c>
     </row>
@@ -10271,12 +10355,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SrTaaiQkROe//NBFUZXbiQ==</t>
+          <t>BoJwdM8kMvx9jWbEvzjXgw==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>cPoTQ1oNUwfqmvqtkVu2SGREk4JzDLUXj0gKtHESxps=</t>
+          <t>fsK2NqP41VIu8Ni6saRw4d5Z8oNL2LPciUaqm+rtm3s=</t>
         </is>
       </c>
     </row>
@@ -10303,12 +10387,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FlgV7IxzIRkRaeti0RQRuw==</t>
+          <t>pqcPX1v3vd8Sp+rX/rSUGg==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>LBSeosPQnBNezo3ce+HT8v8bqz9BNBIVNljP4tBXyio=</t>
+          <t>QnBsn+nGoAfnUjUYkNYkCaXEK/QfsdPLk3vo2cQqKOk=</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10419,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FpgXsnGa5ewUl4UjqZR5sg==</t>
+          <t>exWUAy1oyBkYb1CkWmo1Qw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>LhaxTXUi9QgxlQgW8Uk4y6ywuGeRc1hku079bqU+s5s=</t>
+          <t>KKvHDCjXFAj/85Hs9DDVOj7N/bCPaUgbJm0oj6Uo3Cg=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-29 07:41) - 88 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1993,7 +1993,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="43">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45">
@@ -2101,7 +2101,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="73">
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="74">
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="75">
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="76">
@@ -3229,7 +3229,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="77">
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78">
@@ -4145,12 +4145,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="103">
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4325,12 +4325,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4361,12 +4361,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4397,12 +4397,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4433,12 +4433,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -4541,12 +4541,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3fe0835d-a49b-4cd0-9f89-899820a8df07&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5464,7 +5464,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19">
@@ -5684,7 +5684,7 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23">
@@ -5816,7 +5816,7 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26">
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28">
@@ -6440,7 +6440,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="40">
@@ -6708,7 +6708,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46">
@@ -6752,7 +6752,7 @@
         </is>
       </c>
       <c r="L46" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47">
@@ -6840,7 +6840,7 @@
         </is>
       </c>
       <c r="L48" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49">
@@ -6972,7 +6972,7 @@
         </is>
       </c>
       <c r="L51" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52">
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="L52" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="53">
@@ -7060,7 +7060,7 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="54">
@@ -8371,16 +8371,16 @@
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Informes</t>
+          <t>Grupo Hergo - Jefes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>3fe0835d-a49b-4cd0-9f89-899820a8df07</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L83" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="84">
@@ -9277,12 +9277,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/hG9HEYMYiYCgnkMTVtXpQ==</t>
+          <t>5SJVkGR9sm0iA0bKu/oJzw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>J0lAOmhNZWmw3P74MPJlMCRC7E8sjLH1wFuvrYjPdFU=</t>
+          <t>CWtPuY/jDyoLmD7Zu9L3qdgAuh2SaX4SIEpqdryvJKA=</t>
         </is>
       </c>
     </row>
@@ -9309,12 +9309,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KuBKtKZFWZU5BzOYKzaNMw==</t>
+          <t>TKShgGmT02Kc8sqZX0ClhA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ceTQNsRKNkFyq4cNJGvW5yf+yjXgBJsIloUx6Xw+sLI=</t>
+          <t>NjtcNrzTqrgLrV84/kslIRnGkx7m+YktJYH7uW61ybo=</t>
         </is>
       </c>
     </row>
@@ -9341,12 +9341,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>egpoC3ik5kg0lJmsZka5Qg==</t>
+          <t>O99MSLtesyrgePkZPT8MtQ==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>VfgOXdvx6sSOI6PUJswDVYYm9rHbICJqCtb8BTHkII8=</t>
+          <t>v+As+O56LMBbfSchjo9tO43ozt9F0CElvtfwWSrUhrs=</t>
         </is>
       </c>
     </row>
@@ -9368,12 +9368,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>w0INkPSqtF6Kf7iiANbuew==</t>
+          <t>3PBpuluffW/sOel75AroSg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>vRu0YrhKLmJckCdzfJoxL89YS/CyEsAndB7GHgODFfw=</t>
+          <t>wybPdQViRnQViR9g7Xiv4+eqsmhnLyCA9y/qf6Asrag=</t>
         </is>
       </c>
     </row>
@@ -9400,12 +9400,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>zfyUdHMLbtj7358HHAdknw==</t>
+          <t>dFE+ANStl2SvA5tPTNrUVQ==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>t6+EuFeXGsC8bF5EpIR+PdcR20GxDpDAxm2nBz+Y0X4=</t>
+          <t>nwnj9ydeK9CdmlzigiQM0HK5EoTeQi1ICrlT3L4ZTIA=</t>
         </is>
       </c>
     </row>
@@ -9432,12 +9432,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>odQK0N31Z+jpuB3uonTFDQ==</t>
+          <t>HXNAYtgiCHWnBiTCd0UMHA==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>eM+UUH1ts9jeXWcNBUtxZAQvwMGBe8JDE8ReIgU9x2s=</t>
+          <t>scrLjpCyGXO2BZzCJFUP6i61ReV8g073BST6gPpDYmk=</t>
         </is>
       </c>
     </row>
@@ -9464,12 +9464,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>lcbmMJgj/Xje5zbJhWB3tQ==</t>
+          <t>xTYV9gC5ft2I+OqGS+7gfw==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>wZDwXOeg5ELNjVyHh0knOckvT5Sp5UINAw1hDFBpumU=</t>
+          <t>VspzY8lqCufsCHoqOi+IIlFMvMWetLhWxROwhVY9yb0=</t>
         </is>
       </c>
     </row>
@@ -9491,12 +9491,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>h4tSRGjfzFxxiFCj9acOhg==</t>
+          <t>5VHwVvwkSce9KFsujy67XA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>VhhMnJvENEdFIE48Km7NpPcpjXdGTevomxFMMigZCO8=</t>
+          <t>YoczRBMXLCo6LbpqqWCcWL4BvKghh6rYwFm3LWcebOQ=</t>
         </is>
       </c>
     </row>
@@ -9523,12 +9523,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>q3T9RjMIDYpLSlhxJEhHOQ==;Ngo454r19zrJtCuLWhyioA==</t>
+          <t>lsR3LB4sZA9jQISGUgw3mQ==;M8GWbcrj6RK9+mxLI/P5ZA==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>wQFo08T16Ijwtkb5okHYkvJVBK9f044g8DPuZIOPIy0=;9V4HGfe/XEYltQFolzd/mHgmsIpNR2bw19N4qCXLqVQ=</t>
+          <t>6ewgfqSId3o7jusgxWVcEmwZiHbL74Gfzpn69TdELKI=;FSWMeTIkJpKc6BVj/e4BpvEdZG+Ffg7QlhnE6Z8gZpI=</t>
         </is>
       </c>
     </row>
@@ -9555,12 +9555,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>8NV/9XufmNChW0uy2A3acA==</t>
+          <t>CGi/fha1pJhhaVEFgu+ZCg==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>KymTnxgPrY5uAOI/7Uah68a7hjcn2LIsU87VrlTfAjY=</t>
+          <t>ytyNH3NpDGdrWjHa5C8YXoGGatTvyaJvO6bzNDOgAQw=</t>
         </is>
       </c>
     </row>
@@ -9587,12 +9587,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ciMkZiJCC7FnykR8U6yOjw==</t>
+          <t>SYf+EnbdweyNqHm6cSWExQ==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ZOfc4Z64DVv0MDFxOp12BKcGunnKqf3/L7b0c0jDlFQ=</t>
+          <t>Pprf1RHKve/y0g2IcC8ooQqZ3f9zrhHokHMawdZOiuI=</t>
         </is>
       </c>
     </row>
@@ -9619,12 +9619,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>wq5GU97vWMu9TJoYdS3w9Q==</t>
+          <t>3dpJvSm1iCbucdNeJJKNAA==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>vX6dvzawoBfZst2w1zlRKG7cPSdlcSJwdrDVU/g4QQ0=</t>
+          <t>0+1ScviwzUdeBXDEtHNj1RWU+znSW7iz1TbgAfxHV6k=</t>
         </is>
       </c>
     </row>
@@ -9651,12 +9651,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>hBNL/xfQTGgisr9n2jRjdQ==</t>
+          <t>Kv/DIf5ZZ2AvTIgaimaP0Q==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>YAlwmIEB5UA/wKvxHZ38TcaetUly2l2joqLp5093cyo=</t>
+          <t>7pQ7FhSS8lMabK6050Q1bSKcxurELVDcZpJgeja3c+U=</t>
         </is>
       </c>
     </row>
@@ -9683,12 +9683,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>uGSGrwjViwj/DBzH8ZvqHw==</t>
+          <t>nAeKGdA1FOUmgDvE1BHfMg==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cc5+ug9Ppe3RwWgssGBcyzavmvQgrPZTxZVakNNZH00=</t>
+          <t>DT7owku4AEBAM0C7y1juQU2JDr//Oa8th8+IhGOuMW8=</t>
         </is>
       </c>
     </row>
@@ -9715,12 +9715,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>pSvQqaNidgzR1PePX7wjvw==</t>
+          <t>pbIyco0qTwHY48T4hGBW1Q==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dbuCqFnq3u36lfSCNG8ZJ4eazwJC4xTpehTdyFlgWLM=</t>
+          <t>zSKSsNvZ7W70cDLHjtHotSi46dbgqMrWD51OL1jMvgA=</t>
         </is>
       </c>
     </row>
@@ -9747,12 +9747,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2j5JRQwn6qvFvZyHyO9lWQ==</t>
+          <t>DA1k1eyXjx7P8ptcPPr0fg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>KIWoKVUc+vXZ6B3fQEOH+zj6TSv+daLd/R6rHsmhbhk=</t>
+          <t>yJp3UrES4gP4VhfreXN8BxFPXwi2iPPmSzHO3o5k/BU=</t>
         </is>
       </c>
     </row>
@@ -9779,12 +9779,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>oaoGOPWx6FjExSGtj1ehkQ==</t>
+          <t>UQZzYmGeagQfoK2iZ7aTuA==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>mVk4QaW2q64TzWpj7zX15ZxDr0gI1OXVfGnX39j+dPk=</t>
+          <t>VjM2lq1iwgPeKvXbLo08D19q/nnvoGEs7eeq7sOFT/w=</t>
         </is>
       </c>
     </row>
@@ -9811,12 +9811,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2u0vipAmg0eSN7UFvpuFkw==</t>
+          <t>rlgJS2iD4k/70nvtRZt9Yw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>KYRz3eEe7fI62flWYlpBIE76afm5Mgqb0yt8HUoYOWc=</t>
+          <t>z7UEDv3EFTCKGKzWv7niGk+0xa0hR7I75oYZc1xbEtw=</t>
         </is>
       </c>
     </row>
@@ -9843,12 +9843,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>df8WQifwrFhvsl3PcMYB5g==</t>
+          <t>TIXF9S6EHe2Y764nDdwveg==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RZUdctN8sb+9O8p55pmKRaQ0eWPTDKO8fEJgJRGpItI=</t>
+          <t>lXaKg+nrNlOolz5n2Z8FCbkauIPV5VeRXms0D2tU3sY=</t>
         </is>
       </c>
     </row>
@@ -9875,12 +9875,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>our7ZLcrFIrvt7qxXiBuLQ==</t>
+          <t>RJXWJThzWsD01KwVEMc3xg==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>T5dv1yCGUsGGHSEaAspfuQc4gxJ+77nRgv8GhTefXYE=</t>
+          <t>OKSQKj2lSyYq+y9czeJzsNrULPrio4LqXYoZ0GMx8ak=</t>
         </is>
       </c>
     </row>
@@ -9907,12 +9907,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>nQEo9GVDtE26JXTvDm6ppA==</t>
+          <t>fE+I7K5oTIjMAcEiAuxSTg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>umIcTjAA6hB4YgEQ0vOIzyglUJkHHIMs2ZRhwkHMk44=</t>
+          <t>yS9abYUxCghbefRec691MZNd+pZIkrrkz/AGhbu9K5w=</t>
         </is>
       </c>
     </row>
@@ -9939,12 +9939,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1emADvboG9KOT6SWq4gjGw==</t>
+          <t>2+FEZIfktWFjrYHiDdSEGA==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>+YcpWVnz716x0jbrodxj1DSW1q736NcXlGO0KORsTAw=</t>
+          <t>FagCQMh/r4g7XPtFU33THSTXdneqNVQ/jJx5edfPMzE=</t>
         </is>
       </c>
     </row>
@@ -9971,12 +9971,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>UfYd17/D2Rj5YibWhLRH0Q==</t>
+          <t>JdCH8WsU09HvY86zr2cCwA==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>xbq708nGEHyM4U2HzsA+8LNUYL9Cq53d/zPa3zhFPM0=</t>
+          <t>fwonNasZYviW8iK7SNyVgX4bD7LlmQCC6RB9dvIwbNI=</t>
         </is>
       </c>
     </row>
@@ -10003,12 +10003,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Z2WzhNDJhv54SvEfaMQnJA==</t>
+          <t>rcP2UTuCrS+aumf7t4ZIOg==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>sYU59zndtgjHtfF6tokf2lrb4wI3kBK0F0i5+cYMZAY=</t>
+          <t>S6SC8LWF7j4MHGp0Towj0e+6MB53nT8wSWnmCQf/u+Y=</t>
         </is>
       </c>
     </row>
@@ -10035,12 +10035,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mSn/8daxqNaTjLgCN8o8PA==</t>
+          <t>4ZBbq3cS2ZWp7X67zAJIjQ==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SdBD602yiJUHsiifOCc1rW5fc9PPybrNLfZTXAVKTeg=</t>
+          <t>tx34WQLwRlPcW/v3qaAFBLcMOhlsuZ068z38FSaekiU=</t>
         </is>
       </c>
     </row>
@@ -10067,12 +10067,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>/KkSHbryEQTDSyKuzLUWNg==</t>
+          <t>UMJAVzRcX7Liivi6DyJMtw==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1t0mXUt4t1mBj5R2448B+NVvCmwNxL0rkgYN8IdyW2I=</t>
+          <t>A3Zs+fOEm1FD4UfBj7bGyiUfxP1HneAm9l1qk/7/7qs=</t>
         </is>
       </c>
     </row>
@@ -10099,12 +10099,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>u0NXeN14ll6Lu/HlZX9ysw==</t>
+          <t>39b7XCvrsAp9F4V5k+G8ww==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3dbjsR+iKmXL3z0Z2cFkHtX20AJivSYB5E2ArF2rLio=</t>
+          <t>QKjngOKdxrSfOSGq7XJ5ROQoNA9CAbEJ1iYwhn2GGC4=</t>
         </is>
       </c>
     </row>
@@ -10131,12 +10131,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5VkVrZXqF3G2shfkbrSD9w==</t>
+          <t>N4aUpQlkDCPyy3CRBelcuQ==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>awuxBADzJhtc/wRp/mrMyCsH8vSARbAUkdc0yMN52r0=</t>
+          <t>rKIFR3Bt5FkQ0ILHf5VcU75iBalxSOolQHSgld+4fgA=</t>
         </is>
       </c>
     </row>
@@ -10163,12 +10163,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>DglaGu/LBo6vnwM23y7NYQ==</t>
+          <t>8psdUT4V43PlOrm3GUpu1A==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>bKUh8Dw/XCMeqVfQwUn+5sJ9U7XDw5hUOvYFMqe7kLw=</t>
+          <t>9qmTbikpAUkjgbpPg2eyxu39F83t7v5N2DHGbxl7lPE=</t>
         </is>
       </c>
     </row>
@@ -10195,12 +10195,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>zKeA2AV81IHpQ0wCXnKwaQ==</t>
+          <t>FGqFHAjIGgNVqs4+RjZHqA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>LePCb/ZsLWRp3onwN/stRYlzSRE7sMl/i3M9pG82hoE=</t>
+          <t>q5lWMRYjEedsTkt7uO4+fkrqFbWCl8ANz5Ny6h3yuZ0=</t>
         </is>
       </c>
     </row>
@@ -10227,12 +10227,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>fh7/eotskNRV7WwIf7N/XQ==</t>
+          <t>kSYdRvcbhowZp9ioaoQGiA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>RzweF0eWnJI8vCupYfyycA6yn2ozF9XwrFSAxHYt2zM=</t>
+          <t>KzhQXnTPFMtMLPemiG4haKxbkeOYIvKI02q3sH173gA=</t>
         </is>
       </c>
     </row>
@@ -10259,12 +10259,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>zfJQ+V0xGDwmiHxEmSodug==</t>
+          <t>8x304JPyJ2N1gM03IerW2A==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bkq1Dpw5scpWFsRM4UKr9Jl7l/8CeWNpWqvGR1yquDw=</t>
+          <t>FXV6UGOjXmw3G+IvRHzhS63vtCw5nMQK2MPEoYSyjA8=</t>
         </is>
       </c>
     </row>
@@ -10291,12 +10291,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HTiwy4GJcnqQImzhtWWEnw==</t>
+          <t>fddL/b7PiOREPczlkKHA2A==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>F35uHkaqWJfaFpM27jZJxl8IU/x8I5NWS5W+nHFVGBI=</t>
+          <t>iucyqXbE2BUHSWp9OcQaQkg/ef8tQugpEWmD0RKTPMc=</t>
         </is>
       </c>
     </row>
@@ -10323,12 +10323,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RVxyqRvGJepYwqHxvfOOwg==</t>
+          <t>ODCbhsxmRgwbilEcVggdqg==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MwZzp92NBIhjk0AH9jqPVC20RETYRF4REnw7guSZcVE=</t>
+          <t>IpTyQdxt8vYfH5C4dZvo9oitfAGf3bw3EM2dPmrsf6Y=</t>
         </is>
       </c>
     </row>
@@ -10355,12 +10355,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BoJwdM8kMvx9jWbEvzjXgw==</t>
+          <t>5AnOHYSfpENcRJ2cXLuFoQ==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>fsK2NqP41VIu8Ni6saRw4d5Z8oNL2LPciUaqm+rtm3s=</t>
+          <t>+LJqO0e8HM6XP4vgGHJ8zaiHmMKHKrNO9OrABk0L/Sg=</t>
         </is>
       </c>
     </row>
@@ -10387,12 +10387,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>pqcPX1v3vd8Sp+rX/rSUGg==</t>
+          <t>zZHrRK2kwrH4KD9t+cWDhA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>QnBsn+nGoAfnUjUYkNYkCaXEK/QfsdPLk3vo2cQqKOk=</t>
+          <t>UtYGSIieVMSp3WuO7EEKKmEtsxwM1qR2JC4DmhizR0g=</t>
         </is>
       </c>
     </row>
@@ -10419,12 +10419,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>exWUAy1oyBkYb1CkWmo1Qw==</t>
+          <t>NH/1bxfbbsTjdXbq86CdLA==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>KKvHDCjXFAj/85Hs9DDVOj7N/bCPaUgbJm0oj6Uo3Cg=</t>
+          <t>/EUIuR3kSf+lnQQxjWYuvb+X5wUoJfQDmlRG3iSrRUE=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-29 10:21) - 89 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACCESOS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Categorias'!$A$1:$B$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3965,12 +3965,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3991,22 +3991,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>JEFES</t>
+          <t>GERENCIA</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4fad1e60-e0b1-4cd8-a96c-4a16562120d0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4037,12 +4037,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a89b17b3-7054-43de-af40-580f6642ef37&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4fad1e60-e0b1-4cd8-a96c-4a16562120d0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4068,17 +4068,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>STOCK Y LOGISTICA</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ca658fb8-1f3a-400d-b413-b84dbfc25492&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a89b17b3-7054-43de-af40-580f6642ef37&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4109,12 +4109,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad696dc1-ecc4-4add-92bc-269d1f64e8c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ca658fb8-1f3a-400d-b413-b84dbfc25492&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4140,17 +4140,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VENTAS - COMERCIAL</t>
+          <t>STOCK Y LOGISTICA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad696dc1-ecc4-4add-92bc-269d1f64e8c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="104">
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4325,12 +4325,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4361,12 +4361,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4397,12 +4397,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4433,12 +4433,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -4541,12 +4541,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -4577,12 +4577,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9cc966d7-6002-4a6e-9778-63e56db4b6fd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -4613,12 +4613,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=61dba5db-d24f-47c4-a212-c64465cc56dd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9cc966d7-6002-4a6e-9778-63e56db4b6fd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
@@ -4649,12 +4649,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e2c7bccc-983f-4484-ac5e-6ff109e890ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=61dba5db-d24f-47c4-a212-c64465cc56dd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -4672,8 +4672,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>VENTAS SMK</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e2c7bccc-983f-4484-ac5e-6ff109e890ac&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>INFORME</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H116"/>
+  <autoFilter ref="A1:H117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4684,7 +4720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7433,7 +7469,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -7441,7 +7477,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Informe Hctos</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -7452,7 +7488,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>d4e24e83-9b48-49ff-882e-c5f4392345bf</t>
+          <t>997fd1de-cb5f-4470-afe9-a52a0f251c68</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -7472,12 +7508,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -7485,7 +7521,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -7496,7 +7532,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>4fad1e60-e0b1-4cd8-a96c-4a16562120d0</t>
+          <t>d4e24e83-9b48-49ff-882e-c5f4392345bf</t>
         </is>
       </c>
       <c r="L63" t="n">
@@ -7516,12 +7552,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MARGENES Y COSTOS</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -7529,7 +7565,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -7540,7 +7576,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>0df66729-f27b-49f2-bbd8-9aae3c79ca79</t>
+          <t>4fad1e60-e0b1-4cd8-a96c-4a16562120d0</t>
         </is>
       </c>
       <c r="L64" t="n">
@@ -7560,12 +7596,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>MARGENES Y COSTOS</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MARGENES MC</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -7573,7 +7609,7 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>MARGENES MC</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -7584,7 +7620,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>d0fe6be3-0b91-414d-8ab8-20a749917ed8</t>
+          <t>0df66729-f27b-49f2-bbd8-9aae3c79ca79</t>
         </is>
       </c>
       <c r="L65" t="n">
@@ -7604,12 +7640,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MARGENES Y COSTOS</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>MARGENES MC</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -7617,7 +7653,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>MARGENES MC</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -7628,7 +7664,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>f3324a81-3871-4243-85a2-23f51d9ae770</t>
+          <t>d0fe6be3-0b91-414d-8ab8-20a749917ed8</t>
         </is>
       </c>
       <c r="L66" t="n">
@@ -7648,12 +7684,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>MARGENES Y COSTOS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7661,7 +7697,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Mermas MC</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -7672,7 +7708,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>7abcb544-16b2-46c6-9e30-e033fd764e3d</t>
+          <t>f3324a81-3871-4243-85a2-23f51d9ae770</t>
         </is>
       </c>
       <c r="L67" t="n">
@@ -7692,12 +7728,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7705,7 +7741,7 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Ofertas desempeño</t>
+          <t>Mermas MC</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -7716,7 +7752,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>a89b17b3-7054-43de-af40-580f6642ef37</t>
+          <t>7abcb544-16b2-46c6-9e30-e033fd764e3d</t>
         </is>
       </c>
       <c r="L68" t="n">
@@ -7736,12 +7772,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>STOCK Y LOGISTICA</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7749,7 +7785,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Stock unificado</t>
+          <t>Ofertas desempeño</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -7760,7 +7796,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>c41e244e-dd1d-4c05-bb92-cca5dd11b793</t>
+          <t>a89b17b3-7054-43de-af40-580f6642ef37</t>
         </is>
       </c>
       <c r="L69" t="n">
@@ -7780,12 +7816,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>STOCK Y LOGISTICA</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>VENTAS MENOR COSTE</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -7793,7 +7829,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Ventas Menor Coste</t>
+          <t>Stock unificado</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -7804,7 +7840,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>eef9763b-b2b0-4511-8e24-743e5b681335</t>
+          <t>c41e244e-dd1d-4c05-bb92-cca5dd11b793</t>
         </is>
       </c>
       <c r="L70" t="n">
@@ -7819,17 +7855,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>JEFES</t>
+          <t>GERENCIA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>VENTAS - COMERCIAL</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>VENTAS MENOR COSTE</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -7837,7 +7873,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>Ventas Menor Coste</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -7848,7 +7884,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>f2aecd69-e6f4-4159-9e2d-8b262dfccb70</t>
+          <t>eef9763b-b2b0-4511-8e24-743e5b681335</t>
         </is>
       </c>
       <c r="L71" t="n">
@@ -7873,7 +7909,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7881,7 +7917,7 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -7892,7 +7928,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>ad7033b1-c5ef-4519-b843-eb530bb110c2</t>
+          <t>f2aecd69-e6f4-4159-9e2d-8b262dfccb70</t>
         </is>
       </c>
       <c r="L72" t="n">
@@ -7917,7 +7953,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -7925,7 +7961,7 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>COMPARATIVO VIGENTE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -7936,7 +7972,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8</t>
+          <t>ad7033b1-c5ef-4519-b843-eb530bb110c2</t>
         </is>
       </c>
       <c r="L73" t="n">
@@ -7961,7 +7997,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -7969,7 +8005,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Comportamiento Clientes</t>
+          <t>COMPARATIVO VIGENTE</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -7980,7 +8016,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>1787ebd4-a4bb-4eb3-a825-98d0bae7a62f</t>
+          <t>9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8</t>
         </is>
       </c>
       <c r="L74" t="n">
@@ -8005,7 +8041,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -8013,7 +8049,7 @@
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Consumos por cliente</t>
+          <t>Comportamiento Clientes</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -8024,7 +8060,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>c98743f5-0111-4a4c-8ce7-da33417a325a</t>
+          <t>1787ebd4-a4bb-4eb3-a825-98d0bae7a62f</t>
         </is>
       </c>
       <c r="L75" t="n">
@@ -8049,7 +8085,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -8057,7 +8093,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>Consumos por cliente</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -8068,7 +8104,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>766926ea-349b-4419-8d2c-8204f7ea1313</t>
+          <t>c98743f5-0111-4a4c-8ce7-da33417a325a</t>
         </is>
       </c>
       <c r="L76" t="n">
@@ -8093,7 +8129,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -8101,7 +8137,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Grupo Clientes BLACK 2026</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -8112,7 +8148,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0</t>
+          <t>766926ea-349b-4419-8d2c-8204f7ea1313</t>
         </is>
       </c>
       <c r="L77" t="n">
@@ -8137,7 +8173,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -8145,7 +8181,7 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
+          <t>Grupo Clientes BLACK 2026</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -8156,7 +8192,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>cb91ff77-05db-4f0c-a74d-844bac93f85b</t>
+          <t>3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0</t>
         </is>
       </c>
       <c r="L78" t="n">
@@ -8181,7 +8217,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -8189,7 +8225,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Informe Hctos</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -8200,7 +8236,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>997fd1de-cb5f-4470-afe9-a52a0f251c68</t>
+          <t>cb91ff77-05db-4f0c-a74d-844bac93f85b</t>
         </is>
       </c>
       <c r="L79" t="n">
@@ -8225,7 +8261,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -8233,7 +8269,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Informe Hctos</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -8244,7 +8280,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>da5024b9-7951-4955-9b36-e123275fb22c</t>
+          <t>997fd1de-cb5f-4470-afe9-a52a0f251c68</t>
         </is>
       </c>
       <c r="L80" t="n">
@@ -8269,7 +8305,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -8277,7 +8313,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -8288,7 +8324,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>d4e24e83-9b48-49ff-882e-c5f4392345bf</t>
+          <t>da5024b9-7951-4955-9b36-e123275fb22c</t>
         </is>
       </c>
       <c r="L81" t="n">
@@ -8308,12 +8344,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -8321,7 +8357,7 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -8332,7 +8368,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>4fad1e60-e0b1-4cd8-a96c-4a16562120d0</t>
+          <t>d4e24e83-9b48-49ff-882e-c5f4392345bf</t>
         </is>
       </c>
       <c r="L82" t="n">
@@ -8352,12 +8388,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>VENTAS - COMERCIAL</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -8365,22 +8401,22 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Grupo Hergo - Jefes</t>
+          <t>Informes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
+          <t>4fad1e60-e0b1-4cd8-a96c-4a16562120d0</t>
         </is>
       </c>
       <c r="L83" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -8396,12 +8432,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -8409,22 +8445,22 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Ofertas desempeño</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Informes</t>
+          <t>Grupo Hergo - Jefes</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>a89b17b3-7054-43de-af40-580f6642ef37</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L84" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="85">
@@ -8440,12 +8476,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>VENTAS - COMERCIAL</t>
+          <t>PRECIOS Y OFERTAS</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -8453,7 +8489,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Sin cargo CFH</t>
+          <t>Ofertas desempeño</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -8464,7 +8500,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>9cc966d7-6002-4a6e-9778-63e56db4b6fd</t>
+          <t>a89b17b3-7054-43de-af40-580f6642ef37</t>
         </is>
       </c>
       <c r="L85" t="n">
@@ -8484,12 +8520,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>STOCK Y LOGISTICA</t>
+          <t>VENTAS - COMERCIAL</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -8497,7 +8533,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>Sin cargo CFH</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -8508,7 +8544,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>ca658fb8-1f3a-400d-b413-b84dbfc25492</t>
+          <t>9cc966d7-6002-4a6e-9778-63e56db4b6fd</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -8533,7 +8569,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -8541,7 +8577,7 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -8552,7 +8588,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>ad696dc1-ecc4-4add-92bc-269d1f64e8c8</t>
+          <t>ca658fb8-1f3a-400d-b413-b84dbfc25492</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -8572,12 +8608,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>VENTAS - COMERCIAL</t>
+          <t>STOCK Y LOGISTICA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -8585,7 +8621,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -8596,7 +8632,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>e2c7bccc-983f-4484-ac5e-6ff109e890ac</t>
+          <t>ad696dc1-ecc4-4add-92bc-269d1f64e8c8</t>
         </is>
       </c>
       <c r="L88" t="n">
@@ -8621,7 +8657,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -8629,7 +8665,7 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -8640,17 +8676,61 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
+          <t>e2c7bccc-983f-4484-ac5e-6ff109e890ac</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>VENTAS - COMERCIAL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>VENTA MAYORISTA DETALLE</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Venta Mayorista Detalle</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Informes</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
           <t>61dba5db-d24f-47c4-a212-c64465cc56dd</t>
         </is>
       </c>
-      <c r="L89" t="n">
+      <c r="L90" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L89"/>
+  <autoFilter ref="A1:L90"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9277,12 +9357,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5SJVkGR9sm0iA0bKu/oJzw==</t>
+          <t>Yyb13LyPiqz+WIfu4OMOLg==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CWtPuY/jDyoLmD7Zu9L3qdgAuh2SaX4SIEpqdryvJKA=</t>
+          <t>dUbd/FvAgRSbW7Scft+6nSmpxipn5vN4SkgceMLD95E=</t>
         </is>
       </c>
     </row>
@@ -9309,12 +9389,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TKShgGmT02Kc8sqZX0ClhA==</t>
+          <t>WUPeZ6Y62MuCqLo+c7GlKA==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>NjtcNrzTqrgLrV84/kslIRnGkx7m+YktJYH7uW61ybo=</t>
+          <t>7cVFvQDBmewwli+0OD7pxB5AKkxoNhNJ9O3EwV8F+DE=</t>
         </is>
       </c>
     </row>
@@ -9341,12 +9421,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>O99MSLtesyrgePkZPT8MtQ==</t>
+          <t>+Qhmoa6xtopaMbzAFWXN8Q==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>v+As+O56LMBbfSchjo9tO43ozt9F0CElvtfwWSrUhrs=</t>
+          <t>KfN4SrC+G3H4ybWi8xa71daxkYUjB9teihtJoiTjjN8=</t>
         </is>
       </c>
     </row>
@@ -9368,12 +9448,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3PBpuluffW/sOel75AroSg==</t>
+          <t>m6Vhsv7JRl1kTxklBlVK2g==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>wybPdQViRnQViR9g7Xiv4+eqsmhnLyCA9y/qf6Asrag=</t>
+          <t>IqeG8dqL+BgJj/qMw+se2me+pkSGz1GA74ts+MYyTAQ=</t>
         </is>
       </c>
     </row>
@@ -9400,12 +9480,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>dFE+ANStl2SvA5tPTNrUVQ==</t>
+          <t>9tk2ijwdCxAcch72U8Cg/A==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>nwnj9ydeK9CdmlzigiQM0HK5EoTeQi1ICrlT3L4ZTIA=</t>
+          <t>QyLttpeITBI6a8nArNdISW/zi+vOQfJxhlOhAUybJWU=</t>
         </is>
       </c>
     </row>
@@ -9432,12 +9512,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HXNAYtgiCHWnBiTCd0UMHA==</t>
+          <t>kFuAc2KJtDJwPc9BXAEYhg==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>scrLjpCyGXO2BZzCJFUP6i61ReV8g073BST6gPpDYmk=</t>
+          <t>3g5nRrg7q4cYpZOYJo0/Sko7y3yceiHLanXGlICWtEc=</t>
         </is>
       </c>
     </row>
@@ -9464,12 +9544,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>xTYV9gC5ft2I+OqGS+7gfw==</t>
+          <t>P9nX7pB5oMH0i1L8IgNbjg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>VspzY8lqCufsCHoqOi+IIlFMvMWetLhWxROwhVY9yb0=</t>
+          <t>bSjsGVIq2noov4pvJazkwZejSp2UTPrn0H0e6+o1KWs=</t>
         </is>
       </c>
     </row>
@@ -9491,12 +9571,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5VHwVvwkSce9KFsujy67XA==</t>
+          <t>GJ1+8wXr93jY2Qq/bReFqw==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>YoczRBMXLCo6LbpqqWCcWL4BvKghh6rYwFm3LWcebOQ=</t>
+          <t>uxGNJ83e3c1OWxNGHfa5o2qkF7L6VwxUNPNqY5yPvME=</t>
         </is>
       </c>
     </row>
@@ -9523,12 +9603,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>lsR3LB4sZA9jQISGUgw3mQ==;M8GWbcrj6RK9+mxLI/P5ZA==</t>
+          <t>AFclBb8ptL+gRCTYCZDMfg==;s1Q5q85eG5EP7xIakz8aRg==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>6ewgfqSId3o7jusgxWVcEmwZiHbL74Gfzpn69TdELKI=;FSWMeTIkJpKc6BVj/e4BpvEdZG+Ffg7QlhnE6Z8gZpI=</t>
+          <t>6bkN5E/MOc0tWHxceInvhKJZk7GP7lWE5FbgKMTB4nU=;U+8b0qHWSo96BsHNNtdTlruCh0sCk3WwtPXzOK/LJlY=</t>
         </is>
       </c>
     </row>
@@ -9555,12 +9635,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGi/fha1pJhhaVEFgu+ZCg==</t>
+          <t>8p1QzTgXuTpfdiNnYUZBxw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ytyNH3NpDGdrWjHa5C8YXoGGatTvyaJvO6bzNDOgAQw=</t>
+          <t>MFe0dZvMztU0YlyW/sei50SvTx51yg7I6q2D9CuyOYo=</t>
         </is>
       </c>
     </row>
@@ -9587,12 +9667,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SYf+EnbdweyNqHm6cSWExQ==</t>
+          <t>vfZdg1M7Dy2vmepuCaHlQg==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Pprf1RHKve/y0g2IcC8ooQqZ3f9zrhHokHMawdZOiuI=</t>
+          <t>KZ+OZmrFrlX6HzPKJCRvtOSKzUd2R9QfapF5oenZbTw=</t>
         </is>
       </c>
     </row>
@@ -9619,12 +9699,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3dpJvSm1iCbucdNeJJKNAA==</t>
+          <t>JuKzv2klqq0wIK2wkNOwlw==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0+1ScviwzUdeBXDEtHNj1RWU+znSW7iz1TbgAfxHV6k=</t>
+          <t>WyOnToyCRgY6UsWMJRLsdNWUIjlmgibZGzbuNaDLRxA=</t>
         </is>
       </c>
     </row>
@@ -9651,12 +9731,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kv/DIf5ZZ2AvTIgaimaP0Q==</t>
+          <t>6s1AtCcVuEZkBPk2hwwcnQ==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>7pQ7FhSS8lMabK6050Q1bSKcxurELVDcZpJgeja3c+U=</t>
+          <t>ePUaWL4MRpvnd+xH2DWyl1S/SIGXPnR1/TD/upkC1bs=</t>
         </is>
       </c>
     </row>
@@ -9683,12 +9763,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>nAeKGdA1FOUmgDvE1BHfMg==</t>
+          <t>FcFOzPBoSvoD/+pp61Yu/A==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>DT7owku4AEBAM0C7y1juQU2JDr//Oa8th8+IhGOuMW8=</t>
+          <t>C0YGrVFbEaqMpXhzCgqwaIWr15H7Khxegj7gLOI8P1w=</t>
         </is>
       </c>
     </row>
@@ -9715,12 +9795,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>pbIyco0qTwHY48T4hGBW1Q==</t>
+          <t>21/kM5dPUPaizR6hJxAKfQ==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>zSKSsNvZ7W70cDLHjtHotSi46dbgqMrWD51OL1jMvgA=</t>
+          <t>ImEHMCHYMwJVr0kCErEx6uDJZF5MP3bMYIQfeIK6egw=</t>
         </is>
       </c>
     </row>
@@ -9747,12 +9827,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>DA1k1eyXjx7P8ptcPPr0fg==</t>
+          <t>cyZE2Quqo64gz3pEMkpVzg==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yJp3UrES4gP4VhfreXN8BxFPXwi2iPPmSzHO3o5k/BU=</t>
+          <t>1Cp1GU3tN6osRnvLyls/iST2nIMaOB+pSdKl6GAwhoQ=</t>
         </is>
       </c>
     </row>
@@ -9779,12 +9859,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>UQZzYmGeagQfoK2iZ7aTuA==</t>
+          <t>KXPSzC5fl+i3tS95DdRE7Q==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>VjM2lq1iwgPeKvXbLo08D19q/nnvoGEs7eeq7sOFT/w=</t>
+          <t>6ueKFz+EyoJafZ304Zaq6PD29XFpedGAmh9ZlBXZTcs=</t>
         </is>
       </c>
     </row>
@@ -9811,12 +9891,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>rlgJS2iD4k/70nvtRZt9Yw==</t>
+          <t>yOjrxMuGg/S8SHD8fLtlvA==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>z7UEDv3EFTCKGKzWv7niGk+0xa0hR7I75oYZc1xbEtw=</t>
+          <t>vujqMR1La9prVmzpuH0BV9IeMtj+t35XtWDF07vvYI0=</t>
         </is>
       </c>
     </row>
@@ -9843,12 +9923,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TIXF9S6EHe2Y764nDdwveg==</t>
+          <t>fdYIRtgU13PawQ/RGXq+Og==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>lXaKg+nrNlOolz5n2Z8FCbkauIPV5VeRXms0D2tU3sY=</t>
+          <t>Aa+nvmPtYVMuqBLpb3/nPNS9g3FSm+EENnXiH3KFBjM=</t>
         </is>
       </c>
     </row>
@@ -9875,12 +9955,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RJXWJThzWsD01KwVEMc3xg==</t>
+          <t>Vg7nCcCI4H9k6Xuw7dM3Xw==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>OKSQKj2lSyYq+y9czeJzsNrULPrio4LqXYoZ0GMx8ak=</t>
+          <t>Pw+fGhlHfc7IXCkGpz6A35Jlk87IqfvSjB4QvVr9kxI=</t>
         </is>
       </c>
     </row>
@@ -9907,12 +9987,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>fE+I7K5oTIjMAcEiAuxSTg==</t>
+          <t>P4fblnHcrj+i2WbuHhG3lQ==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>yS9abYUxCghbefRec691MZNd+pZIkrrkz/AGhbu9K5w=</t>
+          <t>yAlm+6KSZG54Qe2yx89HFtYV0RZAhrMRDxoA5kKfwT4=</t>
         </is>
       </c>
     </row>
@@ -9939,12 +10019,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2+FEZIfktWFjrYHiDdSEGA==</t>
+          <t>7BbWNkQ+Q3N5J6e9e62rDw==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>FagCQMh/r4g7XPtFU33THSTXdneqNVQ/jJx5edfPMzE=</t>
+          <t>2drjLTcAyACsOnRtq2igpUfBtO5NX/rqX4SeCBvi6oA=</t>
         </is>
       </c>
     </row>
@@ -9971,12 +10051,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>JdCH8WsU09HvY86zr2cCwA==</t>
+          <t>qRxUgmc0FGsYQmj8s3pZ2g==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>fwonNasZYviW8iK7SNyVgX4bD7LlmQCC6RB9dvIwbNI=</t>
+          <t>cjtoscS4TDBTSLUHwU80gW9qp7lhjNPMRm1pNC2U95Y=</t>
         </is>
       </c>
     </row>
@@ -10003,12 +10083,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>rcP2UTuCrS+aumf7t4ZIOg==</t>
+          <t>MiV37dd4DA3OdAjWNyPqmw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>S6SC8LWF7j4MHGp0Towj0e+6MB53nT8wSWnmCQf/u+Y=</t>
+          <t>Ap0qPNq83uKYEmp0jCbzxjA11OmQI8ADPoF7T5ttnEY=</t>
         </is>
       </c>
     </row>
@@ -10035,12 +10115,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4ZBbq3cS2ZWp7X67zAJIjQ==</t>
+          <t>q6ogW44lf7TqcBAs5wtfIA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>tx34WQLwRlPcW/v3qaAFBLcMOhlsuZ068z38FSaekiU=</t>
+          <t>urWooYqscC5Ccl6uFUoveDHIrTw5U4POz7PrvCGf050=</t>
         </is>
       </c>
     </row>
@@ -10067,12 +10147,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>UMJAVzRcX7Liivi6DyJMtw==</t>
+          <t>p9OrJH2z7OHHx5I8E0n85A==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>A3Zs+fOEm1FD4UfBj7bGyiUfxP1HneAm9l1qk/7/7qs=</t>
+          <t>LZUcUdDf1pCM4SBcOMHoUMCcFwVefRcHqAsGdTKZbA4=</t>
         </is>
       </c>
     </row>
@@ -10099,12 +10179,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>39b7XCvrsAp9F4V5k+G8ww==</t>
+          <t>8XgZC39x94dkxLSBZWT6/w==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>QKjngOKdxrSfOSGq7XJ5ROQoNA9CAbEJ1iYwhn2GGC4=</t>
+          <t>TMGxDCaM+przSIQHaw0Zh9MLgWFz9PDDRSHQ0oUxXZU=</t>
         </is>
       </c>
     </row>
@@ -10131,12 +10211,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>N4aUpQlkDCPyy3CRBelcuQ==</t>
+          <t>cRj4CI/KDkeLIkLh/mjQ5A==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>rKIFR3Bt5FkQ0ILHf5VcU75iBalxSOolQHSgld+4fgA=</t>
+          <t>Jt1MIOXl/IuLFRKVcA9Nn5byhznGG5ho0Q/2ICDkOfw=</t>
         </is>
       </c>
     </row>
@@ -10163,12 +10243,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>8psdUT4V43PlOrm3GUpu1A==</t>
+          <t>Xc8XhaLQ3zZS8o9q0ZxEbw==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>9qmTbikpAUkjgbpPg2eyxu39F83t7v5N2DHGbxl7lPE=</t>
+          <t>38eZdPDU8Q0ja4WrsQVHYWbe9bLavcpz3oNHCl20h0s=</t>
         </is>
       </c>
     </row>
@@ -10195,12 +10275,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FGqFHAjIGgNVqs4+RjZHqA==</t>
+          <t>taTpVnTxeaT8aSHD1Ce80g==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>q5lWMRYjEedsTkt7uO4+fkrqFbWCl8ANz5Ny6h3yuZ0=</t>
+          <t>e70KndQUQwoF7Qz57PLTwYAHmtiJuJ8zwNOuhQur2Fg=</t>
         </is>
       </c>
     </row>
@@ -10227,12 +10307,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>kSYdRvcbhowZp9ioaoQGiA==</t>
+          <t>1qLbzItPOrEJCopMqedrrA==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>KzhQXnTPFMtMLPemiG4haKxbkeOYIvKI02q3sH173gA=</t>
+          <t>8YTjU+m5Tb0PhPAIKmYZ/Ozi+M8J6iDDPkHYWTf5zSE=</t>
         </is>
       </c>
     </row>
@@ -10259,12 +10339,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>8x304JPyJ2N1gM03IerW2A==</t>
+          <t>84Kx+uVk7Z64MPotFtenQA==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>FXV6UGOjXmw3G+IvRHzhS63vtCw5nMQK2MPEoYSyjA8=</t>
+          <t>kzV1kJ6/mrDIrwvx4GKGxb5hLW0vS8g104Q1ZmMvf3A=</t>
         </is>
       </c>
     </row>
@@ -10291,12 +10371,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>fddL/b7PiOREPczlkKHA2A==</t>
+          <t>29F1vgGcerBkn5PX53qd1A==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>iucyqXbE2BUHSWp9OcQaQkg/ef8tQugpEWmD0RKTPMc=</t>
+          <t>nCtPzAuRBrT6Q5XyOTYmGRfoqMs1pY49xSxYshdKc1A=</t>
         </is>
       </c>
     </row>
@@ -10323,12 +10403,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ODCbhsxmRgwbilEcVggdqg==</t>
+          <t>gE+qfKb7ULvxlik9Na6VKA==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>IpTyQdxt8vYfH5C4dZvo9oitfAGf3bw3EM2dPmrsf6Y=</t>
+          <t>nJvfRHZjQhMu0GVagJn4tCIYefcBj4aWQ9NDr1V6tjQ=</t>
         </is>
       </c>
     </row>
@@ -10355,12 +10435,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>5AnOHYSfpENcRJ2cXLuFoQ==</t>
+          <t>NrKAgh3ICVngwcsf1jcr7A==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>+LJqO0e8HM6XP4vgGHJ8zaiHmMKHKrNO9OrABk0L/Sg=</t>
+          <t>eyBSlgVeefcIoqNb7iT1D4nohQhz40PZAjnP1p3Cmjs=</t>
         </is>
       </c>
     </row>
@@ -10387,12 +10467,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>zZHrRK2kwrH4KD9t+cWDhA==</t>
+          <t>Kfw1jJfwwDGpeSRvCfIYew==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>UtYGSIieVMSp3WuO7EEKKmEtsxwM1qR2JC4DmhizR0g=</t>
+          <t>jXDHHvHivKLnc8IqIF++jGXGivjA/cUwSzeVmt+cIuQ=</t>
         </is>
       </c>
     </row>
@@ -10419,12 +10499,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>NH/1bxfbbsTjdXbq86CdLA==</t>
+          <t>GnKaZF206/G5zg9uXgxSnw==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>/EUIuR3kSf+lnQQxjWYuvb+X5wUoJfQDmlRG3iSrRUE=</t>
+          <t>HqgOfN6LItTVyjZpyWhKYj40I1EX6A8bHGLSYfLsCh0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo tableros (2026-10-30 07:41) - 89 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1505,12 +1505,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CONTROL DE COSTOS</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1ef38484-9abb-4187-ab6d-42a823bd9245&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>CONTROL DE COSTOS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1ef38484-9abb-4187-ab6d-42a823bd9245&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -1993,7 +1993,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="43">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44">
@@ -2101,7 +2101,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c89306f-b143-4050-8567-94a4a79d0844&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -2225,12 +2225,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c89306f-b143-4050-8567-94a4a79d0844&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>COMPARATIVO VIGENTE</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="62">
@@ -2705,12 +2705,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPARATIVO VIGENTE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2813,12 +2813,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2885,12 +2885,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="73">
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="74">
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76">
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="82">
@@ -3425,12 +3425,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2c89306f-b143-4050-8567-94a4a79d0844&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
@@ -3461,12 +3461,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0df66729-f27b-49f2-bbd8-9aae3c79ca79&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2c89306f-b143-4050-8567-94a4a79d0844&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -3481,7 +3481,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="92">
@@ -3785,12 +3785,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPARATIVO</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93">
@@ -3821,12 +3821,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -3893,12 +3893,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>COMPARATIVO</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
     <row r="104">
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>AVANCE CCU</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="105">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>SIN CARGO CFH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=46395ec1-f0ac-4b34-9a0c-40fe1322db9f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4273,7 +4273,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>COMPARATIVO</t>
+          <t>HECTOLITROS</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9bce5e20-c4d5-41c4-9dca-0bd7b562c6c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4309,7 +4309,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>AVANCE CCU</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f2aecd69-e6f4-4159-9e2d-8b262dfccb70&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4361,12 +4361,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ad7033b1-c5ef-4519-b843-eb530bb110c2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4397,12 +4397,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1787ebd4-a4bb-4eb3-a825-98d0bae7a62f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4433,12 +4433,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>GRUPO CLIENTES BLACK 2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c98743f5-0111-4a4c-8ce7-da33417a325a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>HECTOLITROS</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=997fd1de-cb5f-4470-afe9-a52a0f251c68&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=766926ea-349b-4419-8d2c-8204f7ea1313&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3a185bf8-fd9f-45ba-9430-d4ed3aea4ce0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -4541,12 +4541,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cb91ff77-05db-4f0c-a74d-844bac93f85b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -4577,12 +4577,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=da5024b9-7951-4955-9b36-e123275fb22c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -4613,12 +4613,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>SIN CARGO CFH</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9cc966d7-6002-4a6e-9778-63e56db4b6fd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4e24e83-9b48-49ff-882e-c5f4392345bf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
@@ -4884,7 +4884,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -4928,7 +4928,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -5104,7 +5104,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
@@ -5720,7 +5720,7 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23">
@@ -5764,7 +5764,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -5808,7 +5808,7 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28">
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -6204,7 +6204,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -6476,7 +6476,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="40">
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -6832,7 +6832,7 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48">
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="L48" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49">
@@ -6920,7 +6920,7 @@
         </is>
       </c>
       <c r="L49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -6964,7 +6964,7 @@
         </is>
       </c>
       <c r="L50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -7052,7 +7052,7 @@
         </is>
       </c>
       <c r="L52" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="53">
@@ -7096,7 +7096,7 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="54">
@@ -7140,7 +7140,7 @@
         </is>
       </c>
       <c r="L54" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
@@ -7228,7 +7228,7 @@
         </is>
       </c>
       <c r="L56" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57">
@@ -7360,7 +7360,7 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -7404,7 +7404,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -7492,7 +7492,7 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66">
@@ -7844,7 +7844,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71">
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="L74" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="75">
@@ -8284,7 +8284,7 @@
         </is>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -8539,16 +8539,16 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Informes</t>
+          <t>Grupo Hergo - Jefes</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>9cc966d7-6002-4a6e-9778-63e56db4b6fd</t>
+          <t>46395ec1-f0ac-4b34-9a0c-40fe1322db9f</t>
         </is>
       </c>
       <c r="L86" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
@@ -9357,12 +9357,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Yyb13LyPiqz+WIfu4OMOLg==</t>
+          <t>YgCU9wMQ86HbKirEKOYOyw==</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dUbd/FvAgRSbW7Scft+6nSmpxipn5vN4SkgceMLD95E=</t>
+          <t>KI+LeJp+WOlVQiaDITvKZsILmomP73J5EWpRpVbyHDs=</t>
         </is>
       </c>
     </row>
@@ -9389,12 +9389,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>WUPeZ6Y62MuCqLo+c7GlKA==</t>
+          <t>C4HMrYEgp3YNVPLY1o4GtQ==</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>7cVFvQDBmewwli+0OD7pxB5AKkxoNhNJ9O3EwV8F+DE=</t>
+          <t>EJneYhu9E25FVj5JfMrKWh31XT3yzXskB4uVJUkPyVw=</t>
         </is>
       </c>
     </row>
@@ -9421,12 +9421,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+Qhmoa6xtopaMbzAFWXN8Q==</t>
+          <t>8XcAK4qXJWZqco3pJOXZ7Q==</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>KfN4SrC+G3H4ybWi8xa71daxkYUjB9teihtJoiTjjN8=</t>
+          <t>vsXqwnqXHDjxHTtq20jMW2VeQGaBNsQXbToxE0QA+JM=</t>
         </is>
       </c>
     </row>
@@ -9448,12 +9448,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>m6Vhsv7JRl1kTxklBlVK2g==</t>
+          <t>4avxrwGRQF/DL/eEJyNyOg==</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IqeG8dqL+BgJj/qMw+se2me+pkSGz1GA74ts+MYyTAQ=</t>
+          <t>b/fX+G8FmDnr6u3YnjYhgULRwIMcncldgX5OAFbsPWk=</t>
         </is>
       </c>
     </row>
@@ -9480,12 +9480,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9tk2ijwdCxAcch72U8Cg/A==</t>
+          <t>mJ6NGlmydZt89BOBGmLb0Q==</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>QyLttpeITBI6a8nArNdISW/zi+vOQfJxhlOhAUybJWU=</t>
+          <t>pX5Sh0zdkgo5pB7yu5Yssjz+BmZXhC9P87fTniTgt/U=</t>
         </is>
       </c>
     </row>
@@ -9512,12 +9512,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>kFuAc2KJtDJwPc9BXAEYhg==</t>
+          <t>OyLLSKTkObbIG2KqQC3qbw==</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3g5nRrg7q4cYpZOYJo0/Sko7y3yceiHLanXGlICWtEc=</t>
+          <t>5cwWnqipSDSHikLIxK7chbyyZNBBQWdzDuA0GvspBjs=</t>
         </is>
       </c>
     </row>
@@ -9544,12 +9544,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>P9nX7pB5oMH0i1L8IgNbjg==</t>
+          <t>jwAmT2mbdGplK1Itzpnoeg==</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>bSjsGVIq2noov4pvJazkwZejSp2UTPrn0H0e6+o1KWs=</t>
+          <t>ZDfJn/mvgo5iY98R/ZVeoBTPw/kTBNOE6xuTMdP6JaM=</t>
         </is>
       </c>
     </row>
@@ -9571,12 +9571,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GJ1+8wXr93jY2Qq/bReFqw==</t>
+          <t>kzZwLsI7y0HJ9exOGL1+IA==</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>uxGNJ83e3c1OWxNGHfa5o2qkF7L6VwxUNPNqY5yPvME=</t>
+          <t>x5ikjOv/EvPlHkLpMRsvQ0pmyxNhN2nJ3TJif5XXjKs=</t>
         </is>
       </c>
     </row>
@@ -9603,12 +9603,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AFclBb8ptL+gRCTYCZDMfg==;s1Q5q85eG5EP7xIakz8aRg==</t>
+          <t>/0/JOY5b1VYADNbByMMhfw==;/s4GYpJzaAyQJusBMIcRYw==</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>6bkN5E/MOc0tWHxceInvhKJZk7GP7lWE5FbgKMTB4nU=;U+8b0qHWSo96BsHNNtdTlruCh0sCk3WwtPXzOK/LJlY=</t>
+          <t>uoT9BC3lB2tF/mMQ2TrXNTMHbBRiBTr6jwesalU8Lb8=;2fGO3iapB/GjHo3wLUxzakbTIM18SzW1w7lUOodsJbM=</t>
         </is>
       </c>
     </row>
@@ -9635,12 +9635,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>8p1QzTgXuTpfdiNnYUZBxw==</t>
+          <t>EQ5LxwxglEmU2lTc6I1Ufw==</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MFe0dZvMztU0YlyW/sei50SvTx51yg7I6q2D9CuyOYo=</t>
+          <t>BUn/mm1IIlMvzaPjK5OE/NDpscPhE0auNHYNOdEVK0Y=</t>
         </is>
       </c>
     </row>
@@ -9667,12 +9667,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>vfZdg1M7Dy2vmepuCaHlQg==</t>
+          <t>P+2wiXhPcDSPZHIIhje05A==</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>KZ+OZmrFrlX6HzPKJCRvtOSKzUd2R9QfapF5oenZbTw=</t>
+          <t>OhV/Ey0fLEC3PeAng37kVCiuXszwhQKqrB3pA1HIKEc=</t>
         </is>
       </c>
     </row>
@@ -9699,12 +9699,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>JuKzv2klqq0wIK2wkNOwlw==</t>
+          <t>kHvZShFDCbxjZSugYhPIBQ==</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WyOnToyCRgY6UsWMJRLsdNWUIjlmgibZGzbuNaDLRxA=</t>
+          <t>AY2XJXP7fe4zR+5Qy26Yrpe9+QZqC7OC7jRaXgggZec=</t>
         </is>
       </c>
     </row>
@@ -9731,12 +9731,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6s1AtCcVuEZkBPk2hwwcnQ==</t>
+          <t>SWD+LiPWF6DerFi077hG4Q==</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ePUaWL4MRpvnd+xH2DWyl1S/SIGXPnR1/TD/upkC1bs=</t>
+          <t>1viary/RTeBtpEcWpnwuZC5sQ4gqh5tew8qx9xDz8ng=</t>
         </is>
       </c>
     </row>
@@ -9763,12 +9763,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FcFOzPBoSvoD/+pp61Yu/A==</t>
+          <t>FZoF7v/kTXYHuQ//fSgnRQ==</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C0YGrVFbEaqMpXhzCgqwaIWr15H7Khxegj7gLOI8P1w=</t>
+          <t>bg+hl1uTYOLg5o0m4UdlUc0WaMnPJ0h7v2tUN8Oj5QI=</t>
         </is>
       </c>
     </row>
@@ -9795,12 +9795,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>21/kM5dPUPaizR6hJxAKfQ==</t>
+          <t>JY7B2imLrNG+2JUe5L23ag==</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ImEHMCHYMwJVr0kCErEx6uDJZF5MP3bMYIQfeIK6egw=</t>
+          <t>oXDTR3izAPTQPSBLA4T/3nWtscnEqFNMGuj2FEtcOfA=</t>
         </is>
       </c>
     </row>
@@ -9827,12 +9827,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>cyZE2Quqo64gz3pEMkpVzg==</t>
+          <t>kfCbUfGAFHTcXxqblRPyNA==</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1Cp1GU3tN6osRnvLyls/iST2nIMaOB+pSdKl6GAwhoQ=</t>
+          <t>ze87XxL4l/LuIb3NXkTj/DcFexsxMV0dUB4H+x0MclM=</t>
         </is>
       </c>
     </row>
@@ -9859,12 +9859,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KXPSzC5fl+i3tS95DdRE7Q==</t>
+          <t>dggo+3FA11zGZTPrQxNdkw==</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6ueKFz+EyoJafZ304Zaq6PD29XFpedGAmh9ZlBXZTcs=</t>
+          <t>F6LZ0cOtzDG2Oah2kNg/NBDAnlTukAKXoWK5RqCW9zk=</t>
         </is>
       </c>
     </row>
@@ -9891,12 +9891,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>yOjrxMuGg/S8SHD8fLtlvA==</t>
+          <t>7WVcMnMCA05lNDDHtW4diw==</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>vujqMR1La9prVmzpuH0BV9IeMtj+t35XtWDF07vvYI0=</t>
+          <t>ZNROLzIRw4pg3id4QZ9wrE6t7WiMMPu/Pxz6IvpIpUk=</t>
         </is>
       </c>
     </row>
@@ -9923,12 +9923,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>fdYIRtgU13PawQ/RGXq+Og==</t>
+          <t>9O6JTWUKlpShFNhmBK4tZQ==</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Aa+nvmPtYVMuqBLpb3/nPNS9g3FSm+EENnXiH3KFBjM=</t>
+          <t>8/sZKBsb5FMZojW0KOXI1M9RFXxCDe2/GdEVJPnYh/Y=</t>
         </is>
       </c>
     </row>
@@ -9955,12 +9955,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Vg7nCcCI4H9k6Xuw7dM3Xw==</t>
+          <t>XCoK/hErBJyOlOEJq2ga6g==</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Pw+fGhlHfc7IXCkGpz6A35Jlk87IqfvSjB4QvVr9kxI=</t>
+          <t>6CCh6ftowogUsQQAeDg2z/cn7XNunC9Hdo/W9J9YQI8=</t>
         </is>
       </c>
     </row>
@@ -9987,12 +9987,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>P4fblnHcrj+i2WbuHhG3lQ==</t>
+          <t>p5bbpWNIxg2gwypUgFBaCg==</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>yAlm+6KSZG54Qe2yx89HFtYV0RZAhrMRDxoA5kKfwT4=</t>
+          <t>i1sFnviiqq0SM7Fsq/hiNe97nr+bJME57yhOeUbZ3NA=</t>
         </is>
       </c>
     </row>
@@ -10019,12 +10019,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7BbWNkQ+Q3N5J6e9e62rDw==</t>
+          <t>AdaEho8UILpwRtonr+R7tg==</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2drjLTcAyACsOnRtq2igpUfBtO5NX/rqX4SeCBvi6oA=</t>
+          <t>MBphDwnhIvwD9zBi/Y8JpFmm+cDLL7JSWIssbaDxI7s=</t>
         </is>
       </c>
     </row>
@@ -10051,12 +10051,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>qRxUgmc0FGsYQmj8s3pZ2g==</t>
+          <t>51QNLHUqJWdG60QsCYOlcA==</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>cjtoscS4TDBTSLUHwU80gW9qp7lhjNPMRm1pNC2U95Y=</t>
+          <t>0dKKzpJZK8O40OpbSYJhcLcOb5Q44gMjCk+iH8WF2J0=</t>
         </is>
       </c>
     </row>
@@ -10083,12 +10083,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MiV37dd4DA3OdAjWNyPqmw==</t>
+          <t>ccf7GPNt+YLTvmtxGJV1Gw==</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Ap0qPNq83uKYEmp0jCbzxjA11OmQI8ADPoF7T5ttnEY=</t>
+          <t>7PoDU6sZybGNBYkM7WtDj1/7OyyU+4AJZhclHt1vnQY=</t>
         </is>
       </c>
     </row>
@@ -10115,12 +10115,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>q6ogW44lf7TqcBAs5wtfIA==</t>
+          <t>SQXiTGlmx90lIg66oqOuhA==</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>urWooYqscC5Ccl6uFUoveDHIrTw5U4POz7PrvCGf050=</t>
+          <t>9Kr1KI5+Ve+KuNRBq4I78HFmatGPXOfVQo3cHskICJM=</t>
         </is>
       </c>
     </row>
@@ -10147,12 +10147,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>p9OrJH2z7OHHx5I8E0n85A==</t>
+          <t>q5Q2xwq53mC+5HOZl2IQRA==</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>LZUcUdDf1pCM4SBcOMHoUMCcFwVefRcHqAsGdTKZbA4=</t>
+          <t>yLDpfsqx8d04EQ/ayCup4/2eRadWQrcRmFnTgUkW6HU=</t>
         </is>
       </c>
     </row>
@@ -10179,12 +10179,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>8XgZC39x94dkxLSBZWT6/w==</t>
+          <t>jMdujo+xlWrTR6zBzXMjPg==</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TMGxDCaM+przSIQHaw0Zh9MLgWFz9PDDRSHQ0oUxXZU=</t>
+          <t>jGCuzCEbB6DoqYwCDLlRlBe2d19G5SzB+565oVtL7kI=</t>
         </is>
       </c>
     </row>
@@ -10211,12 +10211,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>cRj4CI/KDkeLIkLh/mjQ5A==</t>
+          <t>+BfQEVZBZn2L+aGnUudxxw==</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Jt1MIOXl/IuLFRKVcA9Nn5byhznGG5ho0Q/2ICDkOfw=</t>
+          <t>cbxnG0ljPABThJ6WlmVHapq3CINEDI/2R9nnnEh6Ra0=</t>
         </is>
       </c>
     </row>
@@ -10243,12 +10243,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Xc8XhaLQ3zZS8o9q0ZxEbw==</t>
+          <t>ns2vMz8tiVXy1LcG3h1iuw==</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>38eZdPDU8Q0ja4WrsQVHYWbe9bLavcpz3oNHCl20h0s=</t>
+          <t>Zs1K7BgRY+D0SGKuNjFBp2zwb+caf5icO7SncFoKZ3I=</t>
         </is>
       </c>
     </row>
@@ -10275,12 +10275,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>taTpVnTxeaT8aSHD1Ce80g==</t>
+          <t>xOGVVaXtVdVJLGdtwa+vuA==</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e70KndQUQwoF7Qz57PLTwYAHmtiJuJ8zwNOuhQur2Fg=</t>
+          <t>iFm8R9SwrKsUUWDzrS9zpJorH+ouTULa21QIPO5UIxw=</t>
         </is>
       </c>
     </row>
@@ -10307,12 +10307,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1qLbzItPOrEJCopMqedrrA==</t>
+          <t>5U9LCCxVKoVXhsQcxmNUxg==</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>8YTjU+m5Tb0PhPAIKmYZ/Ozi+M8J6iDDPkHYWTf5zSE=</t>
+          <t>yEEaw4UgQbFn/ZR+gab4ZsH2jcAGwGTsrq/0aAdegz8=</t>
         </is>
       </c>
     </row>
@@ -10339,12 +10339,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>84Kx+uVk7Z64MPotFtenQA==</t>
+          <t>4+wg+DlVJibuwWky8bPxFw==</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>kzV1kJ6/mrDIrwvx4GKGxb5hLW0vS8g104Q1ZmMvf3A=</t>
+          <t>ojRTxudYHuQXJrFUTVqKlqqtMn2XZWYOPhYaDkewRlI=</t>
         </is>
       </c>
     </row>
@@ -10371,12 +10371,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>29F1vgGcerBkn5PX53qd1A==</t>
+          <t>dS4RIvBh2VTGf89fVWRIfQ==</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nCtPzAuRBrT6Q5XyOTYmGRfoqMs1pY49xSxYshdKc1A=</t>
+          <t>yWP2mhKyjiIE0Q2Ip4ZU+lbtdY+aBLgfEM9+iH/lIt0=</t>
         </is>
       </c>
     </row>
@@ -10403,12 +10403,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>gE+qfKb7ULvxlik9Na6VKA==</t>
+          <t>P/dtJvEH+MkpuZBMy0a+qw==</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>nJvfRHZjQhMu0GVagJn4tCIYefcBj4aWQ9NDr1V6tjQ=</t>
+          <t>TlwfZ037KJeHyuVGMcIE+glN978eHD8OKi8mn3jjGIo=</t>
         </is>
       </c>
     </row>
@@ -10435,12 +10435,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NrKAgh3ICVngwcsf1jcr7A==</t>
+          <t>ZGhk0zgvfh00G+n9eE9Xbg==</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>eyBSlgVeefcIoqNb7iT1D4nohQhz40PZAjnP1p3Cmjs=</t>
+          <t>QEhjEhtnQVYW8vW+N0GFwo7w5Rwjz2sa8WjNkJ4oxqk=</t>
         </is>
       </c>
     </row>
@@ -10467,12 +10467,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Kfw1jJfwwDGpeSRvCfIYew==</t>
+          <t>2MzrKUhjNFblrROzbrTurA==</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>jXDHHvHivKLnc8IqIF++jGXGivjA/cUwSzeVmt+cIuQ=</t>
+          <t>f5QM/wk7P3IdJCji/oPwB3e4pCRNBgtTtkVKhsZ31CE=</t>
         </is>
       </c>
     </row>
@@ -10499,12 +10499,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GnKaZF206/G5zg9uXgxSnw==</t>
+          <t>IT5r49FLOHRJRPqyXTCsVQ==</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>HqgOfN6LItTVyjZpyWhKYj40I1EX6A8bHGLSYfLsCh0=</t>
+          <t>kzwTbukfdrVcy3P4+HOiNM+bQv1L47pZ1iTmrnID7QU=</t>
         </is>
       </c>
     </row>

</xml_diff>